<commit_message>
Add inventory all-collections filter and size total cards
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="497" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5323D696-6BFB-4B6E-9449-7F1BBAEC2495}"/>
+  <xr:revisionPtr revIDLastSave="531" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E6607B1-5AC2-438B-8617-D875BDDB3DD1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$60</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="142">
   <si>
     <t>CODIGO</t>
   </si>
@@ -471,7 +471,10 @@
     <t>GLITEE</t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 12:06  10-04</t>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 16:33  10-04</t>
   </si>
 </sst>
 </file>
@@ -521,7 +524,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -581,11 +584,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -624,6 +638,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4700,7 +4728,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="B2:N60"/>
+  <dimension ref="B2:P62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
@@ -4742,42 +4770,42 @@
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="6">
-        <v>420100</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
+      <c r="B3" s="17">
+        <v>424900</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>11</v>
       </c>
       <c r="E3" s="1"/>
-      <c r="F3" s="4">
-        <v>40</v>
-      </c>
-      <c r="G3" s="4">
-        <v>50</v>
-      </c>
-      <c r="H3" s="4">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4">
-        <v>48</v>
-      </c>
-      <c r="J3" s="4">
-        <v>28</v>
-      </c>
-      <c r="K3" s="4">
-        <v>14</v>
-      </c>
-      <c r="L3" s="1">
+      <c r="F3" s="15">
+        <v>36</v>
+      </c>
+      <c r="G3" s="15">
+        <v>76</v>
+      </c>
+      <c r="H3" s="1">
+        <v>70</v>
+      </c>
+      <c r="I3" s="15">
+        <v>78</v>
+      </c>
+      <c r="J3" s="15">
+        <v>58</v>
+      </c>
+      <c r="K3" s="15">
+        <v>38</v>
+      </c>
+      <c r="L3" s="14">
         <f>SUM(F3:K3)</f>
-        <v>267</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>420600</v>
+        <v>420100</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -4787,305 +4815,305 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G4" s="4">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="H4" s="4">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="I4" s="4">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="J4" s="4">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="K4" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>176</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
-        <v>423000</v>
+        <v>420600</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G5" s="4">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H5" s="4">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4">
         <v>26</v>
       </c>
       <c r="J5" s="4">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="K5" s="4">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
-        <v>422500</v>
+        <v>423000</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="4">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G6" s="4">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H6" s="4">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="I6" s="4">
+        <v>26</v>
+      </c>
+      <c r="J6" s="4">
         <v>39</v>
       </c>
-      <c r="J6" s="4">
-        <v>30</v>
-      </c>
-      <c r="K6" s="4"/>
+      <c r="K6" s="4">
+        <v>28</v>
+      </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="N6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>422800</v>
+        <v>422500</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G7" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H7" s="4">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="I7" s="4">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="J7" s="4">
-        <v>39</v>
-      </c>
-      <c r="K7" s="4">
-        <v>8</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="K7" s="4"/>
       <c r="L7" s="1">
         <f>SUM(F7:K7)</f>
-        <v>156</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>424400</v>
+        <v>422800</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="4">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="G8" s="4">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="H8" s="4">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="I8" s="4">
+        <v>27</v>
+      </c>
+      <c r="J8" s="4">
         <v>39</v>
       </c>
-      <c r="J8" s="4">
-        <v>9</v>
-      </c>
       <c r="K8" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L8" s="1">
         <f>SUM(F8:K8)</f>
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>424701</v>
+        <v>424400</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G9" s="4">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="H9" s="4">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I9" s="4">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="J9" s="4">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="K9" s="4">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="L9" s="1">
         <f>SUM(F9:K9)</f>
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N9" s="11"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
-        <v>422100</v>
+        <v>424701</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G10" s="4">
+        <v>16</v>
+      </c>
+      <c r="H10" s="4">
         <v>29</v>
       </c>
-      <c r="H10" s="4">
-        <v>30</v>
-      </c>
       <c r="I10" s="4">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="J10" s="4">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="K10" s="4">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="L10" s="1">
         <f>SUM(F10:K10)</f>
-        <v>141</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>422300</v>
+        <v>422100</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G11" s="4">
+        <v>29</v>
+      </c>
+      <c r="H11" s="4">
+        <v>30</v>
+      </c>
+      <c r="I11" s="4">
         <v>27</v>
       </c>
-      <c r="H11" s="4">
-        <v>18</v>
-      </c>
-      <c r="I11" s="4">
-        <v>26</v>
-      </c>
       <c r="J11" s="4">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K11" s="4">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(F11:K11)</f>
-        <v>122</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>424600</v>
+        <v>422300</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G12" s="4">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I12" s="4">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="J12" s="4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K12" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L12" s="1">
         <f>SUM(F12:K12)</f>
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>423308</v>
+        <v>424600</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
@@ -5095,63 +5123,65 @@
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" s="4">
+        <v>19</v>
+      </c>
+      <c r="H13" s="4">
+        <v>43</v>
+      </c>
+      <c r="I13" s="4">
+        <v>18</v>
+      </c>
+      <c r="J13" s="4">
         <v>24</v>
       </c>
-      <c r="H13" s="4">
-        <v>22</v>
-      </c>
-      <c r="I13" s="4">
-        <v>20</v>
-      </c>
-      <c r="J13" s="4">
-        <v>27</v>
-      </c>
       <c r="K13" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L13" s="1">
         <f>SUM(F13:K13)</f>
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
-        <v>421800</v>
+        <v>423308</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="4"/>
+      <c r="F14" s="4">
+        <v>9</v>
+      </c>
       <c r="G14" s="4">
+        <v>24</v>
+      </c>
+      <c r="H14" s="4">
+        <v>22</v>
+      </c>
+      <c r="I14" s="4">
+        <v>20</v>
+      </c>
+      <c r="J14" s="4">
         <v>27</v>
       </c>
-      <c r="H14" s="4">
-        <v>24</v>
-      </c>
-      <c r="I14" s="4">
-        <v>24</v>
-      </c>
-      <c r="J14" s="4">
-        <v>15</v>
-      </c>
       <c r="K14" s="4">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L14" s="1">
         <f>SUM(F14:K14)</f>
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
-        <v>423900</v>
+        <v>421800</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
@@ -5160,66 +5190,64 @@
         <v>6</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="4">
-        <v>14</v>
-      </c>
+      <c r="F15" s="4"/>
       <c r="G15" s="4">
+        <v>27</v>
+      </c>
+      <c r="H15" s="4">
+        <v>24</v>
+      </c>
+      <c r="I15" s="4">
+        <v>24</v>
+      </c>
+      <c r="J15" s="4">
         <v>15</v>
       </c>
-      <c r="H15" s="4">
-        <v>17</v>
-      </c>
-      <c r="I15" s="4">
-        <v>18</v>
-      </c>
-      <c r="J15" s="4">
-        <v>18</v>
-      </c>
       <c r="K15" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L15" s="1">
         <f>SUM(F15:K15)</f>
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>421400</v>
+        <v>423900</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G16" s="4">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H16" s="4">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I16" s="4">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="J16" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K16" s="4">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="L16" s="1">
         <f>SUM(F16:K16)</f>
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423200</v>
+        <v>421400</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
@@ -5229,31 +5257,31 @@
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G17" s="4">
+        <v>5</v>
+      </c>
+      <c r="H17" s="4">
+        <v>7</v>
+      </c>
+      <c r="I17" s="4">
         <v>10</v>
       </c>
-      <c r="H17" s="4">
+      <c r="J17" s="4">
         <v>17</v>
       </c>
-      <c r="I17" s="4">
-        <v>14</v>
-      </c>
-      <c r="J17" s="4">
-        <v>12</v>
-      </c>
       <c r="K17" s="4">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="L17" s="1">
         <f>SUM(F17:K17)</f>
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>421300</v>
+        <v>423200</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
@@ -5263,22 +5291,22 @@
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
+        <v>13</v>
+      </c>
+      <c r="G18" s="4">
         <v>10</v>
       </c>
-      <c r="G18" s="4">
-        <v>18</v>
-      </c>
       <c r="H18" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I18" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J18" s="4">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K18" s="4">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="L18" s="1">
         <f>SUM(F18:K18)</f>
@@ -5287,164 +5315,164 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>420400</v>
+        <v>421300</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G19" s="4">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H19" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I19" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J19" s="4">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K19" s="4">
         <v>11</v>
       </c>
       <c r="L19" s="1">
         <f>SUM(F19:K19)</f>
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="6">
-        <v>423408</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
+      <c r="B20" s="17">
+        <v>423348</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>13</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4">
-        <v>32</v>
-      </c>
-      <c r="H20" s="4">
-        <v>18</v>
-      </c>
-      <c r="I20" s="4">
-        <v>18</v>
-      </c>
-      <c r="J20" s="4">
-        <v>13</v>
-      </c>
-      <c r="K20" s="4"/>
+      <c r="F20" s="15">
+        <v>9</v>
+      </c>
+      <c r="G20" s="15">
+        <v>14</v>
+      </c>
+      <c r="H20" s="1">
+        <v>14</v>
+      </c>
+      <c r="I20" s="15">
+        <v>10</v>
+      </c>
+      <c r="J20" s="15">
+        <v>8</v>
+      </c>
+      <c r="K20" s="15">
+        <v>6</v>
+      </c>
       <c r="L20" s="1">
         <f>SUM(F20:K20)</f>
-        <v>81</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>422700</v>
+        <v>420400</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="G21" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H21" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I21" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J21" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K21" s="4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L21" s="1">
         <f>SUM(F21:K21)</f>
-        <v>36</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>423304</v>
+        <v>423408</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="4">
-        <v>10</v>
-      </c>
+      <c r="F22" s="4"/>
       <c r="G22" s="4">
-        <v>16</v>
-      </c>
-      <c r="H22" s="6">
-        <v>17</v>
+        <v>32</v>
+      </c>
+      <c r="H22" s="4">
+        <v>18</v>
       </c>
       <c r="I22" s="4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J22" s="4">
         <v>13</v>
       </c>
-      <c r="K22" s="4">
-        <v>7</v>
-      </c>
+      <c r="K22" s="4"/>
       <c r="L22" s="1">
         <f>SUM(F22:K22)</f>
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>421100</v>
+        <v>423304</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="4">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G23" s="4">
-        <v>10</v>
-      </c>
-      <c r="H23" s="4">
+        <v>16</v>
+      </c>
+      <c r="H23" s="6">
+        <v>17</v>
+      </c>
+      <c r="I23" s="4">
+        <v>12</v>
+      </c>
+      <c r="J23" s="4">
         <v>13</v>
       </c>
-      <c r="I23" s="4">
-        <v>13</v>
-      </c>
-      <c r="J23" s="4">
-        <v>23</v>
-      </c>
       <c r="K23" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L23" s="1">
         <f>SUM(F23:K23)</f>
@@ -5453,132 +5481,132 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>422000</v>
+        <v>421100</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="4">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="G24" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H24" s="4">
         <v>13</v>
       </c>
       <c r="I24" s="4">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="J24" s="4">
-        <v>5</v>
-      </c>
-      <c r="K24" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="K24" s="4">
+        <v>9</v>
+      </c>
       <c r="L24" s="1">
         <f>SUM(F24:K24)</f>
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>423416</v>
+        <v>422000</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="4">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="G25" s="4">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H25" s="4">
         <v>13</v>
       </c>
       <c r="I25" s="4">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="J25" s="4">
-        <v>9</v>
-      </c>
-      <c r="K25" s="4">
-        <v>5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K25" s="4"/>
       <c r="L25" s="1">
         <f>SUM(F25:K25)</f>
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>423316</v>
+        <v>423416</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G26" s="4">
         <v>14</v>
       </c>
       <c r="H26" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I26" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J26" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K26" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26" s="1">
         <f>SUM(F26:K26)</f>
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>420101</v>
+        <v>423316</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G27" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H27" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I27" s="4">
         <v>13</v>
       </c>
       <c r="J27" s="4">
+        <v>8</v>
+      </c>
+      <c r="K27" s="4">
         <v>4</v>
-      </c>
-      <c r="K27" s="4">
-        <v>5</v>
       </c>
       <c r="L27" s="1">
         <f>SUM(F27:K27)</f>
@@ -5587,7 +5615,7 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>420160</v>
+        <v>420101</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
@@ -5595,191 +5623,197 @@
       <c r="D28" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G28" s="4">
         <v>15</v>
       </c>
       <c r="H28" s="4">
+        <v>15</v>
+      </c>
+      <c r="I28" s="4">
         <v>13</v>
       </c>
-      <c r="I28" s="4">
-        <v>12</v>
-      </c>
       <c r="J28" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K28" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L28" s="1">
         <f>SUM(F28:K28)</f>
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>423404</v>
+        <v>420160</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E29" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F29" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G29" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H29" s="4">
         <v>13</v>
       </c>
       <c r="I29" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J29" s="4">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="K29" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L29" s="1">
         <f>SUM(F29:K29)</f>
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>422101</v>
+        <v>423404</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="G30" s="4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H30" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I30" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J30" s="4">
-        <v>14</v>
-      </c>
-      <c r="K30" s="4"/>
+        <v>11</v>
+      </c>
+      <c r="K30" s="4">
+        <v>4</v>
+      </c>
       <c r="L30" s="1">
         <f>SUM(F30:K30)</f>
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>422200</v>
+        <v>422101</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="4">
-        <v>1</v>
-      </c>
-      <c r="G31" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1</v>
+      </c>
       <c r="H31" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I31" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J31" s="4">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="K31" s="4"/>
       <c r="L31" s="1">
         <f>SUM(F31:K31)</f>
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>424700</v>
+        <v>422200</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="4">
-        <v>19</v>
-      </c>
-      <c r="G32" s="4">
-        <v>8</v>
-      </c>
-      <c r="H32" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4">
+        <v>16</v>
+      </c>
       <c r="I32" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J32" s="4">
-        <v>1</v>
-      </c>
-      <c r="K32" s="4">
-        <v>10</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="K32" s="4"/>
       <c r="L32" s="1">
         <f>SUM(F32:K32)</f>
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>423501</v>
+        <v>424700</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>18</v>
-      </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4">
-        <v>2</v>
-      </c>
-      <c r="I33" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="G33" s="4">
+        <v>8</v>
+      </c>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4">
+        <v>9</v>
+      </c>
       <c r="J33" s="4">
-        <v>23</v>
-      </c>
-      <c r="K33" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K33" s="4">
+        <v>10</v>
+      </c>
       <c r="L33" s="1">
         <f>SUM(F33:K33)</f>
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>424000</v>
+        <v>423501</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
@@ -5789,245 +5823,239 @@
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I34" s="4"/>
       <c r="J34" s="4">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="1">
         <f>SUM(F34:K34)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>421801</v>
+        <v>424000</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E35" s="1"/>
-      <c r="F35" s="4"/>
+      <c r="F35" s="4">
+        <v>23</v>
+      </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4">
-        <v>6</v>
-      </c>
-      <c r="I35" s="4">
-        <v>6</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I35" s="4"/>
       <c r="J35" s="4">
-        <v>18</v>
-      </c>
-      <c r="K35" s="4">
-        <v>10</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="K35" s="4"/>
       <c r="L35" s="1">
         <f>SUM(F35:K35)</f>
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>422900</v>
+        <v>421801</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4">
+        <v>6</v>
+      </c>
+      <c r="I36" s="4">
+        <v>6</v>
+      </c>
+      <c r="J36" s="4">
+        <v>18</v>
+      </c>
+      <c r="K36" s="4">
         <v>10</v>
       </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="4">
-        <v>34</v>
-      </c>
-      <c r="G36" s="4">
-        <v>1</v>
-      </c>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4">
-        <v>2</v>
-      </c>
-      <c r="K36" s="4"/>
       <c r="L36" s="1">
         <f>SUM(F36:K36)</f>
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>424960</v>
-      </c>
-      <c r="C37" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>11</v>
+        <v>422900</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E37" s="1"/>
-      <c r="F37" s="15">
+      <c r="F37" s="4">
+        <v>34</v>
+      </c>
+      <c r="G37" s="4">
+        <v>1</v>
+      </c>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4">
         <v>2</v>
       </c>
-      <c r="G37" s="15">
-        <v>1</v>
-      </c>
-      <c r="H37" s="6">
-        <v>0</v>
-      </c>
-      <c r="I37" s="15">
-        <v>0</v>
-      </c>
-      <c r="J37" s="15">
-        <v>1</v>
-      </c>
-      <c r="K37" s="15">
-        <v>1</v>
-      </c>
-      <c r="L37" s="16">
+      <c r="K37" s="4"/>
+      <c r="L37" s="1">
         <f>SUM(F37:K37)</f>
-        <v>5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>421900</v>
+        <v>422700</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G38" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H38" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I38" s="4">
+        <v>0</v>
+      </c>
+      <c r="J38" s="4">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4">
         <v>4</v>
       </c>
-      <c r="J38" s="4">
-        <v>9</v>
-      </c>
-      <c r="K38" s="4"/>
       <c r="L38" s="1">
         <f>SUM(F38:K38)</f>
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>422701</v>
+        <v>421900</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="4">
-        <v>26</v>
-      </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G39" s="4">
+        <v>8</v>
+      </c>
+      <c r="H39" s="4">
+        <v>9</v>
+      </c>
+      <c r="I39" s="4">
+        <v>4</v>
+      </c>
       <c r="J39" s="4">
-        <v>3</v>
-      </c>
-      <c r="K39" s="4">
-        <v>1</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K39" s="4"/>
       <c r="L39" s="1">
         <f>SUM(F39:K39)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>421901</v>
+        <v>422701</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>4</v>
-      </c>
-      <c r="G40" s="4">
-        <v>8</v>
-      </c>
-      <c r="H40" s="4">
-        <v>6</v>
-      </c>
-      <c r="I40" s="4">
-        <v>5</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
       <c r="J40" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K40" s="4">
         <v>1</v>
       </c>
       <c r="L40" s="1">
         <f>SUM(F40:K40)</f>
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>421402</v>
+        <v>421901</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G41" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H41" s="4">
+        <v>6</v>
+      </c>
+      <c r="I41" s="4">
+        <v>5</v>
+      </c>
+      <c r="J41" s="4">
         <v>4</v>
       </c>
-      <c r="I41" s="4">
-        <v>7</v>
-      </c>
-      <c r="J41" s="4">
-        <v>5</v>
-      </c>
       <c r="K41" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L41" s="1">
         <f>SUM(F41:K41)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>421301</v>
+        <v>421402</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
@@ -6037,49 +6065,53 @@
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="4">
+        <v>1</v>
+      </c>
+      <c r="G42" s="4">
+        <v>6</v>
+      </c>
+      <c r="H42" s="4">
         <v>4</v>
       </c>
-      <c r="G42" s="4">
-        <v>2</v>
-      </c>
-      <c r="H42" s="4">
-        <v>9</v>
-      </c>
       <c r="I42" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J42" s="4">
-        <v>6</v>
-      </c>
-      <c r="K42" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="K42" s="4">
+        <v>4</v>
+      </c>
       <c r="L42" s="1">
         <f>SUM(F42:K42)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>424500</v>
+        <v>421301</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="4">
-        <v>7</v>
-      </c>
-      <c r="G43" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="G43" s="4">
+        <v>2</v>
+      </c>
       <c r="H43" s="4">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I43" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J43" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
@@ -6089,33 +6121,29 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>421401</v>
+        <v>424500</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="4">
-        <v>1</v>
-      </c>
-      <c r="G44" s="4">
-        <v>7</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G44" s="4"/>
       <c r="H44" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I44" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J44" s="4">
-        <v>2</v>
-      </c>
-      <c r="K44" s="4">
-        <v>1</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K44" s="4"/>
       <c r="L44" s="1">
         <f>SUM(F44:K44)</f>
         <v>26</v>
@@ -6123,97 +6151,103 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>421902</v>
+        <v>421401</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4">
+        <v>1</v>
+      </c>
+      <c r="G45" s="4">
+        <v>7</v>
+      </c>
+      <c r="H45" s="4">
+        <v>10</v>
+      </c>
+      <c r="I45" s="4">
+        <v>5</v>
+      </c>
+      <c r="J45" s="4">
         <v>2</v>
       </c>
-      <c r="G45" s="4">
-        <v>6</v>
-      </c>
-      <c r="H45" s="4">
-        <v>6</v>
-      </c>
-      <c r="I45" s="4">
-        <v>5</v>
-      </c>
-      <c r="J45" s="4">
-        <v>4</v>
-      </c>
       <c r="K45" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L45" s="1">
         <f>SUM(F45:K45)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>422190</v>
+        <v>421902</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>139</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E46" s="1"/>
       <c r="F46" s="4">
         <v>2</v>
       </c>
       <c r="G46" s="4">
-        <v>5</v>
-      </c>
-      <c r="H46" s="6">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="H46" s="4">
+        <v>6</v>
       </c>
       <c r="I46" s="4">
         <v>5</v>
       </c>
       <c r="J46" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K46" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L46" s="1">
         <f>SUM(F46:K46)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>424801</v>
+        <v>422190</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="F47" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G47" s="4">
-        <v>10</v>
-      </c>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="H47" s="6">
+        <v>5</v>
+      </c>
+      <c r="I47" s="4">
+        <v>5</v>
+      </c>
       <c r="J47" s="4">
-        <v>9</v>
-      </c>
-      <c r="K47" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K47" s="4">
+        <v>3</v>
+      </c>
       <c r="L47" s="1">
         <f>SUM(F47:K47)</f>
         <v>23</v>
@@ -6221,127 +6255,127 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>423409</v>
+        <v>424801</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G48" s="4">
-        <v>4</v>
-      </c>
-      <c r="H48" s="4">
-        <v>5</v>
-      </c>
-      <c r="I48" s="4">
-        <v>1</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
       <c r="J48" s="4">
-        <v>3</v>
-      </c>
-      <c r="K48" s="4">
-        <v>2</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K48" s="4"/>
       <c r="L48" s="1">
         <f>SUM(F48:K48)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>420900</v>
+        <v>423409</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E49" s="1"/>
-      <c r="F49" s="4"/>
+      <c r="F49" s="4">
+        <v>5</v>
+      </c>
       <c r="G49" s="4">
-        <v>6</v>
-      </c>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="H49" s="4">
+        <v>5</v>
+      </c>
+      <c r="I49" s="4">
+        <v>1</v>
+      </c>
       <c r="J49" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K49" s="4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L49" s="1">
         <f>SUM(F49:K49)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>420501</v>
+        <v>420900</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4">
-        <v>4</v>
-      </c>
-      <c r="H50" s="4">
-        <v>3</v>
-      </c>
-      <c r="I50" s="4">
-        <v>4</v>
-      </c>
-      <c r="J50" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4">
+        <v>5</v>
+      </c>
       <c r="K50" s="4">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L50" s="1">
         <f>SUM(F50:K50)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>424300</v>
+        <v>420501</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="4">
-        <v>8</v>
-      </c>
-      <c r="G51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4">
+        <v>4</v>
+      </c>
       <c r="H51" s="4">
-        <v>1</v>
-      </c>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4">
-        <v>7</v>
-      </c>
-      <c r="K51" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="I51" s="4">
+        <v>4</v>
+      </c>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4">
+        <v>5</v>
+      </c>
       <c r="L51" s="1">
         <f>SUM(F51:K51)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>423500</v>
+        <v>424300</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
@@ -6351,204 +6385,269 @@
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
-        <v>1</v>
-      </c>
-      <c r="G52" s="4">
-        <v>3</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G52" s="4"/>
       <c r="H52" s="4">
-        <v>0</v>
-      </c>
-      <c r="I52" s="4">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I52" s="4"/>
       <c r="J52" s="4">
-        <v>1</v>
-      </c>
-      <c r="K52" s="4">
-        <v>5</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K52" s="4"/>
       <c r="L52" s="1">
         <f>SUM(F52:K52)</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>422601</v>
+        <v>423500</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="4">
-        <v>5</v>
-      </c>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G53" s="4">
+        <v>3</v>
+      </c>
+      <c r="H53" s="4">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4">
+        <v>2</v>
+      </c>
       <c r="J53" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K53" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L53" s="1">
         <f>SUM(F53:K53)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B54" s="6">
+        <v>422601</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B54" s="6">
-        <v>423600</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="E54" s="1"/>
       <c r="F54" s="4">
-        <v>1</v>
-      </c>
-      <c r="G54" s="4">
+        <v>5</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4">
         <v>4</v>
       </c>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4">
-        <v>3</v>
-      </c>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
+      <c r="K54" s="4">
+        <v>1</v>
+      </c>
       <c r="L54" s="1">
         <f>SUM(F54:K54)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>420402</v>
+        <v>423600</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
+      <c r="F55" s="4">
+        <v>1</v>
+      </c>
+      <c r="G55" s="4">
+        <v>4</v>
+      </c>
       <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="4">
-        <v>6</v>
-      </c>
+      <c r="I55" s="4">
+        <v>3</v>
+      </c>
+      <c r="J55" s="4"/>
       <c r="K55" s="4"/>
       <c r="L55" s="1">
         <f>SUM(F55:K55)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>420160</v>
+        <v>420402</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F56" s="4">
-        <v>1</v>
-      </c>
-      <c r="G56" s="4">
-        <v>1</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="E56" s="1"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
       <c r="H56" s="4"/>
-      <c r="I56" s="4">
-        <v>1</v>
-      </c>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4">
-        <v>2</v>
-      </c>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4">
+        <v>6</v>
+      </c>
+      <c r="K56" s="4"/>
       <c r="L56" s="1">
         <f>SUM(F56:K56)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>423309</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>13</v>
+        <v>424960</v>
+      </c>
+      <c r="C57" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>11</v>
       </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4">
-        <v>1</v>
-      </c>
-      <c r="H57" s="4">
-        <v>1</v>
-      </c>
-      <c r="I57" s="4">
-        <v>1</v>
-      </c>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="L57" s="1">
+      <c r="F57" s="15">
+        <v>2</v>
+      </c>
+      <c r="G57" s="15">
+        <v>1</v>
+      </c>
+      <c r="H57" s="6">
+        <v>0</v>
+      </c>
+      <c r="I57" s="15">
+        <v>0</v>
+      </c>
+      <c r="J57" s="15">
+        <v>1</v>
+      </c>
+      <c r="K57" s="15">
+        <v>1</v>
+      </c>
+      <c r="L57" s="16">
         <f>SUM(F57:K57)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>420200</v>
+        <v>420160</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E58" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="F58" s="4">
-        <v>2</v>
-      </c>
-      <c r="G58" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G58" s="4">
+        <v>1</v>
+      </c>
       <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
+      <c r="I58" s="4">
+        <v>1</v>
+      </c>
       <c r="J58" s="4"/>
       <c r="K58" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L58" s="1">
         <f>SUM(F58:K58)</f>
+        <v>5</v>
+      </c>
+      <c r="P58" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B59" s="6">
+        <v>423309</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" s="1"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4">
+        <v>1</v>
+      </c>
+      <c r="H59" s="4">
+        <v>1</v>
+      </c>
+      <c r="I59" s="4">
+        <v>1</v>
+      </c>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+      <c r="L59" s="1">
+        <f>SUM(F59:K59)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="L60" s="10">
-        <f>SUM(L3:L58)</f>
-        <v>3597</v>
+    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B60" s="18">
+        <v>420200</v>
+      </c>
+      <c r="C60" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="20"/>
+      <c r="F60" s="21">
+        <v>2</v>
+      </c>
+      <c r="G60" s="21"/>
+      <c r="H60" s="22"/>
+      <c r="I60" s="21"/>
+      <c r="J60" s="21"/>
+      <c r="K60" s="21">
+        <v>1</v>
+      </c>
+      <c r="L60" s="19">
+        <f>SUM(F60:K60)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="L62" s="10">
+        <f>SUM(L3:L60)</f>
+        <v>4014</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L58" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L58">
-      <sortCondition descending="1" ref="L2:L57"/>
+  <autoFilter ref="B2:L60" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L60">
+      <sortCondition descending="1" ref="L2:L58"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refresh inventory stock from updated workbook and rebuild static site
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="531" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E6607B1-5AC2-438B-8617-D875BDDB3DD1}"/>
+  <xr:revisionPtr revIDLastSave="539" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCDE57F3-53F6-4989-9990-1BCF35609C49}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -599,7 +599,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -628,31 +628,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,10 +660,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -999,19 +987,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
@@ -1798,19 +1786,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2405,19 +2393,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2772,19 +2760,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4365,19 +4353,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4770,36 +4758,36 @@
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="17">
+      <c r="B3" s="6">
         <v>424900</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1"/>
-      <c r="F3" s="15">
+      <c r="F3" s="4">
         <v>36</v>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="4">
         <v>76</v>
       </c>
       <c r="H3" s="1">
         <v>70</v>
       </c>
-      <c r="I3" s="15">
+      <c r="I3" s="4">
         <v>78</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="4">
         <v>58</v>
       </c>
-      <c r="K3" s="15">
+      <c r="K3" s="4">
         <v>38</v>
       </c>
-      <c r="L3" s="14">
-        <f>SUM(F3:K3)</f>
+      <c r="L3" s="1">
+        <f t="shared" ref="L3:L34" si="0">SUM(F3:K3)</f>
         <v>356</v>
       </c>
     </row>
@@ -4833,7 +4821,7 @@
         <v>14</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>267</v>
       </c>
     </row>
@@ -4867,7 +4855,7 @@
         <v>18</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
+        <f t="shared" si="0"/>
         <v>176</v>
       </c>
     </row>
@@ -4901,7 +4889,7 @@
         <v>28</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
+        <f t="shared" si="0"/>
         <v>173</v>
       </c>
       <c r="N6" t="s">
@@ -4936,7 +4924,7 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
+        <f t="shared" si="0"/>
         <v>171</v>
       </c>
     </row>
@@ -4970,7 +4958,7 @@
         <v>8</v>
       </c>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
+        <f t="shared" si="0"/>
         <v>156</v>
       </c>
     </row>
@@ -5004,7 +4992,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
+        <f t="shared" si="0"/>
         <v>153</v>
       </c>
       <c r="N9" s="11"/>
@@ -5039,7 +5027,7 @@
         <v>56</v>
       </c>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>150</v>
       </c>
     </row>
@@ -5073,7 +5061,7 @@
         <v>23</v>
       </c>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
+        <f t="shared" si="0"/>
         <v>141</v>
       </c>
     </row>
@@ -5107,7 +5095,7 @@
         <v>5</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
+        <f t="shared" si="0"/>
         <v>122</v>
       </c>
     </row>
@@ -5141,7 +5129,7 @@
         <v>7</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
+        <f t="shared" si="0"/>
         <v>119</v>
       </c>
     </row>
@@ -5175,7 +5163,7 @@
         <v>8</v>
       </c>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
+        <f t="shared" si="0"/>
         <v>110</v>
       </c>
     </row>
@@ -5207,7 +5195,7 @@
         <v>11</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
+        <f t="shared" si="0"/>
         <v>101</v>
       </c>
     </row>
@@ -5241,7 +5229,7 @@
         <v>9</v>
       </c>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
+        <f t="shared" si="0"/>
         <v>91</v>
       </c>
     </row>
@@ -5275,7 +5263,7 @@
         <v>38</v>
       </c>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
+        <f t="shared" si="0"/>
         <v>88</v>
       </c>
     </row>
@@ -5309,7 +5297,7 @@
         <v>19</v>
       </c>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
+        <f t="shared" si="0"/>
         <v>85</v>
       </c>
     </row>
@@ -5343,42 +5331,42 @@
         <v>11</v>
       </c>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
+        <f t="shared" si="0"/>
         <v>85</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="17">
+      <c r="B20" s="6">
         <v>423348</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="15">
-        <v>9</v>
-      </c>
-      <c r="G20" s="15">
-        <v>14</v>
+      <c r="F20" s="4">
+        <v>5</v>
+      </c>
+      <c r="G20" s="4">
+        <v>10</v>
       </c>
       <c r="H20" s="1">
-        <v>14</v>
-      </c>
-      <c r="I20" s="15">
-        <v>10</v>
-      </c>
-      <c r="J20" s="15">
-        <v>8</v>
-      </c>
-      <c r="K20" s="15">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="I20" s="4">
+        <v>7</v>
+      </c>
+      <c r="J20" s="4">
+        <v>5</v>
+      </c>
+      <c r="K20" s="4">
+        <v>3</v>
       </c>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
-        <v>61</v>
+        <f t="shared" si="0"/>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
@@ -5411,7 +5399,7 @@
         <v>11</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
+        <f t="shared" si="0"/>
         <v>82</v>
       </c>
     </row>
@@ -5441,7 +5429,7 @@
       </c>
       <c r="K22" s="4"/>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
+        <f t="shared" si="0"/>
         <v>81</v>
       </c>
     </row>
@@ -5475,7 +5463,7 @@
         <v>7</v>
       </c>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
+        <f t="shared" si="0"/>
         <v>75</v>
       </c>
     </row>
@@ -5509,7 +5497,7 @@
         <v>9</v>
       </c>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
+        <f t="shared" si="0"/>
         <v>75</v>
       </c>
     </row>
@@ -5541,7 +5529,7 @@
       </c>
       <c r="K25" s="4"/>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
+        <f t="shared" si="0"/>
         <v>69</v>
       </c>
     </row>
@@ -5575,7 +5563,7 @@
         <v>5</v>
       </c>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
+        <f t="shared" si="0"/>
         <v>62</v>
       </c>
     </row>
@@ -5609,7 +5597,7 @@
         <v>4</v>
       </c>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
     </row>
@@ -5643,7 +5631,7 @@
         <v>5</v>
       </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
     </row>
@@ -5679,7 +5667,7 @@
         <v>1</v>
       </c>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
+        <f t="shared" si="0"/>
         <v>57</v>
       </c>
     </row>
@@ -5713,7 +5701,7 @@
         <v>4</v>
       </c>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
     </row>
@@ -5745,7 +5733,7 @@
       </c>
       <c r="K31" s="4"/>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
@@ -5775,7 +5763,7 @@
       </c>
       <c r="K32" s="4"/>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
     </row>
@@ -5807,7 +5795,7 @@
         <v>10</v>
       </c>
       <c r="L33" s="1">
-        <f>SUM(F33:K33)</f>
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
     </row>
@@ -5835,7 +5823,7 @@
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
+        <f t="shared" si="0"/>
         <v>43</v>
       </c>
     </row>
@@ -5863,7 +5851,7 @@
       </c>
       <c r="K35" s="4"/>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" ref="L35:L66" si="1">SUM(F35:K35)</f>
         <v>42</v>
       </c>
     </row>
@@ -5893,7 +5881,7 @@
         <v>10</v>
       </c>
       <c r="L36" s="1">
-        <f>SUM(F36:K36)</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
     </row>
@@ -5921,7 +5909,7 @@
       </c>
       <c r="K37" s="4"/>
       <c r="L37" s="1">
-        <f>SUM(F37:K37)</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
     </row>
@@ -5955,7 +5943,7 @@
         <v>4</v>
       </c>
       <c r="L38" s="1">
-        <f>SUM(F38:K38)</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
     </row>
@@ -5987,7 +5975,7 @@
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="1">
-        <f>SUM(F39:K39)</f>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
     </row>
@@ -6015,7 +6003,7 @@
         <v>1</v>
       </c>
       <c r="L40" s="1">
-        <f>SUM(F40:K40)</f>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
     </row>
@@ -6049,7 +6037,7 @@
         <v>1</v>
       </c>
       <c r="L41" s="1">
-        <f>SUM(F41:K41)</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
     </row>
@@ -6083,7 +6071,7 @@
         <v>4</v>
       </c>
       <c r="L42" s="1">
-        <f>SUM(F42:K42)</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
     </row>
@@ -6115,7 +6103,7 @@
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f>SUM(F43:K43)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
@@ -6145,7 +6133,7 @@
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="1">
-        <f>SUM(F44:K44)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
@@ -6179,7 +6167,7 @@
         <v>1</v>
       </c>
       <c r="L45" s="1">
-        <f>SUM(F45:K45)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
@@ -6213,7 +6201,7 @@
         <v>2</v>
       </c>
       <c r="L46" s="1">
-        <f>SUM(F46:K46)</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
     </row>
@@ -6249,7 +6237,7 @@
         <v>3</v>
       </c>
       <c r="L47" s="1">
-        <f>SUM(F47:K47)</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
     </row>
@@ -6277,7 +6265,7 @@
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f>SUM(F48:K48)</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
     </row>
@@ -6311,7 +6299,7 @@
         <v>2</v>
       </c>
       <c r="L49" s="1">
-        <f>SUM(F49:K49)</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
     </row>
@@ -6339,7 +6327,7 @@
         <v>9</v>
       </c>
       <c r="L50" s="1">
-        <f>SUM(F50:K50)</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
     </row>
@@ -6369,7 +6357,7 @@
         <v>5</v>
       </c>
       <c r="L51" s="1">
-        <f>SUM(F51:K51)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
@@ -6397,7 +6385,7 @@
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f>SUM(F52:K52)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
@@ -6431,7 +6419,7 @@
         <v>5</v>
       </c>
       <c r="L53" s="1">
-        <f>SUM(F53:K53)</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
     </row>
@@ -6459,7 +6447,7 @@
         <v>1</v>
       </c>
       <c r="L54" s="1">
-        <f>SUM(F54:K54)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -6487,7 +6475,7 @@
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
       <c r="L55" s="1">
-        <f>SUM(F55:K55)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
@@ -6511,7 +6499,7 @@
       </c>
       <c r="K56" s="4"/>
       <c r="L56" s="1">
-        <f>SUM(F56:K56)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
@@ -6519,33 +6507,33 @@
       <c r="B57" s="6">
         <v>424960</v>
       </c>
-      <c r="C57" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" s="14" t="s">
+      <c r="C57" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="15">
+      <c r="F57" s="4">
         <v>2</v>
       </c>
-      <c r="G57" s="15">
+      <c r="G57" s="4">
         <v>1</v>
       </c>
       <c r="H57" s="6">
         <v>0</v>
       </c>
-      <c r="I57" s="15">
-        <v>0</v>
-      </c>
-      <c r="J57" s="15">
-        <v>1</v>
-      </c>
-      <c r="K57" s="15">
-        <v>1</v>
-      </c>
-      <c r="L57" s="16">
-        <f>SUM(F57:K57)</f>
+      <c r="I57" s="4">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4">
+        <v>1</v>
+      </c>
+      <c r="K57" s="4">
+        <v>1</v>
+      </c>
+      <c r="L57" s="12">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
@@ -6577,7 +6565,7 @@
         <v>2</v>
       </c>
       <c r="L58" s="1">
-        <f>SUM(F58:K58)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="P58" t="s">
@@ -6608,40 +6596,39 @@
       <c r="J59" s="4"/>
       <c r="K59" s="4"/>
       <c r="L59" s="1">
-        <f>SUM(F59:K59)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
     <row r="60" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B60" s="18">
+      <c r="B60" s="13">
         <v>420200</v>
       </c>
-      <c r="C60" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" s="19" t="s">
+      <c r="C60" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E60" s="20"/>
-      <c r="F60" s="21">
+      <c r="F60" s="15">
         <v>2</v>
       </c>
-      <c r="G60" s="21"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="21"/>
-      <c r="J60" s="21"/>
-      <c r="K60" s="21">
-        <v>1</v>
-      </c>
-      <c r="L60" s="19">
-        <f>SUM(F60:K60)</f>
+      <c r="G60" s="15"/>
+      <c r="H60" s="16"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
+      <c r="K60" s="15">
+        <v>1</v>
+      </c>
+      <c r="L60" s="14">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="L62" s="10">
         <f>SUM(L3:L60)</f>
-        <v>4014</v>
+        <v>3993</v>
       </c>
     </row>
   </sheetData>
@@ -6655,6 +6642,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -6798,22 +6800,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6829,28 +6840,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar stock con ultima data y regenerar web
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="539" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCDE57F3-53F6-4989-9990-1BCF35609C49}"/>
+  <xr:revisionPtr revIDLastSave="890" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F36E9BF-DAF1-4427-8C9B-C750825E18ED}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="145">
   <si>
     <t>CODIGO</t>
   </si>
@@ -474,14 +474,23 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 16:33  10-04</t>
+    <t>GRIS</t>
+  </si>
+  <si>
+    <t>negro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 11:14    14-04</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -498,6 +507,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -524,7 +541,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -584,20 +601,10 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -631,22 +638,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -660,6 +666,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
+<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -981,25 +991,59 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{4918944A-690C-4FAF-86C7-D4C8095E14EF}">
+  <we:reference id="WA200005271" version="2.6.1.0" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005271" version="2.6.1.0" store="WA200005271" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_AI_TABLE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_FILL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_LIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_ASK</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_FORMAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_EXTRACT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_TRANSLATE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_AI_CHOICE</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FB535F-634B-4933-81FF-529A98082563}">
   <dimension ref="B2:L31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
@@ -1786,19 +1830,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2393,19 +2437,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2760,19 +2804,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4353,19 +4397,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4716,13 +4760,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="B2:P62"/>
+  <dimension ref="B2:P65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4757,75 +4801,75 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
-        <v>424900</v>
+        <v>420100</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G3" s="4">
-        <v>76</v>
-      </c>
-      <c r="H3" s="1">
-        <v>70</v>
+        <v>47</v>
+      </c>
+      <c r="H3" s="4">
+        <v>84</v>
       </c>
       <c r="I3" s="4">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="J3" s="4">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="K3" s="4">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="L3" s="1">
-        <f t="shared" ref="L3:L34" si="0">SUM(F3:K3)</f>
-        <v>356</v>
-      </c>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+        <f>SUM(F3:K3)</f>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>420100</v>
+        <v>422500</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G4" s="4">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="H4" s="4">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="I4" s="4">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J4" s="4">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="K4" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="L4" s="1">
-        <f t="shared" si="0"/>
-        <v>267</v>
-      </c>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+        <f>SUM(F4:K4)</f>
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
         <v>420600</v>
       </c>
@@ -4855,11 +4899,11 @@
         <v>18</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F5:K5)</f>
         <v>176</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>423000</v>
       </c>
@@ -4889,46 +4933,48 @@
         <v>28</v>
       </c>
       <c r="L6" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F6:K6)</f>
         <v>173</v>
       </c>
       <c r="N6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>422500</v>
+        <v>423501</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="G7" s="4">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="H7" s="4">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="I7" s="4">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="J7" s="4">
-        <v>30</v>
-      </c>
-      <c r="K7" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="K7" s="4">
+        <v>20</v>
+      </c>
       <c r="L7" s="1">
-        <f t="shared" si="0"/>
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+        <f>SUM(F7:K7)</f>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>422800</v>
       </c>
@@ -4958,11 +5004,11 @@
         <v>8</v>
       </c>
       <c r="L8" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F8:K8)</f>
         <v>156</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
         <v>424400</v>
       </c>
@@ -4992,12 +5038,12 @@
         <v>1</v>
       </c>
       <c r="L9" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F9:K9)</f>
         <v>153</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
         <v>424701</v>
       </c>
@@ -5027,11 +5073,11 @@
         <v>56</v>
       </c>
       <c r="L10" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F10:K10)</f>
         <v>150</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>422100</v>
       </c>
@@ -5061,81 +5107,81 @@
         <v>23</v>
       </c>
       <c r="L11" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F11:K11)</f>
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="6">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="15">
+        <v>423448</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1"/>
+      <c r="F12" s="17">
+        <v>12</v>
+      </c>
+      <c r="G12" s="17">
+        <v>20</v>
+      </c>
+      <c r="H12" s="6">
+        <v>19</v>
+      </c>
+      <c r="I12" s="17">
+        <v>15</v>
+      </c>
+      <c r="J12" s="17">
+        <v>13</v>
+      </c>
+      <c r="K12" s="17">
+        <v>5</v>
+      </c>
+      <c r="L12" s="1">
+        <f>SUM(F12:K12)</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="6">
         <v>422300</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="4">
-        <v>25</v>
-      </c>
-      <c r="G12" s="4">
-        <v>27</v>
-      </c>
-      <c r="H12" s="4">
-        <v>18</v>
-      </c>
-      <c r="I12" s="4">
-        <v>26</v>
-      </c>
-      <c r="J12" s="4">
-        <v>21</v>
-      </c>
-      <c r="K12" s="4">
-        <v>5</v>
-      </c>
-      <c r="L12" s="1">
-        <f t="shared" si="0"/>
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="6">
-        <v>424600</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G13" s="4">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H13" s="4">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I13" s="4">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="J13" s="4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K13" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="0"/>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+        <f>SUM(F13:K13)</f>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
-        <v>423308</v>
+        <v>424600</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
@@ -5145,63 +5191,66 @@
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G14" s="4">
+        <v>19</v>
+      </c>
+      <c r="H14" s="4">
+        <v>43</v>
+      </c>
+      <c r="I14" s="4">
+        <v>18</v>
+      </c>
+      <c r="J14" s="4">
         <v>24</v>
       </c>
-      <c r="H14" s="4">
+      <c r="K14" s="4">
+        <v>7</v>
+      </c>
+      <c r="L14" s="1">
+        <f>SUM(F14:K14)</f>
+        <v>119</v>
+      </c>
+      <c r="O14" s="18"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" s="6">
+        <v>423308</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="4">
+        <v>8</v>
+      </c>
+      <c r="G15" s="4">
         <v>22</v>
       </c>
-      <c r="I14" s="4">
-        <v>20</v>
-      </c>
-      <c r="J14" s="4">
-        <v>27</v>
-      </c>
-      <c r="K14" s="4">
+      <c r="H15" s="4">
+        <v>19</v>
+      </c>
+      <c r="I15" s="4">
+        <v>18</v>
+      </c>
+      <c r="J15" s="4">
+        <v>26</v>
+      </c>
+      <c r="K15" s="4">
         <v>8</v>
       </c>
-      <c r="L14" s="1">
-        <f t="shared" si="0"/>
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="6">
+      <c r="L15" s="1">
+        <f>SUM(F15:K15)</f>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" s="6">
         <v>421800</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4">
-        <v>27</v>
-      </c>
-      <c r="H15" s="4">
-        <v>24</v>
-      </c>
-      <c r="I15" s="4">
-        <v>24</v>
-      </c>
-      <c r="J15" s="4">
-        <v>15</v>
-      </c>
-      <c r="K15" s="4">
-        <v>11</v>
-      </c>
-      <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="6">
-        <v>423900</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
@@ -5211,65 +5260,65 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="4">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H16" s="4">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I16" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J16" s="4">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K16" s="4">
         <v>9</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" si="0"/>
-        <v>91</v>
+        <f>SUM(F16:K16)</f>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>421400</v>
+        <v>423900</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G17" s="4">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H17" s="4">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I17" s="4">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="J17" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K17" s="4">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="L17" s="1">
-        <f t="shared" si="0"/>
-        <v>88</v>
+        <f>SUM(F17:K17)</f>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>423200</v>
+        <v>421400</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
@@ -5279,31 +5328,31 @@
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G18" s="4">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H18" s="4">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I18" s="4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J18" s="4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K18" s="4">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="L18" s="1">
-        <f t="shared" si="0"/>
-        <v>85</v>
+        <f>SUM(F18:K18)</f>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>421300</v>
+        <v>423200</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
@@ -5313,60 +5362,60 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G19" s="4">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H19" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I19" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="J19" s="4">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K19" s="4">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="L19" s="1">
-        <f t="shared" si="0"/>
-        <v>85</v>
+        <f>SUM(F19:K19)</f>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>423348</v>
+        <v>421300</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G20" s="4">
-        <v>10</v>
-      </c>
-      <c r="H20" s="1">
-        <v>10</v>
+        <v>18</v>
+      </c>
+      <c r="H20" s="4">
+        <v>18</v>
       </c>
       <c r="I20" s="4">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J20" s="4">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="K20" s="4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="L20" s="1">
-        <f t="shared" si="0"/>
-        <v>40</v>
+        <f>SUM(F20:K20)</f>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
@@ -5399,13 +5448,13 @@
         <v>11</v>
       </c>
       <c r="L21" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F21:K21)</f>
         <v>82</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>423408</v>
+        <v>421100</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -5414,91 +5463,91 @@
         <v>6</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="4"/>
+      <c r="F22" s="4">
+        <v>7</v>
+      </c>
       <c r="G22" s="4">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="H22" s="4">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I22" s="4">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J22" s="4">
-        <v>13</v>
-      </c>
-      <c r="K22" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="K22" s="4">
+        <v>9</v>
+      </c>
       <c r="L22" s="1">
-        <f t="shared" si="0"/>
-        <v>81</v>
+        <f>SUM(F22:K22)</f>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>423304</v>
+        <v>423408</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="4">
-        <v>10</v>
-      </c>
+      <c r="F23" s="4"/>
       <c r="G23" s="4">
+        <v>30</v>
+      </c>
+      <c r="H23" s="4">
         <v>16</v>
       </c>
-      <c r="H23" s="6">
-        <v>17</v>
-      </c>
       <c r="I23" s="4">
+        <v>16</v>
+      </c>
+      <c r="J23" s="4">
         <v>12</v>
       </c>
-      <c r="J23" s="4">
-        <v>13</v>
-      </c>
-      <c r="K23" s="4">
-        <v>7</v>
-      </c>
+      <c r="K23" s="4"/>
       <c r="L23" s="1">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f>SUM(F23:K23)</f>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>421100</v>
+        <v>422700</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="4">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="G24" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H24" s="4">
         <v>13</v>
       </c>
       <c r="I24" s="4">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="J24" s="4">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="K24" s="4">
         <v>9</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f>SUM(F24:K24)</f>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
@@ -5529,115 +5578,115 @@
       </c>
       <c r="K25" s="4"/>
       <c r="L25" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F25:K25)</f>
         <v>69</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>423416</v>
+        <v>423304</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
+        <v>6</v>
+      </c>
+      <c r="G26" s="4">
         <v>10</v>
       </c>
-      <c r="G26" s="4">
-        <v>14</v>
-      </c>
-      <c r="H26" s="4">
-        <v>13</v>
+      <c r="H26" s="6">
+        <v>11</v>
       </c>
       <c r="I26" s="4">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J26" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K26" s="4">
         <v>5</v>
       </c>
       <c r="L26" s="1">
-        <f t="shared" si="0"/>
-        <v>62</v>
+        <f>SUM(F26:K26)</f>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>423316</v>
+        <v>423416</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G27" s="4">
         <v>14</v>
       </c>
       <c r="H27" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I27" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J27" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K27" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L27" s="1">
-        <f t="shared" si="0"/>
-        <v>59</v>
+        <f>SUM(F27:K27)</f>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>420101</v>
+        <v>423316</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G28" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H28" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I28" s="4">
         <v>13</v>
       </c>
       <c r="J28" s="4">
+        <v>8</v>
+      </c>
+      <c r="K28" s="4">
         <v>4</v>
       </c>
-      <c r="K28" s="4">
-        <v>5</v>
-      </c>
       <c r="L28" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F28:K28)</f>
         <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>420160</v>
+        <v>420101</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
@@ -5645,131 +5694,137 @@
       <c r="D29" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E29" s="1"/>
       <c r="F29" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G29" s="4">
         <v>15</v>
       </c>
       <c r="H29" s="4">
+        <v>15</v>
+      </c>
+      <c r="I29" s="4">
         <v>13</v>
       </c>
-      <c r="I29" s="4">
-        <v>12</v>
-      </c>
       <c r="J29" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K29" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L29" s="1">
-        <f t="shared" si="0"/>
-        <v>57</v>
+        <f>SUM(F29:K29)</f>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>423404</v>
+        <v>420160</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F30" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G30" s="4">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H30" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I30" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J30" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K30" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L30" s="1">
-        <f t="shared" si="0"/>
-        <v>56</v>
+        <f>SUM(F30:K30)</f>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>422101</v>
+        <v>424900</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="F31" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G31" s="4">
-        <v>1</v>
-      </c>
-      <c r="H31" s="4">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="H31" s="1">
+        <v>12</v>
       </c>
       <c r="I31" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J31" s="4">
-        <v>14</v>
-      </c>
-      <c r="K31" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K31" s="4">
+        <v>3</v>
+      </c>
       <c r="L31" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
+        <f>SUM(F31:K31)</f>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>422200</v>
+        <v>422101</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="4">
-        <v>1</v>
-      </c>
-      <c r="G32" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1</v>
+      </c>
       <c r="H32" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I32" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J32" s="4">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="K32" s="4"/>
       <c r="L32" s="1">
-        <f t="shared" si="0"/>
-        <v>48</v>
+        <f>SUM(F32:K32)</f>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>424700</v>
+        <v>422701</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
@@ -5779,237 +5834,257 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G33" s="4">
-        <v>8</v>
-      </c>
-      <c r="H33" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="H33" s="4">
+        <v>0</v>
+      </c>
       <c r="I33" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J33" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K33" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L33" s="1">
-        <f t="shared" si="0"/>
-        <v>47</v>
+        <f>SUM(F33:K33)</f>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>423501</v>
+        <v>424900</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E34" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>142</v>
+      </c>
       <c r="F34" s="4">
-        <v>18</v>
-      </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4">
-        <v>2</v>
-      </c>
-      <c r="I34" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="G34" s="4">
+        <v>14</v>
+      </c>
+      <c r="H34" s="1">
+        <v>15</v>
+      </c>
+      <c r="I34" s="4">
+        <v>8</v>
+      </c>
       <c r="J34" s="4">
-        <v>23</v>
-      </c>
-      <c r="K34" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="K34" s="4">
+        <v>0</v>
+      </c>
       <c r="L34" s="1">
-        <f t="shared" si="0"/>
-        <v>43</v>
+        <f>SUM(F34:K34)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>424000</v>
+        <v>422200</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4">
-        <v>3</v>
-      </c>
-      <c r="I35" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="I35" s="4">
+        <v>6</v>
+      </c>
       <c r="J35" s="4">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="K35" s="4"/>
       <c r="L35" s="1">
-        <f t="shared" ref="L35:L66" si="1">SUM(F35:K35)</f>
-        <v>42</v>
+        <f>SUM(F35:K35)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>421801</v>
+        <v>424700</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E36" s="1"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4">
-        <v>6</v>
-      </c>
+      <c r="F36" s="4">
+        <v>19</v>
+      </c>
+      <c r="G36" s="4">
+        <v>8</v>
+      </c>
+      <c r="H36" s="4"/>
       <c r="I36" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J36" s="4">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="K36" s="4">
         <v>10</v>
       </c>
       <c r="L36" s="1">
-        <f t="shared" si="1"/>
-        <v>40</v>
+        <f>SUM(F36:K36)</f>
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>422900</v>
+        <v>423404</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="G37" s="4">
-        <v>1</v>
-      </c>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
+        <v>10</v>
+      </c>
+      <c r="H37" s="4">
+        <v>10</v>
+      </c>
+      <c r="I37" s="4">
+        <v>6</v>
+      </c>
       <c r="J37" s="4">
-        <v>2</v>
-      </c>
-      <c r="K37" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="K37" s="4">
+        <v>4</v>
+      </c>
       <c r="L37" s="1">
-        <f t="shared" si="1"/>
-        <v>37</v>
+        <f>SUM(F37:K37)</f>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>422700</v>
+        <v>424000</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
-        <v>8</v>
-      </c>
-      <c r="G38" s="4">
-        <v>14</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="G38" s="4"/>
       <c r="H38" s="4">
-        <v>10</v>
-      </c>
-      <c r="I38" s="4">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I38" s="4"/>
       <c r="J38" s="4">
-        <v>0</v>
-      </c>
-      <c r="K38" s="4">
-        <v>4</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="K38" s="4"/>
       <c r="L38" s="1">
-        <f t="shared" si="1"/>
-        <v>36</v>
+        <f>SUM(F38:K38)</f>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>421900</v>
+        <v>423348</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G39" s="4">
-        <v>8</v>
-      </c>
-      <c r="H39" s="4">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="H39" s="6">
+        <v>7</v>
       </c>
       <c r="I39" s="4">
         <v>4</v>
       </c>
       <c r="J39" s="4">
-        <v>9</v>
-      </c>
-      <c r="K39" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K39" s="4">
+        <v>1</v>
+      </c>
       <c r="L39" s="1">
-        <f t="shared" si="1"/>
-        <v>31</v>
+        <f>SUM(F39:K39)</f>
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>422701</v>
+        <v>421801</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" s="1"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4">
+        <v>2</v>
+      </c>
+      <c r="H40" s="4">
         <v>8</v>
       </c>
-      <c r="E40" s="1"/>
-      <c r="F40" s="4">
-        <v>26</v>
-      </c>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
+      <c r="I40" s="4">
+        <v>8</v>
+      </c>
       <c r="J40" s="4">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="K40" s="4">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L40" s="1">
-        <f t="shared" si="1"/>
-        <v>30</v>
+        <f>SUM(F40:K40)</f>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>421901</v>
+        <v>422900</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
@@ -6019,65 +6094,59 @@
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="4">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="G41" s="4">
-        <v>8</v>
-      </c>
-      <c r="H41" s="4">
-        <v>6</v>
-      </c>
-      <c r="I41" s="4">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
       <c r="J41" s="4">
-        <v>4</v>
-      </c>
-      <c r="K41" s="4">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K41" s="4"/>
       <c r="L41" s="1">
-        <f t="shared" si="1"/>
-        <v>28</v>
+        <f>SUM(F41:K41)</f>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>421402</v>
+        <v>421901</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G42" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H42" s="4">
+        <v>6</v>
+      </c>
+      <c r="I42" s="4">
+        <v>5</v>
+      </c>
+      <c r="J42" s="4">
         <v>4</v>
       </c>
-      <c r="I42" s="4">
-        <v>7</v>
-      </c>
-      <c r="J42" s="4">
-        <v>5</v>
-      </c>
       <c r="K42" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L42" s="1">
-        <f t="shared" si="1"/>
-        <v>27</v>
+        <f>SUM(F42:K42)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>421301</v>
+        <v>421402</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>7</v>
@@ -6087,425 +6156,443 @@
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="4">
+        <v>1</v>
+      </c>
+      <c r="G43" s="4">
+        <v>6</v>
+      </c>
+      <c r="H43" s="4">
         <v>4</v>
       </c>
-      <c r="G43" s="4">
-        <v>2</v>
-      </c>
-      <c r="H43" s="4">
-        <v>9</v>
-      </c>
       <c r="I43" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J43" s="4">
-        <v>6</v>
-      </c>
-      <c r="K43" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="K43" s="4">
+        <v>4</v>
+      </c>
       <c r="L43" s="1">
-        <f t="shared" si="1"/>
-        <v>26</v>
+        <f>SUM(F43:K43)</f>
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>424500</v>
+        <v>421301</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="4">
-        <v>7</v>
-      </c>
-      <c r="G44" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="G44" s="4">
+        <v>2</v>
+      </c>
       <c r="H44" s="4">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I44" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J44" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F44:K44)</f>
         <v>26</v>
       </c>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>421401</v>
+        <v>424500</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4">
-        <v>1</v>
-      </c>
-      <c r="G45" s="4">
-        <v>7</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G45" s="4"/>
       <c r="H45" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I45" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J45" s="4">
-        <v>2</v>
-      </c>
-      <c r="K45" s="4">
-        <v>1</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K45" s="4"/>
       <c r="L45" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F45:K45)</f>
         <v>26</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421902</v>
+        <v>421401</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H46" s="4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I46" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J46" s="4">
         <v>4</v>
       </c>
       <c r="K46" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L46" s="1">
-        <f t="shared" si="1"/>
-        <v>25</v>
+        <f>SUM(F46:K46)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>422190</v>
+        <v>421902</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>139</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E47" s="1"/>
       <c r="F47" s="4">
         <v>2</v>
       </c>
       <c r="G47" s="4">
-        <v>5</v>
-      </c>
-      <c r="H47" s="6">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="H47" s="4">
+        <v>6</v>
       </c>
       <c r="I47" s="4">
         <v>5</v>
       </c>
       <c r="J47" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K47" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L47" s="1">
-        <f t="shared" si="1"/>
-        <v>23</v>
+        <f>SUM(F47:K47)</f>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>424801</v>
+        <v>421900</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G48" s="4">
-        <v>10</v>
-      </c>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="H48" s="4">
+        <v>7</v>
+      </c>
+      <c r="I48" s="4">
+        <v>3</v>
+      </c>
       <c r="J48" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F48:K48)</f>
         <v>23</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>423409</v>
+        <v>422190</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E49" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="F49" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G49" s="4">
-        <v>4</v>
-      </c>
-      <c r="H49" s="4">
+        <v>5</v>
+      </c>
+      <c r="H49" s="6">
         <v>5</v>
       </c>
       <c r="I49" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J49" s="4">
         <v>3</v>
       </c>
       <c r="K49" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L49" s="1">
-        <f t="shared" si="1"/>
-        <v>20</v>
+        <f>SUM(F49:K49)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>420900</v>
+        <v>424801</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="1"/>
+      <c r="F50" s="4">
+        <v>4</v>
+      </c>
+      <c r="G50" s="4">
         <v>10</v>
-      </c>
-      <c r="E50" s="1"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4">
-        <v>6</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
       <c r="J50" s="4">
-        <v>5</v>
-      </c>
-      <c r="K50" s="4">
         <v>9</v>
       </c>
+      <c r="K50" s="4"/>
       <c r="L50" s="1">
-        <f t="shared" si="1"/>
-        <v>20</v>
+        <f>SUM(F50:K50)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>420501</v>
+        <v>423409</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="4"/>
+      <c r="F51" s="4">
+        <v>5</v>
+      </c>
       <c r="G51" s="4">
         <v>4</v>
       </c>
       <c r="H51" s="4">
+        <v>5</v>
+      </c>
+      <c r="I51" s="4">
+        <v>1</v>
+      </c>
+      <c r="J51" s="4">
         <v>3</v>
       </c>
-      <c r="I51" s="4">
-        <v>4</v>
-      </c>
-      <c r="J51" s="4"/>
       <c r="K51" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L51" s="1">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <f>SUM(F51:K51)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>424300</v>
+        <v>420900</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E52" s="1"/>
-      <c r="F52" s="4">
+      <c r="F52" s="4"/>
+      <c r="G52" s="4">
         <v>8</v>
       </c>
-      <c r="G52" s="4"/>
       <c r="H52" s="4">
-        <v>1</v>
-      </c>
-      <c r="I52" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="I52" s="4">
+        <v>2</v>
+      </c>
       <c r="J52" s="4">
         <v>7</v>
       </c>
-      <c r="K52" s="4"/>
+      <c r="K52" s="4">
+        <v>11</v>
+      </c>
       <c r="L52" s="1">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <f>SUM(F52:K52)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>423500</v>
+        <v>420501</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E53" s="1"/>
-      <c r="F53" s="4">
-        <v>1</v>
-      </c>
+      <c r="F53" s="4"/>
       <c r="G53" s="4">
+        <v>4</v>
+      </c>
+      <c r="H53" s="4">
         <v>3</v>
       </c>
-      <c r="H53" s="4">
-        <v>0</v>
-      </c>
       <c r="I53" s="4">
-        <v>2</v>
-      </c>
-      <c r="J53" s="4">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J53" s="4"/>
       <c r="K53" s="4">
         <v>5</v>
       </c>
       <c r="L53" s="1">
-        <f t="shared" si="1"/>
-        <v>12</v>
+        <f>SUM(F53:K53)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>422601</v>
+        <v>424300</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E54" s="1"/>
       <c r="F54" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
+      <c r="H54" s="4">
+        <v>1</v>
+      </c>
       <c r="I54" s="4"/>
       <c r="J54" s="4">
-        <v>4</v>
-      </c>
-      <c r="K54" s="4">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K54" s="4"/>
       <c r="L54" s="1">
-        <f t="shared" si="1"/>
-        <v>10</v>
+        <f>SUM(F54:K54)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>423600</v>
+        <v>423500</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G55" s="4">
-        <v>4</v>
-      </c>
-      <c r="H55" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="H55" s="4">
+        <v>0</v>
+      </c>
       <c r="I55" s="4">
-        <v>3</v>
-      </c>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="J55" s="4">
+        <v>1</v>
+      </c>
+      <c r="K55" s="4">
+        <v>5</v>
+      </c>
       <c r="L55" s="1">
-        <f t="shared" si="1"/>
-        <v>8</v>
+        <f>SUM(F55:K55)</f>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>420402</v>
+        <v>422601</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E56" s="1"/>
-      <c r="F56" s="4"/>
+      <c r="F56" s="4">
+        <v>5</v>
+      </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>6</v>
-      </c>
-      <c r="K56" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K56" s="4">
+        <v>1</v>
+      </c>
       <c r="L56" s="1">
-        <f t="shared" si="1"/>
-        <v>6</v>
+        <f>SUM(F56:K56)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>424960</v>
+        <v>423600</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>7</v>
@@ -6515,16 +6602,14 @@
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G57" s="4">
-        <v>1</v>
-      </c>
-      <c r="H57" s="6">
-        <v>0</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="H57" s="4"/>
       <c r="I57" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J57" s="4">
         <v>1</v>
@@ -6532,41 +6617,39 @@
       <c r="K57" s="4">
         <v>1</v>
       </c>
-      <c r="L57" s="12">
-        <f t="shared" si="1"/>
-        <v>5</v>
+      <c r="L57" s="1">
+        <f>SUM(F57:K57)</f>
+        <v>14</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>420160</v>
+        <v>420500</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F58" s="4">
-        <v>1</v>
-      </c>
-      <c r="G58" s="4">
-        <v>1</v>
-      </c>
-      <c r="H58" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1">
+        <v>1</v>
+      </c>
       <c r="I58" s="4">
-        <v>1</v>
-      </c>
-      <c r="J58" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="J58" s="1">
+        <v>1</v>
+      </c>
       <c r="K58" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L58" s="1">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <f>SUM(F58:K58)</f>
+        <v>8</v>
       </c>
       <c r="P58" t="s">
         <v>140</v>
@@ -6574,67 +6657,161 @@
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>423309</v>
+        <v>420402</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="4"/>
-      <c r="G59" s="4">
-        <v>1</v>
-      </c>
-      <c r="H59" s="4">
-        <v>1</v>
-      </c>
-      <c r="I59" s="4">
-        <v>1</v>
-      </c>
-      <c r="J59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4">
+        <v>6</v>
+      </c>
       <c r="K59" s="4"/>
       <c r="L59" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F59:K59)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B60" s="6">
+        <v>424960</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="1"/>
+      <c r="F60" s="4">
+        <v>2</v>
+      </c>
+      <c r="G60" s="4">
+        <v>1</v>
+      </c>
+      <c r="H60" s="6">
+        <v>0</v>
+      </c>
+      <c r="I60" s="4">
+        <v>0</v>
+      </c>
+      <c r="J60" s="4">
+        <v>1</v>
+      </c>
+      <c r="K60" s="4">
+        <v>1</v>
+      </c>
+      <c r="L60" s="12">
+        <f>SUM(F60:K60)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B61" s="6">
+        <v>420160</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F61" s="4">
+        <v>1</v>
+      </c>
+      <c r="G61" s="4">
+        <v>1</v>
+      </c>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4">
+        <v>1</v>
+      </c>
+      <c r="J61" s="4"/>
+      <c r="K61" s="4">
+        <v>2</v>
+      </c>
+      <c r="L61" s="1">
+        <f>SUM(F61:K61)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B62" s="6">
+        <v>423309</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4">
+        <v>1</v>
+      </c>
+      <c r="H62" s="4">
+        <v>1</v>
+      </c>
+      <c r="I62" s="4">
+        <v>1</v>
+      </c>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="1">
+        <f>SUM(F62:K62)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B60" s="13">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B63" s="6">
         <v>420200</v>
       </c>
-      <c r="C60" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" s="14" t="s">
+      <c r="C63" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F60" s="15">
+      <c r="E63" s="1"/>
+      <c r="F63" s="4">
+        <v>1</v>
+      </c>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4">
+        <v>1</v>
+      </c>
+      <c r="L63" s="1">
+        <f>SUM(F63:K63)</f>
         <v>2</v>
       </c>
-      <c r="G60" s="15"/>
-      <c r="H60" s="16"/>
-      <c r="I60" s="15"/>
-      <c r="J60" s="15"/>
-      <c r="K60" s="15">
-        <v>1</v>
-      </c>
-      <c r="L60" s="14">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="L62" s="10">
-        <f>SUM(L3:L60)</f>
-        <v>3993</v>
+    </row>
+    <row r="65" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F65" t="s">
+        <v>143</v>
+      </c>
+      <c r="L65" s="10">
+        <f>SUM(L3:L63)</f>
+        <v>3988</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L60" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L60">
-      <sortCondition descending="1" ref="L2:L58"/>
+  <autoFilter ref="B2:L63" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L63">
+      <sortCondition descending="1" ref="L2:L62"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6804,14 +6981,14 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update inventory seed for GitHub Pages
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="890" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F36E9BF-DAF1-4427-8C9B-C750825E18ED}"/>
+  <xr:revisionPtr revIDLastSave="1112" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F56152C4-3C3D-41A3-9B04-C40365F20785}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="131">
   <si>
     <t>CODIGO</t>
   </si>
@@ -192,54 +192,6 @@
     <t>INVENTARIO COLECCIÓN 38</t>
   </si>
   <si>
-    <t>383400</t>
-  </si>
-  <si>
-    <t>388000</t>
-  </si>
-  <si>
-    <t>389700</t>
-  </si>
-  <si>
-    <t>380200</t>
-  </si>
-  <si>
-    <t>382100</t>
-  </si>
-  <si>
-    <t>382101</t>
-  </si>
-  <si>
-    <t>385800</t>
-  </si>
-  <si>
-    <t>389300</t>
-  </si>
-  <si>
-    <t>387900</t>
-  </si>
-  <si>
-    <t>389201</t>
-  </si>
-  <si>
-    <t>388300</t>
-  </si>
-  <si>
-    <t>385304</t>
-  </si>
-  <si>
-    <t>385371</t>
-  </si>
-  <si>
-    <t>386501</t>
-  </si>
-  <si>
-    <t>381801</t>
-  </si>
-  <si>
-    <t>389401</t>
-  </si>
-  <si>
     <t>INVENTARIO COLECCIÓN 39</t>
   </si>
   <si>
@@ -483,7 +435,13 @@
     <t xml:space="preserve">  </t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 11:14    14-04</t>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 16:09   16-04</t>
+  </si>
+  <si>
+    <t>revisado</t>
   </si>
 </sst>
 </file>
@@ -606,7 +564,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -638,18 +596,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1009,6 +963,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_AI_TABLE</we:customFunctionIds>
@@ -1031,19 +988,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
@@ -1830,19 +1787,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -1880,8 +1837,8 @@
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="8" t="s">
-        <v>56</v>
+      <c r="B5" s="16">
+        <v>389201</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
@@ -1914,8 +1871,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="8" t="s">
-        <v>50</v>
+      <c r="B6" s="16">
+        <v>380200</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -1948,8 +1905,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="8" t="s">
-        <v>47</v>
+      <c r="B7" s="16">
+        <v>383400</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -1982,8 +1939,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
-        <v>51</v>
+      <c r="B8" s="16">
+        <v>382100</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>5</v>
@@ -2016,8 +1973,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="8" t="s">
-        <v>48</v>
+      <c r="B9" s="16">
+        <v>388000</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -2050,8 +2007,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
-        <v>54</v>
+      <c r="B10" s="16">
+        <v>389300</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -2084,8 +2041,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="8" t="s">
-        <v>59</v>
+      <c r="B11" s="16">
+        <v>385371</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
@@ -2118,8 +2075,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="8" t="s">
-        <v>60</v>
+      <c r="B12" s="16">
+        <v>386501</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -2152,8 +2109,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="8" t="s">
-        <v>58</v>
+      <c r="B13" s="16">
+        <v>385304</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -2186,8 +2143,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="8" t="s">
-        <v>57</v>
+      <c r="B14" s="16">
+        <v>388300</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -2220,8 +2177,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="8" t="s">
-        <v>55</v>
+      <c r="B15" s="16">
+        <v>387900</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>5</v>
@@ -2254,8 +2211,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="8" t="s">
-        <v>53</v>
+      <c r="B16" s="16">
+        <v>385800</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>7</v>
@@ -2288,8 +2245,8 @@
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="8" t="s">
-        <v>61</v>
+      <c r="B17" s="16">
+        <v>381801</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>7</v>
@@ -2322,8 +2279,8 @@
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="8" t="s">
-        <v>62</v>
+      <c r="B18" s="16">
+        <v>389401</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>7</v>
@@ -2356,8 +2313,8 @@
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="8" t="s">
-        <v>52</v>
+      <c r="B19" s="16">
+        <v>382101</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>5</v>
@@ -2390,8 +2347,8 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
-        <v>49</v>
+      <c r="B20" s="16">
+        <v>389700</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>7</v>
@@ -2437,19 +2394,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
+      <c r="B3" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2488,10 +2445,10 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>8</v>
@@ -2522,7 +2479,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -2552,7 +2509,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -2582,7 +2539,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -2612,7 +2569,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -2640,7 +2597,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -2666,7 +2623,7 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
@@ -2694,7 +2651,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -2720,7 +2677,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -2744,7 +2701,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -2768,7 +2725,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>7</v>
@@ -2804,19 +2761,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
+      <c r="B3" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2855,7 +2812,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
@@ -2889,7 +2846,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -2923,7 +2880,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -2957,7 +2914,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -2991,7 +2948,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -3025,7 +2982,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -3059,13 +3016,13 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9">
@@ -3093,7 +3050,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>5</v>
@@ -3127,7 +3084,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -3161,7 +3118,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -3195,7 +3152,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>7</v>
@@ -3229,7 +3186,7 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>7</v>
@@ -3263,7 +3220,7 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>7</v>
@@ -3297,7 +3254,7 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>5</v>
@@ -3331,7 +3288,7 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>7</v>
@@ -3365,7 +3322,7 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>7</v>
@@ -3399,7 +3356,7 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="8" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>5</v>
@@ -3433,7 +3390,7 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>7</v>
@@ -3467,7 +3424,7 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>5</v>
@@ -3501,7 +3458,7 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>5</v>
@@ -3535,7 +3492,7 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>7</v>
@@ -3569,13 +3526,13 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9">
@@ -3603,7 +3560,7 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>7</v>
@@ -3637,7 +3594,7 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>7</v>
@@ -3671,13 +3628,13 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="8" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9">
@@ -3705,7 +3662,7 @@
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>5</v>
@@ -3739,7 +3696,7 @@
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>7</v>
@@ -3773,7 +3730,7 @@
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>7</v>
@@ -3807,7 +3764,7 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="8" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>5</v>
@@ -3841,7 +3798,7 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="8" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>7</v>
@@ -3875,7 +3832,7 @@
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="8" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>7</v>
@@ -3909,13 +3866,13 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="C36" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9">
@@ -3943,7 +3900,7 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="8" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>7</v>
@@ -3977,7 +3934,7 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="8" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>7</v>
@@ -4011,7 +3968,7 @@
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="8" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>7</v>
@@ -4045,7 +4002,7 @@
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="8" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>7</v>
@@ -4079,7 +4036,7 @@
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="8" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>7</v>
@@ -4113,13 +4070,13 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="8" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9">
@@ -4147,7 +4104,7 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>5</v>
@@ -4181,7 +4138,7 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="8" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>7</v>
@@ -4215,7 +4172,7 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="8" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>7</v>
@@ -4249,7 +4206,7 @@
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>7</v>
@@ -4283,13 +4240,13 @@
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="8" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="E47" s="9"/>
       <c r="F47" s="9">
@@ -4317,13 +4274,13 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E48" s="9"/>
       <c r="F48" s="9">
@@ -4351,7 +4308,7 @@
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="8" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>7</v>
@@ -4397,19 +4354,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
+      <c r="B3" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4448,10 +4405,10 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>6</v>
@@ -4482,7 +4439,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -4514,7 +4471,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -4548,7 +4505,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>5</v>
@@ -4582,7 +4539,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>5</v>
@@ -4616,7 +4573,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -4650,7 +4607,7 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
@@ -4684,7 +4641,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -4718,7 +4675,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -4760,7 +4717,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="B2:P65"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="B2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
@@ -4801,9 +4759,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
-        <v>420100</v>
+        <v>423500</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>7</v>
@@ -4813,339 +4771,342 @@
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="G3" s="4">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="H3" s="4">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="I3" s="4">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="J3" s="4">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="K3" s="4">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="L3" s="1">
         <f>SUM(F3:K3)</f>
-        <v>251</v>
-      </c>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>422500</v>
+        <v>420100</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G4" s="4">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="H4" s="4">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="I4" s="4">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J4" s="4">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="K4" s="4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>217</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
-        <v>420600</v>
+        <v>422500</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G5" s="4">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H5" s="4">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I5" s="4">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="J5" s="4">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K5" s="4">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
-        <v>423000</v>
+        <v>420600</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="4">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G6" s="4">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H6" s="4">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="I6" s="4">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J6" s="4">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="K6" s="4">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="N6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>423501</v>
+        <v>423000</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G7" s="4">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="H7" s="4">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I7" s="4">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J7" s="4">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="K7" s="4">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="L7" s="1">
         <f>SUM(F7:K7)</f>
-        <v>154</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>422800</v>
+        <v>424701</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H8" s="4">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="I8" s="4">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="J8" s="4">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="K8" s="4">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="L8" s="1">
         <f>SUM(F8:K8)</f>
-        <v>156</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>424400</v>
+        <v>422100</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G9" s="4">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H9" s="4">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I9" s="4">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="J9" s="4">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K9" s="4">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="L9" s="1">
         <f>SUM(F9:K9)</f>
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
-        <v>424701</v>
+        <v>422800</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="4">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H10" s="4">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="I10" s="4">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J10" s="4">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="K10" s="4">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="L10" s="1">
         <f>SUM(F10:K10)</f>
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="M10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>422100</v>
+        <v>420500</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="4">
-        <v>12</v>
-      </c>
-      <c r="G11" s="4">
+      <c r="F11" s="6">
+        <v>14</v>
+      </c>
+      <c r="G11" s="6">
+        <v>28</v>
+      </c>
+      <c r="H11" s="6">
         <v>29</v>
       </c>
-      <c r="H11" s="4">
-        <v>30</v>
-      </c>
       <c r="I11" s="4">
-        <v>27</v>
-      </c>
-      <c r="J11" s="4">
-        <v>20</v>
+        <v>29</v>
+      </c>
+      <c r="J11" s="6">
+        <v>22</v>
       </c>
       <c r="K11" s="4">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(F11:K11)</f>
-        <v>141</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="15">
-        <v>423448</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>6</v>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="6">
+        <v>424400</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E12" s="1"/>
-      <c r="F12" s="17">
-        <v>12</v>
-      </c>
-      <c r="G12" s="17">
-        <v>20</v>
-      </c>
-      <c r="H12" s="6">
-        <v>19</v>
-      </c>
-      <c r="I12" s="17">
-        <v>15</v>
-      </c>
-      <c r="J12" s="17">
-        <v>13</v>
-      </c>
-      <c r="K12" s="17">
-        <v>5</v>
+      <c r="F12" s="4">
+        <v>30</v>
+      </c>
+      <c r="G12" s="4">
+        <v>32</v>
+      </c>
+      <c r="H12" s="4">
+        <v>29</v>
+      </c>
+      <c r="I12" s="4">
+        <v>36</v>
+      </c>
+      <c r="J12" s="4">
+        <v>7</v>
+      </c>
+      <c r="K12" s="4">
+        <v>0</v>
       </c>
       <c r="L12" s="1">
         <f>SUM(F12:K12)</f>
-        <v>84</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
         <v>422300</v>
       </c>
@@ -5179,7 +5140,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
         <v>424600</v>
       </c>
@@ -5212,179 +5173,182 @@
         <f>SUM(F14:K14)</f>
         <v>119</v>
       </c>
-      <c r="O14" s="18"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O14" s="13"/>
+    </row>
+    <row r="15" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
-        <v>423308</v>
+        <v>422701</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G15" s="4">
+        <v>12</v>
+      </c>
+      <c r="H15" s="4">
+        <v>16</v>
+      </c>
+      <c r="I15" s="4">
         <v>22</v>
       </c>
-      <c r="H15" s="4">
-        <v>19</v>
-      </c>
-      <c r="I15" s="4">
-        <v>18</v>
-      </c>
       <c r="J15" s="4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K15" s="4">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="L15" s="1">
         <f>SUM(F15:K15)</f>
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>421800</v>
+        <v>423308</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="4">
         <v>2</v>
       </c>
       <c r="G16" s="4">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H16" s="4">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="I16" s="4">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="J16" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K16" s="4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L16" s="1">
         <f>SUM(F16:K16)</f>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="M16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423900</v>
+        <v>423200</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
+        <v>13</v>
+      </c>
+      <c r="G17" s="4">
+        <v>12</v>
+      </c>
+      <c r="H17" s="4">
+        <v>19</v>
+      </c>
+      <c r="I17" s="4">
+        <v>16</v>
+      </c>
+      <c r="J17" s="4">
         <v>14</v>
       </c>
-      <c r="G17" s="4">
-        <v>15</v>
-      </c>
-      <c r="H17" s="4">
-        <v>17</v>
-      </c>
-      <c r="I17" s="4">
-        <v>18</v>
-      </c>
-      <c r="J17" s="4">
-        <v>18</v>
-      </c>
       <c r="K17" s="4">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="L17" s="1">
         <f>SUM(F17:K17)</f>
-        <v>91</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>421400</v>
+        <v>423900</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G18" s="4">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H18" s="4">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I18" s="4">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="J18" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="K18" s="4">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="L18" s="1">
         <f>SUM(F18:K18)</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>423200</v>
+        <v>421800</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
+        <v>2</v>
+      </c>
+      <c r="G19" s="4">
+        <v>24</v>
+      </c>
+      <c r="H19" s="4">
+        <v>21</v>
+      </c>
+      <c r="I19" s="4">
+        <v>21</v>
+      </c>
+      <c r="J19" s="4">
         <v>13</v>
       </c>
-      <c r="G19" s="4">
-        <v>12</v>
-      </c>
-      <c r="H19" s="4">
-        <v>19</v>
-      </c>
-      <c r="I19" s="4">
-        <v>16</v>
-      </c>
-      <c r="J19" s="4">
-        <v>14</v>
-      </c>
       <c r="K19" s="4">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="L19" s="1">
         <f>SUM(F19:K19)</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
         <v>421300</v>
       </c>
@@ -5418,77 +5382,77 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>420400</v>
+        <v>423448</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="G21" s="4">
-        <v>10</v>
-      </c>
-      <c r="H21" s="4">
+        <v>20</v>
+      </c>
+      <c r="H21" s="6">
+        <v>19</v>
+      </c>
+      <c r="I21" s="4">
         <v>15</v>
       </c>
-      <c r="I21" s="4">
-        <v>9</v>
-      </c>
       <c r="J21" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K21" s="4">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="L21" s="1">
         <f>SUM(F21:K21)</f>
-        <v>82</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>421100</v>
+        <v>420400</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="4">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="G22" s="4">
         <v>10</v>
       </c>
       <c r="H22" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I22" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J22" s="4">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="K22" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L22" s="1">
         <f>SUM(F22:K22)</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>423408</v>
+        <v>421100</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
@@ -5497,126 +5461,132 @@
         <v>6</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="4"/>
+      <c r="F23" s="4">
+        <v>6</v>
+      </c>
       <c r="G23" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H23" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I23" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J23" s="4">
-        <v>12</v>
-      </c>
-      <c r="K23" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="K23" s="4">
+        <v>9</v>
+      </c>
       <c r="L23" s="1">
         <f>SUM(F23:K23)</f>
         <v>74</v>
       </c>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>422700</v>
+        <v>423408</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="4">
-        <v>37</v>
-      </c>
+      <c r="F24" s="4"/>
       <c r="G24" s="4">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="H24" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I24" s="4">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="J24" s="4">
-        <v>4</v>
-      </c>
-      <c r="K24" s="4">
-        <v>9</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="K24" s="4"/>
       <c r="L24" s="1">
         <f>SUM(F24:K24)</f>
-        <v>79</v>
-      </c>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>422000</v>
+        <v>421400</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="4">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4">
+        <v>1</v>
+      </c>
+      <c r="I25" s="4">
+        <v>1</v>
+      </c>
+      <c r="J25" s="4">
         <v>11</v>
       </c>
-      <c r="H25" s="4">
-        <v>13</v>
-      </c>
-      <c r="I25" s="4">
-        <v>5</v>
-      </c>
-      <c r="J25" s="4">
-        <v>5</v>
-      </c>
-      <c r="K25" s="4"/>
+      <c r="K25" s="4">
+        <v>32</v>
+      </c>
       <c r="L25" s="1">
         <f>SUM(F25:K25)</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="M25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>423304</v>
+        <v>422000</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="G26" s="4">
-        <v>10</v>
-      </c>
-      <c r="H26" s="6">
         <v>11</v>
       </c>
+      <c r="H26" s="4">
+        <v>12</v>
+      </c>
       <c r="I26" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J26" s="4">
-        <v>10</v>
-      </c>
-      <c r="K26" s="4">
-        <v>5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K26" s="4"/>
       <c r="L26" s="1">
         <f>SUM(F26:K26)</f>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>423416</v>
       </c>
@@ -5650,7 +5620,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
         <v>423316</v>
       </c>
@@ -5684,9 +5654,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>420101</v>
+        <v>420160</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
@@ -5694,169 +5664,170 @@
       <c r="D29" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="1"/>
+      <c r="E29" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F29" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G29" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H29" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I29" s="4">
         <v>13</v>
       </c>
       <c r="J29" s="4">
+        <v>8</v>
+      </c>
+      <c r="K29" s="4">
         <v>4</v>
-      </c>
-      <c r="K29" s="4">
-        <v>5</v>
       </c>
       <c r="L29" s="1">
         <f>SUM(F29:K29)</f>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+      <c r="M29" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>420160</v>
+        <v>424900</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>14</v>
+        <v>125</v>
       </c>
       <c r="F30" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G30" s="4">
         <v>17</v>
       </c>
-      <c r="H30" s="4">
-        <v>15</v>
+      <c r="H30" s="1">
+        <v>12</v>
       </c>
       <c r="I30" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J30" s="4">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K30" s="4">
         <v>3</v>
       </c>
       <c r="L30" s="1">
         <f>SUM(F30:K30)</f>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>424900</v>
+        <v>422101</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>141</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E31" s="1"/>
       <c r="F31" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G31" s="4">
-        <v>17</v>
-      </c>
-      <c r="H31" s="1">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="H31" s="4">
+        <v>14</v>
       </c>
       <c r="I31" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J31" s="4">
-        <v>3</v>
-      </c>
-      <c r="K31" s="4">
-        <v>3</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="K31" s="4"/>
       <c r="L31" s="1">
         <f>SUM(F31:K31)</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>422101</v>
+        <v>421801</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="4">
-        <v>14</v>
-      </c>
+      <c r="F32" s="4"/>
       <c r="G32" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I32" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J32" s="4">
-        <v>14</v>
-      </c>
-      <c r="K32" s="4"/>
+        <v>20</v>
+      </c>
+      <c r="K32" s="4">
+        <v>12</v>
+      </c>
       <c r="L32" s="1">
         <f>SUM(F32:K32)</f>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>422701</v>
+        <v>423304</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G33" s="4">
-        <v>12</v>
-      </c>
-      <c r="H33" s="4">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="H33" s="6">
+        <v>11</v>
       </c>
       <c r="I33" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J33" s="4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K33" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L33" s="1">
         <f>SUM(F33:K33)</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
         <v>424900</v>
       </c>
@@ -5867,7 +5838,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="F34" s="4">
         <v>6</v>
@@ -5892,7 +5863,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
         <v>422200</v>
       </c>
@@ -5908,7 +5879,7 @@
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I35" s="4">
         <v>6</v>
@@ -5919,10 +5890,10 @@
       <c r="K35" s="4"/>
       <c r="L35" s="1">
         <f>SUM(F35:K35)</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
         <v>424700</v>
       </c>
@@ -5954,165 +5925,167 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>423404</v>
+        <v>420101</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G37" s="4">
+        <v>12</v>
+      </c>
+      <c r="H37" s="4">
+        <v>11</v>
+      </c>
+      <c r="I37" s="4">
         <v>10</v>
       </c>
-      <c r="H37" s="4">
-        <v>10</v>
-      </c>
-      <c r="I37" s="4">
-        <v>6</v>
-      </c>
       <c r="J37" s="4">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K37" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L37" s="1">
         <f>SUM(F37:K37)</f>
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>424000</v>
+        <v>423404</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
-        <v>23</v>
-      </c>
-      <c r="G38" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="G38" s="4">
+        <v>10</v>
+      </c>
       <c r="H38" s="4">
-        <v>3</v>
-      </c>
-      <c r="I38" s="4"/>
+        <v>10</v>
+      </c>
+      <c r="I38" s="4">
+        <v>6</v>
+      </c>
       <c r="J38" s="4">
-        <v>16</v>
-      </c>
-      <c r="K38" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="K38" s="4">
+        <v>4</v>
+      </c>
       <c r="L38" s="1">
         <f>SUM(F38:K38)</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>423348</v>
+        <v>424000</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="4">
+        <v>23</v>
+      </c>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4">
         <v>3</v>
       </c>
-      <c r="G39" s="4">
-        <v>7</v>
-      </c>
-      <c r="H39" s="6">
-        <v>7</v>
-      </c>
-      <c r="I39" s="4">
-        <v>4</v>
-      </c>
+      <c r="I39" s="4"/>
       <c r="J39" s="4">
-        <v>3</v>
-      </c>
-      <c r="K39" s="4">
-        <v>1</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="K39" s="4"/>
       <c r="L39" s="1">
         <f>SUM(F39:K39)</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>421801</v>
+        <v>422900</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E40" s="1"/>
-      <c r="F40" s="4"/>
+      <c r="F40" s="4">
+        <v>34</v>
+      </c>
       <c r="G40" s="4">
+        <v>1</v>
+      </c>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4">
         <v>2</v>
       </c>
-      <c r="H40" s="4">
-        <v>8</v>
-      </c>
-      <c r="I40" s="4">
-        <v>8</v>
-      </c>
-      <c r="J40" s="4">
-        <v>20</v>
-      </c>
-      <c r="K40" s="4">
-        <v>12</v>
-      </c>
+      <c r="K40" s="4"/>
       <c r="L40" s="1">
         <f>SUM(F40:K40)</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>422900</v>
+        <v>421401</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="4">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="G41" s="4">
-        <v>1</v>
-      </c>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="H41" s="4">
+        <v>12</v>
+      </c>
+      <c r="I41" s="4">
+        <v>7</v>
+      </c>
       <c r="J41" s="4">
-        <v>2</v>
-      </c>
-      <c r="K41" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K41" s="4">
+        <v>3</v>
+      </c>
       <c r="L41" s="1">
         <f>SUM(F41:K41)</f>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>421901</v>
+        <v>423501</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
@@ -6125,94 +6098,93 @@
         <v>4</v>
       </c>
       <c r="G42" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H42" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I42" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J42" s="4">
         <v>4</v>
       </c>
       <c r="K42" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L42" s="1">
         <f>SUM(F42:K42)</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>421402</v>
+        <v>420900</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="4">
-        <v>1</v>
-      </c>
+      <c r="F43" s="4"/>
       <c r="G43" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H43" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I43" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J43" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K43" s="4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L43" s="1">
         <f>SUM(F43:K43)</f>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>421301</v>
+        <v>422700</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G44" s="4">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H44" s="4">
-        <v>9</v>
-      </c>
-      <c r="I44" s="4">
-        <v>5</v>
-      </c>
-      <c r="J44" s="4">
-        <v>6</v>
-      </c>
-      <c r="K44" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4">
+        <v>6</v>
+      </c>
       <c r="L44" s="1">
         <f>SUM(F44:K44)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="M44" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>424500</v>
+        <v>421901</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
@@ -6222,27 +6194,31 @@
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4">
-        <v>7</v>
-      </c>
-      <c r="G45" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="G45" s="4">
+        <v>8</v>
+      </c>
       <c r="H45" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I45" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J45" s="4">
-        <v>8</v>
-      </c>
-      <c r="K45" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K45" s="4">
+        <v>1</v>
+      </c>
       <c r="L45" s="1">
         <f>SUM(F45:K45)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421401</v>
+        <v>421402</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
@@ -6255,62 +6231,60 @@
         <v>1</v>
       </c>
       <c r="G46" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H46" s="4">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I46" s="4">
         <v>7</v>
       </c>
       <c r="J46" s="4">
+        <v>5</v>
+      </c>
+      <c r="K46" s="4">
         <v>4</v>
-      </c>
-      <c r="K46" s="4">
-        <v>3</v>
       </c>
       <c r="L46" s="1">
         <f>SUM(F46:K46)</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>421902</v>
+        <v>421301</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="4">
+        <v>4</v>
+      </c>
+      <c r="G47" s="4">
         <v>2</v>
       </c>
-      <c r="G47" s="4">
-        <v>6</v>
-      </c>
       <c r="H47" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I47" s="4">
         <v>5</v>
       </c>
       <c r="J47" s="4">
-        <v>4</v>
-      </c>
-      <c r="K47" s="4">
-        <v>2</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K47" s="4"/>
       <c r="L47" s="1">
         <f>SUM(F47:K47)</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>421900</v>
+        <v>424500</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
@@ -6320,16 +6294,14 @@
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>5</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G48" s="4"/>
       <c r="H48" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I48" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J48" s="4">
         <v>8</v>
@@ -6337,12 +6309,12 @@
       <c r="K48" s="4"/>
       <c r="L48" s="1">
         <f>SUM(F48:K48)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>422190</v>
+        <v>423348</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
@@ -6350,247 +6322,256 @@
       <c r="D49" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>139</v>
-      </c>
+      <c r="E49" s="1"/>
       <c r="F49" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G49" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H49" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I49" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J49" s="4">
         <v>3</v>
       </c>
       <c r="K49" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L49" s="1">
         <f>SUM(F49:K49)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>424801</v>
+        <v>421902</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="4">
+        <v>2</v>
+      </c>
+      <c r="G50" s="4">
+        <v>6</v>
+      </c>
+      <c r="H50" s="4">
+        <v>6</v>
+      </c>
+      <c r="I50" s="4">
+        <v>5</v>
+      </c>
+      <c r="J50" s="4">
         <v>4</v>
       </c>
-      <c r="G50" s="4">
-        <v>10</v>
-      </c>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4">
-        <v>9</v>
-      </c>
-      <c r="K50" s="4"/>
+      <c r="K50" s="4">
+        <v>2</v>
+      </c>
       <c r="L50" s="1">
         <f>SUM(F50:K50)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>423409</v>
+        <v>421900</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G51" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H51" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I51" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51" s="4">
-        <v>3</v>
-      </c>
-      <c r="K51" s="4">
-        <v>2</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K51" s="4"/>
       <c r="L51" s="1">
         <f>SUM(F51:K51)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>420900</v>
+        <v>422190</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E52" s="1"/>
-      <c r="F52" s="4"/>
+        <v>13</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F52" s="4">
+        <v>2</v>
+      </c>
       <c r="G52" s="4">
-        <v>8</v>
-      </c>
-      <c r="H52" s="4">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="H52" s="6">
+        <v>5</v>
       </c>
       <c r="I52" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J52" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K52" s="4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L52" s="1">
         <f>SUM(F52:K52)</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>420501</v>
+        <v>423409</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E53" s="1"/>
-      <c r="F53" s="4"/>
+      <c r="F53" s="4">
+        <v>5</v>
+      </c>
       <c r="G53" s="4">
         <v>4</v>
       </c>
       <c r="H53" s="4">
+        <v>5</v>
+      </c>
+      <c r="I53" s="4">
+        <v>1</v>
+      </c>
+      <c r="J53" s="4">
         <v>3</v>
       </c>
-      <c r="I53" s="4">
-        <v>4</v>
-      </c>
-      <c r="J53" s="4"/>
       <c r="K53" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L53" s="1">
         <f>SUM(F53:K53)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>424300</v>
+        <v>424801</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E54" s="1"/>
       <c r="F54" s="4">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I54" s="4"/>
       <c r="J54" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K54" s="4"/>
       <c r="L54" s="1">
         <f>SUM(F54:K54)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="M54" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>423500</v>
+        <v>420501</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="4">
-        <v>8</v>
-      </c>
+      <c r="F55" s="4"/>
       <c r="G55" s="4">
+        <v>4</v>
+      </c>
+      <c r="H55" s="4">
         <v>3</v>
       </c>
-      <c r="H55" s="4">
-        <v>0</v>
-      </c>
       <c r="I55" s="4">
-        <v>0</v>
-      </c>
-      <c r="J55" s="4">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J55" s="4"/>
       <c r="K55" s="4">
         <v>5</v>
       </c>
       <c r="L55" s="1">
         <f>SUM(F55:K55)</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>422601</v>
+        <v>424300</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
+      <c r="H56" s="4">
+        <v>1</v>
+      </c>
       <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>4</v>
-      </c>
-      <c r="K56" s="4">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K56" s="4"/>
       <c r="L56" s="1">
         <f>SUM(F56:K56)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
         <v>423600</v>
       </c>
@@ -6622,40 +6603,38 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>420500</v>
+        <v>422601</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1">
-        <v>1</v>
-      </c>
-      <c r="I58" s="4">
-        <v>5</v>
-      </c>
-      <c r="J58" s="1">
-        <v>1</v>
+      <c r="F58" s="4">
+        <v>5</v>
+      </c>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4">
+        <v>4</v>
       </c>
       <c r="K58" s="4">
         <v>1</v>
       </c>
       <c r="L58" s="1">
         <f>SUM(F58:K58)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P58" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
         <v>420402</v>
       </c>
@@ -6679,7 +6658,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
         <v>424960</v>
       </c>
@@ -6713,7 +6692,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
         <v>420160</v>
       </c>
@@ -6726,26 +6705,23 @@
       <c r="E61" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F61" s="4">
-        <v>1</v>
-      </c>
-      <c r="G61" s="4">
-        <v>1</v>
-      </c>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
       <c r="H61" s="4"/>
-      <c r="I61" s="4">
-        <v>1</v>
-      </c>
+      <c r="I61" s="4"/>
       <c r="J61" s="4"/>
       <c r="K61" s="4">
         <v>2</v>
       </c>
       <c r="L61" s="1">
         <f>SUM(F61:K61)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="M61" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
         <v>423309</v>
       </c>
@@ -6773,7 +6749,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
         <v>420200</v>
       </c>
@@ -6801,17 +6777,32 @@
     </row>
     <row r="65" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F65" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="L65" s="10">
         <f>SUM(L3:L63)</f>
-        <v>3988</v>
+        <v>4066</v>
+      </c>
+    </row>
+    <row r="69" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F69" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="127" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K127" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B2:L63" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="423900"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L63">
-      <sortCondition descending="1" ref="L2:L62"/>
+      <sortCondition descending="1" ref="L2:L63"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6819,21 +6810,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -6977,31 +6953,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7017,4 +6984,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Republish stock and goals data; improve mobile stock UI
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1112" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F56152C4-3C3D-41A3-9B04-C40365F20785}"/>
+  <xr:revisionPtr revIDLastSave="1314" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE218A92-7FC6-4740-9248-597C3F97F17F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="130">
   <si>
     <t>CODIGO</t>
   </si>
@@ -432,16 +432,13 @@
     <t>negro</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
-  </si>
-  <si>
     <t xml:space="preserve">   </t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 16:09   16-04</t>
-  </si>
-  <si>
     <t>revisado</t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 11:02   17-04</t>
   </si>
 </sst>
 </file>
@@ -564,7 +561,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -597,12 +594,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -988,19 +988,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
@@ -1787,19 +1787,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -1837,7 +1837,7 @@
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="16">
+      <c r="B5" s="14">
         <v>389201</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1871,7 +1871,7 @@
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="16">
+      <c r="B6" s="14">
         <v>380200</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1905,7 +1905,7 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="16">
+      <c r="B7" s="14">
         <v>383400</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -1939,7 +1939,7 @@
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="16">
+      <c r="B8" s="14">
         <v>382100</v>
       </c>
       <c r="C8" s="9" t="s">
@@ -1973,7 +1973,7 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="16">
+      <c r="B9" s="14">
         <v>388000</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -2007,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="16">
+      <c r="B10" s="14">
         <v>389300</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -2041,7 +2041,7 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="16">
+      <c r="B11" s="14">
         <v>385371</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -2075,7 +2075,7 @@
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
+      <c r="B12" s="14">
         <v>386501</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -2109,7 +2109,7 @@
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="16">
+      <c r="B13" s="14">
         <v>385304</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -2143,7 +2143,7 @@
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="16">
+      <c r="B14" s="14">
         <v>388300</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -2177,7 +2177,7 @@
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="16">
+      <c r="B15" s="14">
         <v>387900</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -2211,7 +2211,7 @@
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="16">
+      <c r="B16" s="14">
         <v>385800</v>
       </c>
       <c r="C16" s="9" t="s">
@@ -2245,7 +2245,7 @@
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="16">
+      <c r="B17" s="14">
         <v>381801</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -2279,7 +2279,7 @@
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="16">
+      <c r="B18" s="14">
         <v>389401</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -2313,7 +2313,7 @@
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="16">
+      <c r="B19" s="14">
         <v>382101</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -2347,7 +2347,7 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="16">
+      <c r="B20" s="14">
         <v>389700</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -2394,19 +2394,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2761,19 +2761,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4354,19 +4354,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4789,7 +4789,7 @@
         <v>28</v>
       </c>
       <c r="L3" s="1">
-        <f>SUM(F3:K3)</f>
+        <f t="shared" ref="L3:L41" si="0">SUM(F3:K3)</f>
         <v>290</v>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
         <v>12</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>251</v>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
         <v>5</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
+        <f t="shared" si="0"/>
         <v>201</v>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
         <v>17</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
+        <f t="shared" si="0"/>
         <v>160</v>
       </c>
       <c r="N6" t="s">
@@ -4910,274 +4910,280 @@
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
+        <v>21</v>
+      </c>
+      <c r="G7" s="4">
+        <v>19</v>
+      </c>
+      <c r="H7" s="4">
         <v>22</v>
       </c>
-      <c r="G7" s="4">
-        <v>23</v>
-      </c>
-      <c r="H7" s="4">
-        <v>25</v>
-      </c>
       <c r="I7" s="4">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="J7" s="4">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K7" s="4">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
-        <v>157</v>
+        <f t="shared" si="0"/>
+        <v>153</v>
+      </c>
+      <c r="M7" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>424701</v>
+        <v>422100</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="4">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="H8" s="4">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I8" s="4">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="J8" s="4">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="K8" s="4">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
-        <v>150</v>
+        <f t="shared" si="0"/>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>422100</v>
+        <v>420500</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="1"/>
-      <c r="F9" s="4">
-        <v>12</v>
-      </c>
-      <c r="G9" s="4">
+      <c r="F9" s="6">
+        <v>14</v>
+      </c>
+      <c r="G9" s="6">
+        <v>28</v>
+      </c>
+      <c r="H9" s="6">
         <v>29</v>
       </c>
-      <c r="H9" s="4">
-        <v>30</v>
-      </c>
       <c r="I9" s="4">
-        <v>27</v>
-      </c>
-      <c r="J9" s="4">
-        <v>20</v>
+        <v>29</v>
+      </c>
+      <c r="J9" s="6">
+        <v>22</v>
       </c>
       <c r="K9" s="4">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
-        <v>141</v>
+        <f t="shared" si="0"/>
+        <v>137</v>
+      </c>
+      <c r="M9" t="s">
+        <v>128</v>
       </c>
       <c r="N9" s="11"/>
     </row>
     <row r="10" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
-        <v>422800</v>
+        <v>424400</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="4">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G10" s="4">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H10" s="4">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="I10" s="4">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="J10" s="4">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="K10" s="4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
-        <v>132</v>
+        <f t="shared" si="0"/>
+        <v>134</v>
       </c>
       <c r="M10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>420500</v>
+        <v>422800</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="6">
-        <v>14</v>
-      </c>
-      <c r="G11" s="6">
-        <v>28</v>
-      </c>
-      <c r="H11" s="6">
-        <v>29</v>
+      <c r="F11" s="4">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4">
+        <v>13</v>
+      </c>
+      <c r="H11" s="4">
+        <v>57</v>
       </c>
       <c r="I11" s="4">
-        <v>29</v>
-      </c>
-      <c r="J11" s="6">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="J11" s="4">
+        <v>37</v>
       </c>
       <c r="K11" s="4">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
-        <v>137</v>
+        <f t="shared" si="0"/>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>424400</v>
+        <v>422300</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G12" s="4">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="I12" s="4">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="J12" s="4">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
-        <v>134</v>
+        <f t="shared" si="0"/>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>422300</v>
+        <v>424600</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G13" s="4">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H13" s="4">
+        <v>43</v>
+      </c>
+      <c r="I13" s="4">
         <v>18</v>
       </c>
-      <c r="I13" s="4">
-        <v>26</v>
-      </c>
       <c r="J13" s="4">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K13" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
-        <v>122</v>
+        <f t="shared" si="0"/>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
-        <v>424600</v>
+        <v>420501</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G14" s="4">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H14" s="4">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="I14" s="4">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="J14" s="4">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="K14" s="4">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
-        <v>119</v>
+        <f t="shared" si="0"/>
+        <v>106</v>
       </c>
       <c r="O14" s="13"/>
     </row>
-    <row r="15" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
-        <v>422701</v>
+        <v>424701</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
@@ -5187,136 +5193,143 @@
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G15" s="4">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H15" s="4">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="I15" s="4">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="J15" s="4">
         <v>24</v>
       </c>
       <c r="K15" s="4">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
-        <v>103</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="N15" s="17"/>
     </row>
     <row r="16" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>423308</v>
+        <v>423200</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="4">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="G16" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H16" s="4">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="I16" s="4">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J16" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K16" s="4">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>95</v>
       </c>
       <c r="M16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423200</v>
+        <v>423448</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
+        <v>12</v>
+      </c>
+      <c r="G17" s="4">
+        <v>20</v>
+      </c>
+      <c r="H17" s="6">
+        <v>19</v>
+      </c>
+      <c r="I17" s="4">
+        <v>15</v>
+      </c>
+      <c r="J17" s="4">
         <v>13</v>
       </c>
-      <c r="G17" s="4">
-        <v>12</v>
-      </c>
-      <c r="H17" s="4">
-        <v>19</v>
-      </c>
-      <c r="I17" s="4">
-        <v>16</v>
-      </c>
-      <c r="J17" s="4">
-        <v>14</v>
-      </c>
       <c r="K17" s="4">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>84</v>
+      </c>
+      <c r="M17" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>423900</v>
+        <v>420400</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="G18" s="4">
+        <v>10</v>
+      </c>
+      <c r="H18" s="4">
         <v>15</v>
       </c>
-      <c r="H18" s="4">
-        <v>17</v>
-      </c>
       <c r="I18" s="4">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="J18" s="4">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="K18" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
-        <v>90</v>
+        <f t="shared" si="0"/>
+        <v>82</v>
+      </c>
+      <c r="M18" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>421800</v>
+        <v>421100</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
@@ -5326,232 +5339,245 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G19" s="4">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="H19" s="4">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="I19" s="4">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="J19" s="4">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="K19" s="4">
         <v>9</v>
       </c>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
-        <v>90</v>
+        <f t="shared" si="0"/>
+        <v>74</v>
+      </c>
+      <c r="M19" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>421300</v>
+        <v>423408</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="4">
-        <v>10</v>
-      </c>
+      <c r="F20" s="4"/>
       <c r="G20" s="4">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="H20" s="4">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I20" s="4">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J20" s="4">
-        <v>17</v>
-      </c>
-      <c r="K20" s="4">
-        <v>11</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K20" s="4"/>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
-        <v>85</v>
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="M20" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>423448</v>
+        <v>423900</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
+        <v>13</v>
+      </c>
+      <c r="G21" s="4">
         <v>12</v>
       </c>
-      <c r="G21" s="4">
-        <v>20</v>
-      </c>
-      <c r="H21" s="6">
-        <v>19</v>
+      <c r="H21" s="4">
+        <v>4</v>
       </c>
       <c r="I21" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J21" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K21" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
-        <v>84</v>
+        <f t="shared" si="0"/>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>420400</v>
+        <v>420160</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F22" s="4">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="G22" s="4">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H22" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I22" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J22" s="4">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K22" s="4">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
-        <v>82</v>
+        <f t="shared" si="0"/>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>421100</v>
+        <v>423416</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G23" s="4">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H23" s="4">
         <v>13</v>
       </c>
       <c r="I23" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J23" s="4">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="K23" s="4">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
-        <v>74</v>
+        <f t="shared" si="0"/>
+        <v>62</v>
       </c>
       <c r="M23" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>423408</v>
+        <v>423316</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="4"/>
+      <c r="F24" s="4">
+        <v>6</v>
+      </c>
       <c r="G24" s="4">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="H24" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I24" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J24" s="4">
-        <v>12</v>
-      </c>
-      <c r="K24" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="K24" s="4">
+        <v>4</v>
+      </c>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
-        <v>74</v>
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="M24" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>421400</v>
+        <v>424900</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="4">
+        <v>8</v>
+      </c>
+      <c r="G25" s="4">
+        <v>17</v>
+      </c>
+      <c r="H25" s="1">
         <v>12</v>
       </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="4">
-        <v>7</v>
-      </c>
-      <c r="G25" s="4">
-        <v>0</v>
-      </c>
-      <c r="H25" s="4">
-        <v>1</v>
-      </c>
       <c r="I25" s="4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J25" s="4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K25" s="4">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>56</v>
       </c>
       <c r="M25" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
@@ -5566,436 +5592,430 @@
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G26" s="4">
+        <v>9</v>
+      </c>
+      <c r="H26" s="4">
         <v>11</v>
       </c>
-      <c r="H26" s="4">
-        <v>12</v>
-      </c>
       <c r="I26" s="4">
-        <v>4</v>
-      </c>
-      <c r="J26" s="4">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
-        <v>67</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="M26" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>423416</v>
+        <v>422701</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="4">
+        <v>3</v>
+      </c>
+      <c r="G27" s="4">
+        <v>5</v>
+      </c>
+      <c r="H27" s="4">
+        <v>2</v>
+      </c>
+      <c r="I27" s="4">
         <v>10</v>
       </c>
-      <c r="G27" s="4">
-        <v>14</v>
-      </c>
-      <c r="H27" s="4">
-        <v>13</v>
-      </c>
-      <c r="I27" s="4">
-        <v>11</v>
-      </c>
       <c r="J27" s="4">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="K27" s="4">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
-        <v>62</v>
+        <f t="shared" si="0"/>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>423316</v>
+        <v>420800</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E28" s="1"/>
-      <c r="F28" s="4">
-        <v>6</v>
-      </c>
-      <c r="G28" s="4">
-        <v>14</v>
-      </c>
-      <c r="H28" s="4">
-        <v>14</v>
-      </c>
-      <c r="I28" s="4">
-        <v>13</v>
-      </c>
-      <c r="J28" s="4">
-        <v>8</v>
+      <c r="F28" s="6">
+        <v>6</v>
+      </c>
+      <c r="G28" s="6">
+        <v>10</v>
+      </c>
+      <c r="H28" s="6">
+        <v>12</v>
+      </c>
+      <c r="I28" s="6">
+        <v>12</v>
+      </c>
+      <c r="J28" s="6">
+        <v>6</v>
       </c>
       <c r="K28" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
-        <v>59</v>
+        <f t="shared" si="0"/>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>420160</v>
+        <v>421400</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="E29" s="1"/>
       <c r="F29" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G29" s="4">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I29" s="4">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J29" s="4">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K29" s="4">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
-        <v>63</v>
+        <f t="shared" si="0"/>
+        <v>52</v>
       </c>
       <c r="M29" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>424900</v>
+        <v>422101</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>125</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G30" s="4">
-        <v>17</v>
-      </c>
-      <c r="H30" s="1">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="H30" s="4">
+        <v>14</v>
       </c>
       <c r="I30" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J30" s="4">
-        <v>3</v>
-      </c>
-      <c r="K30" s="4">
-        <v>3</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="K30" s="4"/>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
-        <v>56</v>
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="M30" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>422101</v>
+        <v>421801</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E31" s="1"/>
-      <c r="F31" s="4">
-        <v>14</v>
-      </c>
+      <c r="F31" s="4"/>
       <c r="G31" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I31" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J31" s="4">
-        <v>14</v>
-      </c>
-      <c r="K31" s="4"/>
+        <v>20</v>
+      </c>
+      <c r="K31" s="4">
+        <v>12</v>
+      </c>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>421801</v>
+        <v>423304</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="4"/>
+      <c r="F32" s="4">
+        <v>6</v>
+      </c>
       <c r="G32" s="4">
-        <v>2</v>
-      </c>
-      <c r="H32" s="4">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="H32" s="6">
+        <v>11</v>
       </c>
       <c r="I32" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J32" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K32" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
-        <v>50</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>423304</v>
+        <v>424900</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>126</v>
+      </c>
       <c r="F33" s="4">
         <v>6</v>
       </c>
       <c r="G33" s="4">
-        <v>10</v>
-      </c>
-      <c r="H33" s="6">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="H33" s="1">
+        <v>15</v>
       </c>
       <c r="I33" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J33" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K33" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L33" s="1">
-        <f>SUM(F33:K33)</f>
-        <v>49</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>424900</v>
+        <v>422200</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>126</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>6</v>
-      </c>
-      <c r="G34" s="4">
-        <v>14</v>
-      </c>
-      <c r="H34" s="1">
+        <v>1</v>
+      </c>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4">
         <v>15</v>
       </c>
       <c r="I34" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J34" s="4">
-        <v>5</v>
-      </c>
-      <c r="K34" s="4">
-        <v>0</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
-        <v>48</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>422200</v>
+        <v>424700</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>1</v>
-      </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4">
-        <v>15</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G35" s="4">
+        <v>8</v>
+      </c>
+      <c r="H35" s="4"/>
       <c r="I35" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J35" s="4">
-        <v>25</v>
-      </c>
-      <c r="K35" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K35" s="4">
+        <v>10</v>
+      </c>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
     </row>
     <row r="36" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>424700</v>
+        <v>420101</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="4">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="G36" s="4">
-        <v>8</v>
-      </c>
-      <c r="H36" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="H36" s="4">
+        <v>11</v>
+      </c>
       <c r="I36" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J36" s="4">
         <v>1</v>
       </c>
       <c r="K36" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L36" s="1">
-        <f>SUM(F36:K36)</f>
-        <v>47</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>420101</v>
+        <v>423404</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G37" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H37" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I37" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J37" s="4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K37" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L37" s="1">
-        <f>SUM(F37:K37)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
     <row r="38" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>423404</v>
+        <v>424000</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
-        <v>5</v>
-      </c>
-      <c r="G38" s="4">
-        <v>10</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="G38" s="4"/>
       <c r="H38" s="4">
-        <v>10</v>
-      </c>
-      <c r="I38" s="4">
-        <v>6</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I38" s="4"/>
       <c r="J38" s="4">
-        <v>9</v>
-      </c>
-      <c r="K38" s="4">
-        <v>4</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="K38" s="4"/>
       <c r="L38" s="1">
-        <f>SUM(F38:K38)</f>
-        <v>44</v>
+        <f t="shared" si="0"/>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>424000</v>
+        <v>422900</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>7</v>
@@ -6005,249 +6025,234 @@
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="4">
-        <v>23</v>
-      </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4">
-        <v>3</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="G39" s="4">
+        <v>1</v>
+      </c>
+      <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="1">
-        <f>SUM(F39:K39)</f>
-        <v>42</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>422900</v>
+        <v>421401</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4">
-        <v>1</v>
-      </c>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="H40" s="4">
+        <v>12</v>
+      </c>
+      <c r="I40" s="4">
+        <v>7</v>
+      </c>
       <c r="J40" s="4">
-        <v>2</v>
-      </c>
-      <c r="K40" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K40" s="4">
+        <v>3</v>
+      </c>
       <c r="L40" s="1">
-        <f>SUM(F40:K40)</f>
-        <v>37</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>421401</v>
+        <v>423308</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H41" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I41" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J41" s="4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="K41" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L41" s="1">
-        <f>SUM(F41:K41)</f>
-        <v>36</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="M41" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="42" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>423501</v>
+        <v>420801</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="4">
-        <v>4</v>
-      </c>
-      <c r="G42" s="4">
-        <v>6</v>
-      </c>
-      <c r="H42" s="4">
-        <v>5</v>
-      </c>
-      <c r="I42" s="4">
-        <v>7</v>
-      </c>
-      <c r="J42" s="4">
-        <v>4</v>
-      </c>
-      <c r="K42" s="4">
-        <v>5</v>
-      </c>
+      <c r="F42" s="1"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="4"/>
       <c r="L42" s="1">
-        <f>SUM(F42:K42)</f>
-        <v>31</v>
+        <f>SUM(G42:K42)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>420900</v>
+        <v>420802</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4">
-        <v>8</v>
-      </c>
-      <c r="H43" s="4">
-        <v>2</v>
-      </c>
-      <c r="I43" s="4">
-        <v>2</v>
-      </c>
-      <c r="J43" s="4">
-        <v>7</v>
-      </c>
-      <c r="K43" s="4">
-        <v>11</v>
-      </c>
+      <c r="F43" s="1"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f>SUM(F43:K43)</f>
-        <v>30</v>
+        <f>SUM(G43:K43)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>422700</v>
+        <v>420900</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4">
         <v>8</v>
       </c>
-      <c r="E44" s="1"/>
-      <c r="F44" s="4">
-        <v>6</v>
-      </c>
-      <c r="G44" s="4">
-        <v>9</v>
-      </c>
       <c r="H44" s="4">
-        <v>8</v>
-      </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="I44" s="4">
+        <v>2</v>
+      </c>
+      <c r="J44" s="4">
+        <v>7</v>
+      </c>
       <c r="K44" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L44" s="1">
-        <f>SUM(F44:K44)</f>
-        <v>29</v>
+        <f t="shared" ref="L44:L66" si="1">SUM(F44:K44)</f>
+        <v>30</v>
       </c>
       <c r="M44" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>421901</v>
+        <v>422700</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G45" s="4">
+        <v>9</v>
+      </c>
+      <c r="H45" s="4">
         <v>8</v>
       </c>
-      <c r="H45" s="4">
-        <v>6</v>
-      </c>
-      <c r="I45" s="4">
-        <v>5</v>
-      </c>
-      <c r="J45" s="4">
-        <v>4</v>
-      </c>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
       <c r="K45" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L45" s="1">
-        <f>SUM(F45:K45)</f>
-        <v>28</v>
+        <f t="shared" si="1"/>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421402</v>
+        <v>421901</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G46" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H46" s="4">
+        <v>6</v>
+      </c>
+      <c r="I46" s="4">
+        <v>5</v>
+      </c>
+      <c r="J46" s="4">
         <v>4</v>
       </c>
-      <c r="I46" s="4">
-        <v>7</v>
-      </c>
-      <c r="J46" s="4">
-        <v>5</v>
-      </c>
       <c r="K46" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L46" s="1">
-        <f>SUM(F46:K46)</f>
-        <v>27</v>
+        <f t="shared" si="1"/>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
@@ -6278,7 +6283,7 @@
       </c>
       <c r="K47" s="4"/>
       <c r="L47" s="1">
-        <f>SUM(F47:K47)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
@@ -6308,7 +6313,7 @@
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f>SUM(F48:K48)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
     </row>
@@ -6342,7 +6347,7 @@
         <v>1</v>
       </c>
       <c r="L49" s="1">
-        <f>SUM(F49:K49)</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
     </row>
@@ -6376,259 +6381,267 @@
         <v>2</v>
       </c>
       <c r="L50" s="1">
-        <f>SUM(F50:K50)</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
     </row>
     <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>421900</v>
+        <v>421800</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="4">
-        <v>0</v>
-      </c>
+      <c r="F51" s="4"/>
       <c r="G51" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H51" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I51" s="4">
+        <v>6</v>
+      </c>
+      <c r="J51" s="4">
+        <v>6</v>
+      </c>
+      <c r="K51" s="4">
         <v>3</v>
       </c>
-      <c r="J51" s="4">
-        <v>8</v>
-      </c>
-      <c r="K51" s="4"/>
       <c r="L51" s="1">
-        <f>SUM(F51:K51)</f>
-        <v>23</v>
+        <f t="shared" si="1"/>
+        <v>24</v>
       </c>
     </row>
     <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>422190</v>
+        <v>423501</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>123</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E52" s="1"/>
       <c r="F52" s="4">
         <v>2</v>
       </c>
       <c r="G52" s="4">
-        <v>5</v>
-      </c>
-      <c r="H52" s="6">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="H52" s="4">
+        <v>1</v>
       </c>
       <c r="I52" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J52" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L52" s="1">
-        <f>SUM(F52:K52)</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
     </row>
     <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>423409</v>
+        <v>421900</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G53" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H53" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I53" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J53" s="4">
-        <v>3</v>
-      </c>
-      <c r="K53" s="4">
-        <v>2</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K53" s="4"/>
       <c r="L53" s="1">
-        <f>SUM(F53:K53)</f>
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>424801</v>
+        <v>422190</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E54" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="F54" s="4">
+        <v>2</v>
+      </c>
+      <c r="G54" s="4">
+        <v>5</v>
+      </c>
+      <c r="H54" s="6">
+        <v>5</v>
+      </c>
+      <c r="I54" s="4">
+        <v>5</v>
+      </c>
+      <c r="J54" s="4">
         <v>3</v>
       </c>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4">
-        <v>8</v>
-      </c>
-      <c r="I54" s="4"/>
-      <c r="J54" s="4">
-        <v>8</v>
-      </c>
-      <c r="K54" s="4"/>
+      <c r="K54" s="4">
+        <v>3</v>
+      </c>
       <c r="L54" s="1">
-        <f>SUM(F54:K54)</f>
-        <v>19</v>
+        <f t="shared" si="1"/>
+        <v>23</v>
       </c>
       <c r="M54" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>420501</v>
+        <v>423409</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="4"/>
+      <c r="F55" s="4">
+        <v>5</v>
+      </c>
       <c r="G55" s="4">
         <v>4</v>
       </c>
       <c r="H55" s="4">
+        <v>5</v>
+      </c>
+      <c r="I55" s="4">
+        <v>1</v>
+      </c>
+      <c r="J55" s="4">
         <v>3</v>
       </c>
-      <c r="I55" s="4">
-        <v>4</v>
-      </c>
-      <c r="J55" s="4"/>
       <c r="K55" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L55" s="1">
-        <f>SUM(F55:K55)</f>
-        <v>16</v>
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>424300</v>
+        <v>424801</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="4">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K56" s="4"/>
       <c r="L56" s="1">
-        <f>SUM(F56:K56)</f>
-        <v>16</v>
+        <f t="shared" si="1"/>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>423600</v>
+        <v>424300</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="4">
-        <v>1</v>
-      </c>
-      <c r="G57" s="4">
-        <v>6</v>
-      </c>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4">
-        <v>5</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4">
+        <v>1</v>
+      </c>
+      <c r="I57" s="4"/>
       <c r="J57" s="4">
-        <v>1</v>
-      </c>
-      <c r="K57" s="4">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K57" s="4"/>
       <c r="L57" s="1">
-        <f>SUM(F57:K57)</f>
-        <v>14</v>
+        <f t="shared" si="1"/>
+        <v>16</v>
       </c>
     </row>
     <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>422601</v>
+        <v>423600</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="4">
-        <v>5</v>
-      </c>
-      <c r="G58" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G58" s="4">
+        <v>6</v>
+      </c>
       <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
+      <c r="I58" s="4">
+        <v>5</v>
+      </c>
       <c r="J58" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K58" s="4">
         <v>1</v>
       </c>
       <c r="L58" s="1">
-        <f>SUM(F58:K58)</f>
-        <v>10</v>
+        <f t="shared" si="1"/>
+        <v>14</v>
       </c>
       <c r="P58" t="s">
         <v>124</v>
@@ -6636,157 +6649,240 @@
     </row>
     <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>420402</v>
+        <v>421402</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
+      <c r="G59" s="4">
+        <v>3</v>
+      </c>
+      <c r="H59" s="4">
+        <v>1</v>
+      </c>
+      <c r="I59" s="4">
+        <v>4</v>
+      </c>
       <c r="J59" s="4">
-        <v>6</v>
-      </c>
-      <c r="K59" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K59" s="4">
+        <v>2</v>
+      </c>
       <c r="L59" s="1">
-        <f>SUM(F59:K59)</f>
-        <v>6</v>
+        <f t="shared" si="1"/>
+        <v>13</v>
       </c>
     </row>
     <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
-        <v>424960</v>
+        <v>421300</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="4">
         <v>2</v>
       </c>
-      <c r="G60" s="4">
-        <v>1</v>
-      </c>
-      <c r="H60" s="6">
-        <v>0</v>
-      </c>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
       <c r="I60" s="4">
-        <v>0</v>
-      </c>
-      <c r="J60" s="4">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J60" s="4"/>
       <c r="K60" s="4">
-        <v>1</v>
-      </c>
-      <c r="L60" s="12">
-        <f>SUM(F60:K60)</f>
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="L60" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
-        <v>420160</v>
+        <v>422601</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E61" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F61" s="4"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="4">
+        <v>5</v>
+      </c>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="4"/>
+      <c r="J61" s="4">
+        <v>4</v>
+      </c>
       <c r="K61" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L61" s="1">
-        <f>SUM(F61:K61)</f>
-        <v>2</v>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="M61" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
-        <v>423309</v>
+        <v>420402</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="4"/>
-      <c r="G62" s="4">
-        <v>1</v>
-      </c>
-      <c r="H62" s="4">
-        <v>1</v>
-      </c>
-      <c r="I62" s="4">
-        <v>1</v>
-      </c>
-      <c r="J62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4">
+        <v>6</v>
+      </c>
       <c r="K62" s="4"/>
       <c r="L62" s="1">
-        <f>SUM(F62:K62)</f>
-        <v>3</v>
+        <f t="shared" si="1"/>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
-        <v>420200</v>
+        <v>424960</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="4">
-        <v>1</v>
-      </c>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="G63" s="4">
+        <v>1</v>
+      </c>
+      <c r="H63" s="6">
+        <v>0</v>
+      </c>
+      <c r="I63" s="4">
+        <v>0</v>
+      </c>
+      <c r="J63" s="4">
+        <v>1</v>
+      </c>
       <c r="K63" s="4">
         <v>1</v>
       </c>
-      <c r="L63" s="1">
-        <f>SUM(F63:K63)</f>
+      <c r="L63" s="12">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="6">
+        <v>423309</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E64" s="1"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4">
+        <v>1</v>
+      </c>
+      <c r="H64" s="4">
+        <v>1</v>
+      </c>
+      <c r="I64" s="4">
+        <v>1</v>
+      </c>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="1">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="6">
+        <v>420160</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="65" spans="6:12" x14ac:dyDescent="0.25">
-      <c r="F65" t="s">
+      <c r="L65" s="1">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="6">
+        <v>420200</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="1"/>
+      <c r="F66" s="4">
+        <v>1</v>
+      </c>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4"/>
+      <c r="K66" s="4">
+        <v>1</v>
+      </c>
+      <c r="L66" s="1">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F69" t="s">
         <v>127</v>
       </c>
-      <c r="L65" s="10">
-        <f>SUM(L3:L63)</f>
-        <v>4066</v>
-      </c>
-    </row>
-    <row r="69" spans="6:12" x14ac:dyDescent="0.25">
-      <c r="F69" t="s">
-        <v>128</v>
+      <c r="L69" s="10">
+        <f>SUM(L3:L66)</f>
+        <v>3903</v>
       </c>
     </row>
     <row r="127" spans="11:11" x14ac:dyDescent="0.25">
@@ -6795,14 +6891,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L63" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+  <autoFilter ref="B2:L66" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
     <filterColumn colId="0">
       <filters>
-        <filter val="423900"/>
+        <filter val="424701"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L63">
-      <sortCondition descending="1" ref="L2:L63"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B15:L15">
+      <sortCondition descending="1" ref="L2:L66"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6810,6 +6906,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -6953,7 +7055,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -6962,13 +7064,23 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6986,26 +7098,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update stock bodega source inventory file
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1314" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE218A92-7FC6-4740-9248-597C3F97F17F}"/>
+  <xr:revisionPtr revIDLastSave="1654" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE73E74C-57C4-4700-9B77-FB42ABCE2AE8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="130">
   <si>
     <t>CODIGO</t>
   </si>
@@ -435,10 +435,10 @@
     <t xml:space="preserve">   </t>
   </si>
   <si>
-    <t>revisado</t>
-  </si>
-  <si>
-    <t>ULTIMA ACTUALIZACION 11:02   17-04</t>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 18:19   21-04</t>
   </si>
 </sst>
 </file>
@@ -561,7 +561,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -601,9 +601,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -3709,7 +3710,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H31" s="9">
         <v>0</v>
@@ -3725,7 +3726,7 @@
       </c>
       <c r="L31" s="9">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
@@ -4717,7 +4718,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <sheetPr filterMode="1"/>
   <dimension ref="B2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4759,9 +4759,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
-        <v>423500</v>
+        <v>420100</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>7</v>
@@ -4771,31 +4771,31 @@
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G3" s="4">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="H3" s="4">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="I3" s="4">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="J3" s="4">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="K3" s="4">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="L3" s="1">
-        <f t="shared" ref="L3:L41" si="0">SUM(F3:K3)</f>
-        <v>290</v>
-      </c>
-    </row>
-    <row r="4" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F3:K3)</f>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>420100</v>
+        <v>423500</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -4805,63 +4805,63 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
+        <v>22</v>
+      </c>
+      <c r="G4" s="4">
+        <v>51</v>
+      </c>
+      <c r="H4" s="4">
+        <v>53</v>
+      </c>
+      <c r="I4" s="4">
+        <v>49</v>
+      </c>
+      <c r="J4" s="4">
         <v>37</v>
       </c>
-      <c r="G4" s="4">
-        <v>47</v>
-      </c>
-      <c r="H4" s="4">
-        <v>84</v>
-      </c>
-      <c r="I4" s="4">
-        <v>45</v>
-      </c>
-      <c r="J4" s="4">
-        <v>26</v>
-      </c>
       <c r="K4" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="L4" s="1">
-        <f t="shared" si="0"/>
-        <v>251</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F4:K4)</f>
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
-        <v>422500</v>
+        <v>422200</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="H5" s="4">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="I5" s="4">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="J5" s="4">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="K5" s="4">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" si="0"/>
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F5:K5)</f>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>420600</v>
       </c>
@@ -4891,51 +4891,48 @@
         <v>17</v>
       </c>
       <c r="L6" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F6:K6)</f>
         <v>160</v>
       </c>
       <c r="N6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>423000</v>
+        <v>422500</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G7" s="4">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H7" s="4">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="I7" s="4">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J7" s="4">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K7" s="4">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="L7" s="1">
-        <f t="shared" si="0"/>
-        <v>153</v>
-      </c>
-      <c r="M7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F7:K7)</f>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>422100</v>
       </c>
@@ -4965,120 +4962,117 @@
         <v>23</v>
       </c>
       <c r="L8" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F8:K8)</f>
         <v>141</v>
       </c>
     </row>
-    <row r="9" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>420500</v>
+        <v>424400</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E9" s="1"/>
-      <c r="F9" s="6">
-        <v>14</v>
-      </c>
-      <c r="G9" s="6">
-        <v>28</v>
-      </c>
-      <c r="H9" s="6">
+      <c r="F9" s="4">
+        <v>30</v>
+      </c>
+      <c r="G9" s="4">
+        <v>32</v>
+      </c>
+      <c r="H9" s="4">
         <v>29</v>
       </c>
       <c r="I9" s="4">
-        <v>29</v>
-      </c>
-      <c r="J9" s="6">
-        <v>22</v>
+        <v>36</v>
+      </c>
+      <c r="J9" s="4">
+        <v>7</v>
       </c>
       <c r="K9" s="4">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="L9" s="1">
-        <f t="shared" si="0"/>
-        <v>137</v>
-      </c>
-      <c r="M9" t="s">
-        <v>128</v>
+        <f>SUM(F9:K9)</f>
+        <v>134</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
-        <v>424400</v>
+        <v>422800</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="4">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="H10" s="4">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="I10" s="4">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="J10" s="4">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="K10" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L10" s="1">
-        <f t="shared" si="0"/>
-        <v>134</v>
-      </c>
-      <c r="M10" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F10:K10)</f>
+        <v>132</v>
+      </c>
+      <c r="O10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>422800</v>
+        <v>424600</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G11" s="4">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H11" s="4">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I11" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J11" s="4">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="K11" s="4">
         <v>7</v>
       </c>
       <c r="L11" s="1">
-        <f t="shared" si="0"/>
-        <v>132</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F11:K11)</f>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>422300</v>
       </c>
@@ -5090,65 +5084,66 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G12" s="4">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H12" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I12" s="4">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J12" s="4">
-        <v>21</v>
-      </c>
-      <c r="K12" s="4">
-        <v>5</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K12" s="4"/>
       <c r="L12" s="1">
-        <f t="shared" si="0"/>
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F12:K12)</f>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>424600</v>
+        <v>423000</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G13" s="4">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="H13" s="4">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="I13" s="4">
         <v>18</v>
       </c>
       <c r="J13" s="4">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="K13" s="4">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="0"/>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F13:K13)</f>
+        <v>98</v>
+      </c>
+      <c r="O13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
-        <v>420501</v>
+        <v>423200</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
@@ -5158,26 +5153,26 @@
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G14" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H14" s="4">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I14" s="4">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J14" s="4">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K14" s="4">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L14" s="1">
-        <f t="shared" si="0"/>
-        <v>106</v>
+        <f>SUM(F14:K14)</f>
+        <v>95</v>
       </c>
       <c r="O14" s="13"/>
     </row>
@@ -5193,247 +5188,238 @@
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="4">
+        <v>10</v>
+      </c>
+      <c r="G15" s="4">
+        <v>14</v>
+      </c>
+      <c r="H15" s="4">
+        <v>26</v>
+      </c>
+      <c r="I15" s="4">
         <v>11</v>
       </c>
-      <c r="G15" s="4">
-        <v>16</v>
-      </c>
-      <c r="H15" s="4">
-        <v>29</v>
-      </c>
-      <c r="I15" s="4">
-        <v>14</v>
-      </c>
       <c r="J15" s="4">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K15" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>99</v>
-      </c>
-      <c r="N15" s="17"/>
-    </row>
-    <row r="16" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F15:K15)</f>
+        <v>88</v>
+      </c>
+      <c r="N15" s="11"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>423200</v>
+        <v>420500</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="4">
-        <v>13</v>
-      </c>
-      <c r="G16" s="4">
-        <v>12</v>
-      </c>
-      <c r="H16" s="4">
-        <v>19</v>
+      <c r="F16" s="6">
+        <v>5</v>
+      </c>
+      <c r="G16" s="6">
+        <v>16</v>
+      </c>
+      <c r="H16" s="6">
+        <v>26</v>
       </c>
       <c r="I16" s="4">
         <v>16</v>
       </c>
-      <c r="J16" s="4">
-        <v>14</v>
+      <c r="J16" s="6">
+        <v>15</v>
       </c>
       <c r="K16" s="4">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" si="0"/>
-        <v>95</v>
-      </c>
-      <c r="M16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F16:K16)</f>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423448</v>
+        <v>423900</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
+        <v>13</v>
+      </c>
+      <c r="G17" s="4">
         <v>12</v>
       </c>
-      <c r="G17" s="4">
-        <v>20</v>
-      </c>
-      <c r="H17" s="6">
-        <v>19</v>
+      <c r="H17" s="4">
+        <v>4</v>
       </c>
       <c r="I17" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J17" s="4">
+        <v>16</v>
+      </c>
+      <c r="K17" s="4">
+        <v>7</v>
+      </c>
+      <c r="L17" s="1">
+        <f>SUM(F17:K17)</f>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="6">
+        <v>424900</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F18" s="4">
+        <v>10</v>
+      </c>
+      <c r="G18" s="4">
+        <v>17</v>
+      </c>
+      <c r="H18" s="6">
+        <v>12</v>
+      </c>
+      <c r="I18" s="4">
         <v>13</v>
       </c>
-      <c r="K17" s="4">
-        <v>5</v>
-      </c>
-      <c r="L17" s="1">
-        <f t="shared" si="0"/>
-        <v>84</v>
-      </c>
-      <c r="M17" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="6">
+      <c r="J18" s="4">
+        <v>9</v>
+      </c>
+      <c r="K18" s="4">
+        <v>6</v>
+      </c>
+      <c r="L18" s="1">
+        <f>SUM(F18:K18)</f>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="6">
         <v>420400</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="4">
-        <v>26</v>
-      </c>
-      <c r="G18" s="4">
-        <v>10</v>
-      </c>
-      <c r="H18" s="4">
-        <v>15</v>
-      </c>
-      <c r="I18" s="4">
-        <v>9</v>
-      </c>
-      <c r="J18" s="4">
-        <v>11</v>
-      </c>
-      <c r="K18" s="4">
-        <v>11</v>
-      </c>
-      <c r="L18" s="1">
-        <f t="shared" si="0"/>
-        <v>82</v>
-      </c>
-      <c r="M18" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="6">
-        <v>421100</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G19" s="4">
+        <v>6</v>
+      </c>
+      <c r="H19" s="4">
+        <v>11</v>
+      </c>
+      <c r="I19" s="4">
+        <v>6</v>
+      </c>
+      <c r="J19" s="4">
+        <v>9</v>
+      </c>
+      <c r="K19" s="4">
         <v>10</v>
       </c>
-      <c r="H19" s="4">
+      <c r="L19" s="1">
+        <f>SUM(F19:K19)</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="6">
+        <v>423416</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="4">
+        <v>10</v>
+      </c>
+      <c r="G20" s="4">
+        <v>14</v>
+      </c>
+      <c r="H20" s="4">
         <v>13</v>
       </c>
-      <c r="I19" s="4">
-        <v>13</v>
-      </c>
-      <c r="J19" s="4">
-        <v>23</v>
-      </c>
-      <c r="K19" s="4">
-        <v>9</v>
-      </c>
-      <c r="L19" s="1">
-        <f t="shared" si="0"/>
-        <v>74</v>
-      </c>
-      <c r="M19" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="20" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="6">
-        <v>423408</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4">
-        <v>29</v>
-      </c>
-      <c r="H20" s="4">
-        <v>15</v>
-      </c>
       <c r="I20" s="4">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J20" s="4">
         <v>9</v>
       </c>
-      <c r="K20" s="4"/>
+      <c r="K20" s="4">
+        <v>5</v>
+      </c>
       <c r="L20" s="1">
-        <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-      <c r="M20" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="21" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F20:K20)</f>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>423900</v>
+        <v>423316</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
+        <v>6</v>
+      </c>
+      <c r="G21" s="4">
+        <v>14</v>
+      </c>
+      <c r="H21" s="4">
+        <v>14</v>
+      </c>
+      <c r="I21" s="4">
         <v>13</v>
       </c>
-      <c r="G21" s="4">
-        <v>12</v>
-      </c>
-      <c r="H21" s="4">
+      <c r="J21" s="4">
+        <v>8</v>
+      </c>
+      <c r="K21" s="4">
         <v>4</v>
       </c>
-      <c r="I21" s="4">
-        <v>16</v>
-      </c>
-      <c r="J21" s="4">
-        <v>16</v>
-      </c>
-      <c r="K21" s="4">
-        <v>7</v>
-      </c>
       <c r="L21" s="1">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="22" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F21:K21)</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>420160</v>
+        <v>422000</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -5441,148 +5427,131 @@
       <c r="D22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E22" s="1"/>
       <c r="F22" s="4">
+        <v>34</v>
+      </c>
+      <c r="G22" s="4">
         <v>9</v>
       </c>
-      <c r="G22" s="4">
-        <v>16</v>
-      </c>
       <c r="H22" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I22" s="4">
-        <v>13</v>
-      </c>
-      <c r="J22" s="4">
+        <v>1</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="1">
+        <f>SUM(F22:K22)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="6">
+        <v>422701</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="K22" s="4">
-        <v>4</v>
-      </c>
-      <c r="L22" s="1">
-        <f t="shared" si="0"/>
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="6">
-        <v>423416</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="4">
+        <v>3</v>
+      </c>
+      <c r="G23" s="4">
+        <v>5</v>
+      </c>
+      <c r="H23" s="4">
+        <v>2</v>
+      </c>
+      <c r="I23" s="4">
         <v>10</v>
       </c>
-      <c r="G23" s="4">
-        <v>14</v>
-      </c>
-      <c r="H23" s="4">
-        <v>13</v>
-      </c>
-      <c r="I23" s="4">
+      <c r="J23" s="4">
+        <v>16</v>
+      </c>
+      <c r="K23" s="4">
+        <v>18</v>
+      </c>
+      <c r="L23" s="1">
+        <f>SUM(F23:K23)</f>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="6">
+        <v>420800</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" s="1"/>
+      <c r="F24" s="6">
+        <v>6</v>
+      </c>
+      <c r="G24" s="6">
+        <v>10</v>
+      </c>
+      <c r="H24" s="6">
+        <v>12</v>
+      </c>
+      <c r="I24" s="6">
+        <v>12</v>
+      </c>
+      <c r="J24" s="6">
+        <v>6</v>
+      </c>
+      <c r="K24" s="4">
+        <v>6</v>
+      </c>
+      <c r="L24" s="1">
+        <f>SUM(F24:K24)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="6">
+        <v>421400</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="1"/>
+      <c r="F25" s="4">
+        <v>7</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4">
+        <v>1</v>
+      </c>
+      <c r="I25" s="4">
+        <v>1</v>
+      </c>
+      <c r="J25" s="4">
         <v>11</v>
       </c>
-      <c r="J23" s="4">
-        <v>9</v>
-      </c>
-      <c r="K23" s="4">
-        <v>5</v>
-      </c>
-      <c r="L23" s="1">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-      <c r="M23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="24" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="6">
-        <v>423316</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="4">
-        <v>6</v>
-      </c>
-      <c r="G24" s="4">
-        <v>14</v>
-      </c>
-      <c r="H24" s="4">
-        <v>14</v>
-      </c>
-      <c r="I24" s="4">
-        <v>13</v>
-      </c>
-      <c r="J24" s="4">
-        <v>8</v>
-      </c>
-      <c r="K24" s="4">
-        <v>4</v>
-      </c>
-      <c r="L24" s="1">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="M24" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="25" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="6">
-        <v>424900</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F25" s="4">
-        <v>8</v>
-      </c>
-      <c r="G25" s="4">
-        <v>17</v>
-      </c>
-      <c r="H25" s="1">
-        <v>12</v>
-      </c>
-      <c r="I25" s="4">
-        <v>13</v>
-      </c>
-      <c r="J25" s="4">
-        <v>3</v>
-      </c>
       <c r="K25" s="4">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="L25" s="1">
-        <f t="shared" si="0"/>
-        <v>56</v>
-      </c>
-      <c r="M25" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F25:K25)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>422000</v>
+        <v>422101</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>7</v>
@@ -5592,638 +5561,647 @@
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="G26" s="4">
+        <v>1</v>
+      </c>
+      <c r="H26" s="4">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4">
         <v>9</v>
       </c>
-      <c r="H26" s="4">
-        <v>11</v>
-      </c>
-      <c r="I26" s="4">
-        <v>1</v>
-      </c>
-      <c r="J26" s="4"/>
+      <c r="J26" s="4">
+        <v>14</v>
+      </c>
       <c r="K26" s="4"/>
       <c r="L26" s="1">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-      <c r="M26" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="27" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F26:K26)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>422701</v>
+        <v>421801</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4">
+        <v>2</v>
+      </c>
+      <c r="H27" s="4">
         <v>8</v>
       </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="4">
-        <v>3</v>
-      </c>
-      <c r="G27" s="4">
-        <v>5</v>
-      </c>
-      <c r="H27" s="4">
-        <v>2</v>
-      </c>
       <c r="I27" s="4">
+        <v>8</v>
+      </c>
+      <c r="J27" s="4">
+        <v>20</v>
+      </c>
+      <c r="K27" s="4">
+        <v>12</v>
+      </c>
+      <c r="L27" s="1">
+        <f>SUM(F27:K27)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="6">
+        <v>420160</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J27" s="4">
-        <v>16</v>
-      </c>
-      <c r="K27" s="4">
-        <v>18</v>
-      </c>
-      <c r="L27" s="1">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="6">
-        <v>420800</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="6">
-        <v>6</v>
-      </c>
-      <c r="G28" s="6">
+      <c r="E28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="4">
+        <v>7</v>
+      </c>
+      <c r="G28" s="4">
+        <v>12</v>
+      </c>
+      <c r="H28" s="4">
+        <v>9</v>
+      </c>
+      <c r="I28" s="4">
         <v>10</v>
       </c>
-      <c r="H28" s="6">
-        <v>12</v>
-      </c>
-      <c r="I28" s="6">
-        <v>12</v>
-      </c>
-      <c r="J28" s="6">
+      <c r="J28" s="4">
         <v>6</v>
       </c>
       <c r="K28" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L28" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="29" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F28:K28)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>421400</v>
+        <v>424900</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>126</v>
+      </c>
       <c r="F29" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G29" s="4">
-        <v>0</v>
-      </c>
-      <c r="H29" s="4">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="H29" s="1">
+        <v>15</v>
       </c>
       <c r="I29" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J29" s="4">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K29" s="4">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="L29" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="M29" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="30" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F29:K29)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>422101</v>
+        <v>421100</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G30" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H30" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I30" s="4">
+        <v>7</v>
+      </c>
+      <c r="J30" s="4">
+        <v>20</v>
+      </c>
+      <c r="K30" s="4">
+        <v>7</v>
+      </c>
+      <c r="L30" s="1">
+        <f>SUM(F30:K30)</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="6">
+        <v>424700</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="1"/>
+      <c r="F31" s="4">
+        <v>19</v>
+      </c>
+      <c r="G31" s="4">
+        <v>8</v>
+      </c>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4">
         <v>9</v>
       </c>
-      <c r="J30" s="4">
-        <v>14</v>
-      </c>
-      <c r="K30" s="4"/>
-      <c r="L30" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="M30" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="31" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="6">
-        <v>421801</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4">
-        <v>2</v>
-      </c>
-      <c r="H31" s="4">
-        <v>8</v>
-      </c>
-      <c r="I31" s="4">
-        <v>8</v>
-      </c>
       <c r="J31" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K31" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L31" s="1">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="32" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F31:K31)</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>423304</v>
+        <v>424000</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="4">
-        <v>6</v>
-      </c>
-      <c r="G32" s="4">
+        <v>23</v>
+      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4">
+        <v>3</v>
+      </c>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4">
+        <v>16</v>
+      </c>
+      <c r="K32" s="4"/>
+      <c r="L32" s="1">
+        <f>SUM(F32:K32)</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="6">
+        <v>424300</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H32" s="6">
+      <c r="E33" s="1"/>
+      <c r="F33" s="4">
+        <v>1</v>
+      </c>
+      <c r="G33" s="4">
         <v>11</v>
       </c>
-      <c r="I32" s="4">
-        <v>7</v>
-      </c>
-      <c r="J32" s="4">
+      <c r="H33" s="4">
+        <v>9</v>
+      </c>
+      <c r="I33" s="4">
+        <v>9</v>
+      </c>
+      <c r="J33" s="4">
+        <v>1</v>
+      </c>
+      <c r="K33" s="4">
+        <v>8</v>
+      </c>
+      <c r="L33" s="1">
+        <f>SUM(F33:K33)</f>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34" s="6">
+        <v>422900</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="K32" s="4">
-        <v>5</v>
-      </c>
-      <c r="L32" s="1">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="6">
-        <v>424900</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F33" s="4">
-        <v>6</v>
-      </c>
-      <c r="G33" s="4">
-        <v>14</v>
-      </c>
-      <c r="H33" s="1">
-        <v>15</v>
-      </c>
-      <c r="I33" s="4">
-        <v>8</v>
-      </c>
-      <c r="J33" s="4">
-        <v>5</v>
-      </c>
-      <c r="K33" s="4">
-        <v>0</v>
-      </c>
-      <c r="L33" s="1">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="6">
-        <v>422200</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>1</v>
-      </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4">
-        <v>15</v>
-      </c>
-      <c r="I34" s="4">
-        <v>6</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="G34" s="4">
+        <v>1</v>
+      </c>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
       <c r="J34" s="4">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F34:K34)</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>424700</v>
+        <v>421401</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="G35" s="4">
+        <v>9</v>
+      </c>
+      <c r="H35" s="4">
+        <v>12</v>
+      </c>
+      <c r="I35" s="4">
+        <v>7</v>
+      </c>
+      <c r="J35" s="4">
+        <v>4</v>
+      </c>
+      <c r="K35" s="4">
+        <v>3</v>
+      </c>
+      <c r="L35" s="1">
+        <f>SUM(F35:K35)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B36" s="17">
+        <v>421000</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="6">
+        <v>3</v>
+      </c>
+      <c r="G36" s="6">
         <v>8</v>
       </c>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4">
+      <c r="H36" s="6">
         <v>9</v>
       </c>
-      <c r="J35" s="4">
-        <v>1</v>
-      </c>
-      <c r="K35" s="4">
-        <v>10</v>
-      </c>
-      <c r="L35" s="1">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="36" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="6">
-        <v>420101</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="4">
-        <v>7</v>
-      </c>
-      <c r="G36" s="4">
-        <v>12</v>
-      </c>
-      <c r="H36" s="4">
-        <v>11</v>
-      </c>
-      <c r="I36" s="4">
-        <v>10</v>
-      </c>
-      <c r="J36" s="4">
-        <v>1</v>
-      </c>
-      <c r="K36" s="4">
-        <v>3</v>
+      <c r="I36" s="6">
+        <v>8</v>
+      </c>
+      <c r="J36" s="6">
+        <v>4</v>
+      </c>
+      <c r="K36" s="6">
+        <v>2</v>
       </c>
       <c r="L36" s="1">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="37" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F36:K36)</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>423404</v>
+        <v>423308</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G37" s="4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H37" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I37" s="4">
         <v>6</v>
       </c>
       <c r="J37" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K37" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37" s="1">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F37:K37)</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>424000</v>
+        <v>423408</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="4">
-        <v>23</v>
-      </c>
-      <c r="G38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4">
+        <v>17</v>
+      </c>
       <c r="H38" s="4">
         <v>3</v>
       </c>
-      <c r="I38" s="4"/>
+      <c r="I38" s="4">
+        <v>5</v>
+      </c>
       <c r="J38" s="4">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="K38" s="4"/>
       <c r="L38" s="1">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="39" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F38:K38)</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>422900</v>
+        <v>423448</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="4">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="G39" s="4">
-        <v>1</v>
-      </c>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="H39" s="6">
+        <v>6</v>
+      </c>
+      <c r="I39" s="4">
+        <v>2</v>
+      </c>
       <c r="J39" s="4">
-        <v>2</v>
-      </c>
-      <c r="K39" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="K39" s="4">
+        <v>1</v>
+      </c>
       <c r="L39" s="1">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F39:K39)</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>421401</v>
+        <v>420101</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G40" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H40" s="4">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I40" s="4">
         <v>7</v>
       </c>
-      <c r="J40" s="4">
-        <v>4</v>
-      </c>
+      <c r="J40" s="4"/>
       <c r="K40" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L40" s="1">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="41" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F40:K40)</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>423308</v>
+        <v>422700</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="4">
+        <v>6</v>
+      </c>
+      <c r="G41" s="4">
+        <v>9</v>
+      </c>
+      <c r="H41" s="4">
+        <v>8</v>
+      </c>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4">
+        <v>6</v>
+      </c>
+      <c r="L41" s="1">
+        <f>SUM(F41:K41)</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B42" s="6">
+        <v>421901</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="F42" s="4">
+        <v>4</v>
+      </c>
+      <c r="G42" s="4">
+        <v>8</v>
+      </c>
+      <c r="H42" s="4">
+        <v>6</v>
+      </c>
+      <c r="I42" s="4">
+        <v>5</v>
+      </c>
+      <c r="J42" s="4">
+        <v>4</v>
+      </c>
+      <c r="K42" s="4">
+        <v>1</v>
+      </c>
+      <c r="L42" s="1">
+        <f>SUM(F42:K42)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B43" s="6">
+        <v>421301</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="1"/>
+      <c r="F43" s="4">
+        <v>4</v>
+      </c>
+      <c r="G43" s="4">
         <v>2</v>
       </c>
-      <c r="G41" s="4">
-        <v>8</v>
-      </c>
-      <c r="H41" s="4">
-        <v>5</v>
-      </c>
-      <c r="I41" s="4">
-        <v>6</v>
-      </c>
-      <c r="J41" s="4">
-        <v>11</v>
-      </c>
-      <c r="K41" s="4">
-        <v>2</v>
-      </c>
-      <c r="L41" s="1">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="M41" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="42" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="6">
-        <v>420801</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="1">
-        <f>SUM(G42:K42)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="6">
-        <v>420802</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
+      <c r="H43" s="4">
+        <v>9</v>
+      </c>
+      <c r="I43" s="4">
+        <v>5</v>
+      </c>
+      <c r="J43" s="4">
+        <v>6</v>
+      </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f>SUM(G43:K43)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F43:K43)</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>420900</v>
+        <v>424500</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4">
+      <c r="F44" s="4">
+        <v>7</v>
+      </c>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4">
+        <v>5</v>
+      </c>
+      <c r="I44" s="4">
+        <v>6</v>
+      </c>
+      <c r="J44" s="4">
         <v>8</v>
       </c>
-      <c r="H44" s="4">
-        <v>2</v>
-      </c>
-      <c r="I44" s="4">
-        <v>2</v>
-      </c>
-      <c r="J44" s="4">
-        <v>7</v>
-      </c>
-      <c r="K44" s="4">
-        <v>11</v>
-      </c>
+      <c r="K44" s="4"/>
       <c r="L44" s="1">
-        <f t="shared" ref="L44:L66" si="1">SUM(F44:K44)</f>
-        <v>30</v>
-      </c>
-      <c r="M44" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="45" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F44:K44)</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>422700</v>
+        <v>423348</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G45" s="4">
-        <v>9</v>
-      </c>
-      <c r="H45" s="4">
-        <v>8</v>
-      </c>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="H45" s="6">
+        <v>7</v>
+      </c>
+      <c r="I45" s="4">
+        <v>4</v>
+      </c>
+      <c r="J45" s="4">
+        <v>3</v>
+      </c>
       <c r="K45" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L45" s="1">
-        <f t="shared" si="1"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F45:K45)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421901</v>
+        <v>421902</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
@@ -6233,10 +6211,10 @@
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G46" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H46" s="4">
         <v>6</v>
@@ -6248,48 +6226,50 @@
         <v>4</v>
       </c>
       <c r="K46" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" s="1">
-        <f t="shared" si="1"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="47" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F46:K46)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>421301</v>
+        <v>423501</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G47" s="4">
+        <v>6</v>
+      </c>
+      <c r="H47" s="4">
+        <v>1</v>
+      </c>
+      <c r="I47" s="4">
+        <v>6</v>
+      </c>
+      <c r="J47" s="4">
         <v>2</v>
       </c>
-      <c r="H47" s="4">
-        <v>9</v>
-      </c>
-      <c r="I47" s="4">
-        <v>5</v>
-      </c>
-      <c r="J47" s="4">
-        <v>6</v>
-      </c>
-      <c r="K47" s="4"/>
+      <c r="K47" s="4">
+        <v>6</v>
+      </c>
       <c r="L47" s="1">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F47:K47)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>424500</v>
+        <v>421900</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
@@ -6299,27 +6279,29 @@
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>7</v>
-      </c>
-      <c r="G48" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="G48" s="4">
+        <v>5</v>
+      </c>
       <c r="H48" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I48" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J48" s="4">
         <v>8</v>
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F48:K48)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>423348</v>
+        <v>422190</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
@@ -6327,223 +6309,206 @@
       <c r="D49" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E49" s="1"/>
+      <c r="E49" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="F49" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H49" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I49" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J49" s="4">
         <v>3</v>
       </c>
       <c r="K49" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L49" s="1">
-        <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F49:K49)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>421902</v>
+        <v>424801</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" s="4">
-        <v>6</v>
-      </c>
-      <c r="H50" s="4">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="H50" s="4"/>
       <c r="I50" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J50" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" s="4">
         <v>2</v>
       </c>
       <c r="L50" s="1">
-        <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F50:K50)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>421800</v>
+        <v>420900</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4">
-        <v>1</v>
-      </c>
-      <c r="H51" s="4">
-        <v>8</v>
-      </c>
-      <c r="I51" s="4">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
       <c r="J51" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K51" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L51" s="1">
-        <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F51:K51)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>423501</v>
+        <v>420501</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H52" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I52" s="4">
-        <v>6</v>
-      </c>
-      <c r="J52" s="4">
-        <v>2</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="J52" s="4"/>
       <c r="K52" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L52" s="1">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F52:K52)</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>421900</v>
+        <v>423600</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" s="4">
-        <v>5</v>
-      </c>
-      <c r="H53" s="4">
-        <v>7</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="H53" s="4"/>
       <c r="I53" s="4">
+        <v>5</v>
+      </c>
+      <c r="J53" s="4">
+        <v>1</v>
+      </c>
+      <c r="K53" s="4">
+        <v>1</v>
+      </c>
+      <c r="L53" s="1">
+        <f>SUM(F53:K53)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B54" s="6">
+        <v>421800</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E54" s="1"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4">
+        <v>4</v>
+      </c>
+      <c r="I54" s="4">
         <v>3</v>
       </c>
-      <c r="J53" s="4">
-        <v>8</v>
-      </c>
-      <c r="K53" s="4"/>
-      <c r="L53" s="1">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="6">
-        <v>422190</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="1" t="s">
+      <c r="J54" s="4">
+        <v>4</v>
+      </c>
+      <c r="K54" s="4">
+        <v>2</v>
+      </c>
+      <c r="L54" s="1">
+        <f>SUM(F54:K54)</f>
         <v>13</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F54" s="4">
-        <v>2</v>
-      </c>
-      <c r="G54" s="4">
-        <v>5</v>
-      </c>
-      <c r="H54" s="6">
-        <v>5</v>
-      </c>
-      <c r="I54" s="4">
-        <v>5</v>
-      </c>
-      <c r="J54" s="4">
+    </row>
+    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B55" s="6">
+        <v>421402</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" s="1"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4">
         <v>3</v>
       </c>
-      <c r="K54" s="4">
-        <v>3</v>
-      </c>
-      <c r="L54" s="1">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="M54" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="6">
-        <v>423409</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E55" s="1"/>
-      <c r="F55" s="4">
-        <v>5</v>
-      </c>
-      <c r="G55" s="4">
+      <c r="H55" s="4">
+        <v>1</v>
+      </c>
+      <c r="I55" s="4">
         <v>4</v>
-      </c>
-      <c r="H55" s="4">
-        <v>5</v>
-      </c>
-      <c r="I55" s="4">
-        <v>1</v>
       </c>
       <c r="J55" s="4">
         <v>3</v>
@@ -6552,328 +6517,313 @@
         <v>2</v>
       </c>
       <c r="L55" s="1">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F55:K55)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>424801</v>
+        <v>423304</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E56" s="1"/>
-      <c r="F56" s="4">
-        <v>3</v>
-      </c>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4">
-        <v>8</v>
-      </c>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4">
+        <v>2</v>
+      </c>
+      <c r="H56" s="6"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>8</v>
-      </c>
-      <c r="K56" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="K56" s="4">
+        <v>2</v>
+      </c>
       <c r="L56" s="1">
-        <f t="shared" si="1"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F56:K56)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>424300</v>
+        <v>421300</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G57" s="4"/>
-      <c r="H57" s="4">
-        <v>1</v>
-      </c>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4">
-        <v>7</v>
-      </c>
-      <c r="K57" s="4"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="4">
+        <v>4</v>
+      </c>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4">
+        <v>4</v>
+      </c>
       <c r="L57" s="1">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F57:K57)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>423600</v>
+        <v>422601</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="4">
-        <v>1</v>
-      </c>
-      <c r="G58" s="4">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G58" s="4"/>
       <c r="H58" s="4"/>
-      <c r="I58" s="4">
-        <v>5</v>
-      </c>
+      <c r="I58" s="4"/>
       <c r="J58" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K58" s="4">
         <v>1</v>
       </c>
       <c r="L58" s="1">
-        <f t="shared" si="1"/>
-        <v>14</v>
+        <f>SUM(F58:K58)</f>
+        <v>10</v>
       </c>
       <c r="P58" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>421402</v>
+        <v>423309</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4">
+        <v>1</v>
+      </c>
+      <c r="H59" s="4">
+        <v>1</v>
+      </c>
+      <c r="I59" s="4">
+        <v>1</v>
+      </c>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+      <c r="L59" s="1">
+        <f>SUM(F59:K59)</f>
         <v>3</v>
       </c>
-      <c r="H59" s="4">
-        <v>1</v>
-      </c>
-      <c r="I59" s="4">
-        <v>4</v>
-      </c>
-      <c r="J59" s="4">
-        <v>3</v>
-      </c>
-      <c r="K59" s="4">
-        <v>2</v>
-      </c>
-      <c r="L59" s="1">
-        <f t="shared" si="1"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
-        <v>421300</v>
+        <v>420200</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="4">
-        <v>2</v>
-      </c>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="G60" s="4">
+        <v>60</v>
+      </c>
+      <c r="H60" s="4">
+        <v>40</v>
+      </c>
       <c r="I60" s="4">
-        <v>4</v>
-      </c>
-      <c r="J60" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="J60" s="4">
+        <v>30</v>
+      </c>
       <c r="K60" s="4">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="L60" s="1">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F60:K60)</f>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
-        <v>422601</v>
+        <v>420402</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E61" s="1"/>
-      <c r="F61" s="4">
-        <v>5</v>
-      </c>
+      <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="4">
-        <v>4</v>
-      </c>
-      <c r="K61" s="4">
-        <v>1</v>
-      </c>
+      <c r="J61" s="4"/>
+      <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="M61" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F61:K61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
-        <v>420402</v>
+        <v>424960</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
+      <c r="H62" s="6"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="4">
-        <v>6</v>
-      </c>
+      <c r="J62" s="4"/>
       <c r="K62" s="4"/>
-      <c r="L62" s="1">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="L62" s="12">
+        <f>SUM(F62:K62)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
-        <v>424960</v>
+        <v>423409</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E63" s="1"/>
-      <c r="F63" s="4">
-        <v>2</v>
-      </c>
-      <c r="G63" s="4">
-        <v>1</v>
-      </c>
-      <c r="H63" s="6">
-        <v>0</v>
-      </c>
-      <c r="I63" s="4">
-        <v>0</v>
-      </c>
-      <c r="J63" s="4">
-        <v>1</v>
-      </c>
-      <c r="K63" s="4">
-        <v>1</v>
-      </c>
-      <c r="L63" s="12">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4"/>
+      <c r="L63" s="1">
+        <f>SUM(F63:K63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
-        <v>423309</v>
+        <v>420160</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="F64" s="4"/>
-      <c r="G64" s="4">
-        <v>1</v>
-      </c>
-      <c r="H64" s="4">
-        <v>1</v>
-      </c>
-      <c r="I64" s="4">
-        <v>1</v>
-      </c>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
       <c r="J64" s="4"/>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="65" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F64:K64)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
-        <v>420160</v>
+        <v>423404</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="E65" s="1"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
-      <c r="K65" s="4">
-        <v>2</v>
-      </c>
+      <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+        <f>SUM(F65:K65)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
-        <v>420200</v>
+        <v>420801</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E66" s="1"/>
-      <c r="F66" s="4">
-        <v>1</v>
-      </c>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
-      <c r="J66" s="4"/>
-      <c r="K66" s="4">
-        <v>1</v>
-      </c>
+      <c r="F66" s="1"/>
+      <c r="G66" s="6"/>
+      <c r="H66" s="6"/>
+      <c r="I66" s="6"/>
+      <c r="J66" s="6"/>
+      <c r="K66" s="4"/>
       <c r="L66" s="1">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>SUM(G66:K66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B67" s="6">
+        <v>420802</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="4"/>
+      <c r="H67" s="4"/>
+      <c r="I67" s="4"/>
+      <c r="J67" s="4"/>
+      <c r="K67" s="4"/>
+      <c r="L67" s="1">
+        <f>SUM(G67:K67)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="2:12" x14ac:dyDescent="0.25">
@@ -6882,7 +6832,12 @@
       </c>
       <c r="L69" s="10">
         <f>SUM(L3:L66)</f>
-        <v>3903</v>
+        <v>3676</v>
+      </c>
+    </row>
+    <row r="73" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E73" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="127" spans="11:11" x14ac:dyDescent="0.25">
@@ -6891,14 +6846,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L66" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="424701"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B15:L15">
-      <sortCondition descending="1" ref="L2:L66"/>
+  <autoFilter ref="B2:L67" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L67">
+      <sortCondition descending="1" ref="L2:L67"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6912,6 +6862,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7055,32 +7014,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7096,12 +7054,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar dashboard, stock y datos web
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1654" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE73E74C-57C4-4700-9B77-FB42ABCE2AE8}"/>
+  <xr:revisionPtr revIDLastSave="2221" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{429EDF48-F1A8-46EE-B657-836D4D401900}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="131">
   <si>
     <t>CODIGO</t>
   </si>
@@ -96,9 +96,6 @@
     <t>CLARO</t>
   </si>
   <si>
-    <t>OSURO</t>
-  </si>
-  <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
   <si>
@@ -432,13 +429,19 @@
     <t>negro</t>
   </si>
   <si>
-    <t xml:space="preserve">   </t>
-  </si>
-  <si>
     <t xml:space="preserve">  </t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 18:19   21-04</t>
+    <t xml:space="preserve">MEDIO </t>
+  </si>
+  <si>
+    <t>OSCURO</t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 17:14  29-04</t>
+  </si>
+  <si>
+    <t>REVISADO</t>
   </si>
 </sst>
 </file>
@@ -561,7 +564,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -605,6 +608,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -990,7 +994,7 @@
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -1040,7 +1044,7 @@
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
@@ -1070,7 +1074,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
@@ -1098,7 +1102,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -1126,7 +1130,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -1152,7 +1156,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>5</v>
@@ -1180,7 +1184,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -1204,10 +1208,10 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -1234,7 +1238,7 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>5</v>
@@ -1258,7 +1262,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -1284,7 +1288,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -1312,7 +1316,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -1346,7 +1350,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>7</v>
@@ -1372,7 +1376,7 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>7</v>
@@ -1396,7 +1400,7 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>7</v>
@@ -1428,7 +1432,7 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>7</v>
@@ -1452,7 +1456,7 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>7</v>
@@ -1480,7 +1484,7 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>7</v>
@@ -1512,7 +1516,7 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>7</v>
@@ -1536,7 +1540,7 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>7</v>
@@ -1560,7 +1564,7 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>5</v>
@@ -1584,7 +1588,7 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>5</v>
@@ -1608,7 +1612,7 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>7</v>
@@ -1632,7 +1636,7 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>7</v>
@@ -1656,7 +1660,7 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>5</v>
@@ -1682,7 +1686,7 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>7</v>
@@ -1708,10 +1712,10 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>32</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>33</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
@@ -1730,10 +1734,10 @@
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
@@ -1752,7 +1756,7 @@
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>7</v>
@@ -1789,7 +1793,7 @@
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -2396,7 +2400,7 @@
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -2446,10 +2450,10 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>58</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>8</v>
@@ -2480,7 +2484,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -2510,7 +2514,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -2540,7 +2544,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -2570,7 +2574,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -2598,7 +2602,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -2608,7 +2612,7 @@
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
@@ -2619,12 +2623,12 @@
       <c r="K10" s="9"/>
       <c r="L10" s="9">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
@@ -2652,7 +2656,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -2678,7 +2682,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -2702,7 +2706,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -2726,7 +2730,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>7</v>
@@ -2760,10 +2764,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFAA1C20-0AB4-435A-AEDE-B6C824B1C346}">
   <dimension ref="B3:L49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -2813,7 +2820,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
@@ -2847,7 +2854,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -2881,7 +2888,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -2915,7 +2922,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -2949,7 +2956,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>7</v>
@@ -2983,7 +2990,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -3017,13 +3024,13 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>68</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9">
@@ -3051,7 +3058,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>5</v>
@@ -3085,7 +3092,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -3119,7 +3126,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>7</v>
@@ -3153,7 +3160,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>7</v>
@@ -3187,7 +3194,7 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>7</v>
@@ -3221,7 +3228,7 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>7</v>
@@ -3255,7 +3262,7 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>5</v>
@@ -3289,7 +3296,7 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>7</v>
@@ -3323,7 +3330,7 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>7</v>
@@ -3357,7 +3364,7 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>5</v>
@@ -3391,7 +3398,7 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>7</v>
@@ -3425,7 +3432,7 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>5</v>
@@ -3459,7 +3466,7 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>5</v>
@@ -3493,7 +3500,7 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>7</v>
@@ -3527,13 +3534,13 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>84</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9">
@@ -3561,7 +3568,7 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>7</v>
@@ -3595,7 +3602,7 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>7</v>
@@ -3629,13 +3636,13 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9">
@@ -3663,7 +3670,7 @@
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>5</v>
@@ -3697,7 +3704,7 @@
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>7</v>
@@ -3731,7 +3738,7 @@
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>7</v>
@@ -3765,7 +3772,7 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>5</v>
@@ -3799,7 +3806,7 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>7</v>
@@ -3833,7 +3840,7 @@
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>7</v>
@@ -3867,13 +3874,13 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9">
@@ -3901,7 +3908,7 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>7</v>
@@ -3935,7 +3942,7 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>7</v>
@@ -3969,7 +3976,7 @@
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>7</v>
@@ -4003,7 +4010,7 @@
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>7</v>
@@ -4037,7 +4044,7 @@
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>7</v>
@@ -4071,13 +4078,13 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9">
@@ -4105,7 +4112,7 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>5</v>
@@ -4139,7 +4146,7 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>7</v>
@@ -4173,7 +4180,7 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>7</v>
@@ -4207,7 +4214,7 @@
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>7</v>
@@ -4241,13 +4248,13 @@
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="E47" s="9"/>
       <c r="F47" s="9">
@@ -4275,13 +4282,13 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="E48" s="9"/>
       <c r="F48" s="9">
@@ -4309,7 +4316,7 @@
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>7</v>
@@ -4351,12 +4358,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E9EB22C-7ED7-4D45-8EA1-BD18A384D586}">
-  <dimension ref="B3:L13"/>
+  <dimension ref="B3:L17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -4406,10 +4413,10 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>113</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>114</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>6</v>
@@ -4440,7 +4447,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -4472,7 +4479,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -4506,7 +4513,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>5</v>
@@ -4540,7 +4547,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>5</v>
@@ -4574,7 +4581,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>7</v>
@@ -4608,7 +4615,7 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>7</v>
@@ -4642,7 +4649,7 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>7</v>
@@ -4676,7 +4683,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>7</v>
@@ -4706,6 +4713,11 @@
       <c r="L13" s="9">
         <f t="shared" si="0"/>
         <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -4718,13 +4730,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="B2:P127"/>
+  <dimension ref="A2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4759,43 +4771,49 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
       <c r="B3" s="6">
-        <v>420100</v>
+        <v>423600</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="G3" s="4">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H3" s="4">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="I3" s="4">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J3" s="4">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K3" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="L3" s="1">
         <f>SUM(F3:K3)</f>
-        <v>251</v>
-      </c>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+      <c r="M3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>423500</v>
+        <v>420100</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -4805,29 +4823,32 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="G4" s="4">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="H4" s="4">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="I4" s="4">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="J4" s="4">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="K4" s="4">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>234</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>126</v>
+      </c>
       <c r="B5" s="6">
         <v>422200</v>
       </c>
@@ -4839,510 +4860,527 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5" s="4">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H5" s="4">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I5" s="4">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J5" s="4">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K5" s="4">
         <v>15</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
-        <v>420600</v>
+        <v>423800</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="4">
-        <v>42</v>
-      </c>
-      <c r="G6" s="4">
-        <v>29</v>
-      </c>
-      <c r="H6" s="4">
-        <v>18</v>
-      </c>
-      <c r="I6" s="4">
-        <v>23</v>
-      </c>
-      <c r="J6" s="4">
-        <v>31</v>
-      </c>
-      <c r="K6" s="4">
-        <v>17</v>
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="6">
+        <v>15</v>
+      </c>
+      <c r="G6" s="6">
+        <v>36</v>
+      </c>
+      <c r="H6" s="6">
+        <v>40</v>
+      </c>
+      <c r="I6" s="6">
+        <v>36</v>
+      </c>
+      <c r="J6" s="6">
+        <v>20</v>
+      </c>
+      <c r="K6" s="6">
+        <v>16</v>
       </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="N6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>422500</v>
+        <v>423500</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G7" s="4">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="H7" s="4">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="I7" s="4">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J7" s="4">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="K7" s="4">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L7" s="1">
         <f>SUM(F7:K7)</f>
-        <v>151</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>422100</v>
+        <v>420301</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="4">
-        <v>12</v>
-      </c>
-      <c r="G8" s="4">
-        <v>29</v>
-      </c>
-      <c r="H8" s="4">
-        <v>30</v>
-      </c>
-      <c r="I8" s="4">
-        <v>27</v>
-      </c>
-      <c r="J8" s="4">
-        <v>20</v>
-      </c>
-      <c r="K8" s="4">
-        <v>23</v>
+      <c r="F8" s="6">
+        <v>14</v>
+      </c>
+      <c r="G8" s="6">
+        <v>32</v>
+      </c>
+      <c r="H8" s="6">
+        <v>34</v>
+      </c>
+      <c r="I8" s="6">
+        <v>36</v>
+      </c>
+      <c r="J8" s="6">
+        <v>18</v>
+      </c>
+      <c r="K8" s="6">
+        <v>8</v>
       </c>
       <c r="L8" s="1">
         <f>SUM(F8:K8)</f>
-        <v>141</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="M8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>424400</v>
+        <v>422500</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G9" s="4">
+        <v>11</v>
+      </c>
+      <c r="H9" s="4">
+        <v>43</v>
+      </c>
+      <c r="I9" s="4">
         <v>32</v>
       </c>
-      <c r="H9" s="4">
-        <v>29</v>
-      </c>
-      <c r="I9" s="4">
-        <v>36</v>
-      </c>
       <c r="J9" s="4">
-        <v>7</v>
-      </c>
-      <c r="K9" s="4">
-        <v>0</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="K9" s="4"/>
       <c r="L9" s="1">
         <f>SUM(F9:K9)</f>
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>123</v>
+      </c>
       <c r="B10" s="6">
-        <v>422800</v>
+        <v>420600</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="4">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="G10" s="4">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H10" s="4">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="I10" s="4">
         <v>17</v>
       </c>
       <c r="J10" s="4">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="K10" s="4">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="L10" s="1">
         <f>SUM(F10:K10)</f>
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="O10" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>424600</v>
+        <v>422800</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="4">
-        <v>8</v>
-      </c>
+      <c r="F11" s="4"/>
       <c r="G11" s="4">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="H11" s="4">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="I11" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J11" s="4">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="K11" s="4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(F11:K11)</f>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+      <c r="O11" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>422300</v>
+        <v>424400</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G12" s="4">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="I12" s="4">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="J12" s="4">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="1">
         <f>SUM(F12:K12)</f>
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+      <c r="N12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>423000</v>
+        <v>424701</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G13" s="4">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H13" s="4">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="I13" s="4">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J13" s="4">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="K13" s="4">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="L13" s="1">
         <f>SUM(F13:K13)</f>
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="O13" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>123</v>
+      </c>
       <c r="B14" s="6">
-        <v>423200</v>
+        <v>422300</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G14" s="4">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H14" s="4">
+        <v>11</v>
+      </c>
+      <c r="I14" s="4">
         <v>19</v>
       </c>
-      <c r="I14" s="4">
+      <c r="J14" s="4">
         <v>16</v>
       </c>
-      <c r="J14" s="4">
-        <v>14</v>
-      </c>
-      <c r="K14" s="4">
-        <v>21</v>
-      </c>
+      <c r="K14" s="4"/>
       <c r="L14" s="1">
         <f>SUM(F14:K14)</f>
-        <v>95</v>
-      </c>
-      <c r="O14" s="13"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="O14" s="13" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>123</v>
+      </c>
       <c r="B15" s="6">
-        <v>424701</v>
+        <v>423000</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="4">
         <v>10</v>
       </c>
       <c r="G15" s="4">
+        <v>3</v>
+      </c>
+      <c r="H15" s="4">
+        <v>8</v>
+      </c>
+      <c r="I15" s="4">
         <v>14</v>
       </c>
-      <c r="H15" s="4">
-        <v>26</v>
-      </c>
-      <c r="I15" s="4">
-        <v>11</v>
-      </c>
       <c r="J15" s="4">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="K15" s="4">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="L15" s="1">
         <f>SUM(F15:K15)</f>
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>420500</v>
+        <v>423200</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="6">
-        <v>5</v>
-      </c>
-      <c r="G16" s="6">
-        <v>16</v>
-      </c>
-      <c r="H16" s="6">
-        <v>26</v>
+      <c r="F16" s="4">
+        <v>13</v>
+      </c>
+      <c r="G16" s="4">
+        <v>11</v>
+      </c>
+      <c r="H16" s="4">
+        <v>17</v>
       </c>
       <c r="I16" s="4">
-        <v>16</v>
-      </c>
-      <c r="J16" s="6">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="J16" s="4">
+        <v>12</v>
       </c>
       <c r="K16" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="L16" s="1">
         <f>SUM(F16:K16)</f>
-        <v>87</v>
+        <v>81</v>
+      </c>
+      <c r="O16" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423900</v>
+        <v>420300</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="4">
+      <c r="F17" s="6">
         <v>13</v>
       </c>
-      <c r="G17" s="4">
-        <v>12</v>
-      </c>
-      <c r="H17" s="4">
-        <v>4</v>
-      </c>
-      <c r="I17" s="4">
+      <c r="G17" s="6">
+        <v>15</v>
+      </c>
+      <c r="H17" s="6">
         <v>16</v>
       </c>
-      <c r="J17" s="4">
-        <v>16</v>
-      </c>
-      <c r="K17" s="4">
-        <v>7</v>
-      </c>
-      <c r="L17" s="1">
+      <c r="I17" s="6">
+        <v>15</v>
+      </c>
+      <c r="J17" s="6">
+        <v>11</v>
+      </c>
+      <c r="K17" s="6">
+        <v>10</v>
+      </c>
+      <c r="L17" s="12">
         <f>SUM(F17:K17)</f>
-        <v>68</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>424900</v>
+        <v>422100</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>125</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E18" s="1"/>
       <c r="F18" s="4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G18" s="4">
+        <v>14</v>
+      </c>
+      <c r="H18" s="4">
+        <v>16</v>
+      </c>
+      <c r="I18" s="4">
+        <v>14</v>
+      </c>
+      <c r="J18" s="4">
+        <v>10</v>
+      </c>
+      <c r="K18" s="4">
         <v>17</v>
-      </c>
-      <c r="H18" s="6">
-        <v>12</v>
-      </c>
-      <c r="I18" s="4">
-        <v>13</v>
-      </c>
-      <c r="J18" s="4">
-        <v>9</v>
-      </c>
-      <c r="K18" s="4">
-        <v>6</v>
       </c>
       <c r="L18" s="1">
         <f>SUM(F18:K18)</f>
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>420400</v>
+        <v>423900</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G19" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H19" s="4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I19" s="4">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="J19" s="4">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="K19" s="4">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L19" s="1">
         <f>SUM(F19:K19)</f>
@@ -5351,271 +5389,279 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>423416</v>
+        <v>420400</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="4">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G20" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H20" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I20" s="4">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J20" s="4">
         <v>9</v>
       </c>
       <c r="K20" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L20" s="1">
         <f>SUM(F20:K20)</f>
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>423316</v>
+        <v>424200</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="6">
+        <v>7</v>
+      </c>
+      <c r="G21" s="6">
         <v>13</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="4">
-        <v>6</v>
-      </c>
-      <c r="G21" s="4">
-        <v>14</v>
-      </c>
-      <c r="H21" s="4">
-        <v>14</v>
-      </c>
-      <c r="I21" s="4">
-        <v>13</v>
-      </c>
-      <c r="J21" s="4">
-        <v>8</v>
-      </c>
-      <c r="K21" s="4">
+      <c r="H21" s="6">
+        <v>12</v>
+      </c>
+      <c r="I21" s="6">
+        <v>22</v>
+      </c>
+      <c r="J21" s="6">
         <v>4</v>
       </c>
-      <c r="L21" s="1">
+      <c r="K21" s="6">
+        <v>6</v>
+      </c>
+      <c r="L21" s="12">
         <f>SUM(F21:K21)</f>
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>422000</v>
+        <v>424600</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="4">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="G22" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H22" s="4">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I22" s="4">
-        <v>1</v>
-      </c>
-      <c r="J22" s="4"/>
+        <v>17</v>
+      </c>
+      <c r="J22" s="4">
+        <v>17</v>
+      </c>
       <c r="K22" s="4"/>
       <c r="L22" s="1">
         <f>SUM(F22:K22)</f>
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>422701</v>
+        <v>423416</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G23" s="4">
+        <v>14</v>
+      </c>
+      <c r="H23" s="4">
+        <v>13</v>
+      </c>
+      <c r="I23" s="4">
+        <v>11</v>
+      </c>
+      <c r="J23" s="4">
+        <v>9</v>
+      </c>
+      <c r="K23" s="4">
         <v>5</v>
-      </c>
-      <c r="H23" s="4">
-        <v>2</v>
-      </c>
-      <c r="I23" s="4">
-        <v>10</v>
-      </c>
-      <c r="J23" s="4">
-        <v>16</v>
-      </c>
-      <c r="K23" s="4">
-        <v>18</v>
       </c>
       <c r="L23" s="1">
         <f>SUM(F23:K23)</f>
-        <v>54</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>420800</v>
+        <v>422601</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="6">
-        <v>6</v>
-      </c>
-      <c r="G24" s="6">
-        <v>10</v>
-      </c>
-      <c r="H24" s="6">
-        <v>12</v>
-      </c>
-      <c r="I24" s="6">
-        <v>12</v>
-      </c>
-      <c r="J24" s="6">
-        <v>6</v>
+      <c r="F24" s="4">
+        <v>6</v>
+      </c>
+      <c r="G24" s="4">
+        <v>13</v>
+      </c>
+      <c r="H24" s="4">
+        <v>9</v>
+      </c>
+      <c r="I24" s="4">
+        <v>7</v>
+      </c>
+      <c r="J24" s="4">
+        <v>18</v>
       </c>
       <c r="K24" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L24" s="1">
         <f>SUM(F24:K24)</f>
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>421400</v>
+        <v>423316</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G25" s="4">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H25" s="4">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="I25" s="4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J25" s="4">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K25" s="4">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="L25" s="1">
         <f>SUM(F25:K25)</f>
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>422101</v>
+        <v>424900</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="F26" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G26" s="4">
-        <v>1</v>
-      </c>
-      <c r="H26" s="4">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="H26" s="6">
+        <v>18</v>
       </c>
       <c r="I26" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J26" s="4">
-        <v>14</v>
-      </c>
-      <c r="K26" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="K26" s="4">
+        <v>4</v>
+      </c>
       <c r="L26" s="1">
         <f>SUM(F26:K26)</f>
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>421801</v>
+        <v>425600</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E27" s="1"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4">
-        <v>2</v>
-      </c>
-      <c r="H27" s="4">
-        <v>8</v>
-      </c>
-      <c r="I27" s="4">
-        <v>8</v>
-      </c>
-      <c r="J27" s="4">
-        <v>20</v>
-      </c>
-      <c r="K27" s="4">
-        <v>12</v>
+      <c r="F27" s="6">
+        <v>10</v>
+      </c>
+      <c r="G27" s="6">
+        <v>11</v>
+      </c>
+      <c r="H27" s="6">
+        <v>9</v>
+      </c>
+      <c r="I27" s="6">
+        <v>11</v>
+      </c>
+      <c r="J27" s="6">
+        <v>5</v>
+      </c>
+      <c r="K27" s="6">
+        <v>10</v>
       </c>
       <c r="L27" s="1">
         <f>SUM(F27:K27)</f>
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>420160</v>
+        <v>422000</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
@@ -5623,165 +5669,161 @@
       <c r="D28" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="4">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="G28" s="4">
+        <v>9</v>
+      </c>
+      <c r="H28" s="4">
         <v>12</v>
       </c>
-      <c r="H28" s="4">
-        <v>9</v>
-      </c>
       <c r="I28" s="4">
-        <v>10</v>
-      </c>
-      <c r="J28" s="4">
-        <v>6</v>
-      </c>
-      <c r="K28" s="4">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
       <c r="L28" s="1">
         <f>SUM(F28:K28)</f>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>424900</v>
+        <v>422101</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="1"/>
+      <c r="F29" s="4">
+        <v>14</v>
+      </c>
+      <c r="G29" s="4">
+        <v>1</v>
+      </c>
+      <c r="H29" s="4">
+        <v>14</v>
+      </c>
+      <c r="I29" s="4">
         <v>9</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F29" s="4">
-        <v>6</v>
-      </c>
-      <c r="G29" s="4">
+      <c r="J29" s="4">
         <v>14</v>
       </c>
-      <c r="H29" s="1">
-        <v>15</v>
-      </c>
-      <c r="I29" s="4">
-        <v>8</v>
-      </c>
-      <c r="J29" s="4">
-        <v>5</v>
-      </c>
-      <c r="K29" s="4">
-        <v>0</v>
-      </c>
+      <c r="K29" s="4"/>
       <c r="L29" s="1">
         <f>SUM(F29:K29)</f>
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>421100</v>
+        <v>421400</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G30" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I30" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J30" s="4">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="K30" s="4">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="L30" s="1">
         <f>SUM(F30:K30)</f>
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>424700</v>
+        <v>420800</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E31" s="1"/>
-      <c r="F31" s="4">
-        <v>19</v>
-      </c>
-      <c r="G31" s="4">
-        <v>8</v>
-      </c>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4">
-        <v>9</v>
-      </c>
-      <c r="J31" s="4">
-        <v>1</v>
+      <c r="F31" s="6">
+        <v>6</v>
+      </c>
+      <c r="G31" s="6">
+        <v>10</v>
+      </c>
+      <c r="H31" s="6">
+        <v>12</v>
+      </c>
+      <c r="I31" s="6">
+        <v>12</v>
+      </c>
+      <c r="J31" s="6">
+        <v>6</v>
       </c>
       <c r="K31" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L31" s="1">
         <f>SUM(F31:K31)</f>
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>424000</v>
+        <v>421801</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="4">
-        <v>23</v>
-      </c>
-      <c r="G32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4">
+        <v>2</v>
+      </c>
       <c r="H32" s="4">
-        <v>3</v>
-      </c>
-      <c r="I32" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="I32" s="4">
+        <v>8</v>
+      </c>
       <c r="J32" s="4">
-        <v>16</v>
-      </c>
-      <c r="K32" s="4"/>
+        <v>20</v>
+      </c>
+      <c r="K32" s="4">
+        <v>12</v>
+      </c>
       <c r="L32" s="1">
         <f>SUM(F32:K32)</f>
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>424300</v>
+        <v>420160</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
@@ -5789,227 +5831,223 @@
       <c r="D33" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E33" s="1"/>
+      <c r="E33" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F33" s="4">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G33" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H33" s="4">
         <v>9</v>
       </c>
       <c r="I33" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J33" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K33" s="4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L33" s="1">
         <f>SUM(F33:K33)</f>
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>422900</v>
+        <v>424700</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G34" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
+      <c r="I34" s="4">
+        <v>9</v>
+      </c>
       <c r="J34" s="4">
-        <v>2</v>
-      </c>
-      <c r="K34" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K34" s="4">
+        <v>10</v>
+      </c>
       <c r="L34" s="1">
         <f>SUM(F34:K34)</f>
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>421401</v>
+        <v>421100</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G35" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H35" s="4">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I35" s="4">
         <v>7</v>
       </c>
       <c r="J35" s="4">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="K35" s="4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L35" s="1">
         <f>SUM(F35:K35)</f>
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="17">
-        <v>421000</v>
-      </c>
-      <c r="C36" s="18" t="s">
+      <c r="B36" s="6">
+        <v>420200</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4">
         <v>5</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="H36" s="4">
+        <v>4</v>
+      </c>
+      <c r="I36" s="4">
         <v>12</v>
       </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="6">
-        <v>3</v>
-      </c>
-      <c r="G36" s="6">
+      <c r="J36" s="4">
         <v>8</v>
       </c>
-      <c r="H36" s="6">
-        <v>9</v>
-      </c>
-      <c r="I36" s="6">
-        <v>8</v>
-      </c>
-      <c r="J36" s="6">
-        <v>4</v>
-      </c>
-      <c r="K36" s="6">
-        <v>2</v>
+      <c r="K36" s="4">
+        <v>16</v>
       </c>
       <c r="L36" s="1">
         <f>SUM(F36:K36)</f>
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>423308</v>
+        <v>424000</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>2</v>
-      </c>
-      <c r="G37" s="4">
-        <v>8</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="G37" s="4"/>
       <c r="H37" s="4">
-        <v>5</v>
-      </c>
-      <c r="I37" s="4">
-        <v>6</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I37" s="4"/>
       <c r="J37" s="4">
-        <v>11</v>
-      </c>
-      <c r="K37" s="4">
-        <v>2</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="K37" s="4"/>
       <c r="L37" s="1">
         <f>SUM(F37:K37)</f>
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>423408</v>
+        <v>422701</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="4"/>
+      <c r="F38" s="4">
+        <v>1</v>
+      </c>
       <c r="G38" s="4">
-        <v>17</v>
-      </c>
-      <c r="H38" s="4">
         <v>3</v>
       </c>
+      <c r="H38" s="4"/>
       <c r="I38" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J38" s="4">
-        <v>6</v>
-      </c>
-      <c r="K38" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="K38" s="4">
+        <v>16</v>
+      </c>
       <c r="L38" s="1">
         <f>SUM(F38:K38)</f>
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>423448</v>
+        <v>422600</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>9</v>
+        <v>127</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E39" s="1"/>
-      <c r="F39" s="4">
+      <c r="F39" s="6"/>
+      <c r="G39" s="6">
+        <v>12</v>
+      </c>
+      <c r="H39" s="6">
+        <v>15</v>
+      </c>
+      <c r="I39" s="6">
+        <v>10</v>
+      </c>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6">
         <v>3</v>
-      </c>
-      <c r="G39" s="4">
-        <v>8</v>
-      </c>
-      <c r="H39" s="6">
-        <v>6</v>
-      </c>
-      <c r="I39" s="4">
-        <v>2</v>
-      </c>
-      <c r="J39" s="4">
-        <v>9</v>
-      </c>
-      <c r="K39" s="4">
-        <v>1</v>
       </c>
       <c r="L39" s="1">
         <f>SUM(F39:K39)</f>
-        <v>29</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>420101</v>
+        <v>424300</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
@@ -6019,257 +6057,259 @@
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4">
+        <v>11</v>
+      </c>
+      <c r="H40" s="4">
+        <v>9</v>
+      </c>
+      <c r="I40" s="4">
+        <v>9</v>
+      </c>
+      <c r="J40" s="4">
+        <v>1</v>
+      </c>
+      <c r="K40" s="4">
         <v>8</v>
-      </c>
-      <c r="H40" s="4">
-        <v>7</v>
-      </c>
-      <c r="I40" s="4">
-        <v>7</v>
-      </c>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4">
-        <v>2</v>
       </c>
       <c r="L40" s="1">
         <f>SUM(F40:K40)</f>
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>422700</v>
+        <v>424900</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E41" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="F41" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G41" s="4">
-        <v>9</v>
-      </c>
-      <c r="H41" s="4">
-        <v>8</v>
-      </c>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="H41" s="1">
+        <v>13</v>
+      </c>
+      <c r="I41" s="4">
+        <v>6</v>
+      </c>
+      <c r="J41" s="4">
+        <v>3</v>
+      </c>
       <c r="K41" s="4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L41" s="1">
         <f>SUM(F41:K41)</f>
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>421901</v>
+        <v>421401</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G42" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H42" s="4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I42" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J42" s="4">
         <v>4</v>
       </c>
       <c r="K42" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L42" s="1">
         <f>SUM(F42:K42)</f>
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>421301</v>
+        <v>421000</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="4">
+      <c r="F43" s="6">
+        <v>3</v>
+      </c>
+      <c r="G43" s="6">
+        <v>8</v>
+      </c>
+      <c r="H43" s="6">
+        <v>9</v>
+      </c>
+      <c r="I43" s="6">
+        <v>8</v>
+      </c>
+      <c r="J43" s="6">
         <v>4</v>
       </c>
-      <c r="G43" s="4">
+      <c r="K43" s="6">
         <v>2</v>
       </c>
-      <c r="H43" s="4">
-        <v>9</v>
-      </c>
-      <c r="I43" s="4">
-        <v>5</v>
-      </c>
-      <c r="J43" s="4">
-        <v>6</v>
-      </c>
-      <c r="K43" s="4"/>
       <c r="L43" s="1">
         <f>SUM(F43:K43)</f>
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>424500</v>
+        <v>423408</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="4">
-        <v>7</v>
-      </c>
-      <c r="G44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4">
+        <v>17</v>
+      </c>
       <c r="H44" s="4">
+        <v>3</v>
+      </c>
+      <c r="I44" s="4">
         <v>5</v>
       </c>
-      <c r="I44" s="4">
-        <v>6</v>
-      </c>
       <c r="J44" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="1">
         <f>SUM(F44:K44)</f>
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>423348</v>
+        <v>420500</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E45" s="1"/>
-      <c r="F45" s="4">
-        <v>3</v>
-      </c>
-      <c r="G45" s="4">
-        <v>7</v>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6">
+        <v>6</v>
       </c>
       <c r="H45" s="6">
-        <v>7</v>
-      </c>
-      <c r="I45" s="4">
+        <v>14</v>
+      </c>
+      <c r="I45" s="4"/>
+      <c r="J45" s="6">
+        <v>6</v>
+      </c>
+      <c r="K45" s="4">
         <v>4</v>
-      </c>
-      <c r="J45" s="4">
-        <v>3</v>
-      </c>
-      <c r="K45" s="4">
-        <v>1</v>
       </c>
       <c r="L45" s="1">
         <f>SUM(F45:K45)</f>
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421902</v>
+        <v>423448</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
+        <v>3</v>
+      </c>
+      <c r="G46" s="4">
+        <v>8</v>
+      </c>
+      <c r="H46" s="6">
+        <v>6</v>
+      </c>
+      <c r="I46" s="4">
         <v>2</v>
       </c>
-      <c r="G46" s="4">
-        <v>6</v>
-      </c>
-      <c r="H46" s="4">
-        <v>6</v>
-      </c>
-      <c r="I46" s="4">
-        <v>5</v>
-      </c>
       <c r="J46" s="4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K46" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L46" s="1">
         <f>SUM(F46:K46)</f>
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>423501</v>
+        <v>422700</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G47" s="4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H47" s="4">
-        <v>1</v>
-      </c>
-      <c r="I47" s="4">
-        <v>6</v>
-      </c>
-      <c r="J47" s="4">
-        <v>2</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
       <c r="K47" s="4">
         <v>6</v>
       </c>
       <c r="L47" s="1">
         <f>SUM(F47:K47)</f>
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>421900</v>
+        <v>420101</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
@@ -6279,310 +6319,321 @@
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G48" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H48" s="4">
         <v>7</v>
       </c>
       <c r="I48" s="4">
-        <v>3</v>
-      </c>
-      <c r="J48" s="4">
-        <v>8</v>
-      </c>
-      <c r="K48" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4">
+        <v>2</v>
+      </c>
       <c r="L48" s="1">
         <f>SUM(F48:K48)</f>
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>422190</v>
+        <v>421901</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>123</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E49" s="1"/>
       <c r="F49" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G49" s="4">
-        <v>5</v>
-      </c>
-      <c r="H49" s="6">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="H49" s="4">
+        <v>6</v>
       </c>
       <c r="I49" s="4">
         <v>5</v>
       </c>
       <c r="J49" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K49" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L49" s="1">
         <f>SUM(F49:K49)</f>
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>424801</v>
+        <v>422900</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="4">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="G50" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H50" s="4"/>
-      <c r="I50" s="4">
-        <v>7</v>
-      </c>
+      <c r="I50" s="4"/>
       <c r="J50" s="4">
-        <v>3</v>
-      </c>
-      <c r="K50" s="4">
         <v>2</v>
       </c>
+      <c r="K50" s="4"/>
       <c r="L50" s="1">
         <f>SUM(F50:K50)</f>
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>420900</v>
+        <v>421301</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="F51" s="4">
+        <v>4</v>
+      </c>
+      <c r="G51" s="4">
+        <v>2</v>
+      </c>
+      <c r="H51" s="4">
+        <v>9</v>
+      </c>
+      <c r="I51" s="4">
         <v>5</v>
       </c>
-      <c r="D51" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E51" s="1"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4">
-        <v>5</v>
-      </c>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
       <c r="J51" s="4">
-        <v>4</v>
-      </c>
-      <c r="K51" s="4">
-        <v>10</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K51" s="4"/>
       <c r="L51" s="1">
         <f>SUM(F51:K51)</f>
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>420501</v>
+        <v>421902</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52" s="4">
+        <v>6</v>
+      </c>
+      <c r="H52" s="4">
+        <v>6</v>
+      </c>
+      <c r="I52" s="4">
+        <v>5</v>
+      </c>
+      <c r="J52" s="4">
         <v>4</v>
       </c>
-      <c r="H52" s="4">
-        <v>3</v>
-      </c>
-      <c r="I52" s="4">
-        <v>3</v>
-      </c>
-      <c r="J52" s="4"/>
       <c r="K52" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L52" s="1">
         <f>SUM(F52:K52)</f>
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>423600</v>
+        <v>422190</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="F53" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G53" s="4">
-        <v>6</v>
-      </c>
-      <c r="H53" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="H53" s="6">
+        <v>5</v>
+      </c>
       <c r="I53" s="4">
         <v>5</v>
       </c>
       <c r="J53" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K53" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L53" s="1">
         <f>SUM(F53:K53)</f>
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>421800</v>
+        <v>421900</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E54" s="1"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
+      <c r="F54" s="4">
+        <v>0</v>
+      </c>
+      <c r="G54" s="4">
+        <v>5</v>
+      </c>
       <c r="H54" s="4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I54" s="4">
         <v>3</v>
       </c>
       <c r="J54" s="4">
-        <v>4</v>
-      </c>
-      <c r="K54" s="4">
-        <v>2</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K54" s="4"/>
       <c r="L54" s="1">
         <f>SUM(F54:K54)</f>
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>421402</v>
+        <v>423308</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4">
+        <v>5</v>
+      </c>
+      <c r="H55" s="4">
         <v>3</v>
-      </c>
-      <c r="H55" s="4">
-        <v>1</v>
       </c>
       <c r="I55" s="4">
         <v>4</v>
       </c>
       <c r="J55" s="4">
-        <v>3</v>
-      </c>
-      <c r="K55" s="4">
-        <v>2</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K55" s="4"/>
       <c r="L55" s="1">
         <f>SUM(F55:K55)</f>
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="M55" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>423304</v>
+        <v>424801</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E56" s="1"/>
-      <c r="F56" s="4"/>
+      <c r="F56" s="4">
+        <v>1</v>
+      </c>
       <c r="G56" s="4">
-        <v>2</v>
-      </c>
-      <c r="H56" s="6"/>
-      <c r="I56" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4">
+        <v>7</v>
+      </c>
       <c r="J56" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K56" s="4">
         <v>2</v>
       </c>
       <c r="L56" s="1">
         <f>SUM(F56:K56)</f>
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>421300</v>
+        <v>420900</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="4">
-        <v>2</v>
-      </c>
-      <c r="G57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4">
+        <v>5</v>
+      </c>
       <c r="H57" s="4"/>
-      <c r="I57" s="4">
+      <c r="I57" s="4"/>
+      <c r="J57" s="4">
         <v>4</v>
       </c>
-      <c r="J57" s="4"/>
       <c r="K57" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L57" s="1">
         <f>SUM(F57:K57)</f>
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>422601</v>
+        <v>424500</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>10</v>
@@ -6592,90 +6643,96 @@
         <v>5</v>
       </c>
       <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
+      <c r="H58" s="4">
+        <v>3</v>
+      </c>
+      <c r="I58" s="4">
+        <v>4</v>
+      </c>
       <c r="J58" s="4">
-        <v>4</v>
-      </c>
-      <c r="K58" s="4">
-        <v>1</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K58" s="4"/>
       <c r="L58" s="1">
         <f>SUM(F58:K58)</f>
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="P58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>423309</v>
+        <v>423501</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E59" s="1"/>
-      <c r="F59" s="4"/>
+      <c r="F59" s="4">
+        <v>2</v>
+      </c>
       <c r="G59" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H59" s="4">
         <v>1</v>
       </c>
       <c r="I59" s="4">
-        <v>1</v>
-      </c>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="J59" s="4">
+        <v>1</v>
+      </c>
+      <c r="K59" s="4">
+        <v>6</v>
+      </c>
       <c r="L59" s="1">
         <f>SUM(F59:K59)</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
-        <v>420200</v>
+        <v>420501</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="4">
         <v>1</v>
       </c>
       <c r="G60" s="4">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="H60" s="4">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="I60" s="4">
-        <v>50</v>
-      </c>
-      <c r="J60" s="4">
-        <v>30</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="J60" s="4"/>
       <c r="K60" s="4">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="L60" s="1">
         <f>SUM(F60:K60)</f>
-        <v>212</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
-        <v>420402</v>
+        <v>421800</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>6</v>
@@ -6683,172 +6740,433 @@
       <c r="E61" s="1"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="4"/>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
+      <c r="H61" s="4">
+        <v>4</v>
+      </c>
+      <c r="I61" s="4">
+        <v>3</v>
+      </c>
+      <c r="J61" s="4">
+        <v>4</v>
+      </c>
+      <c r="K61" s="4">
+        <v>2</v>
+      </c>
       <c r="L61" s="1">
         <f>SUM(F61:K61)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
-        <v>424960</v>
+        <v>421402</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="6"/>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="12">
+      <c r="G62" s="4">
+        <v>3</v>
+      </c>
+      <c r="H62" s="4">
+        <v>1</v>
+      </c>
+      <c r="I62" s="4">
+        <v>4</v>
+      </c>
+      <c r="J62" s="4">
+        <v>3</v>
+      </c>
+      <c r="K62" s="4">
+        <v>2</v>
+      </c>
+      <c r="L62" s="1">
         <f>SUM(F62:K62)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
-        <v>423409</v>
+        <v>423304</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
+      <c r="G63" s="4">
+        <v>1</v>
+      </c>
+      <c r="H63" s="6"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
+      <c r="J63" s="4">
+        <v>7</v>
+      </c>
+      <c r="K63" s="4">
+        <v>2</v>
+      </c>
       <c r="L63" s="1">
         <f>SUM(F63:K63)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
-        <v>420160</v>
+        <v>421300</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F64" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="E64" s="1"/>
+      <c r="F64" s="4">
+        <v>2</v>
+      </c>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
+      <c r="I64" s="4">
+        <v>4</v>
+      </c>
       <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
+      <c r="K64" s="4">
+        <v>4</v>
+      </c>
       <c r="L64" s="1">
         <f>SUM(F64:K64)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="2:12" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
-        <v>423404</v>
+        <v>423348</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
+      <c r="G65" s="4">
+        <v>4</v>
+      </c>
+      <c r="H65" s="6">
+        <v>4</v>
+      </c>
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
         <f>SUM(F65:K65)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B66" s="6">
-        <v>420801</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B66" s="17">
+        <v>422401</v>
+      </c>
+      <c r="C66" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="E66" s="1"/>
-      <c r="F66" s="1"/>
-      <c r="G66" s="6"/>
-      <c r="H66" s="6"/>
-      <c r="I66" s="6"/>
-      <c r="J66" s="6"/>
-      <c r="K66" s="4"/>
+      <c r="F66" s="1">
+        <v>1</v>
+      </c>
+      <c r="G66" s="1">
+        <v>1</v>
+      </c>
+      <c r="H66" s="1">
+        <v>1</v>
+      </c>
+      <c r="I66" s="1">
+        <v>1</v>
+      </c>
+      <c r="J66" s="1">
+        <v>1</v>
+      </c>
+      <c r="K66" s="1">
+        <v>1</v>
+      </c>
       <c r="L66" s="1">
-        <f>SUM(G66:K66)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="2:12" x14ac:dyDescent="0.25">
+        <f>SUM(F66:K66)</f>
+        <v>6</v>
+      </c>
+      <c r="M66" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
-        <v>420802</v>
+        <v>423309</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E67" s="1"/>
-      <c r="F67" s="1"/>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-      <c r="I67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="4">
+        <v>1</v>
+      </c>
+      <c r="H67" s="4">
+        <v>1</v>
+      </c>
+      <c r="I67" s="4">
+        <v>1</v>
+      </c>
       <c r="J67" s="4"/>
       <c r="K67" s="4"/>
       <c r="L67" s="1">
-        <f>SUM(G67:K67)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="F69" t="s">
-        <v>127</v>
-      </c>
-      <c r="L69" s="10">
+        <f>SUM(F67:K67)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B68" s="6">
+        <v>422400</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" s="1"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="6"/>
+      <c r="J68" s="6">
+        <v>2</v>
+      </c>
+      <c r="K68" s="6"/>
+      <c r="L68" s="1">
+        <f>SUM(F68:K68)</f>
+        <v>2</v>
+      </c>
+      <c r="M68" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B69" s="6">
+        <v>424960</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" s="1"/>
+      <c r="F69" s="4"/>
+      <c r="G69" s="4"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="4"/>
+      <c r="J69" s="4"/>
+      <c r="K69" s="4"/>
+      <c r="L69" s="12">
+        <f>SUM(F69:K69)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B70" s="6">
+        <v>423409</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E70" s="1"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="4"/>
+      <c r="K70" s="4"/>
+      <c r="L70" s="1">
+        <f>SUM(F70:K70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B71" s="6">
+        <v>423404</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E71" s="1"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4"/>
+      <c r="L71" s="1">
+        <f>SUM(F71:K71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B72" s="6">
+        <v>420802</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+      <c r="J72" s="4"/>
+      <c r="K72" s="4"/>
+      <c r="L72" s="1">
+        <f>SUM(G72:K72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B73" s="6">
+        <v>420801</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="4"/>
+      <c r="L73" s="1">
+        <f>SUM(G73:K73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B74" s="6">
+        <v>420402</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E74" s="1"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="4"/>
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="4"/>
+      <c r="L74" s="1">
+        <f>SUM(F74:K74)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B75" s="6">
+        <v>420160</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F75" s="4"/>
+      <c r="G75" s="4"/>
+      <c r="H75" s="4"/>
+      <c r="I75" s="4"/>
+      <c r="J75" s="4"/>
+      <c r="K75" s="4"/>
+      <c r="L75" s="1">
+        <f>SUM(F75:K75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B76" s="6">
+        <v>421001</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+      <c r="I76" s="1"/>
+      <c r="J76" s="1"/>
+      <c r="K76" s="1"/>
+      <c r="L76" s="1"/>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B77" s="19"/>
+      <c r="C77" s="19"/>
+      <c r="D77" s="19"/>
+      <c r="E77" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F77" s="19"/>
+      <c r="G77" s="19"/>
+      <c r="H77" s="19"/>
+      <c r="I77" s="19"/>
+      <c r="J77" s="19"/>
+      <c r="K77" s="19"/>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="L79" s="10">
         <f>SUM(L3:L66)</f>
-        <v>3676</v>
-      </c>
-    </row>
-    <row r="73" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E73" t="s">
-        <v>124</v>
+        <v>3772</v>
       </c>
     </row>
     <row r="127" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K127" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L67" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L67">
-      <sortCondition descending="1" ref="L2:L67"/>
+  <autoFilter ref="B2:L77" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L77">
+      <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6856,21 +7174,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7014,31 +7317,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7054,4 +7348,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Mejorar stock bodega y actualizar inventario
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2221" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{429EDF48-F1A8-46EE-B657-836D4D401900}"/>
+  <xr:revisionPtr revIDLastSave="2619" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C26B8896-F80D-4768-948E-298C60752D26}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -18,15 +18,17 @@
     <sheet name="cole39" sheetId="6" r:id="rId3"/>
     <sheet name="COLE 40" sheetId="8" r:id="rId4"/>
     <sheet name="COLE 41" sheetId="9" r:id="rId5"/>
-    <sheet name="principal 42" sheetId="4" r:id="rId6"/>
+    <sheet name="COLE 42" sheetId="4" r:id="rId6"/>
+    <sheet name="COLE 43" sheetId="10" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cole 37'!$B$3:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'cole 38'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'COLE 42'!$B$2:$L$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$B$3:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'principal 42'!$B$2:$L$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="130">
   <si>
     <t>CODIGO</t>
   </si>
@@ -438,10 +440,7 @@
     <t>OSCURO</t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 17:14  29-04</t>
-  </si>
-  <si>
-    <t>REVISADO</t>
+    <t>ULTIMA ACTUALIZACION 15:11  06-05-2026</t>
   </si>
 </sst>
 </file>
@@ -564,7 +563,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -604,11 +603,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4776,44 +4770,39 @@
         <v>123</v>
       </c>
       <c r="B3" s="6">
-        <v>423600</v>
+        <v>422200</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G3" s="4">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="H3" s="4">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="I3" s="4">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J3" s="4">
-        <v>28</v>
-      </c>
-      <c r="K3" s="4">
-        <v>24</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="K3" s="4"/>
       <c r="L3" s="1">
         <f>SUM(F3:K3)</f>
-        <v>208</v>
-      </c>
-      <c r="M3" t="s">
-        <v>130</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>420100</v>
+        <v>423500</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -4823,26 +4812,26 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="G4" s="4">
+        <v>35</v>
+      </c>
+      <c r="H4" s="4">
+        <v>36</v>
+      </c>
+      <c r="I4" s="4">
         <v>33</v>
       </c>
-      <c r="H4" s="4">
-        <v>69</v>
-      </c>
-      <c r="I4" s="4">
-        <v>42</v>
-      </c>
       <c r="J4" s="4">
+        <v>43</v>
+      </c>
+      <c r="K4" s="4">
         <v>23</v>
-      </c>
-      <c r="K4" s="4">
-        <v>9</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>205</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -4850,72 +4839,73 @@
         <v>126</v>
       </c>
       <c r="B5" s="6">
-        <v>422200</v>
+        <v>423600</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G5" s="4">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H5" s="4">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I5" s="4">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="J5" s="4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K5" s="4">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
-        <v>423800</v>
+        <v>420600</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" s="6">
-        <v>15</v>
-      </c>
-      <c r="G6" s="6">
-        <v>36</v>
-      </c>
-      <c r="H6" s="6">
-        <v>40</v>
-      </c>
-      <c r="I6" s="6">
-        <v>36</v>
-      </c>
-      <c r="J6" s="6">
-        <v>20</v>
-      </c>
-      <c r="K6" s="6">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="4">
+        <v>38</v>
+      </c>
+      <c r="G6" s="4">
+        <v>22</v>
+      </c>
+      <c r="H6" s="4">
+        <v>10</v>
+      </c>
+      <c r="I6" s="4">
+        <v>17</v>
+      </c>
+      <c r="J6" s="4">
+        <v>26</v>
+      </c>
+      <c r="K6" s="4">
+        <v>13</v>
       </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>163</v>
+        <v>126</v>
+      </c>
+      <c r="M6" t="s">
+        <v>123</v>
       </c>
       <c r="N6" t="s">
         <v>129</v>
@@ -4923,7 +4913,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>423500</v>
+        <v>420100</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
@@ -4933,95 +4923,88 @@
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G7" s="4">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H7" s="4">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="I7" s="4">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="J7" s="4">
-        <v>27</v>
-      </c>
-      <c r="K7" s="4">
-        <v>10</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K7" s="4"/>
       <c r="L7" s="1">
         <f>SUM(F7:K7)</f>
-        <v>153</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>420301</v>
+        <v>424400</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="6">
-        <v>14</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="F8" s="4">
+        <v>27</v>
+      </c>
+      <c r="G8" s="4">
+        <v>27</v>
+      </c>
+      <c r="H8" s="4">
+        <v>24</v>
+      </c>
+      <c r="I8" s="4">
         <v>32</v>
       </c>
-      <c r="H8" s="6">
-        <v>34</v>
-      </c>
-      <c r="I8" s="6">
-        <v>36</v>
-      </c>
-      <c r="J8" s="6">
-        <v>18</v>
-      </c>
-      <c r="K8" s="6">
-        <v>8</v>
-      </c>
+      <c r="J8" s="4">
+        <v>3</v>
+      </c>
+      <c r="K8" s="4"/>
       <c r="L8" s="1">
         <f>SUM(F8:K8)</f>
-        <v>142</v>
-      </c>
-      <c r="M8" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>422500</v>
+        <v>422300</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G9" s="4">
+        <v>19</v>
+      </c>
+      <c r="H9" s="4">
         <v>11</v>
       </c>
-      <c r="H9" s="4">
-        <v>43</v>
-      </c>
       <c r="I9" s="4">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="J9" s="4">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
         <f>SUM(F9:K9)</f>
-        <v>139</v>
+        <v>83</v>
       </c>
       <c r="N9" s="11"/>
     </row>
@@ -5030,36 +5013,36 @@
         <v>123</v>
       </c>
       <c r="B10" s="6">
-        <v>420600</v>
+        <v>420300</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="1"/>
+      <c r="F10" s="6">
+        <v>13</v>
+      </c>
+      <c r="G10" s="6">
+        <v>15</v>
+      </c>
+      <c r="H10" s="6">
+        <v>16</v>
+      </c>
+      <c r="I10" s="6">
+        <v>15</v>
+      </c>
+      <c r="J10" s="6">
+        <v>11</v>
+      </c>
+      <c r="K10" s="6">
         <v>10</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="4">
-        <v>38</v>
-      </c>
-      <c r="G10" s="4">
-        <v>22</v>
-      </c>
-      <c r="H10" s="4">
-        <v>10</v>
-      </c>
-      <c r="I10" s="4">
-        <v>17</v>
-      </c>
-      <c r="J10" s="4">
-        <v>26</v>
-      </c>
-      <c r="K10" s="4">
-        <v>13</v>
-      </c>
-      <c r="L10" s="1">
+      <c r="L10" s="12">
         <f>SUM(F10:K10)</f>
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
@@ -5067,7 +5050,7 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>422800</v>
+        <v>420400</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>5</v>
@@ -5076,25 +5059,27 @@
         <v>6</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="4"/>
+      <c r="F11" s="4">
+        <v>26</v>
+      </c>
       <c r="G11" s="4">
+        <v>6</v>
+      </c>
+      <c r="H11" s="4">
         <v>9</v>
       </c>
-      <c r="H11" s="4">
-        <v>55</v>
-      </c>
       <c r="I11" s="4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J11" s="4">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="K11" s="4">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(F11:K11)</f>
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
@@ -5102,34 +5087,36 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>424400</v>
+        <v>423200</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G12" s="4">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="H12" s="4">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I12" s="4">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="J12" s="4">
-        <v>3</v>
-      </c>
-      <c r="K12" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="K12" s="4">
+        <v>14</v>
+      </c>
       <c r="L12" s="1">
         <f>SUM(F12:K12)</f>
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="N12" t="s">
         <v>123</v>
@@ -5137,36 +5124,36 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>424701</v>
+        <v>422500</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" s="4">
+        <v>1</v>
+      </c>
+      <c r="H13" s="4">
+        <v>14</v>
+      </c>
+      <c r="I13" s="4">
+        <v>15</v>
+      </c>
+      <c r="J13" s="4">
         <v>13</v>
       </c>
-      <c r="H13" s="4">
-        <v>28</v>
-      </c>
-      <c r="I13" s="4">
-        <v>11</v>
-      </c>
-      <c r="J13" s="4">
-        <v>23</v>
-      </c>
       <c r="K13" s="4">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="L13" s="1">
         <f>SUM(F13:K13)</f>
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
@@ -5177,34 +5164,34 @@
         <v>123</v>
       </c>
       <c r="B14" s="6">
-        <v>422300</v>
+        <v>424600</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G14" s="4">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H14" s="4">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I14" s="4">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J14" s="4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="1">
         <f>SUM(F14:K14)</f>
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
@@ -5215,71 +5202,63 @@
         <v>123</v>
       </c>
       <c r="B15" s="6">
-        <v>423000</v>
+        <v>422800</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="4">
-        <v>10</v>
-      </c>
+      <c r="F15" s="4"/>
       <c r="G15" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="4">
-        <v>8</v>
-      </c>
-      <c r="I15" s="4">
-        <v>14</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="I15" s="4"/>
       <c r="J15" s="4">
         <v>28</v>
       </c>
-      <c r="K15" s="4">
-        <v>19</v>
-      </c>
+      <c r="K15" s="4"/>
       <c r="L15" s="1">
         <f>SUM(F15:K15)</f>
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="N15" s="11"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>423200</v>
+        <v>422000</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="4">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="G16" s="4">
+        <v>10</v>
+      </c>
+      <c r="H16" s="4">
         <v>11</v>
       </c>
-      <c r="H16" s="4">
-        <v>17</v>
-      </c>
       <c r="I16" s="4">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="J16" s="4">
-        <v>12</v>
-      </c>
-      <c r="K16" s="4">
-        <v>14</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K16" s="4"/>
       <c r="L16" s="1">
         <f>SUM(F16:K16)</f>
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
@@ -5287,306 +5266,300 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>420300</v>
+        <v>423316</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="6">
+      <c r="F17" s="4">
+        <v>6</v>
+      </c>
+      <c r="G17" s="4">
+        <v>14</v>
+      </c>
+      <c r="H17" s="4">
+        <v>14</v>
+      </c>
+      <c r="I17" s="4">
         <v>13</v>
       </c>
-      <c r="G17" s="6">
-        <v>15</v>
-      </c>
-      <c r="H17" s="6">
-        <v>16</v>
-      </c>
-      <c r="I17" s="6">
-        <v>15</v>
-      </c>
-      <c r="J17" s="6">
-        <v>11</v>
-      </c>
-      <c r="K17" s="6">
-        <v>10</v>
-      </c>
-      <c r="L17" s="12">
+      <c r="J17" s="4">
+        <v>8</v>
+      </c>
+      <c r="K17" s="4">
+        <v>4</v>
+      </c>
+      <c r="L17" s="1">
         <f>SUM(F17:K17)</f>
-        <v>80</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>422100</v>
+        <v>422101</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G18" s="4">
+        <v>1</v>
+      </c>
+      <c r="H18" s="4">
+        <v>15</v>
+      </c>
+      <c r="I18" s="4">
+        <v>9</v>
+      </c>
+      <c r="J18" s="4">
         <v>14</v>
       </c>
-      <c r="H18" s="4">
-        <v>16</v>
-      </c>
-      <c r="I18" s="4">
-        <v>14</v>
-      </c>
-      <c r="J18" s="4">
-        <v>10</v>
-      </c>
-      <c r="K18" s="4">
-        <v>17</v>
-      </c>
+      <c r="K18" s="4"/>
       <c r="L18" s="1">
         <f>SUM(F18:K18)</f>
-        <v>79</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>423900</v>
+        <v>421400</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4">
+        <v>1</v>
+      </c>
+      <c r="J19" s="4">
         <v>11</v>
       </c>
-      <c r="H19" s="4">
-        <v>3</v>
-      </c>
-      <c r="I19" s="4">
-        <v>16</v>
-      </c>
-      <c r="J19" s="4">
-        <v>16</v>
-      </c>
       <c r="K19" s="4">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="L19" s="1">
         <f>SUM(F19:K19)</f>
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>420400</v>
+        <v>420800</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="4">
-        <v>24</v>
-      </c>
-      <c r="G20" s="4">
-        <v>6</v>
-      </c>
-      <c r="H20" s="4">
-        <v>11</v>
-      </c>
-      <c r="I20" s="4">
-        <v>6</v>
-      </c>
-      <c r="J20" s="4">
-        <v>9</v>
+      <c r="F20" s="6">
+        <v>6</v>
+      </c>
+      <c r="G20" s="6">
+        <v>10</v>
+      </c>
+      <c r="H20" s="6">
+        <v>12</v>
+      </c>
+      <c r="I20" s="6">
+        <v>12</v>
+      </c>
+      <c r="J20" s="6">
+        <v>6</v>
       </c>
       <c r="K20" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L20" s="1">
         <f>SUM(F20:K20)</f>
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>424200</v>
+        <v>421801</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="6">
-        <v>7</v>
-      </c>
-      <c r="G21" s="6">
-        <v>13</v>
-      </c>
-      <c r="H21" s="6">
+      <c r="F21" s="4"/>
+      <c r="G21" s="4">
+        <v>2</v>
+      </c>
+      <c r="H21" s="4">
+        <v>8</v>
+      </c>
+      <c r="I21" s="4">
+        <v>8</v>
+      </c>
+      <c r="J21" s="4">
+        <v>20</v>
+      </c>
+      <c r="K21" s="4">
         <v>12</v>
       </c>
-      <c r="I21" s="6">
-        <v>22</v>
-      </c>
-      <c r="J21" s="6">
-        <v>4</v>
-      </c>
-      <c r="K21" s="6">
-        <v>6</v>
-      </c>
-      <c r="L21" s="12">
+      <c r="L21" s="1">
         <f>SUM(F21:K21)</f>
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>424600</v>
+        <v>420160</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F22" s="4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G22" s="4">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H22" s="4">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="I22" s="4">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="J22" s="4">
-        <v>17</v>
-      </c>
-      <c r="K22" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="K22" s="4">
+        <v>5</v>
+      </c>
       <c r="L22" s="1">
         <f>SUM(F22:K22)</f>
-        <v>64</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>423416</v>
+        <v>421100</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G23" s="4">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H23" s="4">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I23" s="4">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J23" s="4">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K23" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L23" s="1">
         <f>SUM(F23:K23)</f>
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>422601</v>
+        <v>422700</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G24" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H24" s="4">
-        <v>9</v>
-      </c>
-      <c r="I24" s="4">
-        <v>7</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="I24" s="4"/>
       <c r="J24" s="4">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="K24" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L24" s="1">
         <f>SUM(F24:K24)</f>
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>423316</v>
+        <v>423000</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="4">
-        <v>6</v>
-      </c>
-      <c r="G25" s="4">
-        <v>14</v>
-      </c>
-      <c r="H25" s="4">
-        <v>14</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
       <c r="I25" s="4">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J25" s="4">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="K25" s="4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L25" s="1">
         <f>SUM(F25:K25)</f>
-        <v>59</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
@@ -5594,40 +5567,40 @@
         <v>424900</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F26" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G26" s="4">
-        <v>10</v>
-      </c>
-      <c r="H26" s="6">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="H26" s="1">
+        <v>13</v>
       </c>
       <c r="I26" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J26" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K26" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L26" s="1">
         <f>SUM(F26:K26)</f>
-        <v>58</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>425600</v>
+        <v>424900</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>7</v>
@@ -5635,63 +5608,67 @@
       <c r="D27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="6">
-        <v>10</v>
-      </c>
-      <c r="G27" s="6">
-        <v>11</v>
+      <c r="E27" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4">
+        <v>14</v>
       </c>
       <c r="H27" s="6">
         <v>9</v>
       </c>
-      <c r="I27" s="6">
-        <v>11</v>
-      </c>
-      <c r="J27" s="6">
-        <v>5</v>
-      </c>
-      <c r="K27" s="6">
-        <v>10</v>
+      <c r="I27" s="4">
+        <v>9</v>
+      </c>
+      <c r="J27" s="4">
+        <v>1</v>
+      </c>
+      <c r="K27" s="4">
+        <v>1</v>
       </c>
       <c r="L27" s="1">
         <f>SUM(F27:K27)</f>
-        <v>56</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>422000</v>
+        <v>421000</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E28" s="1"/>
-      <c r="F28" s="4">
-        <v>34</v>
-      </c>
-      <c r="G28" s="4">
+      <c r="F28" s="6">
+        <v>3</v>
+      </c>
+      <c r="G28" s="6">
+        <v>8</v>
+      </c>
+      <c r="H28" s="6">
         <v>9</v>
       </c>
-      <c r="H28" s="4">
-        <v>12</v>
-      </c>
-      <c r="I28" s="4">
-        <v>1</v>
-      </c>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
+      <c r="I28" s="6">
+        <v>8</v>
+      </c>
+      <c r="J28" s="6">
+        <v>4</v>
+      </c>
+      <c r="K28" s="6">
+        <v>2</v>
+      </c>
       <c r="L28" s="1">
         <f>SUM(F28:K28)</f>
-        <v>56</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>422101</v>
+        <v>424000</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
@@ -5701,353 +5678,347 @@
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="4">
-        <v>14</v>
-      </c>
-      <c r="G29" s="4">
-        <v>1</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G29" s="4"/>
       <c r="H29" s="4">
-        <v>14</v>
-      </c>
-      <c r="I29" s="4">
-        <v>9</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I29" s="4"/>
       <c r="J29" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K29" s="4"/>
       <c r="L29" s="1">
         <f>SUM(F29:K29)</f>
-        <v>52</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>421400</v>
+        <v>422701</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>7</v>
-      </c>
-      <c r="G30" s="4">
-        <v>0</v>
-      </c>
-      <c r="H30" s="4">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
       <c r="I30" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J30" s="4">
         <v>11</v>
       </c>
       <c r="K30" s="4">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="L30" s="1">
         <f>SUM(F30:K30)</f>
-        <v>52</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>420800</v>
+        <v>423448</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E31" s="1"/>
-      <c r="F31" s="6">
-        <v>6</v>
-      </c>
-      <c r="G31" s="6">
-        <v>10</v>
+      <c r="F31" s="4">
+        <v>3</v>
+      </c>
+      <c r="G31" s="4">
+        <v>8</v>
       </c>
       <c r="H31" s="6">
-        <v>12</v>
-      </c>
-      <c r="I31" s="6">
-        <v>12</v>
-      </c>
-      <c r="J31" s="6">
-        <v>6</v>
+        <v>6</v>
+      </c>
+      <c r="I31" s="4">
+        <v>2</v>
+      </c>
+      <c r="J31" s="4">
+        <v>9</v>
       </c>
       <c r="K31" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L31" s="1">
         <f>SUM(F31:K31)</f>
-        <v>52</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>421801</v>
+        <v>420101</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="4"/>
+      <c r="F32" s="4">
+        <v>5</v>
+      </c>
       <c r="G32" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H32" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I32" s="4">
-        <v>8</v>
-      </c>
-      <c r="J32" s="4">
-        <v>20</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="J32" s="4"/>
       <c r="K32" s="4">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L32" s="1">
         <f>SUM(F32:K32)</f>
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>420160</v>
+        <v>424701</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>7</v>
-      </c>
-      <c r="G33" s="4">
-        <v>12</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G33" s="4"/>
       <c r="H33" s="4">
-        <v>9</v>
-      </c>
-      <c r="I33" s="4">
-        <v>10</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="I33" s="4"/>
       <c r="J33" s="4">
-        <v>6</v>
-      </c>
-      <c r="K33" s="4">
-        <v>5</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="K33" s="4"/>
       <c r="L33" s="1">
         <f>SUM(F33:K33)</f>
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>424700</v>
+        <v>421901</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G34" s="4">
         <v>8</v>
       </c>
-      <c r="H34" s="4"/>
+      <c r="H34" s="4">
+        <v>6</v>
+      </c>
       <c r="I34" s="4">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J34" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K34" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L34" s="1">
         <f>SUM(F34:K34)</f>
-        <v>47</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>421100</v>
+        <v>422900</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="G35" s="4">
-        <v>4</v>
-      </c>
-      <c r="H35" s="4">
-        <v>6</v>
-      </c>
-      <c r="I35" s="4">
-        <v>7</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
       <c r="J35" s="4">
-        <v>20</v>
-      </c>
-      <c r="K35" s="4">
-        <v>7</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K35" s="4"/>
       <c r="L35" s="1">
         <f>SUM(F35:K35)</f>
-        <v>47</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>420200</v>
+        <v>421902</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E36" s="1"/>
-      <c r="F36" s="4"/>
+      <c r="F36" s="4">
+        <v>2</v>
+      </c>
       <c r="G36" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H36" s="4">
+        <v>6</v>
+      </c>
+      <c r="I36" s="4">
+        <v>5</v>
+      </c>
+      <c r="J36" s="4">
         <v>4</v>
       </c>
-      <c r="I36" s="4">
-        <v>12</v>
-      </c>
-      <c r="J36" s="4">
-        <v>8</v>
-      </c>
       <c r="K36" s="4">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="L36" s="1">
         <f>SUM(F36:K36)</f>
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>424000</v>
+        <v>420501</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4">
-        <v>3</v>
-      </c>
-      <c r="I37" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="I37" s="4">
+        <v>5</v>
+      </c>
       <c r="J37" s="4">
-        <v>16</v>
-      </c>
-      <c r="K37" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="K37" s="4">
+        <v>4</v>
+      </c>
       <c r="L37" s="1">
         <f>SUM(F37:K37)</f>
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>422701</v>
+        <v>420301</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="4">
-        <v>1</v>
-      </c>
-      <c r="G38" s="4">
-        <v>3</v>
-      </c>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4">
-        <v>8</v>
-      </c>
-      <c r="J38" s="4">
-        <v>14</v>
-      </c>
-      <c r="K38" s="4">
-        <v>16</v>
+      <c r="F38" s="6">
+        <v>17</v>
+      </c>
+      <c r="G38" s="6">
+        <v>34</v>
+      </c>
+      <c r="H38" s="6">
+        <v>37</v>
+      </c>
+      <c r="I38" s="6">
+        <v>29</v>
+      </c>
+      <c r="J38" s="6">
+        <v>33</v>
+      </c>
+      <c r="K38" s="6">
+        <v>15</v>
       </c>
       <c r="L38" s="1">
         <f>SUM(F38:K38)</f>
-        <v>42</v>
+        <v>165</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>422600</v>
+        <v>422190</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E39" s="1"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F39" s="4">
+        <v>2</v>
+      </c>
+      <c r="G39" s="4">
+        <v>5</v>
       </c>
       <c r="H39" s="6">
-        <v>15</v>
-      </c>
-      <c r="I39" s="6">
-        <v>10</v>
-      </c>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6">
+        <v>5</v>
+      </c>
+      <c r="I39" s="4">
+        <v>5</v>
+      </c>
+      <c r="J39" s="4">
+        <v>3</v>
+      </c>
+      <c r="K39" s="4">
         <v>3</v>
       </c>
       <c r="L39" s="1">
         <f>SUM(F39:K39)</f>
-        <v>40</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>424300</v>
+        <v>421900</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
@@ -6057,259 +6028,235 @@
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="4">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H40" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I40" s="4">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J40" s="4">
-        <v>1</v>
-      </c>
-      <c r="K40" s="4">
         <v>8</v>
       </c>
+      <c r="K40" s="4"/>
       <c r="L40" s="1">
         <f>SUM(F40:K40)</f>
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>424900</v>
+        <v>423501</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>125</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E41" s="1"/>
       <c r="F41" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G41" s="4">
-        <v>12</v>
-      </c>
-      <c r="H41" s="1">
-        <v>13</v>
+        <v>6</v>
+      </c>
+      <c r="H41" s="4">
+        <v>1</v>
       </c>
       <c r="I41" s="4">
         <v>6</v>
       </c>
       <c r="J41" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K41" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L41" s="1">
         <f>SUM(F41:K41)</f>
-        <v>38</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>421401</v>
+        <v>423308</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="4">
-        <v>1</v>
-      </c>
+      <c r="F42" s="4"/>
       <c r="G42" s="4">
+        <v>5</v>
+      </c>
+      <c r="H42" s="4">
+        <v>3</v>
+      </c>
+      <c r="I42" s="4">
+        <v>4</v>
+      </c>
+      <c r="J42" s="4">
         <v>9</v>
       </c>
-      <c r="H42" s="4">
-        <v>12</v>
-      </c>
-      <c r="I42" s="4">
-        <v>7</v>
-      </c>
-      <c r="J42" s="4">
-        <v>4</v>
-      </c>
-      <c r="K42" s="4">
-        <v>3</v>
-      </c>
+      <c r="K42" s="4"/>
       <c r="L42" s="1">
         <f>SUM(F42:K42)</f>
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>421000</v>
+        <v>423408</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="6">
-        <v>3</v>
-      </c>
-      <c r="G43" s="6">
-        <v>8</v>
-      </c>
-      <c r="H43" s="6">
-        <v>9</v>
-      </c>
-      <c r="I43" s="6">
-        <v>8</v>
-      </c>
-      <c r="J43" s="6">
+      <c r="F43" s="4"/>
+      <c r="G43" s="4">
+        <v>14</v>
+      </c>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4">
+        <v>2</v>
+      </c>
+      <c r="J43" s="4">
         <v>4</v>
       </c>
-      <c r="K43" s="6">
-        <v>2</v>
-      </c>
+      <c r="K43" s="4"/>
       <c r="L43" s="1">
         <f>SUM(F43:K43)</f>
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>423408</v>
+        <v>424801</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="4"/>
+      <c r="F44" s="4">
+        <v>1</v>
+      </c>
       <c r="G44" s="4">
-        <v>17</v>
-      </c>
-      <c r="H44" s="4">
+        <v>7</v>
+      </c>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4">
+        <v>7</v>
+      </c>
+      <c r="J44" s="4">
         <v>3</v>
       </c>
-      <c r="I44" s="4">
-        <v>5</v>
-      </c>
-      <c r="J44" s="4">
-        <v>6</v>
-      </c>
-      <c r="K44" s="4"/>
+      <c r="K44" s="4">
+        <v>2</v>
+      </c>
       <c r="L44" s="1">
         <f>SUM(F44:K44)</f>
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>420500</v>
+        <v>420900</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E45" s="1"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6">
-        <v>6</v>
-      </c>
-      <c r="H45" s="6">
-        <v>14</v>
-      </c>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4">
+        <v>5</v>
+      </c>
+      <c r="H45" s="4"/>
       <c r="I45" s="4"/>
-      <c r="J45" s="6">
-        <v>6</v>
+      <c r="J45" s="4">
+        <v>4</v>
       </c>
       <c r="K45" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L45" s="1">
         <f>SUM(F45:K45)</f>
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>423448</v>
+        <v>423900</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
-        <v>3</v>
-      </c>
-      <c r="G46" s="4">
+        <v>2</v>
+      </c>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4">
+        <v>9</v>
+      </c>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4">
         <v>8</v>
       </c>
-      <c r="H46" s="6">
-        <v>6</v>
-      </c>
-      <c r="I46" s="4">
-        <v>2</v>
-      </c>
-      <c r="J46" s="4">
-        <v>9</v>
-      </c>
-      <c r="K46" s="4">
-        <v>1</v>
-      </c>
+      <c r="K46" s="4"/>
       <c r="L46" s="1">
         <f>SUM(F46:K46)</f>
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>422700</v>
+        <v>422100</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E47" s="1"/>
-      <c r="F47" s="4">
-        <v>6</v>
-      </c>
-      <c r="G47" s="4">
-        <v>9</v>
-      </c>
-      <c r="H47" s="4">
-        <v>8</v>
-      </c>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
       <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
+      <c r="J47" s="4">
+        <v>5</v>
+      </c>
       <c r="K47" s="4">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="L47" s="1">
         <f>SUM(F47:K47)</f>
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>420101</v>
+        <v>424500</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
@@ -6321,341 +6268,314 @@
       <c r="F48" s="4">
         <v>5</v>
       </c>
-      <c r="G48" s="4">
-        <v>8</v>
-      </c>
+      <c r="G48" s="4"/>
       <c r="H48" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I48" s="4">
-        <v>7</v>
-      </c>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4">
-        <v>2</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J48" s="4">
+        <v>6</v>
+      </c>
+      <c r="K48" s="4"/>
       <c r="L48" s="1">
         <f>SUM(F48:K48)</f>
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>421901</v>
+        <v>424700</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G49" s="4">
-        <v>8</v>
-      </c>
-      <c r="H49" s="4">
-        <v>6</v>
-      </c>
-      <c r="I49" s="4">
-        <v>5</v>
-      </c>
-      <c r="J49" s="4">
-        <v>4</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
       <c r="K49" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L49" s="1">
         <f>SUM(F49:K49)</f>
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>422900</v>
+        <v>420802</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1"/>
-      <c r="F50" s="4">
-        <v>23</v>
-      </c>
+      <c r="F50" s="1"/>
       <c r="G50" s="4">
         <v>1</v>
       </c>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
+      <c r="H50" s="4">
+        <v>5</v>
+      </c>
+      <c r="I50" s="4">
+        <v>5</v>
+      </c>
       <c r="J50" s="4">
-        <v>2</v>
-      </c>
-      <c r="K50" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K50" s="4">
+        <v>3</v>
+      </c>
       <c r="L50" s="1">
-        <f>SUM(F50:K50)</f>
-        <v>26</v>
+        <f>SUM(G50:K50)</f>
+        <v>17</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>421301</v>
+        <v>420200</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="4">
-        <v>4</v>
-      </c>
-      <c r="G51" s="4">
-        <v>2</v>
-      </c>
-      <c r="H51" s="4">
-        <v>9</v>
-      </c>
-      <c r="I51" s="4">
-        <v>5</v>
-      </c>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
       <c r="J51" s="4">
-        <v>6</v>
-      </c>
-      <c r="K51" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="K51" s="4">
+        <v>13</v>
+      </c>
       <c r="L51" s="1">
         <f>SUM(F51:K51)</f>
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>421902</v>
+        <v>421301</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
-        <v>2</v>
-      </c>
-      <c r="G52" s="4">
-        <v>6</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G52" s="4"/>
       <c r="H52" s="4">
         <v>6</v>
       </c>
       <c r="I52" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J52" s="4">
         <v>4</v>
       </c>
-      <c r="K52" s="4">
-        <v>2</v>
-      </c>
+      <c r="K52" s="4"/>
       <c r="L52" s="1">
         <f>SUM(F52:K52)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>422190</v>
+        <v>424300</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F53" s="4">
-        <v>2</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="F53" s="4"/>
       <c r="G53" s="4">
         <v>5</v>
       </c>
-      <c r="H53" s="6">
-        <v>5</v>
-      </c>
+      <c r="H53" s="4"/>
       <c r="I53" s="4">
-        <v>5</v>
-      </c>
-      <c r="J53" s="4">
         <v>3</v>
       </c>
+      <c r="J53" s="4"/>
       <c r="K53" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L53" s="1">
         <f>SUM(F53:K53)</f>
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>421900</v>
+        <v>421402</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E54" s="1"/>
-      <c r="F54" s="4">
-        <v>0</v>
-      </c>
+      <c r="F54" s="4"/>
       <c r="G54" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H54" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I54" s="4">
+        <v>4</v>
+      </c>
+      <c r="J54" s="4">
         <v>3</v>
       </c>
-      <c r="J54" s="4">
-        <v>8</v>
-      </c>
-      <c r="K54" s="4"/>
+      <c r="K54" s="4">
+        <v>2</v>
+      </c>
       <c r="L54" s="1">
         <f>SUM(F54:K54)</f>
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>423308</v>
+        <v>425600</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4">
-        <v>5</v>
-      </c>
-      <c r="H55" s="4">
-        <v>3</v>
-      </c>
-      <c r="I55" s="4">
-        <v>4</v>
-      </c>
-      <c r="J55" s="4">
-        <v>9</v>
-      </c>
-      <c r="K55" s="4"/>
+      <c r="F55" s="6">
+        <v>2</v>
+      </c>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6">
+        <v>2</v>
+      </c>
+      <c r="K55" s="6">
+        <v>7</v>
+      </c>
       <c r="L55" s="1">
         <f>SUM(F55:K55)</f>
-        <v>21</v>
-      </c>
-      <c r="M55" t="s">
-        <v>130</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>424801</v>
+        <v>423304</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E56" s="1"/>
-      <c r="F56" s="4">
-        <v>1</v>
-      </c>
+      <c r="F56" s="4"/>
       <c r="G56" s="4">
-        <v>7</v>
-      </c>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4">
-        <v>7</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H56" s="6"/>
+      <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K56" s="4">
         <v>2</v>
       </c>
       <c r="L56" s="1">
         <f>SUM(F56:K56)</f>
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>420900</v>
+        <v>421300</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4">
-        <v>5</v>
-      </c>
+      <c r="F57" s="4">
+        <v>2</v>
+      </c>
+      <c r="G57" s="4"/>
       <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4">
+      <c r="I57" s="4">
         <v>4</v>
       </c>
+      <c r="J57" s="4"/>
       <c r="K57" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L57" s="1">
         <f>SUM(F57:K57)</f>
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>424500</v>
+        <v>424960</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="4">
-        <v>5</v>
-      </c>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="G58" s="4">
+        <v>2</v>
+      </c>
+      <c r="H58" s="6">
+        <v>2</v>
       </c>
       <c r="I58" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J58" s="4">
-        <v>6</v>
-      </c>
-      <c r="K58" s="4"/>
-      <c r="L58" s="1">
+        <v>1</v>
+      </c>
+      <c r="K58" s="4">
+        <v>1</v>
+      </c>
+      <c r="L58" s="12">
         <f>SUM(F58:K58)</f>
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
@@ -6663,103 +6583,91 @@
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>423501</v>
+        <v>421800</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E59" s="1"/>
-      <c r="F59" s="4">
-        <v>2</v>
-      </c>
-      <c r="G59" s="4">
-        <v>4</v>
-      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
       <c r="H59" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I59" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J59" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L59" s="1">
         <f>SUM(F59:K59)</f>
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
-        <v>420501</v>
+        <v>423348</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E60" s="1"/>
-      <c r="F60" s="4">
-        <v>1</v>
-      </c>
+      <c r="F60" s="4"/>
       <c r="G60" s="4">
-        <v>4</v>
-      </c>
-      <c r="H60" s="4">
+        <v>2</v>
+      </c>
+      <c r="H60" s="6">
+        <v>2</v>
+      </c>
+      <c r="I60" s="4">
+        <v>1</v>
+      </c>
+      <c r="J60" s="4">
         <v>3</v>
       </c>
-      <c r="I60" s="4">
-        <v>3</v>
-      </c>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4">
-        <v>5</v>
-      </c>
+      <c r="K60" s="4"/>
       <c r="L60" s="1">
         <f>SUM(F60:K60)</f>
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
-        <v>421800</v>
+        <v>422601</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E61" s="1"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
-      <c r="H61" s="4">
-        <v>4</v>
-      </c>
-      <c r="I61" s="4">
-        <v>3</v>
-      </c>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4"/>
       <c r="J61" s="4">
-        <v>4</v>
-      </c>
-      <c r="K61" s="4">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K61" s="4"/>
       <c r="L61" s="1">
         <f>SUM(F61:K61)</f>
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
-        <v>421402</v>
+        <v>421401</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>7</v>
@@ -6770,167 +6678,150 @@
       <c r="E62" s="1"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H62" s="4">
-        <v>1</v>
-      </c>
-      <c r="I62" s="4">
         <v>4</v>
       </c>
-      <c r="J62" s="4">
-        <v>3</v>
-      </c>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
       <c r="K62" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L62" s="1">
         <f>SUM(F62:K62)</f>
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
-        <v>423304</v>
+        <v>421001</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E63" s="1"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4">
-        <v>1</v>
-      </c>
-      <c r="H63" s="6"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4">
-        <v>7</v>
-      </c>
-      <c r="K63" s="4">
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1">
+        <v>2</v>
+      </c>
+      <c r="I63" s="1">
+        <v>1</v>
+      </c>
+      <c r="J63" s="1">
+        <v>1</v>
+      </c>
+      <c r="K63" s="1">
         <v>2</v>
       </c>
       <c r="L63" s="1">
-        <f>SUM(F63:K63)</f>
-        <v>10</v>
+        <f>SUM(H63:K63)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
-        <v>421300</v>
+        <v>420500</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E64" s="1"/>
-      <c r="F64" s="4">
-        <v>2</v>
-      </c>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4">
-        <v>4</v>
-      </c>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4">
-        <v>4</v>
-      </c>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6">
+        <v>1</v>
+      </c>
+      <c r="H64" s="6">
+        <v>2</v>
+      </c>
+      <c r="I64" s="4"/>
+      <c r="J64" s="6">
+        <v>2</v>
+      </c>
+      <c r="K64" s="4"/>
       <c r="L64" s="1">
         <f>SUM(F64:K64)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
-        <v>423348</v>
+        <v>420402</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="4"/>
-      <c r="G65" s="4">
-        <v>4</v>
-      </c>
-      <c r="H65" s="6">
-        <v>4</v>
-      </c>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
+      <c r="J65" s="4">
+        <v>5</v>
+      </c>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
         <f>SUM(F65:K65)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B66" s="17">
-        <v>422401</v>
-      </c>
-      <c r="C66" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D66" s="18" t="s">
-        <v>12</v>
+      <c r="B66" s="6">
+        <v>423416</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="E66" s="1"/>
-      <c r="F66" s="1">
-        <v>1</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-      <c r="H66" s="1">
-        <v>1</v>
-      </c>
-      <c r="I66" s="1">
-        <v>1</v>
-      </c>
-      <c r="J66" s="1">
-        <v>1</v>
-      </c>
-      <c r="K66" s="1">
-        <v>1</v>
-      </c>
+      <c r="F66" s="4">
+        <v>1</v>
+      </c>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4">
+        <v>1</v>
+      </c>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4">
+        <v>2</v>
+      </c>
+      <c r="K66" s="4"/>
       <c r="L66" s="1">
         <f>SUM(F66:K66)</f>
-        <v>6</v>
-      </c>
-      <c r="M66" t="s">
-        <v>130</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
-        <v>423309</v>
+        <v>422600</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E67" s="1"/>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4">
-        <v>1</v>
-      </c>
-      <c r="H67" s="4">
-        <v>1</v>
-      </c>
-      <c r="I67" s="4">
-        <v>1</v>
-      </c>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6"/>
+      <c r="J67" s="6"/>
+      <c r="K67" s="6">
+        <v>3</v>
+      </c>
       <c r="L67" s="1">
         <f>SUM(F67:K67)</f>
         <v>3</v>
@@ -6938,70 +6829,73 @@
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="6">
-        <v>422400</v>
+        <v>423309</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E68" s="1"/>
-      <c r="F68" s="6"/>
-      <c r="G68" s="6"/>
-      <c r="H68" s="6"/>
-      <c r="I68" s="6"/>
-      <c r="J68" s="6">
-        <v>2</v>
-      </c>
-      <c r="K68" s="6"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4">
+        <v>1</v>
+      </c>
+      <c r="H68" s="4">
+        <v>1</v>
+      </c>
+      <c r="I68" s="4">
+        <v>1</v>
+      </c>
+      <c r="J68" s="4"/>
+      <c r="K68" s="4"/>
       <c r="L68" s="1">
         <f>SUM(F68:K68)</f>
-        <v>2</v>
-      </c>
-      <c r="M68" t="s">
-        <v>130</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="6">
-        <v>424960</v>
+        <v>422400</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E69" s="1"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
       <c r="H69" s="6"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="12">
+      <c r="I69" s="6"/>
+      <c r="J69" s="6">
+        <v>2</v>
+      </c>
+      <c r="K69" s="6"/>
+      <c r="L69" s="1">
         <f>SUM(F69:K69)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="6">
-        <v>423409</v>
+        <v>422401</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E70" s="1"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
       <c r="L70" s="1">
         <f>SUM(F70:K70)</f>
         <v>0</v>
@@ -7009,21 +6903,23 @@
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
-        <v>423404</v>
+        <v>423800</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E71" s="1"/>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
-      <c r="J71" s="4"/>
-      <c r="K71" s="4"/>
+        <v>11</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F71" s="6"/>
+      <c r="G71" s="6"/>
+      <c r="H71" s="6"/>
+      <c r="I71" s="6"/>
+      <c r="J71" s="6"/>
+      <c r="K71" s="6"/>
       <c r="L71" s="1">
         <f>SUM(F71:K71)</f>
         <v>0</v>
@@ -7031,54 +6927,54 @@
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
-        <v>420802</v>
+        <v>424200</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-      <c r="I72" s="4"/>
-      <c r="J72" s="4"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="1">
-        <f>SUM(G72:K72)</f>
+      <c r="F72" s="6"/>
+      <c r="G72" s="6"/>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="6"/>
+      <c r="L72" s="12">
+        <f>SUM(F72:K72)</f>
         <v>0</v>
       </c>
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="6">
-        <v>420801</v>
+        <v>423409</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E73" s="1"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="6"/>
-      <c r="H73" s="6"/>
-      <c r="I73" s="6"/>
-      <c r="J73" s="6"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="4"/>
+      <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f>SUM(G73:K73)</f>
+        <f>SUM(F73:K73)</f>
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="6">
-        <v>420402</v>
+        <v>423404</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>6</v>
@@ -7097,65 +6993,67 @@
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" s="6">
-        <v>420160</v>
+        <v>420801</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
-      <c r="H75" s="4"/>
-      <c r="I75" s="4"/>
-      <c r="J75" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="6"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6"/>
+      <c r="J75" s="6"/>
       <c r="K75" s="4"/>
       <c r="L75" s="1">
-        <f>SUM(F75:K75)</f>
+        <f>SUM(G75:K75)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B76" s="6">
-        <v>421001</v>
+        <v>420160</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1"/>
-      <c r="K76" s="1"/>
-      <c r="L76" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F76" s="4"/>
+      <c r="G76" s="4"/>
+      <c r="H76" s="4"/>
+      <c r="I76" s="4"/>
+      <c r="J76" s="4"/>
+      <c r="K76" s="4"/>
+      <c r="L76" s="1">
+        <f>SUM(F76:K76)</f>
+        <v>0</v>
+      </c>
+      <c r="M76" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B77" s="19"/>
-      <c r="C77" s="19"/>
-      <c r="D77" s="19"/>
-      <c r="E77" s="19" t="s">
+      <c r="E77" t="s">
         <v>123</v>
       </c>
-      <c r="F77" s="19"/>
-      <c r="G77" s="19"/>
-      <c r="H77" s="19"/>
-      <c r="I77" s="19"/>
-      <c r="J77" s="19"/>
-      <c r="K77" s="19"/>
     </row>
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L79" s="10">
-        <f>SUM(L3:L66)</f>
-        <v>3772</v>
+        <f>SUM(L3:L78)</f>
+        <v>2833</v>
+      </c>
+    </row>
+    <row r="83" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O83" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="127" spans="11:11" x14ac:dyDescent="0.25">
@@ -7169,6 +7067,52 @@
       <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
   </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
+  <dimension ref="B3:L3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="3">
+        <v>36</v>
+      </c>
+      <c r="G3" s="3">
+        <v>38</v>
+      </c>
+      <c r="H3" s="3">
+        <v>40</v>
+      </c>
+      <c r="I3" s="3">
+        <v>42</v>
+      </c>
+      <c r="J3" s="3">
+        <v>44</v>
+      </c>
+      <c r="K3" s="3">
+        <v>46</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B3:L3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7361,14 +7305,14 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>

</xml_diff>

<commit_message>
Corregir stock bodega y refresco de inventario
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2619" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C26B8896-F80D-4768-948E-298C60752D26}"/>
+  <xr:revisionPtr revIDLastSave="2631" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21404990-CE57-4093-A4A2-1C3476524D88}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="130">
   <si>
     <t>CODIGO</t>
   </si>
@@ -440,7 +440,7 @@
     <t>OSCURO</t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 15:11  06-05-2026</t>
+    <t>ULTIMA ACTUALIZACION 12:15  07-05-2026</t>
   </si>
 </sst>
 </file>
@@ -983,10 +983,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FB535F-634B-4933-81FF-529A98082563}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="B2:L31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="s">
         <v>15</v>
       </c>
@@ -1001,7 +1002,7 @@
       <c r="K2" s="16"/>
       <c r="L2" s="16"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
@@ -1036,7 +1037,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="8" t="s">
         <v>38</v>
       </c>
@@ -1066,7 +1067,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="8" t="s">
         <v>19</v>
       </c>
@@ -1094,7 +1095,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>40</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="8" t="s">
         <v>42</v>
       </c>
@@ -1148,7 +1149,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>41</v>
       </c>
@@ -1176,7 +1177,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>18</v>
       </c>
@@ -1200,7 +1201,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="8" t="s">
         <v>43</v>
       </c>
@@ -1230,7 +1231,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="8" t="s">
         <v>44</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1280,7 +1281,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="8" t="s">
         <v>23</v>
       </c>
@@ -1308,7 +1309,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="8" t="s">
         <v>30</v>
       </c>
@@ -1342,7 +1343,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="8" t="s">
         <v>36</v>
       </c>
@@ -1368,7 +1369,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="8" t="s">
         <v>33</v>
       </c>
@@ -1392,7 +1393,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="8" t="s">
         <v>37</v>
       </c>
@@ -1424,7 +1425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
@@ -1448,7 +1449,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="8" t="s">
         <v>20</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="8" t="s">
         <v>29</v>
       </c>
@@ -1508,7 +1509,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="8" t="s">
         <v>39</v>
       </c>
@@ -1532,7 +1533,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="8" t="s">
         <v>25</v>
       </c>
@@ -1556,7 +1557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="8" t="s">
         <v>24</v>
       </c>
@@ -1580,7 +1581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="8" t="s">
         <v>28</v>
       </c>
@@ -1604,7 +1605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="8" t="s">
         <v>35</v>
       </c>
@@ -1628,7 +1629,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="8" t="s">
         <v>27</v>
       </c>
@@ -1652,7 +1653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="8" t="s">
         <v>17</v>
       </c>
@@ -1678,7 +1679,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="8" t="s">
         <v>22</v>
       </c>
@@ -1704,7 +1705,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="8" t="s">
         <v>31</v>
       </c>
@@ -1726,7 +1727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
@@ -1748,7 +1749,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="8" t="s">
         <v>26</v>
       </c>
@@ -1782,10 +1783,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011174A9-0248-46ED-981A-FD90D8DB99B2}">
+  <sheetPr codeName="Hoja2"/>
   <dimension ref="B3:L20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
       <c r="B3" s="15" t="s">
         <v>45</v>
       </c>
@@ -1800,7 +1802,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1835,7 +1837,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="14">
         <v>389201</v>
       </c>
@@ -1869,7 +1871,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="14">
         <v>380200</v>
       </c>
@@ -1903,7 +1905,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="14">
         <v>383400</v>
       </c>
@@ -1937,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="14">
         <v>382100</v>
       </c>
@@ -1971,7 +1973,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="14">
         <v>388000</v>
       </c>
@@ -2005,7 +2007,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="14">
         <v>389300</v>
       </c>
@@ -2039,7 +2041,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="14">
         <v>385371</v>
       </c>
@@ -2073,7 +2075,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="14">
         <v>386501</v>
       </c>
@@ -2107,7 +2109,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="14">
         <v>385304</v>
       </c>
@@ -2141,7 +2143,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="14">
         <v>388300</v>
       </c>
@@ -2175,7 +2177,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="14">
         <v>387900</v>
       </c>
@@ -2209,7 +2211,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="14">
         <v>385800</v>
       </c>
@@ -2243,7 +2245,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="14">
         <v>381801</v>
       </c>
@@ -2277,7 +2279,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="14">
         <v>389401</v>
       </c>
@@ -2311,7 +2313,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="14">
         <v>382101</v>
       </c>
@@ -2345,7 +2347,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="14">
         <v>389700</v>
       </c>
@@ -2389,10 +2391,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE2264EF-F28E-4311-81D5-A7BF6F5FC77F}">
+  <sheetPr codeName="Hoja3"/>
   <dimension ref="B3:L15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
       <c r="B3" s="15" t="s">
         <v>46</v>
       </c>
@@ -2407,7 +2410,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -2442,7 +2445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="8" t="s">
         <v>56</v>
       </c>
@@ -2476,7 +2479,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>52</v>
       </c>
@@ -2506,7 +2509,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="8" t="s">
         <v>47</v>
       </c>
@@ -2536,7 +2539,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>50</v>
       </c>
@@ -2566,7 +2569,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
@@ -2594,7 +2597,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="8" t="s">
         <v>53</v>
       </c>
@@ -2620,7 +2623,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="8" t="s">
         <v>55</v>
       </c>
@@ -2648,7 +2651,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="8" t="s">
         <v>54</v>
       </c>
@@ -2674,7 +2677,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="8" t="s">
         <v>48</v>
       </c>
@@ -2698,7 +2701,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="8" t="s">
         <v>49</v>
       </c>
@@ -2722,7 +2725,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="8" t="s">
         <v>58</v>
       </c>
@@ -2756,13 +2759,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFAA1C20-0AB4-435A-AEDE-B6C824B1C346}">
+  <sheetPr codeName="Hoja4"/>
   <dimension ref="B3:L49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
       <c r="B3" s="15" t="s">
         <v>59</v>
       </c>
@@ -2777,7 +2781,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -2812,7 +2816,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="8" t="s">
         <v>60</v>
       </c>
@@ -2846,7 +2850,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>61</v>
       </c>
@@ -2880,7 +2884,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="8" t="s">
         <v>62</v>
       </c>
@@ -2914,7 +2918,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>64</v>
       </c>
@@ -2948,7 +2952,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>63</v>
       </c>
@@ -2982,7 +2986,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="8" t="s">
         <v>65</v>
       </c>
@@ -3016,7 +3020,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="8" t="s">
         <v>66</v>
       </c>
@@ -3050,7 +3054,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="8" t="s">
         <v>68</v>
       </c>
@@ -3084,7 +3088,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="8" t="s">
         <v>69</v>
       </c>
@@ -3118,7 +3122,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="8" t="s">
         <v>70</v>
       </c>
@@ -3152,7 +3156,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="8" t="s">
         <v>71</v>
       </c>
@@ -3186,7 +3190,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="8" t="s">
         <v>72</v>
       </c>
@@ -3220,7 +3224,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="8" t="s">
         <v>73</v>
       </c>
@@ -3254,7 +3258,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="8" t="s">
         <v>74</v>
       </c>
@@ -3288,7 +3292,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="8" t="s">
         <v>75</v>
       </c>
@@ -3322,7 +3326,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="8" t="s">
         <v>76</v>
       </c>
@@ -3356,7 +3360,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="8" t="s">
         <v>77</v>
       </c>
@@ -3390,7 +3394,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="8" t="s">
         <v>78</v>
       </c>
@@ -3424,7 +3428,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="8" t="s">
         <v>79</v>
       </c>
@@ -3458,7 +3462,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="8" t="s">
         <v>80</v>
       </c>
@@ -3492,7 +3496,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="8" t="s">
         <v>81</v>
       </c>
@@ -3526,7 +3530,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="8" t="s">
         <v>82</v>
       </c>
@@ -3560,7 +3564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="8" t="s">
         <v>84</v>
       </c>
@@ -3594,7 +3598,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="8" t="s">
         <v>85</v>
       </c>
@@ -3628,7 +3632,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="8" t="s">
         <v>86</v>
       </c>
@@ -3662,7 +3666,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="8" t="s">
         <v>89</v>
       </c>
@@ -3696,7 +3700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="8" t="s">
         <v>88</v>
       </c>
@@ -3730,7 +3734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="8" t="s">
         <v>90</v>
       </c>
@@ -3764,7 +3768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="8" t="s">
         <v>91</v>
       </c>
@@ -3798,7 +3802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="8" t="s">
         <v>92</v>
       </c>
@@ -3832,7 +3836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="8" t="s">
         <v>93</v>
       </c>
@@ -3866,7 +3870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="8" t="s">
         <v>94</v>
       </c>
@@ -3900,7 +3904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="8" t="s">
         <v>96</v>
       </c>
@@ -3934,7 +3938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="8" t="s">
         <v>97</v>
       </c>
@@ -3968,7 +3972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="8" t="s">
         <v>98</v>
       </c>
@@ -4002,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="8" t="s">
         <v>99</v>
       </c>
@@ -4036,7 +4040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="8" t="s">
         <v>100</v>
       </c>
@@ -4070,7 +4074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="8" t="s">
         <v>101</v>
       </c>
@@ -4104,7 +4108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="8" t="s">
         <v>102</v>
       </c>
@@ -4138,7 +4142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="8" t="s">
         <v>103</v>
       </c>
@@ -4172,7 +4176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="8" t="s">
         <v>104</v>
       </c>
@@ -4206,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="8" t="s">
         <v>105</v>
       </c>
@@ -4240,7 +4244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="8" t="s">
         <v>106</v>
       </c>
@@ -4274,7 +4278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="8" t="s">
         <v>108</v>
       </c>
@@ -4308,7 +4312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B49" s="8" t="s">
         <v>110</v>
       </c>
@@ -4352,10 +4356,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E9EB22C-7ED7-4D45-8EA1-BD18A384D586}">
+  <sheetPr codeName="Hoja5"/>
   <dimension ref="B3:L17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
       <c r="B3" s="15" t="s">
         <v>111</v>
       </c>
@@ -4370,7 +4375,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4405,7 +4410,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="8" t="s">
         <v>112</v>
       </c>
@@ -4439,7 +4444,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>121</v>
       </c>
@@ -4471,7 +4476,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="8" t="s">
         <v>114</v>
       </c>
@@ -4505,7 +4510,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="8" t="s">
         <v>116</v>
       </c>
@@ -4539,7 +4544,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="8" t="s">
         <v>115</v>
       </c>
@@ -4573,7 +4578,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="8" t="s">
         <v>117</v>
       </c>
@@ -4607,7 +4612,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="8" t="s">
         <v>118</v>
       </c>
@@ -4641,7 +4646,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="8" t="s">
         <v>119</v>
       </c>
@@ -4675,7 +4680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="8" t="s">
         <v>120</v>
       </c>
@@ -4709,7 +4714,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J17" t="s">
         <v>123</v>
       </c>
@@ -4724,13 +4729,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+  <sheetPr codeName="Hoja6" filterMode="1"/>
   <dimension ref="A2:P127"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4765,7 +4771,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -4796,11 +4802,11 @@
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="1">
-        <f>SUM(F3:K3)</f>
+        <f t="shared" ref="L3:L49" si="0">SUM(F3:K3)</f>
         <v>205</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B4" s="6">
         <v>423500</v>
       </c>
@@ -4830,11 +4836,11 @@
         <v>23</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>126</v>
       </c>
@@ -4849,29 +4855,29 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G5" s="4">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H5" s="4">
+        <v>43</v>
+      </c>
+      <c r="I5" s="4">
+        <v>39</v>
+      </c>
+      <c r="J5" s="4">
         <v>32</v>
       </c>
-      <c r="I5" s="4">
-        <v>27</v>
-      </c>
-      <c r="J5" s="4">
-        <v>24</v>
-      </c>
       <c r="K5" s="4">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6">
         <v>420600</v>
       </c>
@@ -4901,7 +4907,7 @@
         <v>13</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
+        <f t="shared" si="0"/>
         <v>126</v>
       </c>
       <c r="M6" t="s">
@@ -4911,7 +4917,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6">
         <v>420100</v>
       </c>
@@ -4939,11 +4945,11 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
+        <f t="shared" si="0"/>
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6">
         <v>424400</v>
       </c>
@@ -4971,11 +4977,11 @@
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
+        <f t="shared" si="0"/>
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6">
         <v>422300</v>
       </c>
@@ -5003,12 +5009,12 @@
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
+        <f t="shared" si="0"/>
         <v>83</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>123</v>
       </c>
@@ -5041,14 +5047,14 @@
         <v>10</v>
       </c>
       <c r="L10" s="12">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6">
         <v>420400</v>
       </c>
@@ -5078,14 +5084,14 @@
         <v>16</v>
       </c>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
+        <f t="shared" si="0"/>
         <v>72</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B12" s="6">
         <v>423200</v>
       </c>
@@ -5115,14 +5121,14 @@
         <v>14</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
+        <f t="shared" si="0"/>
         <v>71</v>
       </c>
       <c r="N12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6">
         <v>422500</v>
       </c>
@@ -5152,14 +5158,14 @@
         <v>17</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>123</v>
       </c>
@@ -5190,14 +5196,14 @@
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>123</v>
       </c>
@@ -5224,12 +5230,12 @@
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="B16" s="6">
         <v>422000</v>
       </c>
@@ -5257,14 +5263,14 @@
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B17" s="6">
         <v>423316</v>
       </c>
@@ -5294,11 +5300,11 @@
         <v>4</v>
       </c>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B18" s="6">
         <v>422101</v>
       </c>
@@ -5326,11 +5332,11 @@
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B19" s="6">
         <v>421400</v>
       </c>
@@ -5360,11 +5366,11 @@
         <v>32</v>
       </c>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B20" s="6">
         <v>420800</v>
       </c>
@@ -5394,11 +5400,11 @@
         <v>6</v>
       </c>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B21" s="6">
         <v>421801</v>
       </c>
@@ -5426,11 +5432,11 @@
         <v>12</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B22" s="6">
         <v>420160</v>
       </c>
@@ -5462,11 +5468,11 @@
         <v>5</v>
       </c>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B23" s="6">
         <v>421100</v>
       </c>
@@ -5496,11 +5502,11 @@
         <v>7</v>
       </c>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B24" s="6">
         <v>422700</v>
       </c>
@@ -5528,11 +5534,11 @@
         <v>10</v>
       </c>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="6">
         <v>423000</v>
       </c>
@@ -5558,11 +5564,11 @@
         <v>9</v>
       </c>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B26" s="6">
         <v>424900</v>
       </c>
@@ -5594,11 +5600,11 @@
         <v>0</v>
       </c>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="6">
         <v>424900</v>
       </c>
@@ -5628,11 +5634,11 @@
         <v>1</v>
       </c>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B28" s="6">
         <v>421000</v>
       </c>
@@ -5662,11 +5668,11 @@
         <v>2</v>
       </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B29" s="6">
         <v>424000</v>
       </c>
@@ -5690,11 +5696,11 @@
       </c>
       <c r="K29" s="4"/>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B30" s="6">
         <v>422701</v>
       </c>
@@ -5720,11 +5726,11 @@
         <v>14</v>
       </c>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6">
         <v>423448</v>
       </c>
@@ -5754,11 +5760,11 @@
         <v>1</v>
       </c>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B32" s="6">
         <v>420101</v>
       </c>
@@ -5786,11 +5792,11 @@
         <v>2</v>
       </c>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B33" s="6">
         <v>424701</v>
       </c>
@@ -5814,11 +5820,11 @@
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="1">
-        <f>SUM(F33:K33)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B34" s="6">
         <v>421901</v>
       </c>
@@ -5848,11 +5854,11 @@
         <v>1</v>
       </c>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="6">
         <v>422900</v>
       </c>
@@ -5876,11 +5882,11 @@
       </c>
       <c r="K35" s="4"/>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6">
         <v>421902</v>
       </c>
@@ -5910,11 +5916,11 @@
         <v>2</v>
       </c>
       <c r="L36" s="1">
-        <f>SUM(F36:K36)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="6">
         <v>420501</v>
       </c>
@@ -5942,11 +5948,11 @@
         <v>4</v>
       </c>
       <c r="L37" s="1">
-        <f>SUM(F37:K37)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B38" s="6">
         <v>420301</v>
       </c>
@@ -5976,11 +5982,11 @@
         <v>15</v>
       </c>
       <c r="L38" s="1">
-        <f>SUM(F38:K38)</f>
+        <f t="shared" si="0"/>
         <v>165</v>
       </c>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="6">
         <v>422190</v>
       </c>
@@ -6012,11 +6018,11 @@
         <v>3</v>
       </c>
       <c r="L39" s="1">
-        <f>SUM(F39:K39)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="6">
         <v>421900</v>
       </c>
@@ -6044,11 +6050,11 @@
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="1">
-        <f>SUM(F40:K40)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="6">
         <v>423501</v>
       </c>
@@ -6078,11 +6084,11 @@
         <v>6</v>
       </c>
       <c r="L41" s="1">
-        <f>SUM(F41:K41)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="6">
         <v>423308</v>
       </c>
@@ -6108,11 +6114,11 @@
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="1">
-        <f>SUM(F42:K42)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B43" s="6">
         <v>423408</v>
       </c>
@@ -6136,11 +6142,11 @@
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f>SUM(F43:K43)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="6">
         <v>424801</v>
       </c>
@@ -6168,11 +6174,11 @@
         <v>2</v>
       </c>
       <c r="L44" s="1">
-        <f>SUM(F44:K44)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="6">
         <v>420900</v>
       </c>
@@ -6196,11 +6202,11 @@
         <v>10</v>
       </c>
       <c r="L45" s="1">
-        <f>SUM(F45:K45)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="6">
         <v>423900</v>
       </c>
@@ -6224,11 +6230,11 @@
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="1">
-        <f>SUM(F46:K46)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="6">
         <v>422100</v>
       </c>
@@ -6250,11 +6256,11 @@
         <v>13</v>
       </c>
       <c r="L47" s="1">
-        <f>SUM(F47:K47)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="6">
         <v>424500</v>
       </c>
@@ -6280,11 +6286,11 @@
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f>SUM(F48:K48)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="6">
         <v>424700</v>
       </c>
@@ -6308,11 +6314,11 @@
         <v>5</v>
       </c>
       <c r="L49" s="1">
-        <f>SUM(F49:K49)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="6">
         <v>420802</v>
       </c>
@@ -6344,7 +6350,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="6">
         <v>420200</v>
       </c>
@@ -6366,11 +6372,11 @@
         <v>13</v>
       </c>
       <c r="L51" s="1">
-        <f>SUM(F51:K51)</f>
+        <f t="shared" ref="L51:L62" si="1">SUM(F51:K51)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B52" s="6">
         <v>421301</v>
       </c>
@@ -6396,11 +6402,11 @@
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f>SUM(F52:K52)</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B53" s="6">
         <v>424300</v>
       </c>
@@ -6424,11 +6430,11 @@
         <v>6</v>
       </c>
       <c r="L53" s="1">
-        <f>SUM(F53:K53)</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B54" s="6">
         <v>421402</v>
       </c>
@@ -6456,11 +6462,11 @@
         <v>2</v>
       </c>
       <c r="L54" s="1">
-        <f>SUM(F54:K54)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B55" s="6">
         <v>425600</v>
       </c>
@@ -6484,11 +6490,11 @@
         <v>7</v>
       </c>
       <c r="L55" s="1">
-        <f>SUM(F55:K55)</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B56" s="6">
         <v>423304</v>
       </c>
@@ -6512,11 +6518,11 @@
         <v>2</v>
       </c>
       <c r="L56" s="1">
-        <f>SUM(F56:K56)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B57" s="6">
         <v>421300</v>
       </c>
@@ -6540,11 +6546,11 @@
         <v>4</v>
       </c>
       <c r="L57" s="1">
-        <f>SUM(F57:K57)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B58" s="6">
         <v>424960</v>
       </c>
@@ -6574,14 +6580,14 @@
         <v>1</v>
       </c>
       <c r="L58" s="12">
-        <f>SUM(F58:K58)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B59" s="6">
         <v>421800</v>
       </c>
@@ -6607,11 +6613,11 @@
         <v>1</v>
       </c>
       <c r="L59" s="1">
-        <f>SUM(F59:K59)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B60" s="6">
         <v>423348</v>
       </c>
@@ -6637,11 +6643,11 @@
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="1">
-        <f>SUM(F60:K60)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="6">
         <v>422601</v>
       </c>
@@ -6661,11 +6667,11 @@
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f>SUM(F61:K61)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="6">
         <v>421401</v>
       </c>
@@ -6689,11 +6695,11 @@
         <v>1</v>
       </c>
       <c r="L62" s="1">
-        <f>SUM(F62:K62)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B63" s="6">
         <v>421001</v>
       </c>
@@ -6723,7 +6729,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B64" s="6">
         <v>420500</v>
       </c>
@@ -6747,11 +6753,11 @@
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f>SUM(F64:K64)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L64:L74" si="2">SUM(F64:K64)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="6">
         <v>420402</v>
       </c>
@@ -6771,11 +6777,11 @@
       </c>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f>SUM(F65:K65)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="6">
         <v>423416</v>
       </c>
@@ -6799,11 +6805,11 @@
       </c>
       <c r="K66" s="4"/>
       <c r="L66" s="1">
-        <f>SUM(F66:K66)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="6">
         <v>422600</v>
       </c>
@@ -6823,11 +6829,11 @@
         <v>3</v>
       </c>
       <c r="L67" s="1">
-        <f>SUM(F67:K67)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="6">
         <v>423309</v>
       </c>
@@ -6851,11 +6857,11 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f>SUM(F68:K68)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="6">
         <v>422400</v>
       </c>
@@ -6875,11 +6881,11 @@
       </c>
       <c r="K69" s="6"/>
       <c r="L69" s="1">
-        <f>SUM(F69:K69)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="6">
         <v>422401</v>
       </c>
@@ -6897,11 +6903,11 @@
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
       <c r="L70" s="1">
-        <f>SUM(F70:K70)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="6">
         <v>423800</v>
       </c>
@@ -6921,11 +6927,11 @@
       <c r="J71" s="6"/>
       <c r="K71" s="6"/>
       <c r="L71" s="1">
-        <f>SUM(F71:K71)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="6">
         <v>424200</v>
       </c>
@@ -6943,11 +6949,11 @@
       <c r="J72" s="6"/>
       <c r="K72" s="6"/>
       <c r="L72" s="12">
-        <f>SUM(F72:K72)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="6">
         <v>423409</v>
       </c>
@@ -6965,11 +6971,11 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f>SUM(F73:K73)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="6">
         <v>423404</v>
       </c>
@@ -6987,11 +6993,11 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f>SUM(F74:K74)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="6">
         <v>420801</v>
       </c>
@@ -7013,7 +7019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="B76" s="6">
         <v>420160</v>
       </c>
@@ -7040,30 +7046,35 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="E77" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:13" x14ac:dyDescent="0.35">
       <c r="L79" s="10">
         <f>SUM(L3:L78)</f>
-        <v>2833</v>
-      </c>
-    </row>
-    <row r="83" spans="15:15" x14ac:dyDescent="0.25">
+        <v>2889</v>
+      </c>
+    </row>
+    <row r="83" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O83" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="127" spans="11:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K127" t="s">
         <v>123</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B2:L77" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L77">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="423000"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B25:L25">
       <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
   </autoFilter>
@@ -7073,10 +7084,11 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr codeName="Hoja7"/>
+  <dimension ref="B3:L4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
@@ -7109,6 +7121,11 @@
       </c>
       <c r="L3" s="2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -7118,6 +7135,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7261,15 +7287,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -7277,6 +7294,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7290,14 +7315,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizar stock bodega con coleccion 43
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2631" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21404990-CE57-4093-A4A2-1C3476524D88}"/>
+  <xr:revisionPtr revIDLastSave="2878" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E45A504F-C099-40E6-9150-FF1D30549160}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="132">
   <si>
     <t>CODIGO</t>
   </si>
@@ -441,6 +441,12 @@
   </si>
   <si>
     <t>ULTIMA ACTUALIZACION 12:15  07-05-2026</t>
+  </si>
+  <si>
+    <t>WIDE</t>
+  </si>
+  <si>
+    <t>WIDE LEG</t>
   </si>
 </sst>
 </file>
@@ -563,7 +569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -603,6 +609,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -983,11 +990,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FB535F-634B-4933-81FF-529A98082563}">
-  <sheetPr codeName="Hoja1"/>
   <dimension ref="B2:L31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
         <v>15</v>
       </c>
@@ -1002,7 +1008,7 @@
       <c r="K2" s="16"/>
       <c r="L2" s="16"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
@@ -1037,7 +1043,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
         <v>38</v>
       </c>
@@ -1067,7 +1073,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>19</v>
       </c>
@@ -1095,7 +1101,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>40</v>
       </c>
@@ -1123,7 +1129,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
         <v>42</v>
       </c>
@@ -1149,7 +1155,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>41</v>
       </c>
@@ -1177,7 +1183,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
         <v>18</v>
       </c>
@@ -1201,7 +1207,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>43</v>
       </c>
@@ -1231,7 +1237,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>44</v>
       </c>
@@ -1255,7 +1261,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1281,7 +1287,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>23</v>
       </c>
@@ -1309,7 +1315,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
         <v>30</v>
       </c>
@@ -1343,7 +1349,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>36</v>
       </c>
@@ -1369,7 +1375,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>33</v>
       </c>
@@ -1393,7 +1399,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>37</v>
       </c>
@@ -1425,7 +1431,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
@@ -1449,7 +1455,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
         <v>20</v>
       </c>
@@ -1477,7 +1483,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
         <v>29</v>
       </c>
@@ -1509,7 +1515,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="8" t="s">
         <v>39</v>
       </c>
@@ -1533,7 +1539,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
         <v>25</v>
       </c>
@@ -1557,7 +1563,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
         <v>24</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>28</v>
       </c>
@@ -1605,7 +1611,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>35</v>
       </c>
@@ -1629,7 +1635,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
         <v>27</v>
       </c>
@@ -1653,7 +1659,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="8" t="s">
         <v>17</v>
       </c>
@@ -1679,7 +1685,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
         <v>22</v>
       </c>
@@ -1705,7 +1711,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="8" t="s">
         <v>31</v>
       </c>
@@ -1727,7 +1733,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
         <v>34</v>
       </c>
@@ -1749,7 +1755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
         <v>26</v>
       </c>
@@ -1783,11 +1789,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011174A9-0248-46ED-981A-FD90D8DB99B2}">
-  <sheetPr codeName="Hoja2"/>
   <dimension ref="B3:L20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>45</v>
       </c>
@@ -1802,7 +1807,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1837,7 +1842,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="14">
         <v>389201</v>
       </c>
@@ -1871,7 +1876,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="14">
         <v>380200</v>
       </c>
@@ -1905,7 +1910,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="14">
         <v>383400</v>
       </c>
@@ -1939,7 +1944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="14">
         <v>382100</v>
       </c>
@@ -1973,7 +1978,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="14">
         <v>388000</v>
       </c>
@@ -2007,7 +2012,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="14">
         <v>389300</v>
       </c>
@@ -2041,7 +2046,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="14">
         <v>385371</v>
       </c>
@@ -2075,7 +2080,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="14">
         <v>386501</v>
       </c>
@@ -2109,7 +2114,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="14">
         <v>385304</v>
       </c>
@@ -2143,7 +2148,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="14">
         <v>388300</v>
       </c>
@@ -2177,7 +2182,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="14">
         <v>387900</v>
       </c>
@@ -2211,7 +2216,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="14">
         <v>385800</v>
       </c>
@@ -2245,7 +2250,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="14">
         <v>381801</v>
       </c>
@@ -2279,7 +2284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="14">
         <v>389401</v>
       </c>
@@ -2313,7 +2318,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="14">
         <v>382101</v>
       </c>
@@ -2347,7 +2352,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="14">
         <v>389700</v>
       </c>
@@ -2391,11 +2396,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE2264EF-F28E-4311-81D5-A7BF6F5FC77F}">
-  <sheetPr codeName="Hoja3"/>
   <dimension ref="B3:L15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>46</v>
       </c>
@@ -2410,7 +2414,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -2445,7 +2449,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>56</v>
       </c>
@@ -2479,7 +2483,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>52</v>
       </c>
@@ -2509,7 +2513,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
         <v>47</v>
       </c>
@@ -2539,7 +2543,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>50</v>
       </c>
@@ -2569,7 +2573,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
@@ -2597,7 +2601,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>53</v>
       </c>
@@ -2623,7 +2627,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>55</v>
       </c>
@@ -2651,7 +2655,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>54</v>
       </c>
@@ -2677,7 +2681,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>48</v>
       </c>
@@ -2701,7 +2705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
         <v>49</v>
       </c>
@@ -2725,7 +2729,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>58</v>
       </c>
@@ -2759,14 +2763,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFAA1C20-0AB4-435A-AEDE-B6C824B1C346}">
-  <sheetPr codeName="Hoja4"/>
   <dimension ref="B3:L49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>59</v>
       </c>
@@ -2781,7 +2784,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -2816,7 +2819,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>60</v>
       </c>
@@ -2850,7 +2853,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>61</v>
       </c>
@@ -2884,7 +2887,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
         <v>62</v>
       </c>
@@ -2918,7 +2921,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>64</v>
       </c>
@@ -2952,7 +2955,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
         <v>63</v>
       </c>
@@ -2986,7 +2989,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>65</v>
       </c>
@@ -3020,7 +3023,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>66</v>
       </c>
@@ -3054,7 +3057,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>68</v>
       </c>
@@ -3088,7 +3091,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>69</v>
       </c>
@@ -3122,7 +3125,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
         <v>70</v>
       </c>
@@ -3156,7 +3159,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>71</v>
       </c>
@@ -3190,7 +3193,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>72</v>
       </c>
@@ -3224,7 +3227,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>73</v>
       </c>
@@ -3258,7 +3261,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>74</v>
       </c>
@@ -3292,7 +3295,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
         <v>75</v>
       </c>
@@ -3326,7 +3329,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
         <v>76</v>
       </c>
@@ -3360,7 +3363,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="8" t="s">
         <v>77</v>
       </c>
@@ -3394,7 +3397,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
         <v>78</v>
       </c>
@@ -3428,7 +3431,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
         <v>79</v>
       </c>
@@ -3462,7 +3465,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>80</v>
       </c>
@@ -3496,7 +3499,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>81</v>
       </c>
@@ -3530,7 +3533,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
         <v>82</v>
       </c>
@@ -3564,7 +3567,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="8" t="s">
         <v>84</v>
       </c>
@@ -3598,7 +3601,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
         <v>85</v>
       </c>
@@ -3632,7 +3635,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="8" t="s">
         <v>86</v>
       </c>
@@ -3666,7 +3669,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
         <v>89</v>
       </c>
@@ -3700,7 +3703,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
         <v>88</v>
       </c>
@@ -3734,7 +3737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>90</v>
       </c>
@@ -3768,7 +3771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="8" t="s">
         <v>91</v>
       </c>
@@ -3802,7 +3805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="8" t="s">
         <v>92</v>
       </c>
@@ -3836,7 +3839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="8" t="s">
         <v>93</v>
       </c>
@@ -3870,7 +3873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
         <v>94</v>
       </c>
@@ -3904,7 +3907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="8" t="s">
         <v>96</v>
       </c>
@@ -3938,7 +3941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="8" t="s">
         <v>97</v>
       </c>
@@ -3972,7 +3975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="8" t="s">
         <v>98</v>
       </c>
@@ -4006,7 +4009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="8" t="s">
         <v>99</v>
       </c>
@@ -4040,7 +4043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="8" t="s">
         <v>100</v>
       </c>
@@ -4074,7 +4077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="8" t="s">
         <v>101</v>
       </c>
@@ -4108,7 +4111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
         <v>102</v>
       </c>
@@ -4142,7 +4145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="8" t="s">
         <v>103</v>
       </c>
@@ -4176,7 +4179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="8" t="s">
         <v>104</v>
       </c>
@@ -4210,7 +4213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
         <v>105</v>
       </c>
@@ -4244,7 +4247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="8" t="s">
         <v>106</v>
       </c>
@@ -4278,7 +4281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
         <v>108</v>
       </c>
@@ -4312,7 +4315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="8" t="s">
         <v>110</v>
       </c>
@@ -4356,11 +4359,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E9EB22C-7ED7-4D45-8EA1-BD18A384D586}">
-  <sheetPr codeName="Hoja5"/>
   <dimension ref="B3:L17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>111</v>
       </c>
@@ -4375,7 +4377,7 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>0</v>
       </c>
@@ -4410,7 +4412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">
         <v>112</v>
       </c>
@@ -4444,7 +4446,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>121</v>
       </c>
@@ -4476,7 +4478,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
         <v>114</v>
       </c>
@@ -4510,7 +4512,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>116</v>
       </c>
@@ -4544,7 +4546,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
         <v>115</v>
       </c>
@@ -4578,7 +4580,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>117</v>
       </c>
@@ -4612,7 +4614,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>118</v>
       </c>
@@ -4646,7 +4648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>119</v>
       </c>
@@ -4680,7 +4682,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>120</v>
       </c>
@@ -4714,9 +4716,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J17" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -4729,14 +4731,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <sheetPr codeName="Hoja6" filterMode="1"/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A2:P127"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4771,144 +4773,144 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>123</v>
       </c>
       <c r="B3" s="6">
-        <v>422200</v>
+        <v>423600</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
+        <v>24</v>
+      </c>
+      <c r="G3" s="4">
+        <v>46</v>
+      </c>
+      <c r="H3" s="4">
+        <v>43</v>
+      </c>
+      <c r="I3" s="4">
+        <v>39</v>
+      </c>
+      <c r="J3" s="4">
+        <v>32</v>
+      </c>
+      <c r="K3" s="4">
+        <v>25</v>
+      </c>
+      <c r="L3" s="1">
+        <f>SUM(F3:K3)</f>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="6">
+        <v>422200</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="G3" s="4">
-        <v>60</v>
-      </c>
-      <c r="H3" s="4">
-        <v>53</v>
-      </c>
-      <c r="I3" s="4">
-        <v>48</v>
-      </c>
-      <c r="J3" s="4">
-        <v>31</v>
-      </c>
-      <c r="K3" s="4"/>
-      <c r="L3" s="1">
-        <f t="shared" ref="L3:L49" si="0">SUM(F3:K3)</f>
-        <v>205</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="6">
-        <v>423500</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" s="4">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="H4" s="4">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="I4" s="4">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="J4" s="4">
-        <v>43</v>
-      </c>
-      <c r="K4" s="4">
-        <v>23</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="K4" s="4"/>
       <c r="L4" s="1">
-        <f t="shared" si="0"/>
-        <v>186</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F4:K4)</f>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>126</v>
       </c>
       <c r="B5" s="6">
-        <v>423600</v>
+        <v>423500</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="H5" s="4">
+        <v>36</v>
+      </c>
+      <c r="I5" s="4">
+        <v>33</v>
+      </c>
+      <c r="J5" s="4">
         <v>43</v>
       </c>
-      <c r="I5" s="4">
-        <v>39</v>
-      </c>
-      <c r="J5" s="4">
+      <c r="K5" s="4">
+        <v>23</v>
+      </c>
+      <c r="L5" s="1">
+        <f>SUM(F5:K5)</f>
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="6">
+        <v>420301</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="6">
+        <v>14</v>
+      </c>
+      <c r="G6" s="6">
         <v>32</v>
       </c>
-      <c r="K5" s="4">
-        <v>25</v>
-      </c>
-      <c r="L5" s="1">
-        <f t="shared" si="0"/>
-        <v>209</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="6">
-        <v>420600</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="4">
-        <v>38</v>
-      </c>
-      <c r="G6" s="4">
-        <v>22</v>
-      </c>
-      <c r="H6" s="4">
-        <v>10</v>
-      </c>
-      <c r="I6" s="4">
-        <v>17</v>
-      </c>
-      <c r="J6" s="4">
+      <c r="H6" s="6">
+        <v>34</v>
+      </c>
+      <c r="I6" s="6">
         <v>26</v>
       </c>
-      <c r="K6" s="4">
-        <v>13</v>
+      <c r="J6" s="6">
+        <v>28</v>
+      </c>
+      <c r="K6" s="6">
+        <v>8</v>
       </c>
       <c r="L6" s="1">
-        <f t="shared" si="0"/>
-        <v>126</v>
+        <f>SUM(F6:K6)</f>
+        <v>142</v>
       </c>
       <c r="M6" t="s">
         <v>123</v>
@@ -4917,9 +4919,9 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>420100</v>
+        <v>420600</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
@@ -4929,29 +4931,29 @@
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G7" s="4">
-        <v>22</v>
-      </c>
-      <c r="H7" s="4">
-        <v>52</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H7" s="4"/>
       <c r="I7" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J7" s="4">
+        <v>18</v>
+      </c>
+      <c r="K7" s="4">
         <v>8</v>
       </c>
-      <c r="K7" s="4"/>
       <c r="L7" s="1">
-        <f t="shared" si="0"/>
-        <v>121</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F7:K7)</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
-        <v>424400</v>
+        <v>420100</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
@@ -4964,903 +4966,887 @@
         <v>27</v>
       </c>
       <c r="G8" s="4">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H8" s="4">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="I8" s="4">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="J8" s="4">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="1">
-        <f t="shared" si="0"/>
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F8:K8)</f>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
-        <v>422300</v>
+        <v>424400</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G9" s="4">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H9" s="4">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="I9" s="4">
-        <v>19</v>
-      </c>
-      <c r="J9" s="4">
-        <v>16</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f t="shared" si="0"/>
-        <v>83</v>
+        <f>SUM(F9:K9)</f>
+        <v>110</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>123</v>
       </c>
       <c r="B10" s="6">
-        <v>420300</v>
+        <v>422300</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="6">
-        <v>13</v>
-      </c>
-      <c r="G10" s="6">
-        <v>15</v>
-      </c>
-      <c r="H10" s="6">
+      <c r="F10" s="4">
+        <v>18</v>
+      </c>
+      <c r="G10" s="4">
+        <v>19</v>
+      </c>
+      <c r="H10" s="4">
+        <v>11</v>
+      </c>
+      <c r="I10" s="4">
+        <v>19</v>
+      </c>
+      <c r="J10" s="4">
         <v>16</v>
       </c>
-      <c r="I10" s="6">
-        <v>15</v>
-      </c>
-      <c r="J10" s="6">
-        <v>11</v>
-      </c>
-      <c r="K10" s="6">
-        <v>10</v>
-      </c>
-      <c r="L10" s="12">
-        <f t="shared" si="0"/>
-        <v>80</v>
+      <c r="K10" s="4"/>
+      <c r="L10" s="1">
+        <f>SUM(F10:K10)</f>
+        <v>83</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>420400</v>
+        <v>420300</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="4">
-        <v>26</v>
-      </c>
-      <c r="G11" s="4">
-        <v>6</v>
-      </c>
-      <c r="H11" s="4">
-        <v>9</v>
-      </c>
-      <c r="I11" s="4">
-        <v>7</v>
-      </c>
-      <c r="J11" s="4">
-        <v>8</v>
-      </c>
-      <c r="K11" s="4">
+      <c r="F11" s="6">
+        <v>13</v>
+      </c>
+      <c r="G11" s="6">
+        <v>15</v>
+      </c>
+      <c r="H11" s="6">
         <v>16</v>
       </c>
-      <c r="L11" s="1">
-        <f t="shared" si="0"/>
-        <v>72</v>
+      <c r="I11" s="6">
+        <v>15</v>
+      </c>
+      <c r="J11" s="6">
+        <v>11</v>
+      </c>
+      <c r="K11" s="6">
+        <v>10</v>
+      </c>
+      <c r="L11" s="12">
+        <f>SUM(F11:K11)</f>
+        <v>80</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>423200</v>
+        <v>420400</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="G12" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H12" s="4">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I12" s="4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J12" s="4">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K12" s="4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L12" s="1">
-        <f t="shared" si="0"/>
-        <v>71</v>
+        <f>SUM(F12:K12)</f>
+        <v>72</v>
       </c>
       <c r="N12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>422500</v>
+        <v>423200</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="4">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G13" s="4">
         <v>1</v>
       </c>
       <c r="H13" s="4">
+        <v>17</v>
+      </c>
+      <c r="I13" s="4">
         <v>14</v>
       </c>
-      <c r="I13" s="4">
-        <v>15</v>
-      </c>
       <c r="J13" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K13" s="4">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="0"/>
-        <v>68</v>
+        <f>SUM(F13:K13)</f>
+        <v>71</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>123</v>
       </c>
       <c r="B14" s="6">
-        <v>424600</v>
+        <v>422500</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>4</v>
-      </c>
-      <c r="G14" s="4">
-        <v>4</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G14" s="4"/>
       <c r="H14" s="4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I14" s="4">
+        <v>15</v>
+      </c>
+      <c r="J14" s="4">
+        <v>13</v>
+      </c>
+      <c r="K14" s="4">
         <v>17</v>
       </c>
-      <c r="J14" s="4">
-        <v>17</v>
-      </c>
-      <c r="K14" s="4"/>
       <c r="L14" s="1">
-        <f t="shared" si="0"/>
-        <v>64</v>
+        <f>SUM(F14:K14)</f>
+        <v>65</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>123</v>
       </c>
       <c r="B15" s="6">
-        <v>422800</v>
+        <v>424600</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="4"/>
+      <c r="F15" s="4">
+        <v>4</v>
+      </c>
       <c r="G15" s="4">
         <v>4</v>
       </c>
       <c r="H15" s="4">
-        <v>29</v>
-      </c>
-      <c r="I15" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="I15" s="4">
+        <v>17</v>
+      </c>
       <c r="J15" s="4">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>61</v>
+        <f>SUM(F15:K15)</f>
+        <v>64</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>422000</v>
+        <v>422800</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="4">
-        <v>34</v>
-      </c>
+      <c r="F16" s="4"/>
       <c r="G16" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H16" s="4">
-        <v>11</v>
-      </c>
-      <c r="I16" s="4">
-        <v>3</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="I16" s="4"/>
       <c r="J16" s="4">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F16:K16)</f>
         <v>61</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>423316</v>
+        <v>422000</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="4">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="G17" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H17" s="4">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I17" s="4">
+        <v>3</v>
+      </c>
+      <c r="J17" s="4">
+        <v>3</v>
+      </c>
+      <c r="K17" s="4"/>
+      <c r="L17" s="1">
+        <f>SUM(F17:K17)</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="6">
+        <v>423316</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="J17" s="4">
-        <v>8</v>
-      </c>
-      <c r="K17" s="4">
-        <v>4</v>
-      </c>
-      <c r="L17" s="1">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="6">
-        <v>422101</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="4">
+        <v>6</v>
+      </c>
+      <c r="G18" s="4">
         <v>14</v>
       </c>
-      <c r="G18" s="4">
-        <v>1</v>
-      </c>
       <c r="H18" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I18" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J18" s="4">
-        <v>14</v>
-      </c>
-      <c r="K18" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="K18" s="4">
+        <v>4</v>
+      </c>
       <c r="L18" s="1">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F18:K18)</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>421400</v>
+        <v>422101</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G19" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="4">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I19" s="4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J19" s="4">
-        <v>11</v>
-      </c>
-      <c r="K19" s="4">
+        <v>14</v>
+      </c>
+      <c r="K19" s="4"/>
+      <c r="L19" s="1">
+        <f>SUM(F19:K19)</f>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="6">
+        <v>421400</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="4">
+        <v>7</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4">
+        <v>1</v>
+      </c>
+      <c r="J20" s="4">
+        <v>12</v>
+      </c>
+      <c r="K20" s="4">
         <v>32</v>
       </c>
-      <c r="L19" s="1">
-        <f t="shared" si="0"/>
+      <c r="L20" s="1">
+        <f>SUM(F20:K20)</f>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="6">
+        <v>420800</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="6">
+        <v>6</v>
+      </c>
+      <c r="G21" s="6">
+        <v>10</v>
+      </c>
+      <c r="H21" s="6">
+        <v>12</v>
+      </c>
+      <c r="I21" s="6">
+        <v>12</v>
+      </c>
+      <c r="J21" s="6">
+        <v>6</v>
+      </c>
+      <c r="K21" s="4">
+        <v>6</v>
+      </c>
+      <c r="L21" s="1">
+        <f>SUM(F21:K21)</f>
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="6">
-        <v>420800</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="6">
-        <v>6</v>
-      </c>
-      <c r="G20" s="6">
+    <row r="22" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="6">
+        <v>421801</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4">
+        <v>2</v>
+      </c>
+      <c r="I22" s="4">
+        <v>3</v>
+      </c>
+      <c r="J22" s="4">
+        <v>13</v>
+      </c>
+      <c r="K22" s="4">
         <v>10</v>
       </c>
-      <c r="H20" s="6">
+      <c r="L22" s="1">
+        <f>SUM(F22:K22)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="6">
+        <v>420160</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="4">
+        <v>7</v>
+      </c>
+      <c r="G23" s="4">
         <v>12</v>
       </c>
-      <c r="I20" s="6">
-        <v>12</v>
-      </c>
-      <c r="J20" s="6">
-        <v>6</v>
-      </c>
-      <c r="K20" s="4">
-        <v>6</v>
-      </c>
-      <c r="L20" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="6">
-        <v>421801</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4">
-        <v>2</v>
-      </c>
-      <c r="H21" s="4">
-        <v>8</v>
-      </c>
-      <c r="I21" s="4">
-        <v>8</v>
-      </c>
-      <c r="J21" s="4">
-        <v>20</v>
-      </c>
-      <c r="K21" s="4">
-        <v>12</v>
-      </c>
-      <c r="L21" s="1">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="6">
-        <v>420160</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="H23" s="4">
+        <v>9</v>
+      </c>
+      <c r="I23" s="4">
         <v>10</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="4">
-        <v>7</v>
-      </c>
-      <c r="G22" s="4">
-        <v>12</v>
-      </c>
-      <c r="H22" s="4">
-        <v>9</v>
-      </c>
-      <c r="I22" s="4">
-        <v>10</v>
-      </c>
-      <c r="J22" s="4">
-        <v>6</v>
-      </c>
-      <c r="K22" s="4">
-        <v>5</v>
-      </c>
-      <c r="L22" s="1">
-        <f t="shared" si="0"/>
+      <c r="J23" s="4">
+        <v>6</v>
+      </c>
+      <c r="K23" s="4">
+        <v>5</v>
+      </c>
+      <c r="L23" s="1">
+        <f>SUM(F23:K23)</f>
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="6">
+    <row r="24" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="6">
         <v>421100</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="4">
-        <v>3</v>
-      </c>
-      <c r="G23" s="4">
-        <v>4</v>
-      </c>
-      <c r="H23" s="4">
-        <v>6</v>
-      </c>
-      <c r="I23" s="4">
-        <v>6</v>
-      </c>
-      <c r="J23" s="4">
-        <v>20</v>
-      </c>
-      <c r="K23" s="4">
-        <v>7</v>
-      </c>
-      <c r="L23" s="1">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="6">
-        <v>422700</v>
-      </c>
       <c r="C24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G24" s="4">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H24" s="4">
         <v>6</v>
       </c>
-      <c r="I24" s="4"/>
+      <c r="I24" s="4">
+        <v>6</v>
+      </c>
       <c r="J24" s="4">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K24" s="4">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F24:K24)</f>
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>423000</v>
+        <v>422700</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="4">
         <v>10</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4">
-        <v>4</v>
-      </c>
+      <c r="G25" s="4">
+        <v>14</v>
+      </c>
+      <c r="H25" s="4">
+        <v>6</v>
+      </c>
+      <c r="I25" s="4"/>
       <c r="J25" s="4">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="K25" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L25" s="1">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F25:K25)</f>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>424900</v>
+        <v>423000</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>125</v>
-      </c>
+      <c r="E26" s="1"/>
       <c r="F26" s="4">
+        <v>10</v>
+      </c>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4">
         <v>4</v>
       </c>
-      <c r="G26" s="4">
-        <v>12</v>
-      </c>
-      <c r="H26" s="1">
-        <v>13</v>
-      </c>
-      <c r="I26" s="4">
-        <v>6</v>
-      </c>
       <c r="J26" s="4">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="K26" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L26" s="1">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F26:K26)</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>424900</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F27" s="4">
+        <v>4</v>
+      </c>
+      <c r="G27" s="4">
+        <v>12</v>
+      </c>
+      <c r="H27" s="1">
+        <v>13</v>
+      </c>
+      <c r="I27" s="4">
+        <v>6</v>
+      </c>
+      <c r="J27" s="4">
+        <v>3</v>
+      </c>
+      <c r="K27" s="4">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1">
+        <f>SUM(F27:K27)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="6">
+        <v>424900</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4">
+      <c r="F28" s="4">
+        <v>9</v>
+      </c>
+      <c r="G28" s="4">
         <v>14</v>
       </c>
-      <c r="H27" s="6">
-        <v>9</v>
-      </c>
-      <c r="I27" s="4">
-        <v>9</v>
-      </c>
-      <c r="J27" s="4">
-        <v>1</v>
-      </c>
-      <c r="K27" s="4">
-        <v>1</v>
-      </c>
-      <c r="L27" s="1">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="6">
+      <c r="H28" s="6">
+        <v>15</v>
+      </c>
+      <c r="I28" s="4">
+        <v>6</v>
+      </c>
+      <c r="J28" s="4">
+        <v>4</v>
+      </c>
+      <c r="K28" s="4">
+        <v>4</v>
+      </c>
+      <c r="L28" s="1">
+        <f>SUM(F28:K28)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="6">
         <v>421000</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="C29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="6">
-        <v>3</v>
-      </c>
-      <c r="G28" s="6">
-        <v>8</v>
-      </c>
-      <c r="H28" s="6">
-        <v>9</v>
-      </c>
-      <c r="I28" s="6">
-        <v>8</v>
-      </c>
-      <c r="J28" s="6">
-        <v>4</v>
-      </c>
-      <c r="K28" s="6">
-        <v>2</v>
-      </c>
-      <c r="L28" s="1">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="6">
+      <c r="E29" s="1"/>
+      <c r="F29" s="6">
+        <v>5</v>
+      </c>
+      <c r="G29" s="6">
+        <v>15</v>
+      </c>
+      <c r="H29" s="6">
+        <v>17</v>
+      </c>
+      <c r="I29" s="6">
+        <v>16</v>
+      </c>
+      <c r="J29" s="6">
+        <v>11</v>
+      </c>
+      <c r="K29" s="6">
+        <v>12</v>
+      </c>
+      <c r="L29" s="1">
+        <f>SUM(F29:K29)</f>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="6">
         <v>424000</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="1" t="s">
+      <c r="C30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E29" s="1"/>
-      <c r="F29" s="4">
-        <v>20</v>
-      </c>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4">
-        <v>3</v>
-      </c>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4">
-        <v>10</v>
-      </c>
-      <c r="K29" s="4"/>
-      <c r="L29" s="1">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="6">
-        <v>422701</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4">
-        <v>4</v>
-      </c>
+      <c r="H30" s="4">
+        <v>3</v>
+      </c>
+      <c r="I30" s="4"/>
       <c r="J30" s="4">
-        <v>11</v>
-      </c>
-      <c r="K30" s="4">
-        <v>14</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="K30" s="4"/>
       <c r="L30" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F30:K30)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>423448</v>
+        <v>422701</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="4">
-        <v>3</v>
-      </c>
-      <c r="G31" s="4">
-        <v>8</v>
-      </c>
-      <c r="H31" s="6">
-        <v>6</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
       <c r="I31" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J31" s="4">
+        <v>11</v>
+      </c>
+      <c r="K31" s="4">
+        <v>14</v>
+      </c>
+      <c r="L31" s="1">
+        <f>SUM(F31:K31)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="6">
+        <v>423448</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K31" s="4">
-        <v>1</v>
-      </c>
-      <c r="L31" s="1">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="6">
+      <c r="D32" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4">
+        <v>4</v>
+      </c>
+      <c r="K32" s="4"/>
+      <c r="L32" s="1">
+        <f>SUM(F32:K32)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="6">
         <v>420101</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="C33" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E32" s="1"/>
-      <c r="F32" s="4">
-        <v>5</v>
-      </c>
-      <c r="G32" s="4">
-        <v>8</v>
-      </c>
-      <c r="H32" s="4">
-        <v>7</v>
-      </c>
-      <c r="I32" s="4">
-        <v>7</v>
-      </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4">
-        <v>2</v>
-      </c>
-      <c r="L32" s="1">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="6">
-        <v>424701</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>2</v>
-      </c>
-      <c r="G33" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="G33" s="4">
+        <v>7</v>
+      </c>
       <c r="H33" s="4">
-        <v>13</v>
-      </c>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4">
-        <v>13</v>
-      </c>
-      <c r="K33" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="I33" s="4">
+        <v>7</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4">
+        <v>2</v>
+      </c>
       <c r="L33" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F33:K33)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>421901</v>
+        <v>424701</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
-        <v>4</v>
-      </c>
-      <c r="G34" s="4">
-        <v>8</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G34" s="4"/>
       <c r="H34" s="4">
-        <v>6</v>
-      </c>
-      <c r="I34" s="4">
-        <v>5</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="I34" s="4"/>
       <c r="J34" s="4">
-        <v>4</v>
-      </c>
-      <c r="K34" s="4">
-        <v>1</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F34:K34)</f>
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>422900</v>
+        <v>421901</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
@@ -5870,25 +5856,31 @@
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="4">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="G35" s="4">
-        <v>1</v>
-      </c>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="H35" s="4">
+        <v>6</v>
+      </c>
+      <c r="I35" s="4">
+        <v>5</v>
+      </c>
       <c r="J35" s="4">
-        <v>2</v>
-      </c>
-      <c r="K35" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K35" s="4">
+        <v>1</v>
+      </c>
       <c r="L35" s="1">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F35:K35)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>421902</v>
+        <v>422900</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
@@ -5898,95 +5890,89 @@
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="4">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="G36" s="4">
-        <v>6</v>
-      </c>
-      <c r="H36" s="4">
-        <v>6</v>
-      </c>
-      <c r="I36" s="4">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
       <c r="J36" s="4">
-        <v>4</v>
-      </c>
-      <c r="K36" s="4">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K36" s="4"/>
       <c r="L36" s="1">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F36:K36)</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>420501</v>
+        <v>421902</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4">
+        <v>2</v>
+      </c>
+      <c r="G37" s="4">
+        <v>6</v>
+      </c>
+      <c r="H37" s="4">
+        <v>6</v>
+      </c>
+      <c r="I37" s="4">
+        <v>5</v>
+      </c>
+      <c r="J37" s="4">
+        <v>4</v>
+      </c>
+      <c r="K37" s="4">
+        <v>2</v>
+      </c>
+      <c r="L37" s="1">
+        <f>SUM(F37:K37)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="6">
+        <v>420501</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="1"/>
+      <c r="F38" s="4">
         <v>3</v>
       </c>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4">
-        <v>5</v>
-      </c>
-      <c r="I37" s="4">
-        <v>5</v>
-      </c>
-      <c r="J37" s="4">
-        <v>7</v>
-      </c>
-      <c r="K37" s="4">
+      <c r="G38" s="4"/>
+      <c r="H38" s="4">
+        <v>5</v>
+      </c>
+      <c r="I38" s="4">
+        <v>5</v>
+      </c>
+      <c r="J38" s="4">
+        <v>7</v>
+      </c>
+      <c r="K38" s="4">
         <v>4</v>
       </c>
-      <c r="L37" s="1">
-        <f t="shared" si="0"/>
+      <c r="L38" s="1">
+        <f>SUM(F38:K38)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="6">
-        <v>420301</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" s="1"/>
-      <c r="F38" s="6">
-        <v>17</v>
-      </c>
-      <c r="G38" s="6">
-        <v>34</v>
-      </c>
-      <c r="H38" s="6">
-        <v>37</v>
-      </c>
-      <c r="I38" s="6">
-        <v>29</v>
-      </c>
-      <c r="J38" s="6">
-        <v>33</v>
-      </c>
-      <c r="K38" s="6">
-        <v>15</v>
-      </c>
-      <c r="L38" s="1">
-        <f t="shared" si="0"/>
-        <v>165</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
         <v>422190</v>
       </c>
@@ -6018,11 +6004,11 @@
         <v>3</v>
       </c>
       <c r="L39" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F39:K39)</f>
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
         <v>421900</v>
       </c>
@@ -6037,7 +6023,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H40" s="4">
         <v>7</v>
@@ -6050,11 +6036,11 @@
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="41" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F40:K40)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
         <v>423501</v>
       </c>
@@ -6084,11 +6070,11 @@
         <v>6</v>
       </c>
       <c r="L41" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F41:K41)</f>
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
         <v>423308</v>
       </c>
@@ -6114,11 +6100,11 @@
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F42:K42)</f>
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
         <v>423408</v>
       </c>
@@ -6142,11 +6128,11 @@
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F43:K43)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
         <v>424801</v>
       </c>
@@ -6158,27 +6144,23 @@
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="4">
-        <v>1</v>
-      </c>
-      <c r="G44" s="4">
-        <v>7</v>
-      </c>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4">
-        <v>7</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4">
+        <v>10</v>
+      </c>
+      <c r="I44" s="4"/>
       <c r="J44" s="4">
-        <v>3</v>
-      </c>
-      <c r="K44" s="4">
-        <v>2</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K44" s="4"/>
       <c r="L44" s="1">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F44:K44)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
         <v>420900</v>
       </c>
@@ -6202,11 +6184,11 @@
         <v>10</v>
       </c>
       <c r="L45" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F45:K45)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
         <v>423900</v>
       </c>
@@ -6230,11 +6212,11 @@
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F46:K46)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
         <v>422100</v>
       </c>
@@ -6256,11 +6238,11 @@
         <v>13</v>
       </c>
       <c r="L47" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F47:K47)</f>
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="2:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
         <v>424500</v>
       </c>
@@ -6272,25 +6254,23 @@
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G48" s="4"/>
-      <c r="H48" s="4">
+      <c r="H48" s="4"/>
+      <c r="I48" s="4">
         <v>3</v>
       </c>
-      <c r="I48" s="4">
-        <v>4</v>
-      </c>
       <c r="J48" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F48:K48)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
         <v>424700</v>
       </c>
@@ -6314,11 +6294,11 @@
         <v>5</v>
       </c>
       <c r="L49" s="1">
-        <f t="shared" si="0"/>
+        <f>SUM(F49:K49)</f>
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
         <v>420802</v>
       </c>
@@ -6350,7 +6330,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
         <v>420200</v>
       </c>
@@ -6362,21 +6342,25 @@
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
+      <c r="G51" s="4">
+        <v>1</v>
+      </c>
+      <c r="H51" s="4">
+        <v>1</v>
+      </c>
       <c r="I51" s="4"/>
       <c r="J51" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L51" s="1">
-        <f t="shared" ref="L51:L62" si="1">SUM(F51:K51)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F51:K51)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
         <v>421301</v>
       </c>
@@ -6402,11 +6386,11 @@
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F52:K52)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
         <v>424300</v>
       </c>
@@ -6421,7 +6405,9 @@
       <c r="G53" s="4">
         <v>5</v>
       </c>
-      <c r="H53" s="4"/>
+      <c r="H53" s="4">
+        <v>2</v>
+      </c>
       <c r="I53" s="4">
         <v>3</v>
       </c>
@@ -6430,11 +6416,11 @@
         <v>6</v>
       </c>
       <c r="L53" s="1">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F53:K53)</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
         <v>421402</v>
       </c>
@@ -6462,11 +6448,11 @@
         <v>2</v>
       </c>
       <c r="L54" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F54:K54)</f>
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
         <v>425600</v>
       </c>
@@ -6490,11 +6476,11 @@
         <v>7</v>
       </c>
       <c r="L55" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F55:K55)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
         <v>423304</v>
       </c>
@@ -6506,23 +6492,21 @@
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="4"/>
-      <c r="G56" s="4">
-        <v>1</v>
-      </c>
+      <c r="G56" s="4"/>
       <c r="H56" s="6"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K56" s="4">
         <v>2</v>
       </c>
       <c r="L56" s="1">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F56:K56)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
         <v>421300</v>
       </c>
@@ -6546,11 +6530,11 @@
         <v>4</v>
       </c>
       <c r="L57" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F57:K57)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
         <v>424960</v>
       </c>
@@ -6580,14 +6564,14 @@
         <v>1</v>
       </c>
       <c r="L58" s="12">
-        <f t="shared" si="1"/>
+        <f>SUM(F58:K58)</f>
         <v>9</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
         <v>421800</v>
       </c>
@@ -6613,11 +6597,11 @@
         <v>1</v>
       </c>
       <c r="L59" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F59:K59)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
         <v>423348</v>
       </c>
@@ -6643,11 +6627,11 @@
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F60:K60)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
         <v>422601</v>
       </c>
@@ -6667,11 +6651,11 @@
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F61:K61)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
         <v>421401</v>
       </c>
@@ -6695,11 +6679,11 @@
         <v>1</v>
       </c>
       <c r="L62" s="1">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F62:K62)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
         <v>421001</v>
       </c>
@@ -6729,7 +6713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
         <v>420500</v>
       </c>
@@ -6753,11 +6737,11 @@
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f t="shared" ref="L64:L74" si="2">SUM(F64:K64)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F64:K64)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
         <v>420402</v>
       </c>
@@ -6777,11 +6761,11 @@
       </c>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="66" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F65:K65)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
         <v>423416</v>
       </c>
@@ -6805,11 +6789,11 @@
       </c>
       <c r="K66" s="4"/>
       <c r="L66" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F66:K66)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
         <v>422600</v>
       </c>
@@ -6829,11 +6813,11 @@
         <v>3</v>
       </c>
       <c r="L67" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F67:K67)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="6">
         <v>423309</v>
       </c>
@@ -6857,11 +6841,11 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F68:K68)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" s="6">
         <v>422400</v>
       </c>
@@ -6881,11 +6865,11 @@
       </c>
       <c r="K69" s="6"/>
       <c r="L69" s="1">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F69:K69)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" s="6">
         <v>422401</v>
       </c>
@@ -6903,11 +6887,11 @@
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
       <c r="L70" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F70:K70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
         <v>423800</v>
       </c>
@@ -6927,11 +6911,11 @@
       <c r="J71" s="6"/>
       <c r="K71" s="6"/>
       <c r="L71" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F71:K71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
         <v>424200</v>
       </c>
@@ -6943,17 +6927,25 @@
       </c>
       <c r="E72" s="1"/>
       <c r="F72" s="6"/>
-      <c r="G72" s="6"/>
+      <c r="G72" s="6">
+        <v>1</v>
+      </c>
       <c r="H72" s="6"/>
-      <c r="I72" s="6"/>
-      <c r="J72" s="6"/>
-      <c r="K72" s="6"/>
+      <c r="I72" s="6">
+        <v>9</v>
+      </c>
+      <c r="J72" s="6">
+        <v>1</v>
+      </c>
+      <c r="K72" s="6">
+        <v>3</v>
+      </c>
       <c r="L72" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F72:K72)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" s="6">
         <v>423409</v>
       </c>
@@ -6971,11 +6963,11 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F73:K73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" s="6">
         <v>423404</v>
       </c>
@@ -6993,11 +6985,11 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+        <f>SUM(F74:K74)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="6">
         <v>420801</v>
       </c>
@@ -7019,7 +7011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" s="6">
         <v>420160</v>
       </c>
@@ -7046,23 +7038,23 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="2:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L79" s="10">
         <f>SUM(L3:L78)</f>
-        <v>2889</v>
-      </c>
-    </row>
-    <row r="83" spans="15:15" x14ac:dyDescent="0.35">
+        <v>2819</v>
+      </c>
+    </row>
+    <row r="83" spans="15:15" x14ac:dyDescent="0.25">
       <c r="O83" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="127" spans="11:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K127" t="s">
         <v>123</v>
       </c>
@@ -7071,10 +7063,10 @@
   <autoFilter ref="B2:L77" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
     <filterColumn colId="0">
       <filters>
-        <filter val="423000"/>
+        <filter val="423200"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B25:L25">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L77">
       <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
   </autoFilter>
@@ -7084,11 +7076,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <sheetPr codeName="Hoja7"/>
-  <dimension ref="B3:L4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B3:L10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
@@ -7123,9 +7114,146 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
-        <v>123</v>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="1">
+        <v>432900</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1">
+        <v>36</v>
+      </c>
+      <c r="G4" s="1">
+        <v>85</v>
+      </c>
+      <c r="H4" s="1">
+        <v>94</v>
+      </c>
+      <c r="I4" s="1">
+        <v>95</v>
+      </c>
+      <c r="J4" s="1">
+        <v>67</v>
+      </c>
+      <c r="K4" s="1">
+        <v>49</v>
+      </c>
+      <c r="L4" s="1">
+        <f>SUM(F4:K4)</f>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>431800</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1">
+        <v>27</v>
+      </c>
+      <c r="G5" s="1">
+        <v>54</v>
+      </c>
+      <c r="H5" s="1">
+        <v>56</v>
+      </c>
+      <c r="I5" s="1">
+        <v>38</v>
+      </c>
+      <c r="J5" s="1">
+        <v>36</v>
+      </c>
+      <c r="K5" s="1">
+        <v>24</v>
+      </c>
+      <c r="L5" s="1">
+        <f>SUM(F5:K5)</f>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>430900</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1">
+        <v>18</v>
+      </c>
+      <c r="G6" s="1">
+        <v>51</v>
+      </c>
+      <c r="H6" s="1">
+        <v>55</v>
+      </c>
+      <c r="I6" s="1">
+        <v>48</v>
+      </c>
+      <c r="J6" s="1">
+        <v>35</v>
+      </c>
+      <c r="K6" s="1">
+        <v>26</v>
+      </c>
+      <c r="L6" s="1">
+        <f>SUM(F6:K6)</f>
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="17">
+        <v>432300</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="17">
+        <v>56</v>
+      </c>
+      <c r="G7" s="17">
+        <v>115</v>
+      </c>
+      <c r="H7" s="17">
+        <v>132</v>
+      </c>
+      <c r="I7" s="17">
+        <v>122</v>
+      </c>
+      <c r="J7" s="17">
+        <v>85</v>
+      </c>
+      <c r="K7" s="17">
+        <v>66</v>
+      </c>
+      <c r="L7" s="1">
+        <f>SUM(F7:K7)</f>
+        <v>576</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <f>SUM(L4:L7)</f>
+        <v>1470</v>
       </c>
     </row>
   </sheetData>
@@ -7135,15 +7263,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7287,6 +7406,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -7294,14 +7422,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7315,6 +7435,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizar stock bodega con nueva coleccion 43
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2878" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E45A504F-C099-40E6-9150-FF1D30549160}"/>
+  <xr:revisionPtr revIDLastSave="2899" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36FB4087-2DEE-4BD4-8FC2-80894B0D490C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="132">
   <si>
     <t>CODIGO</t>
   </si>
@@ -569,7 +569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -609,7 +609,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -626,10 +625,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4731,7 +4726,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4773,7 +4767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -4806,11 +4800,11 @@
         <v>25</v>
       </c>
       <c r="L3" s="1">
-        <f>SUM(F3:K3)</f>
+        <f t="shared" ref="L3:L49" si="0">SUM(F3:K3)</f>
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
         <v>422200</v>
       </c>
@@ -4838,11 +4832,11 @@
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>205</v>
       </c>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>126</v>
       </c>
@@ -4875,11 +4869,11 @@
         <v>23</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
+        <f t="shared" si="0"/>
         <v>186</v>
       </c>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>420301</v>
       </c>
@@ -4909,7 +4903,7 @@
         <v>8</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
+        <f t="shared" si="0"/>
         <v>142</v>
       </c>
       <c r="M6" t="s">
@@ -4919,7 +4913,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
         <v>420600</v>
       </c>
@@ -4947,11 +4941,11 @@
         <v>8</v>
       </c>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
+        <f t="shared" si="0"/>
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>420100</v>
       </c>
@@ -4979,11 +4973,11 @@
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
+        <f t="shared" si="0"/>
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
         <v>424400</v>
       </c>
@@ -5009,12 +5003,12 @@
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
+        <f t="shared" si="0"/>
         <v>110</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>123</v>
       </c>
@@ -5045,14 +5039,14 @@
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>83</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>420300</v>
       </c>
@@ -5082,14 +5076,14 @@
         <v>10</v>
       </c>
       <c r="L11" s="12">
-        <f>SUM(F11:K11)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>420400</v>
       </c>
@@ -5119,7 +5113,7 @@
         <v>16</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
+        <f t="shared" si="0"/>
         <v>72</v>
       </c>
       <c r="N12" t="s">
@@ -5156,14 +5150,14 @@
         <v>14</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
+        <f t="shared" si="0"/>
         <v>71</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>123</v>
       </c>
@@ -5194,14 +5188,14 @@
         <v>17</v>
       </c>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
+        <f t="shared" si="0"/>
         <v>65</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>123</v>
       </c>
@@ -5232,12 +5226,12 @@
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
         <v>422800</v>
       </c>
@@ -5261,14 +5255,14 @@
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
         <v>422000</v>
       </c>
@@ -5296,11 +5290,11 @@
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
         <v>423316</v>
       </c>
@@ -5330,11 +5324,11 @@
         <v>4</v>
       </c>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
         <v>422101</v>
       </c>
@@ -5362,11 +5356,11 @@
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
         <v>421400</v>
       </c>
@@ -5396,11 +5390,11 @@
         <v>32</v>
       </c>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
         <v>420800</v>
       </c>
@@ -5430,11 +5424,11 @@
         <v>6</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
         <v>421801</v>
       </c>
@@ -5460,11 +5454,11 @@
         <v>10</v>
       </c>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
         <v>420160</v>
       </c>
@@ -5496,11 +5490,11 @@
         <v>5</v>
       </c>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
         <v>421100</v>
       </c>
@@ -5530,11 +5524,11 @@
         <v>7</v>
       </c>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
         <v>422700</v>
       </c>
@@ -5562,11 +5556,11 @@
         <v>10</v>
       </c>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
         <v>423000</v>
       </c>
@@ -5592,11 +5586,11 @@
         <v>9</v>
       </c>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>424900</v>
       </c>
@@ -5628,11 +5622,11 @@
         <v>0</v>
       </c>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
         <v>424900</v>
       </c>
@@ -5664,11 +5658,11 @@
         <v>4</v>
       </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
         <v>421000</v>
       </c>
@@ -5698,11 +5692,11 @@
         <v>12</v>
       </c>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
+        <f t="shared" si="0"/>
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
         <v>424000</v>
       </c>
@@ -5726,11 +5720,11 @@
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
         <v>422701</v>
       </c>
@@ -5756,11 +5750,11 @@
         <v>14</v>
       </c>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
         <v>423448</v>
       </c>
@@ -5780,11 +5774,11 @@
       </c>
       <c r="K32" s="4"/>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
         <v>420101</v>
       </c>
@@ -5812,11 +5806,11 @@
         <v>2</v>
       </c>
       <c r="L33" s="1">
-        <f>SUM(F33:K33)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
         <v>424701</v>
       </c>
@@ -5840,11 +5834,11 @@
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
         <v>421901</v>
       </c>
@@ -5874,11 +5868,11 @@
         <v>1</v>
       </c>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
         <v>422900</v>
       </c>
@@ -5902,11 +5896,11 @@
       </c>
       <c r="K36" s="4"/>
       <c r="L36" s="1">
-        <f>SUM(F36:K36)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
         <v>421902</v>
       </c>
@@ -5936,11 +5930,11 @@
         <v>2</v>
       </c>
       <c r="L37" s="1">
-        <f>SUM(F37:K37)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
         <v>420501</v>
       </c>
@@ -5968,11 +5962,11 @@
         <v>4</v>
       </c>
       <c r="L38" s="1">
-        <f>SUM(F38:K38)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
         <v>422190</v>
       </c>
@@ -6004,11 +5998,11 @@
         <v>3</v>
       </c>
       <c r="L39" s="1">
-        <f>SUM(F39:K39)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
         <v>421900</v>
       </c>
@@ -6036,11 +6030,11 @@
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="1">
-        <f>SUM(F40:K40)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
         <v>423501</v>
       </c>
@@ -6070,11 +6064,11 @@
         <v>6</v>
       </c>
       <c r="L41" s="1">
-        <f>SUM(F41:K41)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
         <v>423308</v>
       </c>
@@ -6100,11 +6094,11 @@
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="1">
-        <f>SUM(F42:K42)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
         <v>423408</v>
       </c>
@@ -6128,11 +6122,11 @@
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="1">
-        <f>SUM(F43:K43)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
         <v>424801</v>
       </c>
@@ -6156,11 +6150,11 @@
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="1">
-        <f>SUM(F44:K44)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
         <v>420900</v>
       </c>
@@ -6184,11 +6178,11 @@
         <v>10</v>
       </c>
       <c r="L45" s="1">
-        <f>SUM(F45:K45)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
         <v>423900</v>
       </c>
@@ -6212,11 +6206,11 @@
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="1">
-        <f>SUM(F46:K46)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
         <v>422100</v>
       </c>
@@ -6238,11 +6232,11 @@
         <v>13</v>
       </c>
       <c r="L47" s="1">
-        <f>SUM(F47:K47)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
         <v>424500</v>
       </c>
@@ -6266,11 +6260,11 @@
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="1">
-        <f>SUM(F48:K48)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
         <v>424700</v>
       </c>
@@ -6294,11 +6288,11 @@
         <v>5</v>
       </c>
       <c r="L49" s="1">
-        <f>SUM(F49:K49)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
         <v>420802</v>
       </c>
@@ -6330,7 +6324,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
         <v>420200</v>
       </c>
@@ -6356,11 +6350,11 @@
         <v>11</v>
       </c>
       <c r="L51" s="1">
-        <f>SUM(F51:K51)</f>
+        <f t="shared" ref="L51:L62" si="1">SUM(F51:K51)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
         <v>421301</v>
       </c>
@@ -6386,11 +6380,11 @@
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f>SUM(F52:K52)</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
         <v>424300</v>
       </c>
@@ -6416,11 +6410,11 @@
         <v>6</v>
       </c>
       <c r="L53" s="1">
-        <f>SUM(F53:K53)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
         <v>421402</v>
       </c>
@@ -6448,11 +6442,11 @@
         <v>2</v>
       </c>
       <c r="L54" s="1">
-        <f>SUM(F54:K54)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
         <v>425600</v>
       </c>
@@ -6476,11 +6470,11 @@
         <v>7</v>
       </c>
       <c r="L55" s="1">
-        <f>SUM(F55:K55)</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
         <v>423304</v>
       </c>
@@ -6502,11 +6496,11 @@
         <v>2</v>
       </c>
       <c r="L56" s="1">
-        <f>SUM(F56:K56)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
         <v>421300</v>
       </c>
@@ -6530,11 +6524,11 @@
         <v>4</v>
       </c>
       <c r="L57" s="1">
-        <f>SUM(F57:K57)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
         <v>424960</v>
       </c>
@@ -6564,14 +6558,14 @@
         <v>1</v>
       </c>
       <c r="L58" s="12">
-        <f>SUM(F58:K58)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
         <v>421800</v>
       </c>
@@ -6597,11 +6591,11 @@
         <v>1</v>
       </c>
       <c r="L59" s="1">
-        <f>SUM(F59:K59)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
         <v>423348</v>
       </c>
@@ -6627,11 +6621,11 @@
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="1">
-        <f>SUM(F60:K60)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
         <v>422601</v>
       </c>
@@ -6651,11 +6645,11 @@
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f>SUM(F61:K61)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
         <v>421401</v>
       </c>
@@ -6679,11 +6673,11 @@
         <v>1</v>
       </c>
       <c r="L62" s="1">
-        <f>SUM(F62:K62)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
         <v>421001</v>
       </c>
@@ -6713,7 +6707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
         <v>420500</v>
       </c>
@@ -6737,11 +6731,11 @@
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f>SUM(F64:K64)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L64:L74" si="2">SUM(F64:K64)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
         <v>420402</v>
       </c>
@@ -6761,11 +6755,11 @@
       </c>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f>SUM(F65:K65)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="66" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
         <v>423416</v>
       </c>
@@ -6789,11 +6783,11 @@
       </c>
       <c r="K66" s="4"/>
       <c r="L66" s="1">
-        <f>SUM(F66:K66)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
         <v>422600</v>
       </c>
@@ -6813,11 +6807,11 @@
         <v>3</v>
       </c>
       <c r="L67" s="1">
-        <f>SUM(F67:K67)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="6">
         <v>423309</v>
       </c>
@@ -6841,11 +6835,11 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f>SUM(F68:K68)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="6">
         <v>422400</v>
       </c>
@@ -6865,11 +6859,11 @@
       </c>
       <c r="K69" s="6"/>
       <c r="L69" s="1">
-        <f>SUM(F69:K69)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="6">
         <v>422401</v>
       </c>
@@ -6887,11 +6881,11 @@
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
       <c r="L70" s="1">
-        <f>SUM(F70:K70)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
         <v>423800</v>
       </c>
@@ -6911,11 +6905,11 @@
       <c r="J71" s="6"/>
       <c r="K71" s="6"/>
       <c r="L71" s="1">
-        <f>SUM(F71:K71)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
         <v>424200</v>
       </c>
@@ -6941,11 +6935,11 @@
         <v>3</v>
       </c>
       <c r="L72" s="12">
-        <f>SUM(F72:K72)</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="6">
         <v>423409</v>
       </c>
@@ -6963,11 +6957,11 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f>SUM(F73:K73)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="6">
         <v>423404</v>
       </c>
@@ -6985,11 +6979,11 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f>SUM(F74:K74)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" s="6">
         <v>420801</v>
       </c>
@@ -7011,7 +7005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B76" s="6">
         <v>420160</v>
       </c>
@@ -7038,7 +7032,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>123</v>
       </c>
@@ -7061,11 +7055,6 @@
     </row>
   </sheetData>
   <autoFilter ref="B2:L77" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="423200"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L77">
       <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
@@ -7076,10 +7065,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:L10"/>
+  <dimension ref="B3:M10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
@@ -7114,7 +7103,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>432900</v>
       </c>
@@ -7126,29 +7115,29 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="G4" s="1">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="H4" s="1">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="I4" s="1">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="J4" s="1">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="K4" s="1">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>426</v>
-      </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>431800</v>
       </c>
@@ -7160,29 +7149,32 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="G5" s="1">
+        <v>117</v>
+      </c>
+      <c r="H5" s="1">
+        <v>127</v>
+      </c>
+      <c r="I5" s="1">
+        <v>98</v>
+      </c>
+      <c r="J5" s="1">
+        <v>79</v>
+      </c>
+      <c r="K5" s="1">
         <v>54</v>
-      </c>
-      <c r="H5" s="1">
-        <v>56</v>
-      </c>
-      <c r="I5" s="1">
-        <v>38</v>
-      </c>
-      <c r="J5" s="1">
-        <v>36</v>
-      </c>
-      <c r="K5" s="1">
-        <v>24</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>235</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+        <v>531</v>
+      </c>
+      <c r="M5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>430900</v>
       </c>
@@ -7216,33 +7208,33 @@
         <v>233</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="17">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
         <v>432300</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="17" t="s">
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>131</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="F7" s="17">
+      <c r="F7" s="1">
         <v>56</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="1">
         <v>115</v>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="1">
         <v>132</v>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="1">
         <v>122</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="1">
         <v>85</v>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="1">
         <v>66</v>
       </c>
       <c r="L7" s="1">
@@ -7250,10 +7242,10 @@
         <v>576</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L10">
         <f>SUM(L4:L7)</f>
-        <v>1470</v>
+        <v>1900</v>
       </c>
     </row>
   </sheetData>
@@ -7263,6 +7255,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7406,22 +7413,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7437,28 +7453,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar datos de produccion e inventario
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2899" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36FB4087-2DEE-4BD4-8FC2-80894B0D490C}"/>
+  <xr:revisionPtr revIDLastSave="3438" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE9101E6-FED5-4DC0-9E5F-9FBA180ACA68}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'COLE 42'!$B$2:$L$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$B$3:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$B$3:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="133">
   <si>
     <t>CODIGO</t>
   </si>
@@ -440,13 +440,16 @@
     <t>OSCURO</t>
   </si>
   <si>
-    <t>ULTIMA ACTUALIZACION 12:15  07-05-2026</t>
-  </si>
-  <si>
     <t>WIDE</t>
   </si>
   <si>
     <t>WIDE LEG</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>ULTIMA ACTUALIZACION 10:147  25-05-2026</t>
   </si>
 </sst>
 </file>
@@ -504,7 +507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -564,12 +567,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -605,10 +621,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -625,6 +648,14 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
+<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
+</file>
+
+<file path=xl/namedSheetViews/namedSheetView2.xml><?xml version="1.0" encoding="utf-8"?>
+<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -989,19 +1020,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
@@ -1788,19 +1819,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2395,19 +2426,19 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -2765,19 +2796,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
@@ -4358,357 +4389,381 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="B4" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="15">
         <v>36</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="15">
         <v>38</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="15">
         <v>40</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="15">
         <v>42</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="15">
         <v>44</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="15">
         <v>46</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="L4" s="15" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9">
-        <v>0</v>
-      </c>
-      <c r="G5" s="9">
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
         <v>14</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="4">
         <v>26</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="4">
         <v>13</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="4">
         <v>20</v>
       </c>
-      <c r="K5" s="9">
-        <v>7</v>
-      </c>
-      <c r="L5" s="9">
+      <c r="K5" s="4">
+        <v>7</v>
+      </c>
+      <c r="L5" s="4">
         <f t="shared" ref="L5:L13" si="0">SUM(F5:K5)</f>
         <v>80</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9">
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
         <v>4</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="4">
         <v>11</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="4">
         <v>12</v>
       </c>
-      <c r="I6" s="9">
-        <v>6</v>
-      </c>
-      <c r="J6" s="9">
-        <v>5</v>
-      </c>
-      <c r="K6" s="9">
-        <v>2</v>
-      </c>
-      <c r="L6" s="9">
+      <c r="I6" s="4">
+        <v>6</v>
+      </c>
+      <c r="J6" s="4">
+        <v>5</v>
+      </c>
+      <c r="K6" s="4">
+        <v>2</v>
+      </c>
+      <c r="L6" s="4">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9">
-        <v>0</v>
-      </c>
-      <c r="G7" s="9">
-        <v>0</v>
-      </c>
-      <c r="H7" s="9">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
         <v>4</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="4">
         <v>3</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="4">
         <v>13</v>
       </c>
-      <c r="K7" s="9">
-        <v>0</v>
-      </c>
-      <c r="L7" s="9">
+      <c r="K7" s="4">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9">
-        <v>0</v>
-      </c>
-      <c r="G8" s="9">
-        <v>0</v>
-      </c>
-      <c r="H8" s="9">
-        <v>5</v>
-      </c>
-      <c r="I8" s="9">
-        <v>7</v>
-      </c>
-      <c r="J8" s="9">
-        <v>5</v>
-      </c>
-      <c r="K8" s="9">
-        <v>2</v>
-      </c>
-      <c r="L8" s="9">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>5</v>
+      </c>
+      <c r="I8" s="4">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9">
-        <v>0</v>
-      </c>
-      <c r="G9" s="9">
-        <v>0</v>
-      </c>
-      <c r="H9" s="9">
-        <v>0</v>
-      </c>
-      <c r="I9" s="9">
+      <c r="E9" s="4"/>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
         <v>4</v>
       </c>
-      <c r="J9" s="9">
-        <v>5</v>
-      </c>
-      <c r="K9" s="9">
-        <v>1</v>
-      </c>
-      <c r="L9" s="9">
+      <c r="J9" s="4">
+        <v>5</v>
+      </c>
+      <c r="K9" s="4">
+        <v>1</v>
+      </c>
+      <c r="L9" s="4">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="C10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9">
-        <v>0</v>
-      </c>
-      <c r="G10" s="9">
-        <v>0</v>
-      </c>
-      <c r="H10" s="9">
-        <v>1</v>
-      </c>
-      <c r="I10" s="9">
-        <v>6</v>
-      </c>
-      <c r="J10" s="9">
-        <v>0</v>
-      </c>
-      <c r="K10" s="9">
-        <v>2</v>
-      </c>
-      <c r="L10" s="9">
+      <c r="E10" s="4"/>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4">
+        <v>6</v>
+      </c>
+      <c r="J10" s="4">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4">
+        <v>2</v>
+      </c>
+      <c r="L10" s="4">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9">
-        <v>1</v>
-      </c>
-      <c r="G11" s="9">
-        <v>0</v>
-      </c>
-      <c r="H11" s="9">
-        <v>1</v>
-      </c>
-      <c r="I11" s="9">
+      <c r="C11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4">
         <v>4</v>
       </c>
-      <c r="J11" s="9">
-        <v>0</v>
-      </c>
-      <c r="K11" s="9">
-        <v>2</v>
-      </c>
-      <c r="L11" s="9">
+      <c r="J11" s="4">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4">
+        <v>2</v>
+      </c>
+      <c r="L11" s="4">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="C12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9">
-        <v>0</v>
-      </c>
-      <c r="G12" s="9">
-        <v>0</v>
-      </c>
-      <c r="H12" s="9">
-        <v>1</v>
-      </c>
-      <c r="I12" s="9">
-        <v>7</v>
-      </c>
-      <c r="J12" s="9">
-        <v>0</v>
-      </c>
-      <c r="K12" s="9">
-        <v>0</v>
-      </c>
-      <c r="L12" s="9">
+      <c r="E12" s="4"/>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4">
+        <v>7</v>
+      </c>
+      <c r="J12" s="4">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="C13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9">
-        <v>1</v>
-      </c>
-      <c r="G13" s="9">
-        <v>1</v>
-      </c>
-      <c r="H13" s="9">
-        <v>1</v>
-      </c>
-      <c r="I13" s="9">
-        <v>1</v>
-      </c>
-      <c r="J13" s="9">
-        <v>1</v>
-      </c>
-      <c r="K13" s="9">
-        <v>1</v>
-      </c>
-      <c r="L13" s="9">
-        <f t="shared" si="0"/>
-        <v>6</v>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4">
+        <v>1</v>
+      </c>
+      <c r="G13" s="4">
+        <v>1</v>
+      </c>
+      <c r="H13" s="4">
+        <v>1</v>
+      </c>
+      <c r="I13" s="4">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4">
+        <v>1</v>
+      </c>
+      <c r="L13" s="4">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <v>416500</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="4">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1">
+        <f>SUM(F14:K14)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.25">
@@ -4726,13 +4781,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="A2:P127"/>
+  <dimension ref="B2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -4767,79 +4823,75 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>123</v>
-      </c>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
-        <v>423600</v>
+        <v>422200</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="4">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G3" s="4">
+        <v>51</v>
+      </c>
+      <c r="H3" s="4">
         <v>46</v>
       </c>
-      <c r="H3" s="4">
-        <v>43</v>
-      </c>
       <c r="I3" s="4">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="J3" s="4">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K3" s="4">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="L3" s="1">
-        <f t="shared" ref="L3:L49" si="0">SUM(F3:K3)</f>
-        <v>209</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <f>SUM(F3:K3)</f>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
-        <v>422200</v>
+        <v>423600</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="4">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="G4" s="4">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="H4" s="4">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="I4" s="4">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="J4" s="4">
-        <v>31</v>
-      </c>
-      <c r="K4" s="4"/>
+        <v>27</v>
+      </c>
+      <c r="K4" s="4">
+        <v>25</v>
+      </c>
       <c r="L4" s="1">
-        <f t="shared" si="0"/>
-        <v>205</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>126</v>
-      </c>
+        <f>SUM(F4:K4)</f>
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
         <v>423500</v>
       </c>
@@ -4851,29 +4903,29 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G5" s="4">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H5" s="4">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I5" s="4">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="J5" s="4">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="K5" s="4">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" si="0"/>
-        <v>186</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <f>SUM(F5:K5)</f>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>420301</v>
       </c>
@@ -4885,101 +4937,105 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="6">
+        <v>7</v>
+      </c>
+      <c r="G6" s="6">
+        <v>23</v>
+      </c>
+      <c r="H6" s="6">
+        <v>26</v>
+      </c>
+      <c r="I6" s="6">
+        <v>28</v>
+      </c>
+      <c r="J6" s="6">
         <v>14</v>
       </c>
-      <c r="G6" s="6">
-        <v>32</v>
-      </c>
-      <c r="H6" s="6">
-        <v>34</v>
-      </c>
-      <c r="I6" s="6">
-        <v>26</v>
-      </c>
-      <c r="J6" s="6">
-        <v>28</v>
-      </c>
       <c r="K6" s="6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L6" s="1">
-        <f t="shared" si="0"/>
-        <v>142</v>
+        <f>SUM(F6:K6)</f>
+        <v>102</v>
       </c>
       <c r="M6" t="s">
         <v>123</v>
       </c>
       <c r="N6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
-        <v>420600</v>
+        <v>423200</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="4">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G7" s="4">
-        <v>3</v>
-      </c>
-      <c r="H7" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="H7" s="4">
+        <v>15</v>
+      </c>
       <c r="I7" s="4">
+        <v>13</v>
+      </c>
+      <c r="J7" s="4">
+        <v>13</v>
+      </c>
+      <c r="K7" s="4">
+        <v>16</v>
+      </c>
+      <c r="L7" s="1">
+        <f>SUM(F7:K7)</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="6">
+        <v>421000</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="1"/>
+      <c r="F8" s="6">
+        <v>5</v>
+      </c>
+      <c r="G8" s="6">
+        <v>15</v>
+      </c>
+      <c r="H8" s="6">
+        <v>15</v>
+      </c>
+      <c r="I8" s="6">
+        <v>15</v>
+      </c>
+      <c r="J8" s="6">
         <v>10</v>
       </c>
-      <c r="J7" s="4">
-        <v>18</v>
-      </c>
-      <c r="K7" s="4">
-        <v>8</v>
-      </c>
-      <c r="L7" s="1">
-        <f t="shared" si="0"/>
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="6">
+      <c r="K8" s="6">
+        <v>10</v>
+      </c>
+      <c r="L8" s="1">
+        <f>SUM(F8:K8)</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="6">
         <v>420100</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="4">
-        <v>27</v>
-      </c>
-      <c r="G8" s="4">
-        <v>22</v>
-      </c>
-      <c r="H8" s="4">
-        <v>52</v>
-      </c>
-      <c r="I8" s="4">
-        <v>12</v>
-      </c>
-      <c r="J8" s="4">
-        <v>8</v>
-      </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="1">
-        <f t="shared" si="0"/>
-        <v>121</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="6">
-        <v>424400</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
@@ -4989,31 +5045,30 @@
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="4">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="G9" s="4">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="I9" s="4">
-        <v>32</v>
-      </c>
-      <c r="J9" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="J9" s="4">
+        <v>3</v>
+      </c>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f t="shared" si="0"/>
-        <v>110</v>
+        <f>SUM(F9:K9)</f>
+        <v>66</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>123</v>
-      </c>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
-        <v>422300</v>
+        <v>422800</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -5022,241 +5077,235 @@
         <v>6</v>
       </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="4">
-        <v>18</v>
-      </c>
+      <c r="F10" s="4"/>
       <c r="G10" s="4">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H10" s="4">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="I10" s="4">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="1">
-        <f t="shared" si="0"/>
-        <v>83</v>
+        <f>SUM(F10:K10)</f>
+        <v>66</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
-        <v>420300</v>
+        <v>422000</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="6">
-        <v>13</v>
-      </c>
-      <c r="G11" s="6">
-        <v>15</v>
-      </c>
-      <c r="H11" s="6">
-        <v>16</v>
-      </c>
-      <c r="I11" s="6">
-        <v>15</v>
-      </c>
-      <c r="J11" s="6">
-        <v>11</v>
-      </c>
-      <c r="K11" s="6">
-        <v>10</v>
-      </c>
-      <c r="L11" s="12">
-        <f t="shared" si="0"/>
-        <v>80</v>
+      <c r="F11" s="4">
+        <v>35</v>
+      </c>
+      <c r="G11" s="4">
+        <v>9</v>
+      </c>
+      <c r="H11" s="4">
+        <v>12</v>
+      </c>
+      <c r="I11" s="4">
+        <v>4</v>
+      </c>
+      <c r="J11" s="4">
+        <v>3</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="1">
+        <f>SUM(F11:K11)</f>
+        <v>63</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
-        <v>420400</v>
+        <v>424400</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="4">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G12" s="4">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="H12" s="4">
         <v>9</v>
       </c>
       <c r="I12" s="4">
-        <v>7</v>
-      </c>
-      <c r="J12" s="4">
-        <v>8</v>
-      </c>
-      <c r="K12" s="4">
-        <v>16</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
       <c r="L12" s="1">
-        <f t="shared" si="0"/>
-        <v>72</v>
+        <f>SUM(F12:K12)</f>
+        <v>56</v>
       </c>
       <c r="N12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
-        <v>423200</v>
+        <v>420800</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E13" s="1"/>
-      <c r="F13" s="4">
+      <c r="F13" s="6">
+        <v>6</v>
+      </c>
+      <c r="G13" s="6">
+        <v>11</v>
+      </c>
+      <c r="H13" s="6">
+        <v>14</v>
+      </c>
+      <c r="I13" s="6">
         <v>13</v>
       </c>
-      <c r="G13" s="4">
-        <v>1</v>
-      </c>
-      <c r="H13" s="4">
-        <v>17</v>
-      </c>
-      <c r="I13" s="4">
-        <v>14</v>
-      </c>
-      <c r="J13" s="4">
-        <v>12</v>
+      <c r="J13" s="6">
+        <v>6</v>
       </c>
       <c r="K13" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="0"/>
-        <v>71</v>
+        <f>SUM(F13:K13)</f>
+        <v>56</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>123</v>
-      </c>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
-        <v>422500</v>
+        <v>420400</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="4">
-        <v>8</v>
-      </c>
-      <c r="G14" s="4"/>
+        <v>25</v>
+      </c>
+      <c r="G14" s="4">
+        <v>4</v>
+      </c>
       <c r="H14" s="4">
+        <v>5</v>
+      </c>
+      <c r="I14" s="4">
+        <v>4</v>
+      </c>
+      <c r="J14" s="4">
+        <v>5</v>
+      </c>
+      <c r="K14" s="4">
         <v>12</v>
       </c>
-      <c r="I14" s="4">
-        <v>15</v>
-      </c>
-      <c r="J14" s="4">
-        <v>13</v>
-      </c>
-      <c r="K14" s="4">
-        <v>17</v>
-      </c>
       <c r="L14" s="1">
-        <f t="shared" si="0"/>
-        <v>65</v>
+        <f>SUM(F14:K14)</f>
+        <v>55</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>123</v>
-      </c>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
-        <v>424600</v>
+        <v>421400</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G15" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="I15" s="4">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="J15" s="4">
-        <v>17</v>
-      </c>
-      <c r="K15" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="K15" s="4">
+        <v>32</v>
+      </c>
       <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>64</v>
+        <f>SUM(F15:K15)</f>
+        <v>53</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
-        <v>422800</v>
+        <v>422101</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="4"/>
+      <c r="F16" s="4">
+        <v>14</v>
+      </c>
       <c r="G16" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H16" s="4">
-        <v>29</v>
-      </c>
-      <c r="I16" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="I16" s="4">
+        <v>9</v>
+      </c>
       <c r="J16" s="4">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="1">
-        <f t="shared" si="0"/>
-        <v>61</v>
+        <f>SUM(F16:K16)</f>
+        <v>52</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
@@ -5264,139 +5313,143 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
-        <v>422000</v>
+        <v>424900</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="F17" s="4">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="G17" s="4">
-        <v>10</v>
-      </c>
-      <c r="H17" s="4">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="H17" s="6">
+        <v>15</v>
       </c>
       <c r="I17" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J17" s="4">
-        <v>3</v>
-      </c>
-      <c r="K17" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K17" s="4">
+        <v>4</v>
+      </c>
       <c r="L17" s="1">
-        <f t="shared" si="0"/>
-        <v>61</v>
+        <f>SUM(F17:K17)</f>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
-        <v>423316</v>
+        <v>420160</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F18" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G18" s="4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H18" s="4">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I18" s="4">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J18" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K18" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L18" s="1">
-        <f t="shared" si="0"/>
-        <v>59</v>
+        <f>SUM(F18:K18)</f>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>422101</v>
+        <v>422701</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G19" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H19" s="4">
+        <v>3</v>
+      </c>
+      <c r="I19" s="4">
+        <v>7</v>
+      </c>
+      <c r="J19" s="4">
+        <v>13</v>
+      </c>
+      <c r="K19" s="4">
         <v>15</v>
       </c>
-      <c r="I19" s="4">
-        <v>9</v>
-      </c>
-      <c r="J19" s="4">
-        <v>14</v>
-      </c>
-      <c r="K19" s="4"/>
       <c r="L19" s="1">
-        <f t="shared" si="0"/>
-        <v>53</v>
+        <f>SUM(F19:K19)</f>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>421400</v>
+        <v>424600</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="4">
-        <v>7</v>
-      </c>
-      <c r="G20" s="4">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G20" s="4"/>
       <c r="H20" s="4">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="I20" s="4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J20" s="4">
-        <v>12</v>
-      </c>
-      <c r="K20" s="4">
-        <v>32</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="K20" s="4"/>
       <c r="L20" s="1">
-        <f t="shared" si="0"/>
-        <v>53</v>
+        <f>SUM(F20:K20)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>420800</v>
+        <v>421100</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
@@ -5405,328 +5458,322 @@
         <v>6</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="6">
-        <v>6</v>
-      </c>
-      <c r="G21" s="6">
-        <v>10</v>
-      </c>
-      <c r="H21" s="6">
-        <v>12</v>
-      </c>
-      <c r="I21" s="6">
-        <v>12</v>
-      </c>
-      <c r="J21" s="6">
-        <v>6</v>
+      <c r="F21" s="4">
+        <v>3</v>
+      </c>
+      <c r="G21" s="4">
+        <v>4</v>
+      </c>
+      <c r="H21" s="4">
+        <v>6</v>
+      </c>
+      <c r="I21" s="4">
+        <v>6</v>
+      </c>
+      <c r="J21" s="4">
+        <v>20</v>
       </c>
       <c r="K21" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L21" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
+        <f>SUM(F21:K21)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>421801</v>
+        <v>422700</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="F22" s="4">
+        <v>10</v>
+      </c>
+      <c r="G22" s="4">
+        <v>14</v>
+      </c>
       <c r="H22" s="4">
-        <v>2</v>
-      </c>
-      <c r="I22" s="4">
-        <v>3</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="I22" s="4"/>
       <c r="J22" s="4">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="K22" s="4">
         <v>10</v>
       </c>
       <c r="L22" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
+        <f>SUM(F22:K22)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
-        <v>420160</v>
+        <v>423000</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="1"/>
+      <c r="F23" s="4">
         <v>10</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="4">
-        <v>7</v>
-      </c>
-      <c r="G23" s="4">
-        <v>12</v>
-      </c>
-      <c r="H23" s="4">
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4">
+        <v>4</v>
+      </c>
+      <c r="J23" s="4">
+        <v>21</v>
+      </c>
+      <c r="K23" s="4">
         <v>9</v>
       </c>
-      <c r="I23" s="4">
-        <v>10</v>
-      </c>
-      <c r="J23" s="4">
-        <v>6</v>
-      </c>
-      <c r="K23" s="4">
-        <v>5</v>
-      </c>
       <c r="L23" s="1">
-        <f t="shared" si="0"/>
-        <v>49</v>
+        <f>SUM(F23:K23)</f>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
-        <v>421100</v>
+        <v>422300</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="4">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G24" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H24" s="4">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I24" s="4">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="J24" s="4">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="K24" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L24" s="1">
-        <f t="shared" si="0"/>
-        <v>46</v>
+        <f>SUM(F24:K24)</f>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
-        <v>422700</v>
+        <v>424900</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="F25" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G25" s="4">
-        <v>14</v>
-      </c>
-      <c r="H25" s="4">
-        <v>6</v>
-      </c>
-      <c r="I25" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="H25" s="1">
+        <v>13</v>
+      </c>
+      <c r="I25" s="4">
+        <v>6</v>
+      </c>
       <c r="J25" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K25" s="4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L25" s="1">
-        <f t="shared" si="0"/>
-        <v>46</v>
+        <f>SUM(F25:K25)</f>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
-        <v>423000</v>
+        <v>420600</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>10</v>
-      </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+        <v>13</v>
+      </c>
+      <c r="G26" s="4">
+        <v>2</v>
+      </c>
+      <c r="H26" s="4">
+        <v>1</v>
+      </c>
       <c r="I26" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J26" s="4">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="K26" s="4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L26" s="1">
-        <f t="shared" si="0"/>
-        <v>45</v>
+        <f>SUM(F26:K26)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
-        <v>424900</v>
+        <v>422500</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="4">
+        <v>8</v>
+      </c>
+      <c r="G27" s="4">
+        <v>2</v>
+      </c>
+      <c r="H27" s="4">
+        <v>4</v>
+      </c>
+      <c r="I27" s="4">
         <v>9</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="J27" s="4">
         <v>11</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F27" s="4">
-        <v>4</v>
-      </c>
-      <c r="G27" s="4">
-        <v>12</v>
-      </c>
-      <c r="H27" s="1">
-        <v>13</v>
-      </c>
-      <c r="I27" s="4">
-        <v>6</v>
-      </c>
-      <c r="J27" s="4">
-        <v>3</v>
-      </c>
-      <c r="K27" s="4">
-        <v>0</v>
-      </c>
+      <c r="K27" s="4"/>
       <c r="L27" s="1">
-        <f t="shared" si="0"/>
-        <v>38</v>
+        <f>SUM(F27:K27)</f>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>424900</v>
+        <v>424000</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>124</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="4">
-        <v>9</v>
-      </c>
-      <c r="G28" s="4">
-        <v>14</v>
-      </c>
-      <c r="H28" s="6">
-        <v>15</v>
-      </c>
-      <c r="I28" s="4">
-        <v>6</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4">
+        <v>3</v>
+      </c>
+      <c r="I28" s="4"/>
       <c r="J28" s="4">
-        <v>4</v>
-      </c>
-      <c r="K28" s="4">
-        <v>4</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="K28" s="4"/>
       <c r="L28" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
+        <f>SUM(F28:K28)</f>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>421000</v>
+        <v>420101</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E29" s="1"/>
-      <c r="F29" s="6">
-        <v>5</v>
-      </c>
-      <c r="G29" s="6">
-        <v>15</v>
-      </c>
-      <c r="H29" s="6">
-        <v>17</v>
-      </c>
-      <c r="I29" s="6">
-        <v>16</v>
-      </c>
-      <c r="J29" s="6">
-        <v>11</v>
-      </c>
-      <c r="K29" s="6">
-        <v>12</v>
+      <c r="F29" s="4">
+        <v>7</v>
+      </c>
+      <c r="G29" s="4">
+        <v>7</v>
+      </c>
+      <c r="H29" s="4">
+        <v>7</v>
+      </c>
+      <c r="I29" s="4">
+        <v>7</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4">
+        <v>2</v>
       </c>
       <c r="L29" s="1">
-        <f t="shared" si="0"/>
-        <v>76</v>
+        <f>SUM(F29:K29)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
-        <v>424000</v>
+        <v>421801</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E30" s="1"/>
-      <c r="F30" s="4">
-        <v>20</v>
-      </c>
-      <c r="G30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4">
+        <v>1</v>
+      </c>
       <c r="H30" s="4">
-        <v>3</v>
-      </c>
-      <c r="I30" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="I30" s="4">
+        <v>4</v>
+      </c>
       <c r="J30" s="4">
-        <v>10</v>
-      </c>
-      <c r="K30" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="K30" s="4">
+        <v>11</v>
+      </c>
       <c r="L30" s="1">
-        <f t="shared" si="0"/>
-        <v>33</v>
+        <f>SUM(F30:K30)</f>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>422701</v>
+        <v>424701</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
@@ -5736,51 +5783,65 @@
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="4">
-        <v>1</v>
-      </c>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1</v>
+      </c>
+      <c r="H31" s="4">
+        <v>13</v>
+      </c>
       <c r="I31" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J31" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K31" s="4">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="L31" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
+        <f>SUM(F31:K31)</f>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
-        <v>423448</v>
+        <v>421901</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="4"/>
+      <c r="F32" s="4">
+        <v>4</v>
+      </c>
+      <c r="G32" s="4">
+        <v>8</v>
+      </c>
+      <c r="H32" s="4">
+        <v>6</v>
+      </c>
+      <c r="I32" s="4">
+        <v>5</v>
+      </c>
       <c r="J32" s="4">
         <v>4</v>
       </c>
-      <c r="K32" s="4"/>
+      <c r="K32" s="4">
+        <v>1</v>
+      </c>
       <c r="L32" s="1">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>SUM(F32:K32)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
-        <v>420101</v>
+        <v>422900</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>7</v>
@@ -5790,119 +5851,123 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="G33" s="4">
-        <v>7</v>
-      </c>
-      <c r="H33" s="4">
-        <v>7</v>
-      </c>
-      <c r="I33" s="4">
-        <v>7</v>
-      </c>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4">
+        <v>2</v>
+      </c>
+      <c r="K33" s="4"/>
       <c r="L33" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
+        <f>SUM(F33:K33)</f>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
-        <v>424701</v>
+        <v>421902</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="4">
         <v>2</v>
       </c>
-      <c r="G34" s="4"/>
+      <c r="G34" s="4">
+        <v>6</v>
+      </c>
       <c r="H34" s="4">
-        <v>13</v>
-      </c>
-      <c r="I34" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="I34" s="4">
+        <v>5</v>
+      </c>
       <c r="J34" s="4">
-        <v>13</v>
-      </c>
-      <c r="K34" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K34" s="4">
+        <v>2</v>
+      </c>
       <c r="L34" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
+        <f>SUM(F34:K34)</f>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
-        <v>421901</v>
+        <v>422190</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>122</v>
+      </c>
       <c r="F35" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G35" s="4">
-        <v>8</v>
-      </c>
-      <c r="H35" s="4">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="H35" s="6">
+        <v>5</v>
       </c>
       <c r="I35" s="4">
         <v>5</v>
       </c>
       <c r="J35" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K35" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L35" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
+        <f>SUM(F35:K35)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>422900</v>
+        <v>424801</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="4">
-        <v>23</v>
-      </c>
-      <c r="G36" s="4">
-        <v>1</v>
-      </c>
-      <c r="H36" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4">
+        <v>10</v>
+      </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K36" s="4"/>
       <c r="L36" s="1">
-        <f t="shared" si="0"/>
-        <v>26</v>
+        <f>SUM(F36:K36)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>421902</v>
+        <v>421900</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
@@ -5911,27 +5976,19 @@
         <v>10</v>
       </c>
       <c r="E37" s="1"/>
-      <c r="F37" s="4">
-        <v>2</v>
-      </c>
-      <c r="G37" s="4">
-        <v>6</v>
-      </c>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
       <c r="H37" s="4">
-        <v>6</v>
-      </c>
-      <c r="I37" s="4">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="I37" s="4"/>
       <c r="J37" s="4">
         <v>4</v>
       </c>
-      <c r="K37" s="4">
-        <v>2</v>
-      </c>
+      <c r="K37" s="4"/>
       <c r="L37" s="1">
-        <f t="shared" si="0"/>
-        <v>25</v>
+        <f>SUM(F37:K37)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
@@ -5946,537 +6003,533 @@
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
-        <v>3</v>
-      </c>
-      <c r="G38" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1</v>
+      </c>
       <c r="H38" s="4">
         <v>5</v>
       </c>
       <c r="I38" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J38" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K38" s="4">
         <v>4</v>
       </c>
       <c r="L38" s="1">
-        <f t="shared" si="0"/>
-        <v>24</v>
+        <f>SUM(F38:K38)</f>
+        <v>21</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
-        <v>422190</v>
+        <v>420900</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F39" s="4">
-        <v>2</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E39" s="1"/>
+      <c r="F39" s="4"/>
       <c r="G39" s="4">
         <v>5</v>
       </c>
-      <c r="H39" s="6">
-        <v>5</v>
-      </c>
-      <c r="I39" s="4">
-        <v>5</v>
-      </c>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
       <c r="J39" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K39" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L39" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
+        <f>SUM(F39:K39)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
-        <v>421900</v>
+        <v>423900</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="4">
-        <v>0</v>
-      </c>
-      <c r="G40" s="4">
-        <v>4</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G40" s="4"/>
       <c r="H40" s="4">
-        <v>7</v>
-      </c>
-      <c r="I40" s="4">
-        <v>3</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="I40" s="4"/>
       <c r="J40" s="4">
         <v>8</v>
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="1">
-        <f t="shared" si="0"/>
-        <v>22</v>
+        <f>SUM(F40:K40)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
-        <v>423501</v>
+        <v>422100</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E41" s="1"/>
-      <c r="F41" s="4">
-        <v>2</v>
-      </c>
-      <c r="G41" s="4">
-        <v>6</v>
-      </c>
-      <c r="H41" s="4">
-        <v>1</v>
-      </c>
-      <c r="I41" s="4">
-        <v>6</v>
-      </c>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
       <c r="J41" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K41" s="4">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="L41" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
+        <f>SUM(F41:K41)</f>
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
-        <v>423308</v>
+        <v>420802</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="4"/>
+      <c r="F42" s="1"/>
       <c r="G42" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H42" s="4">
+        <v>5</v>
+      </c>
+      <c r="I42" s="4">
+        <v>5</v>
+      </c>
+      <c r="J42" s="4">
         <v>3</v>
       </c>
-      <c r="I42" s="4">
-        <v>4</v>
-      </c>
-      <c r="J42" s="4">
-        <v>9</v>
-      </c>
-      <c r="K42" s="4"/>
+      <c r="K42" s="4">
+        <v>3</v>
+      </c>
       <c r="L42" s="1">
-        <f t="shared" si="0"/>
-        <v>21</v>
+        <f>SUM(G42:K42)</f>
+        <v>17</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
-        <v>423408</v>
+        <v>424700</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4">
-        <v>14</v>
-      </c>
+      <c r="F43" s="4">
+        <v>11</v>
+      </c>
+      <c r="G43" s="4"/>
       <c r="H43" s="4"/>
-      <c r="I43" s="4">
-        <v>2</v>
-      </c>
-      <c r="J43" s="4">
-        <v>4</v>
-      </c>
-      <c r="K43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4">
+        <v>5</v>
+      </c>
       <c r="L43" s="1">
-        <f t="shared" si="0"/>
-        <v>20</v>
+        <f>SUM(F43:K43)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>424801</v>
+        <v>424300</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="4">
+      <c r="F44" s="4"/>
+      <c r="G44" s="4">
+        <v>6</v>
+      </c>
+      <c r="H44" s="4">
         <v>4</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4">
-        <v>10</v>
-      </c>
-      <c r="I44" s="4"/>
+      <c r="I44" s="4">
+        <v>4</v>
+      </c>
       <c r="J44" s="4">
-        <v>9</v>
-      </c>
-      <c r="K44" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K44" s="4">
+        <v>6</v>
+      </c>
       <c r="L44" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
+        <f>SUM(F44:K44)</f>
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>420900</v>
+        <v>420200</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4">
-        <v>5</v>
-      </c>
-      <c r="H45" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="H45" s="4">
+        <v>1</v>
+      </c>
       <c r="I45" s="4"/>
       <c r="J45" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K45" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L45" s="1">
-        <f t="shared" si="0"/>
-        <v>19</v>
+        <f>SUM(F45:K45)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>423900</v>
+        <v>421301</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G46" s="4"/>
       <c r="H46" s="4">
-        <v>9</v>
-      </c>
-      <c r="I46" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="I46" s="4">
+        <v>2</v>
+      </c>
       <c r="J46" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="1">
-        <f t="shared" si="0"/>
-        <v>19</v>
+        <f>SUM(F46:K46)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>422100</v>
+        <v>423501</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E47" s="1"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
+      <c r="F47" s="4">
+        <v>2</v>
+      </c>
+      <c r="G47" s="4">
+        <v>3</v>
+      </c>
       <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
+      <c r="I47" s="4">
+        <v>3</v>
+      </c>
       <c r="J47" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K47" s="4">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="L47" s="1">
-        <f t="shared" si="0"/>
-        <v>18</v>
+        <f>SUM(F47:K47)</f>
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>424500</v>
+        <v>424200</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E48" s="1"/>
-      <c r="F48" s="4">
-        <v>4</v>
-      </c>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4">
+      <c r="F48" s="6"/>
+      <c r="G48" s="6">
+        <v>1</v>
+      </c>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6">
+        <v>9</v>
+      </c>
+      <c r="J48" s="6">
+        <v>1</v>
+      </c>
+      <c r="K48" s="6">
         <v>3</v>
       </c>
-      <c r="J48" s="4">
-        <v>3</v>
-      </c>
-      <c r="K48" s="4"/>
-      <c r="L48" s="1">
-        <f t="shared" si="0"/>
-        <v>10</v>
+      <c r="L48" s="12">
+        <f>SUM(F48:K48)</f>
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6">
-        <v>424700</v>
+        <v>421402</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E49" s="1"/>
-      <c r="F49" s="4">
-        <v>11</v>
-      </c>
+      <c r="F49" s="4"/>
       <c r="G49" s="4">
-        <v>1</v>
-      </c>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="H49" s="4">
+        <v>1</v>
+      </c>
+      <c r="I49" s="4">
+        <v>4</v>
+      </c>
+      <c r="J49" s="4">
+        <v>3</v>
+      </c>
       <c r="K49" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L49" s="1">
-        <f t="shared" si="0"/>
-        <v>17</v>
+        <f>SUM(F49:K49)</f>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>420802</v>
+        <v>425600</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="4">
-        <v>1</v>
-      </c>
-      <c r="H50" s="4">
-        <v>5</v>
-      </c>
-      <c r="I50" s="4">
-        <v>5</v>
-      </c>
-      <c r="J50" s="4">
-        <v>3</v>
-      </c>
-      <c r="K50" s="4">
-        <v>3</v>
+      <c r="F50" s="6">
+        <v>2</v>
+      </c>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6">
+        <v>2</v>
+      </c>
+      <c r="K50" s="6">
+        <v>7</v>
       </c>
       <c r="L50" s="1">
-        <f>SUM(G50:K50)</f>
-        <v>17</v>
+        <f>SUM(F50:K50)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>420200</v>
+        <v>423408</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4">
-        <v>1</v>
-      </c>
-      <c r="H51" s="4">
-        <v>1</v>
-      </c>
-      <c r="I51" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4">
+        <v>2</v>
+      </c>
       <c r="J51" s="4">
-        <v>2</v>
-      </c>
-      <c r="K51" s="4">
-        <v>11</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K51" s="4"/>
       <c r="L51" s="1">
-        <f t="shared" ref="L51:L62" si="1">SUM(F51:K51)</f>
-        <v>15</v>
+        <f>SUM(F51:K51)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>421301</v>
+        <v>424500</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
         <v>3</v>
       </c>
       <c r="G52" s="4"/>
-      <c r="H52" s="4">
-        <v>6</v>
-      </c>
+      <c r="H52" s="4"/>
       <c r="I52" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J52" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f t="shared" si="1"/>
-        <v>15</v>
+        <f>SUM(F52:K52)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>424300</v>
+        <v>421300</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E53" s="1"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4">
-        <v>5</v>
-      </c>
-      <c r="H53" s="4">
-        <v>2</v>
-      </c>
+      <c r="F53" s="4">
+        <v>2</v>
+      </c>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
       <c r="I53" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J53" s="4"/>
       <c r="K53" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L53" s="1">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <f>SUM(F53:K53)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
-        <v>421402</v>
+        <v>424960</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E54" s="1"/>
-      <c r="F54" s="4"/>
+      <c r="F54" s="4">
+        <v>1</v>
+      </c>
       <c r="G54" s="4">
-        <v>3</v>
-      </c>
-      <c r="H54" s="4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H54" s="6">
+        <v>2</v>
       </c>
       <c r="I54" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J54" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K54" s="4">
-        <v>2</v>
-      </c>
-      <c r="L54" s="1">
-        <f t="shared" si="1"/>
-        <v>13</v>
+        <v>1</v>
+      </c>
+      <c r="L54" s="12">
+        <f>SUM(F54:K54)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
-        <v>425600</v>
+        <v>421800</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="6">
-        <v>2</v>
-      </c>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
-      <c r="I55" s="6"/>
-      <c r="J55" s="6">
-        <v>2</v>
-      </c>
-      <c r="K55" s="6">
-        <v>7</v>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4">
+        <v>3</v>
+      </c>
+      <c r="I55" s="4">
+        <v>2</v>
+      </c>
+      <c r="J55" s="4">
+        <v>2</v>
+      </c>
+      <c r="K55" s="4">
+        <v>1</v>
       </c>
       <c r="L55" s="1">
-        <f t="shared" si="1"/>
-        <v>11</v>
+        <f>SUM(F55:K55)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
-        <v>423304</v>
+        <v>423348</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>7</v>
@@ -6486,80 +6539,81 @@
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="6"/>
-      <c r="I56" s="4"/>
+      <c r="G56" s="4">
+        <v>2</v>
+      </c>
+      <c r="H56" s="6">
+        <v>2</v>
+      </c>
+      <c r="I56" s="4">
+        <v>1</v>
+      </c>
       <c r="J56" s="4">
-        <v>6</v>
-      </c>
-      <c r="K56" s="4">
-        <v>2</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K56" s="4"/>
       <c r="L56" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F56:K56)</f>
         <v>8</v>
       </c>
     </row>
     <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>421300</v>
+        <v>422601</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
-      <c r="I57" s="4">
+      <c r="I57" s="4"/>
+      <c r="J57" s="4">
         <v>4</v>
       </c>
-      <c r="J57" s="4"/>
       <c r="K57" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L57" s="1">
-        <f t="shared" si="1"/>
+        <f>SUM(F57:K57)</f>
         <v>10</v>
+      </c>
+      <c r="M57" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>424960</v>
+        <v>421401</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E58" s="1"/>
-      <c r="F58" s="4">
-        <v>1</v>
-      </c>
+      <c r="F58" s="4"/>
       <c r="G58" s="4">
         <v>2</v>
       </c>
-      <c r="H58" s="6">
-        <v>2</v>
-      </c>
-      <c r="I58" s="4">
-        <v>2</v>
-      </c>
-      <c r="J58" s="4">
-        <v>1</v>
-      </c>
+      <c r="H58" s="4">
+        <v>4</v>
+      </c>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
       <c r="K58" s="4">
         <v>1</v>
       </c>
-      <c r="L58" s="12">
-        <f t="shared" si="1"/>
-        <v>9</v>
+      <c r="L58" s="1">
+        <f>SUM(F58:K58)</f>
+        <v>7</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
@@ -6567,73 +6621,71 @@
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
-        <v>421800</v>
+        <v>421001</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E59" s="1"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4">
-        <v>3</v>
-      </c>
-      <c r="I59" s="4">
-        <v>2</v>
-      </c>
-      <c r="J59" s="4">
-        <v>2</v>
-      </c>
-      <c r="K59" s="4">
-        <v>1</v>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1">
+        <v>2</v>
+      </c>
+      <c r="I59" s="1">
+        <v>1</v>
+      </c>
+      <c r="J59" s="1">
+        <v>1</v>
+      </c>
+      <c r="K59" s="1">
+        <v>2</v>
       </c>
       <c r="L59" s="1">
-        <f t="shared" si="1"/>
-        <v>8</v>
+        <f>SUM(H59:K59)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
-        <v>423348</v>
+        <v>420500</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E60" s="1"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4">
-        <v>2</v>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6">
+        <v>1</v>
       </c>
       <c r="H60" s="6">
         <v>2</v>
       </c>
-      <c r="I60" s="4">
-        <v>1</v>
-      </c>
-      <c r="J60" s="4">
-        <v>3</v>
+      <c r="I60" s="4"/>
+      <c r="J60" s="6">
+        <v>2</v>
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="1">
-        <f t="shared" si="1"/>
-        <v>8</v>
+        <f>SUM(F60:K60)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
-        <v>422601</v>
+        <v>420402</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E61" s="1"/>
       <c r="F61" s="4"/>
@@ -6641,179 +6693,163 @@
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <f>SUM(F61:K61)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
-        <v>421401</v>
+        <v>423448</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="4"/>
-      <c r="G62" s="4">
-        <v>2</v>
-      </c>
-      <c r="H62" s="4">
+      <c r="G62" s="4"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4">
         <v>4</v>
       </c>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4">
-        <v>1</v>
-      </c>
+      <c r="K62" s="4"/>
       <c r="L62" s="1">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <f>SUM(F62:K62)</f>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
-        <v>421001</v>
+        <v>422600</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>5</v>
+        <v>127</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E63" s="1"/>
-      <c r="F63" s="1"/>
-      <c r="G63" s="1"/>
-      <c r="H63" s="1">
-        <v>2</v>
-      </c>
-      <c r="I63" s="1">
-        <v>1</v>
-      </c>
-      <c r="J63" s="1">
-        <v>1</v>
-      </c>
-      <c r="K63" s="1">
-        <v>2</v>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6"/>
+      <c r="K63" s="6">
+        <v>3</v>
       </c>
       <c r="L63" s="1">
-        <f>SUM(H63:K63)</f>
-        <v>6</v>
+        <f>SUM(F63:K63)</f>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
-        <v>420500</v>
+        <v>423309</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E64" s="1"/>
-      <c r="F64" s="6"/>
-      <c r="G64" s="6">
-        <v>1</v>
-      </c>
-      <c r="H64" s="6">
-        <v>2</v>
-      </c>
-      <c r="I64" s="4"/>
-      <c r="J64" s="6">
-        <v>2</v>
-      </c>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4">
+        <v>1</v>
+      </c>
+      <c r="H64" s="4">
+        <v>1</v>
+      </c>
+      <c r="I64" s="4">
+        <v>1</v>
+      </c>
+      <c r="J64" s="4"/>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f t="shared" ref="L64:L74" si="2">SUM(F64:K64)</f>
-        <v>5</v>
+        <f>SUM(F64:K64)</f>
+        <v>3</v>
       </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
-        <v>420402</v>
+        <v>423308</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
+      <c r="G65" s="4">
+        <v>2</v>
+      </c>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="4">
-        <v>5</v>
-      </c>
+      <c r="J65" s="4"/>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f t="shared" si="2"/>
-        <v>5</v>
+        <f>SUM(F65:K65)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
-        <v>423416</v>
+        <v>422400</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E66" s="1"/>
-      <c r="F66" s="4">
-        <v>1</v>
-      </c>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4">
-        <v>1</v>
-      </c>
-      <c r="I66" s="4"/>
-      <c r="J66" s="4">
-        <v>2</v>
-      </c>
-      <c r="K66" s="4"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6"/>
+      <c r="H66" s="6"/>
+      <c r="I66" s="6"/>
+      <c r="J66" s="6">
+        <v>2</v>
+      </c>
+      <c r="K66" s="6"/>
       <c r="L66" s="1">
-        <f t="shared" si="2"/>
-        <v>4</v>
+        <f>SUM(F66:K66)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
-        <v>422600</v>
+        <v>423316</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E67" s="1"/>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
-      <c r="J67" s="6"/>
-      <c r="K67" s="6">
-        <v>3</v>
-      </c>
+      <c r="F67" s="4"/>
+      <c r="G67" s="4"/>
+      <c r="H67" s="4"/>
+      <c r="I67" s="4"/>
+      <c r="J67" s="4"/>
+      <c r="K67" s="4"/>
       <c r="L67" s="1">
-        <f t="shared" si="2"/>
-        <v>3</v>
+        <f>SUM(F67:K67)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="6">
-        <v>423309</v>
+        <v>423304</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>7</v>
@@ -6823,95 +6859,85 @@
       </c>
       <c r="E68" s="1"/>
       <c r="F68" s="4"/>
-      <c r="G68" s="4">
-        <v>1</v>
-      </c>
-      <c r="H68" s="4">
-        <v>1</v>
-      </c>
-      <c r="I68" s="4">
-        <v>1</v>
-      </c>
+      <c r="G68" s="4"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="4"/>
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f t="shared" si="2"/>
-        <v>3</v>
+        <f>SUM(F68:K68)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="6">
-        <v>422400</v>
+        <v>423416</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E69" s="1"/>
-      <c r="F69" s="6"/>
-      <c r="G69" s="6"/>
-      <c r="H69" s="6"/>
-      <c r="I69" s="6"/>
-      <c r="J69" s="6">
-        <v>2</v>
-      </c>
-      <c r="K69" s="6"/>
+      <c r="F69" s="4"/>
+      <c r="G69" s="4"/>
+      <c r="H69" s="4"/>
+      <c r="I69" s="4"/>
+      <c r="J69" s="4"/>
+      <c r="K69" s="4"/>
       <c r="L69" s="1">
-        <f t="shared" si="2"/>
-        <v>2</v>
+        <f>SUM(F69:K69)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="6">
-        <v>422401</v>
+        <v>420300</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E70" s="1"/>
-      <c r="F70" s="1"/>
-      <c r="G70" s="1"/>
-      <c r="H70" s="1"/>
-      <c r="I70" s="1"/>
-      <c r="J70" s="1"/>
-      <c r="K70" s="1"/>
-      <c r="L70" s="1">
-        <f t="shared" si="2"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
+      <c r="J70" s="6"/>
+      <c r="K70" s="6"/>
+      <c r="L70" s="12">
+        <f>SUM(F70:K70)</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
-        <v>423800</v>
+        <v>422401</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F71" s="6"/>
-      <c r="G71" s="6"/>
-      <c r="H71" s="6"/>
-      <c r="I71" s="6"/>
-      <c r="J71" s="6"/>
-      <c r="K71" s="6"/>
+        <v>12</v>
+      </c>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
       <c r="L71" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F71:K71)</f>
         <v>0</v>
       </c>
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
-        <v>424200</v>
+        <v>423800</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>7</v>
@@ -6919,24 +6945,18 @@
       <c r="D72" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E72" s="1"/>
+      <c r="E72" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="F72" s="6"/>
-      <c r="G72" s="6">
-        <v>1</v>
-      </c>
+      <c r="G72" s="6"/>
       <c r="H72" s="6"/>
-      <c r="I72" s="6">
-        <v>9</v>
-      </c>
-      <c r="J72" s="6">
-        <v>1</v>
-      </c>
-      <c r="K72" s="6">
-        <v>3</v>
-      </c>
-      <c r="L72" s="12">
-        <f t="shared" si="2"/>
-        <v>14</v>
+      <c r="I72" s="6"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="6"/>
+      <c r="L72" s="1">
+        <f>SUM(F72:K72)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.25">
@@ -6957,7 +6977,7 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F73:K73)</f>
         <v>0</v>
       </c>
     </row>
@@ -6979,7 +6999,7 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f t="shared" si="2"/>
+        <f>SUM(F74:K74)</f>
         <v>0</v>
       </c>
     </row>
@@ -7040,7 +7060,7 @@
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L79" s="10">
         <f>SUM(L3:L78)</f>
-        <v>2819</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="83" spans="15:15" x14ac:dyDescent="0.25">
@@ -7065,10 +7085,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:M10"/>
+  <dimension ref="B3:L14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
@@ -7103,112 +7123,109 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
-        <v>432900</v>
+        <v>431400</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G4" s="1">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H4" s="1">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I4" s="1">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="J4" s="1">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K4" s="1">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>560</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
-        <v>431800</v>
+        <v>430100</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>130</v>
+        <v>6</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="G5" s="1">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="H5" s="1">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="I5" s="1">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J5" s="1">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K5" s="1">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>531</v>
-      </c>
-      <c r="M5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
-        <v>430900</v>
+        <v>432100</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G6" s="1">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="H6" s="1">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="I6" s="1">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="J6" s="1">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="K6" s="1">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>233</v>
-      </c>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>432300</v>
       </c>
@@ -7216,60 +7233,224 @@
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="G7" s="1">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="H7" s="1">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="I7" s="1">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="J7" s="1">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="K7" s="1">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="L7" s="1">
         <f>SUM(F7:K7)</f>
-        <v>576</v>
-      </c>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="L10">
-        <f>SUM(L4:L7)</f>
-        <v>1900</v>
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>432900</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1">
+        <v>35</v>
+      </c>
+      <c r="G8" s="1">
+        <v>95</v>
+      </c>
+      <c r="H8" s="1">
+        <v>100</v>
+      </c>
+      <c r="I8" s="1">
+        <v>91</v>
+      </c>
+      <c r="J8" s="1">
+        <v>62</v>
+      </c>
+      <c r="K8" s="1">
+        <v>57</v>
+      </c>
+      <c r="L8" s="1">
+        <f>SUM(F8:K8)</f>
+        <v>440</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>430900</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1">
+        <v>30</v>
+      </c>
+      <c r="G9" s="1">
+        <v>87</v>
+      </c>
+      <c r="H9" s="1">
+        <v>102</v>
+      </c>
+      <c r="I9" s="1">
+        <v>96</v>
+      </c>
+      <c r="J9" s="1">
+        <v>77</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46</v>
+      </c>
+      <c r="L9" s="1">
+        <f>SUM(F9:K9)</f>
+        <v>438</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>431800</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1">
+        <v>30</v>
+      </c>
+      <c r="G10" s="1">
+        <v>80</v>
+      </c>
+      <c r="H10" s="1">
+        <v>87</v>
+      </c>
+      <c r="I10" s="1">
+        <v>70</v>
+      </c>
+      <c r="J10" s="1">
+        <v>57</v>
+      </c>
+      <c r="K10" s="1">
+        <v>41</v>
+      </c>
+      <c r="L10" s="1">
+        <f>SUM(F10:K10)</f>
+        <v>365</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>434100</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1">
+        <v>29</v>
+      </c>
+      <c r="G11" s="1">
+        <v>62</v>
+      </c>
+      <c r="H11" s="1">
+        <v>64</v>
+      </c>
+      <c r="I11" s="1">
+        <v>61</v>
+      </c>
+      <c r="J11" s="1">
+        <v>38</v>
+      </c>
+      <c r="K11" s="1">
+        <v>34</v>
+      </c>
+      <c r="L11" s="1">
+        <f>SUM(F11:K11)</f>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="19">
+        <v>433900</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1"/>
+      <c r="F12" s="19">
+        <v>30</v>
+      </c>
+      <c r="G12" s="19">
+        <v>64</v>
+      </c>
+      <c r="H12" s="19">
+        <v>57</v>
+      </c>
+      <c r="I12" s="19">
+        <v>62</v>
+      </c>
+      <c r="J12" s="19">
+        <v>41</v>
+      </c>
+      <c r="K12" s="19">
+        <v>39</v>
+      </c>
+      <c r="L12" s="19">
+        <f>SUM(F12:K12)</f>
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="I13" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <f>SUM(L4:L13)</f>
+        <v>3806</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:L3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}"/>
+  <autoFilter ref="B3:L13" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:L13">
+      <sortCondition descending="1" ref="L3:L13"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7413,31 +7594,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7453,4 +7625,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar datos y recarga desde seed
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3438" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE9101E6-FED5-4DC0-9E5F-9FBA180ACA68}"/>
+  <xr:revisionPtr revIDLastSave="3517" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E62BF79-4C01-4116-88CC-5F073E178EE6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -27,10 +27,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'COLE 40'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'COLE 41'!$B$4:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'COLE 42'!$B$2:$L$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$B$3:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$B$3:$L$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="133">
   <si>
     <t>CODIGO</t>
   </si>
@@ -446,10 +446,10 @@
     <t>WIDE LEG</t>
   </si>
   <si>
-    <t>_</t>
-  </si>
-  <si>
     <t>ULTIMA ACTUALIZACION 10:147  25-05-2026</t>
+  </si>
+  <si>
+    <t>WID LEG</t>
   </si>
 </sst>
 </file>
@@ -507,7 +507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -580,6 +580,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -631,7 +642,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4781,6 +4792,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
+  <sheetPr filterMode="1"/>
   <dimension ref="B2:P127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4823,7 +4835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B3" s="6">
         <v>422200</v>
       </c>
@@ -4853,11 +4865,11 @@
         <v>20</v>
       </c>
       <c r="L3" s="1">
-        <f>SUM(F3:K3)</f>
+        <f t="shared" ref="L3:L41" si="0">SUM(F3:K3)</f>
         <v>212</v>
       </c>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" s="6">
         <v>423600</v>
       </c>
@@ -4887,11 +4899,11 @@
         <v>25</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6">
         <v>423500</v>
       </c>
@@ -4921,11 +4933,11 @@
         <v>11</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
+        <f t="shared" si="0"/>
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>420301</v>
       </c>
@@ -4937,35 +4949,35 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="6">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G6" s="6">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H6" s="6">
+        <v>34</v>
+      </c>
+      <c r="I6" s="6">
         <v>26</v>
       </c>
-      <c r="I6" s="6">
+      <c r="J6" s="6">
         <v>28</v>
       </c>
-      <c r="J6" s="6">
-        <v>14</v>
-      </c>
       <c r="K6" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
-        <v>102</v>
+        <f t="shared" si="0"/>
+        <v>142</v>
       </c>
       <c r="M6" t="s">
         <v>123</v>
       </c>
       <c r="N6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6">
         <v>423200</v>
       </c>
@@ -4995,11 +5007,11 @@
         <v>16</v>
       </c>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
+        <f t="shared" si="0"/>
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6">
         <v>421000</v>
       </c>
@@ -5029,11 +5041,11 @@
         <v>10</v>
       </c>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6">
         <v>420100</v>
       </c>
@@ -5061,12 +5073,12 @@
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6">
         <v>422800</v>
       </c>
@@ -5092,14 +5104,14 @@
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
       <c r="O10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>422000</v>
       </c>
@@ -5127,14 +5139,14 @@
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
+        <f t="shared" si="0"/>
         <v>63</v>
       </c>
       <c r="O11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>424400</v>
       </c>
@@ -5149,7 +5161,7 @@
         <v>17</v>
       </c>
       <c r="G12" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H12" s="4">
         <v>9</v>
@@ -5160,14 +5172,14 @@
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
-        <v>56</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
       <c r="N12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
         <v>420800</v>
       </c>
@@ -5197,14 +5209,14 @@
         <v>6</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="O13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
         <v>420400</v>
       </c>
@@ -5234,14 +5246,14 @@
         <v>12</v>
       </c>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
         <v>421400</v>
       </c>
@@ -5271,12 +5283,12 @@
         <v>32</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
       <c r="N15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
         <v>422101</v>
       </c>
@@ -5304,14 +5316,14 @@
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="O16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
         <v>424900</v>
       </c>
@@ -5343,11 +5355,11 @@
         <v>4</v>
       </c>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
         <v>420160</v>
       </c>
@@ -5379,111 +5391,109 @@
         <v>5</v>
       </c>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
-        <v>422701</v>
+        <v>424600</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="4">
-        <v>4</v>
-      </c>
-      <c r="G19" s="4">
         <v>3</v>
       </c>
+      <c r="G19" s="4"/>
       <c r="H19" s="4">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="I19" s="4">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="J19" s="4">
-        <v>13</v>
-      </c>
-      <c r="K19" s="4">
-        <v>15</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="K19" s="4"/>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
-        <v>424600</v>
+        <v>421100</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="4">
+        <v>2</v>
+      </c>
+      <c r="G20" s="4">
         <v>3</v>
       </c>
-      <c r="G20" s="4"/>
       <c r="H20" s="4">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I20" s="4">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="J20" s="4">
-        <v>14</v>
-      </c>
-      <c r="K20" s="4"/>
+        <v>20</v>
+      </c>
+      <c r="K20" s="4">
+        <v>7</v>
+      </c>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
-        <v>421100</v>
+        <v>422700</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G21" s="4">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H21" s="4">
         <v>6</v>
       </c>
-      <c r="I21" s="4">
-        <v>6</v>
-      </c>
+      <c r="I21" s="4"/>
       <c r="J21" s="4">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="K21" s="4">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
-        <v>422700</v>
+        <v>422701</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -5493,27 +5503,29 @@
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G22" s="4">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H22" s="4">
-        <v>6</v>
-      </c>
-      <c r="I22" s="4"/>
+        <v>3</v>
+      </c>
+      <c r="I22" s="4">
+        <v>7</v>
+      </c>
       <c r="J22" s="4">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="K22" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
         <v>423000</v>
       </c>
@@ -5539,11 +5551,11 @@
         <v>9</v>
       </c>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
         <v>422300</v>
       </c>
@@ -5573,11 +5585,11 @@
         <v>1</v>
       </c>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
+        <f t="shared" si="0"/>
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
         <v>424900</v>
       </c>
@@ -5609,11 +5621,11 @@
         <v>0</v>
       </c>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
         <v>420600</v>
       </c>
@@ -5625,29 +5637,26 @@
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="4">
-        <v>13</v>
-      </c>
-      <c r="G26" s="4">
-        <v>2</v>
-      </c>
-      <c r="H26" s="4">
-        <v>1</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
       <c r="I26" s="4">
-        <v>1</v>
-      </c>
-      <c r="J26" s="4">
-        <v>13</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="J26" s="4"/>
       <c r="K26" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="M26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>422500</v>
       </c>
@@ -5675,41 +5684,47 @@
       </c>
       <c r="K27" s="4"/>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
-        <v>424000</v>
+        <v>424701</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="4">
-        <v>20</v>
-      </c>
-      <c r="G28" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="G28" s="4">
+        <v>1</v>
+      </c>
       <c r="H28" s="4">
-        <v>3</v>
-      </c>
-      <c r="I28" s="4"/>
+        <v>13</v>
+      </c>
+      <c r="I28" s="4">
+        <v>1</v>
+      </c>
       <c r="J28" s="4">
-        <v>10</v>
-      </c>
-      <c r="K28" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="K28" s="4">
+        <v>1</v>
+      </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
-        <v>420101</v>
+        <v>424000</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
@@ -5719,27 +5734,21 @@
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="4">
-        <v>7</v>
-      </c>
-      <c r="G29" s="4">
-        <v>7</v>
-      </c>
-      <c r="H29" s="4">
-        <v>7</v>
-      </c>
-      <c r="I29" s="4">
-        <v>7</v>
-      </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4">
-        <v>2</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4">
+        <v>10</v>
+      </c>
+      <c r="K29" s="4"/>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
         <v>421801</v>
       </c>
@@ -5767,45 +5776,43 @@
         <v>11</v>
       </c>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
-        <v>424701</v>
+        <v>420101</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="4">
+        <v>7</v>
+      </c>
+      <c r="G31" s="4">
+        <v>7</v>
+      </c>
+      <c r="H31" s="4">
+        <v>7</v>
+      </c>
+      <c r="I31" s="4">
+        <v>7</v>
+      </c>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4">
         <v>2</v>
       </c>
-      <c r="G31" s="4">
-        <v>1</v>
-      </c>
-      <c r="H31" s="4">
-        <v>13</v>
-      </c>
-      <c r="I31" s="4">
-        <v>1</v>
-      </c>
-      <c r="J31" s="4">
-        <v>16</v>
-      </c>
-      <c r="K31" s="4">
-        <v>1</v>
-      </c>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="6">
         <v>421901</v>
       </c>
@@ -5835,11 +5842,11 @@
         <v>1</v>
       </c>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="6">
         <v>422900</v>
       </c>
@@ -5851,7 +5858,7 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="4">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="G33" s="4">
         <v>1</v>
@@ -5863,11 +5870,11 @@
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="1">
-        <f>SUM(F33:K33)</f>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="6">
         <v>421902</v>
       </c>
@@ -5897,11 +5904,11 @@
         <v>2</v>
       </c>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="6">
         <v>422190</v>
       </c>
@@ -5933,41 +5940,47 @@
         <v>3</v>
       </c>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6">
-        <v>424801</v>
+        <v>420501</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="4">
         <v>4</v>
       </c>
-      <c r="G36" s="4"/>
+      <c r="G36" s="4">
+        <v>1</v>
+      </c>
       <c r="H36" s="4">
-        <v>10</v>
-      </c>
-      <c r="I36" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="I36" s="4">
+        <v>1</v>
+      </c>
       <c r="J36" s="4">
-        <v>5</v>
-      </c>
-      <c r="K36" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="K36" s="4">
+        <v>4</v>
+      </c>
       <c r="L36" s="1">
         <f>SUM(F36:K36)</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="6">
-        <v>421900</v>
+        <v>424300</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
@@ -5977,55 +5990,55 @@
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="G37" s="4">
+        <v>6</v>
+      </c>
       <c r="H37" s="4">
-        <v>2</v>
-      </c>
-      <c r="I37" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="I37" s="4">
+        <v>4</v>
+      </c>
       <c r="J37" s="4">
-        <v>4</v>
-      </c>
-      <c r="K37" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="K37" s="4">
+        <v>6</v>
+      </c>
       <c r="L37" s="1">
         <f>SUM(F37:K37)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" s="6">
-        <v>420501</v>
+        <v>424801</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="4">
         <v>4</v>
       </c>
-      <c r="G38" s="4">
-        <v>1</v>
-      </c>
+      <c r="G38" s="4"/>
       <c r="H38" s="4">
-        <v>5</v>
-      </c>
-      <c r="I38" s="4">
-        <v>1</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I38" s="4"/>
       <c r="J38" s="4">
-        <v>6</v>
-      </c>
-      <c r="K38" s="4">
-        <v>4</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K38" s="4"/>
       <c r="L38" s="1">
         <f>SUM(F38:K38)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="6">
         <v>420900</v>
       </c>
@@ -6053,7 +6066,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="6">
         <v>423900</v>
       </c>
@@ -6081,7 +6094,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
         <v>422100</v>
       </c>
@@ -6107,7 +6120,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
         <v>420802</v>
       </c>
@@ -6118,9 +6131,11 @@
         <v>6</v>
       </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
+      <c r="F42" s="6">
+        <v>1</v>
+      </c>
       <c r="G42" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H42" s="4">
         <v>5</v>
@@ -6136,10 +6151,10 @@
       </c>
       <c r="L42" s="1">
         <f>SUM(G42:K42)</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
         <v>424700</v>
       </c>
@@ -6167,303 +6182,301 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
-        <v>424300</v>
+        <v>420200</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H44" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I44" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J44" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L44" s="1">
         <f>SUM(F44:K44)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="6">
-        <v>420200</v>
+        <v>421301</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E45" s="1"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4">
-        <v>1</v>
-      </c>
+      <c r="F45" s="4">
+        <v>3</v>
+      </c>
+      <c r="G45" s="4"/>
       <c r="H45" s="4">
-        <v>1</v>
-      </c>
-      <c r="I45" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="I45" s="4">
+        <v>2</v>
+      </c>
       <c r="J45" s="4">
-        <v>2</v>
-      </c>
-      <c r="K45" s="4">
-        <v>11</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K45" s="4"/>
       <c r="L45" s="1">
         <f>SUM(F45:K45)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="6">
-        <v>421301</v>
+        <v>423501</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="4">
+        <v>2</v>
+      </c>
+      <c r="G46" s="4">
         <v>3</v>
       </c>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4">
-        <v>6</v>
-      </c>
+      <c r="H46" s="4"/>
       <c r="I46" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J46" s="4">
-        <v>4</v>
-      </c>
-      <c r="K46" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="K46" s="4">
+        <v>6</v>
+      </c>
       <c r="L46" s="1">
         <f>SUM(F46:K46)</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" s="6">
-        <v>423501</v>
+        <v>424200</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E47" s="1"/>
-      <c r="F47" s="4">
-        <v>2</v>
-      </c>
-      <c r="G47" s="4">
+      <c r="F47" s="6"/>
+      <c r="G47" s="6">
+        <v>1</v>
+      </c>
+      <c r="H47" s="6"/>
+      <c r="I47" s="6">
+        <v>9</v>
+      </c>
+      <c r="J47" s="6">
+        <v>1</v>
+      </c>
+      <c r="K47" s="6">
         <v>3</v>
       </c>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4">
-        <v>3</v>
-      </c>
-      <c r="J47" s="4">
-        <v>0</v>
-      </c>
-      <c r="K47" s="4">
-        <v>6</v>
-      </c>
-      <c r="L47" s="1">
+      <c r="L47" s="12">
         <f>SUM(F47:K47)</f>
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="6">
-        <v>424200</v>
+        <v>421402</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" s="1"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4">
+        <v>3</v>
+      </c>
+      <c r="H48" s="4">
+        <v>1</v>
+      </c>
+      <c r="I48" s="4">
+        <v>4</v>
+      </c>
+      <c r="J48" s="4">
+        <v>3</v>
+      </c>
+      <c r="K48" s="4">
+        <v>2</v>
+      </c>
+      <c r="L48" s="1">
+        <f>SUM(F48:K48)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="6">
+        <v>425600</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E48" s="1"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6">
-        <v>1</v>
-      </c>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6">
-        <v>9</v>
-      </c>
-      <c r="J48" s="6">
-        <v>1</v>
-      </c>
-      <c r="K48" s="6">
-        <v>3</v>
-      </c>
-      <c r="L48" s="12">
-        <f>SUM(F48:K48)</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B49" s="6">
-        <v>421402</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="E49" s="1"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4">
-        <v>3</v>
-      </c>
-      <c r="H49" s="4">
-        <v>1</v>
-      </c>
-      <c r="I49" s="4">
-        <v>4</v>
-      </c>
-      <c r="J49" s="4">
-        <v>3</v>
-      </c>
-      <c r="K49" s="4">
+      <c r="F49" s="6">
         <v>2</v>
+      </c>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6">
+        <v>2</v>
+      </c>
+      <c r="K49" s="6">
+        <v>7</v>
       </c>
       <c r="L49" s="1">
         <f>SUM(F49:K49)</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="6">
-        <v>425600</v>
+        <v>423408</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1"/>
-      <c r="F50" s="6">
+      <c r="F50" s="4"/>
+      <c r="G50" s="4">
+        <v>4</v>
+      </c>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4">
         <v>2</v>
       </c>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6">
-        <v>2</v>
-      </c>
-      <c r="K50" s="6">
-        <v>7</v>
-      </c>
+      <c r="J50" s="4">
+        <v>4</v>
+      </c>
+      <c r="K50" s="4"/>
       <c r="L50" s="1">
         <f>SUM(F50:K50)</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="6">
-        <v>423408</v>
+        <v>421300</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4">
-        <v>4</v>
-      </c>
+      <c r="F51" s="4">
+        <v>2</v>
+      </c>
+      <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4">
-        <v>2</v>
-      </c>
-      <c r="J51" s="4">
         <v>4</v>
       </c>
-      <c r="K51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4">
+        <v>4</v>
+      </c>
       <c r="L51" s="1">
         <f>SUM(F51:K51)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="6">
-        <v>424500</v>
+        <v>422601</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
-      <c r="I52" s="4">
-        <v>3</v>
-      </c>
+      <c r="I52" s="4"/>
       <c r="J52" s="4">
-        <v>3</v>
-      </c>
-      <c r="K52" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="K52" s="4">
+        <v>1</v>
+      </c>
       <c r="L52" s="1">
         <f>SUM(F52:K52)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="6">
-        <v>421300</v>
+        <v>424500</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4">
-        <v>4</v>
-      </c>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4">
-        <v>4</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="J53" s="4">
+        <v>3</v>
+      </c>
+      <c r="K53" s="4"/>
       <c r="L53" s="1">
         <f>SUM(F53:K53)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="6">
         <v>424960</v>
       </c>
@@ -6497,7 +6510,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" s="6">
         <v>421800</v>
       </c>
@@ -6508,26 +6521,30 @@
         <v>6</v>
       </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
+      <c r="F55" s="4">
+        <v>3</v>
+      </c>
+      <c r="G55" s="4">
+        <v>2</v>
+      </c>
       <c r="H55" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I55" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J55" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K55" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L55" s="1">
         <f>SUM(F55:K55)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" s="6">
         <v>423348</v>
       </c>
@@ -6557,69 +6574,67 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" s="6">
-        <v>422601</v>
+        <v>421401</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="4">
-        <v>5</v>
-      </c>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4">
+        <v>2</v>
+      </c>
+      <c r="H57" s="4">
+        <v>4</v>
+      </c>
       <c r="I57" s="4"/>
-      <c r="J57" s="4">
-        <v>4</v>
-      </c>
+      <c r="J57" s="4"/>
       <c r="K57" s="4">
         <v>1</v>
       </c>
       <c r="L57" s="1">
         <f>SUM(F57:K57)</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="M57" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" s="6">
-        <v>421401</v>
+        <v>421900</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="4"/>
-      <c r="G58" s="4">
+      <c r="G58" s="4"/>
+      <c r="H58" s="4">
         <v>2</v>
       </c>
-      <c r="H58" s="4">
+      <c r="I58" s="4"/>
+      <c r="J58" s="4">
         <v>4</v>
       </c>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4">
-        <v>1</v>
-      </c>
+      <c r="K58" s="4"/>
       <c r="L58" s="1">
         <f>SUM(F58:K58)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P58" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" s="6">
         <v>421001</v>
       </c>
@@ -6649,7 +6664,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" s="6">
         <v>420500</v>
       </c>
@@ -6677,7 +6692,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="6">
         <v>420402</v>
       </c>
@@ -6697,11 +6712,11 @@
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="1">
-        <f>SUM(F61:K61)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L60:L74" si="1">SUM(F61:K61)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
         <v>423448</v>
       </c>
@@ -6721,11 +6736,11 @@
       </c>
       <c r="K62" s="4"/>
       <c r="L62" s="1">
-        <f>SUM(F62:K62)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" s="6">
         <v>422600</v>
       </c>
@@ -6745,11 +6760,11 @@
         <v>3</v>
       </c>
       <c r="L63" s="1">
-        <f>SUM(F63:K63)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="B64" s="6">
         <v>423309</v>
       </c>
@@ -6773,11 +6788,11 @@
       <c r="J64" s="4"/>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f>SUM(F64:K64)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="6">
         <v>423308</v>
       </c>
@@ -6797,11 +6812,11 @@
       <c r="J65" s="4"/>
       <c r="K65" s="4"/>
       <c r="L65" s="1">
-        <f>SUM(F65:K65)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
         <v>422400</v>
       </c>
@@ -6821,11 +6836,11 @@
       </c>
       <c r="K66" s="6"/>
       <c r="L66" s="1">
-        <f>SUM(F66:K66)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" s="6">
         <v>423316</v>
       </c>
@@ -6843,11 +6858,11 @@
       <c r="J67" s="4"/>
       <c r="K67" s="4"/>
       <c r="L67" s="1">
-        <f>SUM(F67:K67)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="6">
         <v>423304</v>
       </c>
@@ -6865,11 +6880,11 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f>SUM(F68:K68)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" s="6">
         <v>423416</v>
       </c>
@@ -6887,11 +6902,11 @@
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
       <c r="L69" s="1">
-        <f>SUM(F69:K69)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" s="6">
         <v>420300</v>
       </c>
@@ -6909,11 +6924,11 @@
       <c r="J70" s="6"/>
       <c r="K70" s="6"/>
       <c r="L70" s="12">
-        <f>SUM(F70:K70)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
         <v>422401</v>
       </c>
@@ -6931,11 +6946,11 @@
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
       <c r="L71" s="1">
-        <f>SUM(F71:K71)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
         <v>423800</v>
       </c>
@@ -6955,11 +6970,11 @@
       <c r="J72" s="6"/>
       <c r="K72" s="6"/>
       <c r="L72" s="1">
-        <f>SUM(F72:K72)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" s="6">
         <v>423409</v>
       </c>
@@ -6977,11 +6992,11 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f>SUM(F73:K73)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" s="6">
         <v>423404</v>
       </c>
@@ -6999,11 +7014,11 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f>SUM(F74:K74)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="6">
         <v>420801</v>
       </c>
@@ -7025,7 +7040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" s="6">
         <v>420160</v>
       </c>
@@ -7052,7 +7067,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>123</v>
       </c>
@@ -7060,7 +7075,7 @@
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L79" s="10">
         <f>SUM(L3:L78)</f>
-        <v>2291</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="83" spans="15:15" x14ac:dyDescent="0.25">
@@ -7075,7 +7090,12 @@
     </row>
   </sheetData>
   <autoFilter ref="B2:L77" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:L77">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="420200"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B36:L60">
       <sortCondition descending="1" ref="L2:L77"/>
     </sortState>
   </autoFilter>
@@ -7085,7 +7105,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:L14"/>
+  <dimension ref="B3:L15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -7125,85 +7145,85 @@
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
-        <v>431400</v>
+        <v>430100</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="G4" s="1">
+        <v>107</v>
+      </c>
+      <c r="H4" s="1">
         <v>111</v>
       </c>
-      <c r="H4" s="1">
-        <v>127</v>
-      </c>
       <c r="I4" s="1">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J4" s="1">
         <v>81</v>
       </c>
       <c r="K4" s="1">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="L4" s="1">
         <f>SUM(F4:K4)</f>
-        <v>539</v>
+        <v>495</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
-        <v>430100</v>
+        <v>432100</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G5" s="1">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H5" s="1">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="I5" s="1">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J5" s="1">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="K5" s="1">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L5" s="1">
         <f>SUM(F5:K5)</f>
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
-        <v>432100</v>
+        <v>431400</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1">
         <v>99</v>
@@ -7212,17 +7232,17 @@
         <v>115</v>
       </c>
       <c r="I6" s="1">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="J6" s="1">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K6" s="1">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L6" s="1">
         <f>SUM(F6:K6)</f>
-        <v>493</v>
+        <v>485</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -7363,81 +7383,121 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
-        <v>434100</v>
+        <v>433300</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>132</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G11" s="1">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H11" s="1">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I11" s="1">
         <v>61</v>
       </c>
       <c r="J11" s="1">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="K11" s="1">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L11" s="1">
         <f>SUM(F11:K11)</f>
-        <v>288</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="19">
+      <c r="B12" s="1">
         <v>433900</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="19" t="s">
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="1"/>
-      <c r="F12" s="19">
+      <c r="F12" s="1">
+        <v>22</v>
+      </c>
+      <c r="G12" s="1">
+        <v>52</v>
+      </c>
+      <c r="H12" s="1">
+        <v>45</v>
+      </c>
+      <c r="I12" s="1">
+        <v>50</v>
+      </c>
+      <c r="J12" s="1">
+        <v>35</v>
+      </c>
+      <c r="K12" s="1">
+        <v>35</v>
+      </c>
+      <c r="L12" s="1">
+        <f>SUM(F12:K12)</f>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <v>434100</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1">
+        <v>21</v>
+      </c>
+      <c r="G13" s="1">
+        <v>50</v>
+      </c>
+      <c r="H13" s="1">
+        <v>52</v>
+      </c>
+      <c r="I13" s="1">
+        <v>49</v>
+      </c>
+      <c r="J13" s="1">
+        <v>32</v>
+      </c>
+      <c r="K13" s="1">
         <v>30</v>
       </c>
-      <c r="G12" s="19">
-        <v>64</v>
-      </c>
-      <c r="H12" s="19">
-        <v>57</v>
-      </c>
-      <c r="I12" s="19">
-        <v>62</v>
-      </c>
-      <c r="J12" s="19">
-        <v>41</v>
-      </c>
-      <c r="K12" s="19">
-        <v>39</v>
-      </c>
-      <c r="L12" s="19">
-        <f>SUM(F12:K12)</f>
-        <v>293</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="I13" t="s">
-        <v>131</v>
+      <c r="L13" s="1">
+        <f>SUM(F13:K13)</f>
+        <v>234</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="L14">
+      <c r="B14" s="19">
+        <v>431000</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L15">
         <f>SUM(L4:L13)</f>
-        <v>3806</v>
+        <v>3941</v>
       </c>
     </row>
   </sheetData>
@@ -7639,14 +7699,14 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar web con nuevos datos de seed
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3966" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F53D0A4-CF49-4881-976E-0F8AE34AE6FB}"/>
+  <xr:revisionPtr revIDLastSave="4096" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{437C3FDC-339C-414F-A66D-383F4A9F321F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="135">
   <si>
     <t>CODIGO</t>
   </si>
@@ -450,6 +450,12 @@
   </si>
   <si>
     <t>ULTIMA ACTUALIZACION  9:57  27-05-2026</t>
+  </si>
+  <si>
+    <t>BURDEO</t>
+  </si>
+  <si>
+    <t>CAFÉ</t>
   </si>
 </sst>
 </file>
@@ -483,7 +489,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +510,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -585,7 +603,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -631,7 +649,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -648,14 +667,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
-</file>
-
-<file path=xl/namedSheetViews/namedSheetView2.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4853,7 +4864,7 @@
         <v>20</v>
       </c>
       <c r="L3" s="1">
-        <f>SUM(F3:K3)</f>
+        <f t="shared" ref="L3:L32" si="0">SUM(F3:K3)</f>
         <v>212</v>
       </c>
     </row>
@@ -4887,7 +4898,7 @@
         <v>8</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
+        <f t="shared" si="0"/>
         <v>142</v>
       </c>
     </row>
@@ -4921,7 +4932,7 @@
         <v>17</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
+        <f t="shared" si="0"/>
         <v>125</v>
       </c>
     </row>
@@ -4955,7 +4966,7 @@
         <v>11</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
+        <f t="shared" si="0"/>
         <v>121</v>
       </c>
       <c r="M6" t="s">
@@ -4995,7 +5006,7 @@
         <v>10</v>
       </c>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
@@ -5025,7 +5036,7 @@
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
     </row>
@@ -5057,7 +5068,7 @@
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
+        <f t="shared" si="0"/>
         <v>63</v>
       </c>
       <c r="N9" s="11"/>
@@ -5086,7 +5097,7 @@
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>62</v>
       </c>
       <c r="O10" t="s">
@@ -5119,7 +5130,7 @@
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
       <c r="O11" t="s">
@@ -5156,7 +5167,7 @@
         <v>6</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="N12" t="s">
@@ -5193,7 +5204,7 @@
         <v>12</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="O13" t="s">
@@ -5228,7 +5239,7 @@
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="O14" s="13" t="s">
@@ -5267,7 +5278,7 @@
         <v>4</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="N15" s="11"/>
@@ -5304,7 +5315,7 @@
         <v>5</v>
       </c>
       <c r="L16" s="1">
-        <f>SUM(F16:K16)</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
       <c r="O16" t="s">
@@ -5337,7 +5348,7 @@
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
     </row>
@@ -5369,7 +5380,7 @@
         <v>10</v>
       </c>
       <c r="L18" s="1">
-        <f>SUM(F18:K18)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
@@ -5403,7 +5414,7 @@
         <v>15</v>
       </c>
       <c r="L19" s="1">
-        <f>SUM(F19:K19)</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
@@ -5437,7 +5448,7 @@
         <v>7</v>
       </c>
       <c r="L20" s="1">
-        <f>SUM(F20:K20)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
@@ -5467,7 +5478,7 @@
         <v>9</v>
       </c>
       <c r="L21" s="1">
-        <f>SUM(F21:K21)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
@@ -5503,7 +5514,7 @@
         <v>0</v>
       </c>
       <c r="L22" s="1">
-        <f>SUM(F22:K22)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
@@ -5531,7 +5542,7 @@
       </c>
       <c r="K23" s="4"/>
       <c r="L23" s="1">
-        <f>SUM(F23:K23)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
@@ -5563,7 +5574,7 @@
       </c>
       <c r="K24" s="4"/>
       <c r="L24" s="1">
-        <f>SUM(F24:K24)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
@@ -5597,7 +5608,7 @@
         <v>1</v>
       </c>
       <c r="L25" s="1">
-        <f>SUM(F25:K25)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
@@ -5629,7 +5640,7 @@
         <v>11</v>
       </c>
       <c r="L26" s="1">
-        <f>SUM(F26:K26)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="M26" t="s">
@@ -5660,7 +5671,7 @@
         <v>24</v>
       </c>
       <c r="L27" s="1">
-        <f>SUM(F27:K27)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
@@ -5692,7 +5703,7 @@
         <v>2</v>
       </c>
       <c r="L28" s="1">
-        <f>SUM(F28:K28)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
@@ -5726,7 +5737,7 @@
         <v>1</v>
       </c>
       <c r="L29" s="1">
-        <f>SUM(F29:K29)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
@@ -5752,7 +5763,7 @@
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="1">
-        <f>SUM(F30:K30)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
@@ -5786,7 +5797,7 @@
         <v>2</v>
       </c>
       <c r="L31" s="1">
-        <f>SUM(F31:K31)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
@@ -5822,7 +5833,7 @@
         <v>3</v>
       </c>
       <c r="L32" s="1">
-        <f>SUM(F32:K32)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
@@ -5882,7 +5893,7 @@
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="1">
-        <f>SUM(F34:K34)</f>
+        <f t="shared" ref="L34:L56" si="1">SUM(F34:K34)</f>
         <v>19</v>
       </c>
     </row>
@@ -5910,7 +5921,7 @@
       </c>
       <c r="K35" s="4"/>
       <c r="L35" s="1">
-        <f>SUM(F35:K35)</f>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
@@ -5938,7 +5949,7 @@
         <v>10</v>
       </c>
       <c r="L36" s="1">
-        <f>SUM(F36:K36)</f>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
@@ -5966,7 +5977,7 @@
       </c>
       <c r="K37" s="4"/>
       <c r="L37" s="1">
-        <f>SUM(F37:K37)</f>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
@@ -5992,7 +6003,7 @@
         <v>13</v>
       </c>
       <c r="L38" s="1">
-        <f>SUM(F38:K38)</f>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
     </row>
@@ -6020,7 +6031,7 @@
         <v>8</v>
       </c>
       <c r="L39" s="1">
-        <f>SUM(F39:K39)</f>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
     </row>
@@ -6044,7 +6055,7 @@
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="1">
-        <f>SUM(F40:K40)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
@@ -6070,7 +6081,7 @@
         <v>5</v>
       </c>
       <c r="L41" s="1">
-        <f>SUM(F41:K41)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
@@ -6100,7 +6111,7 @@
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="1">
-        <f>SUM(F42:K42)</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
@@ -6132,7 +6143,7 @@
         <v>6</v>
       </c>
       <c r="L43" s="1">
-        <f>SUM(F43:K43)</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
@@ -6162,7 +6173,7 @@
         <v>3</v>
       </c>
       <c r="L44" s="12">
-        <f>SUM(F44:K44)</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
@@ -6192,7 +6203,7 @@
         <v>5</v>
       </c>
       <c r="L45" s="1">
-        <f>SUM(F45:K45)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
@@ -6224,7 +6235,7 @@
         <v>2</v>
       </c>
       <c r="L46" s="1">
-        <f>SUM(F46:K46)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
@@ -6252,7 +6263,7 @@
         <v>7</v>
       </c>
       <c r="L47" s="1">
-        <f>SUM(F47:K47)</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
     </row>
@@ -6280,7 +6291,7 @@
         <v>1</v>
       </c>
       <c r="L48" s="1">
-        <f>SUM(F48:K48)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -6308,7 +6319,7 @@
       </c>
       <c r="K49" s="4"/>
       <c r="L49" s="1">
-        <f>SUM(F49:K49)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -6336,7 +6347,7 @@
         <v>4</v>
       </c>
       <c r="L50" s="1">
-        <f>SUM(F50:K50)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -6364,7 +6375,7 @@
         <v>1</v>
       </c>
       <c r="L51" s="1">
-        <f>SUM(F51:K51)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -6392,7 +6403,7 @@
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="1">
-        <f>SUM(F52:K52)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -6426,7 +6437,7 @@
         <v>1</v>
       </c>
       <c r="L53" s="12">
-        <f>SUM(F53:K53)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -6456,7 +6467,7 @@
       </c>
       <c r="K54" s="4"/>
       <c r="L54" s="1">
-        <f>SUM(F54:K54)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
@@ -6484,7 +6495,7 @@
         <v>1</v>
       </c>
       <c r="L55" s="1">
-        <f>SUM(F55:K55)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
     </row>
@@ -6510,7 +6521,7 @@
       </c>
       <c r="K56" s="4"/>
       <c r="L56" s="1">
-        <f>SUM(F56:K56)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
@@ -6571,7 +6582,7 @@
       </c>
       <c r="K58" s="4"/>
       <c r="L58" s="1">
-        <f>SUM(F58:K58)</f>
+        <f t="shared" ref="L58:L74" si="2">SUM(F58:K58)</f>
         <v>5</v>
       </c>
       <c r="P58" t="s">
@@ -6598,7 +6609,7 @@
       </c>
       <c r="K59" s="4"/>
       <c r="L59" s="1">
-        <f>SUM(F59:K59)</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
@@ -6622,7 +6633,7 @@
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="1">
-        <f>SUM(F60:K60)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
@@ -6646,7 +6657,7 @@
         <v>3</v>
       </c>
       <c r="L61" s="1">
-        <f>SUM(F61:K61)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
@@ -6674,7 +6685,7 @@
       <c r="J62" s="4"/>
       <c r="K62" s="4"/>
       <c r="L62" s="1">
-        <f>SUM(F62:K62)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
@@ -6700,7 +6711,7 @@
       <c r="J63" s="4"/>
       <c r="K63" s="4"/>
       <c r="L63" s="1">
-        <f>SUM(F63:K63)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
@@ -6724,7 +6735,7 @@
       <c r="J64" s="4"/>
       <c r="K64" s="4"/>
       <c r="L64" s="1">
-        <f>SUM(F64:K64)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
@@ -6748,7 +6759,7 @@
       </c>
       <c r="K65" s="6"/>
       <c r="L65" s="1">
-        <f>SUM(F65:K65)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
@@ -6770,7 +6781,7 @@
       <c r="J66" s="4"/>
       <c r="K66" s="4"/>
       <c r="L66" s="1">
-        <f>SUM(F66:K66)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6792,7 +6803,7 @@
       <c r="J67" s="4"/>
       <c r="K67" s="4"/>
       <c r="L67" s="1">
-        <f>SUM(F67:K67)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6814,7 +6825,7 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="1">
-        <f>SUM(F68:K68)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6836,7 +6847,7 @@
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
       <c r="L69" s="1">
-        <f>SUM(F69:K69)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6858,7 +6869,7 @@
       <c r="J70" s="6"/>
       <c r="K70" s="6"/>
       <c r="L70" s="12">
-        <f>SUM(F70:K70)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6880,7 +6891,7 @@
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
       <c r="L71" s="1">
-        <f>SUM(F71:K71)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6904,7 +6915,7 @@
       <c r="J72" s="6"/>
       <c r="K72" s="6"/>
       <c r="L72" s="1">
-        <f>SUM(F72:K72)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6926,7 +6937,7 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="1">
-        <f>SUM(F73:K73)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6948,7 +6959,7 @@
       <c r="J74" s="4"/>
       <c r="K74" s="4"/>
       <c r="L74" s="1">
-        <f>SUM(F74:K74)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7044,7 +7055,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:L19"/>
+  <dimension ref="B3:L21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -7094,7 +7105,7 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G4" s="1">
         <v>102</v>
@@ -7112,12 +7123,12 @@
         <v>56</v>
       </c>
       <c r="L4" s="1">
-        <f>SUM(F4:K4)</f>
-        <v>473</v>
+        <f t="shared" ref="L4:L19" si="0">SUM(F4:K4)</f>
+        <v>472</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="1">
+      <c r="B5" s="19">
         <v>432100</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -7128,7 +7139,7 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G5" s="1">
         <v>94</v>
@@ -7146,8 +7157,8 @@
         <v>57</v>
       </c>
       <c r="L5" s="1">
-        <f>SUM(F5:K5)</f>
-        <v>454</v>
+        <f t="shared" si="0"/>
+        <v>453</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
@@ -7162,26 +7173,26 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G6" s="1">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H6" s="1">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I6" s="1">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="J6" s="1">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K6" s="1">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="L6" s="1">
-        <f>SUM(F6:K6)</f>
-        <v>453</v>
+        <f t="shared" si="0"/>
+        <v>464</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -7202,10 +7213,10 @@
         <v>94</v>
       </c>
       <c r="H7" s="1">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I7" s="1">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J7" s="1">
         <v>69</v>
@@ -7214,12 +7225,12 @@
         <v>52</v>
       </c>
       <c r="L7" s="1">
-        <f>SUM(F7:K7)</f>
-        <v>451</v>
+        <f t="shared" si="0"/>
+        <v>445</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="1">
+      <c r="B8" s="19">
         <v>430900</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -7230,16 +7241,16 @@
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G8" s="1">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H8" s="1">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I8" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J8" s="1">
         <v>75</v>
@@ -7248,8 +7259,8 @@
         <v>44</v>
       </c>
       <c r="L8" s="1">
-        <f>SUM(F8:K8)</f>
-        <v>420</v>
+        <f t="shared" si="0"/>
+        <v>410</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -7276,14 +7287,14 @@
         <v>86</v>
       </c>
       <c r="J9" s="1">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K9" s="1">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="L9" s="1">
-        <f>SUM(F9:K9)</f>
-        <v>415</v>
+        <f t="shared" si="0"/>
+        <v>411</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -7316,12 +7327,12 @@
         <v>38</v>
       </c>
       <c r="L10" s="1">
-        <f>SUM(F10:K10)</f>
+        <f t="shared" si="0"/>
         <v>331</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="1">
+      <c r="B11" s="19">
         <v>434100</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -7332,16 +7343,16 @@
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G11" s="1">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="H11" s="1">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="I11" s="1">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="J11" s="1">
         <v>31</v>
@@ -7350,12 +7361,12 @@
         <v>29</v>
       </c>
       <c r="L11" s="1">
-        <f>SUM(F11:K11)</f>
-        <v>218</v>
+        <f t="shared" si="0"/>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="1">
+      <c r="B12" s="19">
         <v>433300</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -7366,26 +7377,26 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="G12" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="H12" s="1">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="I12" s="1">
         <v>45</v>
       </c>
       <c r="J12" s="1">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="K12" s="1">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="L12" s="1">
-        <f>SUM(F12:K12)</f>
-        <v>215</v>
+        <f t="shared" si="0"/>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -7403,27 +7414,27 @@
         <v>7</v>
       </c>
       <c r="G13" s="1">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H13" s="1">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I13" s="1">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J13" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K13" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L13" s="1">
-        <f>SUM(F13:K13)</f>
-        <v>172</v>
+        <f t="shared" si="0"/>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="1">
+      <c r="B14" s="19">
         <v>435600</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -7434,30 +7445,30 @@
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G14" s="1">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H14" s="1">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="I14" s="1">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="J14" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K14" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L14" s="1">
-        <f>SUM(F14:K14)</f>
-        <v>129</v>
+        <f t="shared" si="0"/>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="1">
+      <c r="B15" s="19">
         <v>433900</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -7471,13 +7482,13 @@
         <v>4</v>
       </c>
       <c r="G15" s="1">
+        <v>17</v>
+      </c>
+      <c r="H15" s="1">
         <v>20</v>
       </c>
-      <c r="H15" s="1">
-        <v>23</v>
-      </c>
       <c r="I15" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J15" s="1">
         <v>22</v>
@@ -7486,78 +7497,154 @@
         <v>26</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(F15:K15)</f>
-        <v>124</v>
+        <f t="shared" si="0"/>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="19">
+      <c r="B16" s="20">
         <v>435601</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="C16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="19">
-        <v>3</v>
-      </c>
-      <c r="G16" s="19">
-        <v>30</v>
-      </c>
-      <c r="H16" s="19">
-        <v>3</v>
-      </c>
-      <c r="I16" s="19">
-        <v>23</v>
-      </c>
-      <c r="J16" s="19">
-        <v>22</v>
-      </c>
-      <c r="K16" s="19">
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>14</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>16</v>
+      </c>
+      <c r="J16" s="1">
+        <v>17</v>
+      </c>
+      <c r="K16" s="1">
         <v>21</v>
       </c>
-      <c r="L16" s="19">
-        <f>SUM(F16:K16)</f>
-        <v>102</v>
+      <c r="L16" s="1">
+        <f t="shared" si="0"/>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
+        <v>436104</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" s="1">
+        <v>26</v>
+      </c>
+      <c r="G17" s="1">
+        <v>50</v>
+      </c>
+      <c r="H17" s="1">
+        <v>52</v>
+      </c>
+      <c r="I17" s="1">
+        <v>47</v>
+      </c>
+      <c r="J17" s="1">
+        <v>41</v>
+      </c>
+      <c r="K17" s="1">
+        <v>27</v>
+      </c>
+      <c r="L17" s="1">
+        <f t="shared" si="0"/>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="1">
+        <v>436148</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="1">
+        <v>7</v>
+      </c>
+      <c r="G18" s="1">
+        <v>16</v>
+      </c>
+      <c r="H18" s="1">
+        <v>22</v>
+      </c>
+      <c r="I18" s="1">
+        <v>21</v>
+      </c>
+      <c r="J18" s="1">
+        <v>9</v>
+      </c>
+      <c r="K18" s="1">
+        <v>8</v>
+      </c>
+      <c r="L18" s="1">
+        <f t="shared" si="0"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="19">
         <v>431300</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1">
-        <v>1</v>
-      </c>
-      <c r="H17" s="1">
-        <v>12</v>
-      </c>
-      <c r="I17" s="1">
-        <v>3</v>
-      </c>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1">
-        <v>3</v>
-      </c>
-      <c r="L17" s="1">
-        <f>SUM(F17:K17)</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="L19">
-        <f>SUM(L4:L18)</f>
-        <v>3976</v>
+      <c r="C19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <f>SUM(L4:L20)</f>
+        <v>4047</v>
       </c>
     </row>
   </sheetData>
@@ -7571,12 +7658,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -7585,7 +7666,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -7729,23 +7810,13 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -7753,7 +7824,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7769,4 +7840,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar pedidos, stock y trazabilidad
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4096" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{437C3FDC-339C-414F-A66D-383F4A9F321F}"/>
+  <xr:revisionPtr revIDLastSave="4242" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A26F9DA4-83EA-4D95-BC9C-13DA87DE479D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -489,7 +489,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -521,6 +521,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -603,7 +609,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -649,8 +655,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4914,26 +4925,26 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="4">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G5" s="4">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H5" s="4">
+        <v>16</v>
+      </c>
+      <c r="I5" s="4">
         <v>17</v>
       </c>
-      <c r="I5" s="4">
-        <v>18</v>
-      </c>
       <c r="J5" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K5" s="4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L5" s="1">
         <f t="shared" si="0"/>
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
@@ -4954,7 +4965,7 @@
         <v>27</v>
       </c>
       <c r="H6" s="4">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="I6" s="4">
         <v>28</v>
@@ -4967,7 +4978,7 @@
       </c>
       <c r="L6" s="1">
         <f t="shared" si="0"/>
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="M6" t="s">
         <v>123</v>
@@ -5464,22 +5475,22 @@
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J21" s="4">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K21" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L21" s="1">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
@@ -7020,7 +7031,7 @@
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="L79" s="10">
         <f>SUM(L3:L78)</f>
-        <v>2105</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="83" spans="7:15" x14ac:dyDescent="0.25">
@@ -7055,11 +7066,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:L21"/>
+  <dimension ref="A3:L21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" style="22"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -7093,8 +7107,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="1">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="19">
         <v>430100</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -7127,7 +7141,8 @@
         <v>472</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="20"/>
       <c r="B5" s="19">
         <v>432100</v>
       </c>
@@ -7139,30 +7154,31 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H5" s="1">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I5" s="1">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J5" s="1">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K5" s="1">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L5" s="1">
         <f t="shared" si="0"/>
-        <v>453</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="1">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="20"/>
+      <c r="B6" s="19">
         <v>431400</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -7173,30 +7189,30 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G6" s="1">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H6" s="1">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I6" s="1">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J6" s="1">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K6" s="1">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L6" s="1">
         <f t="shared" si="0"/>
-        <v>464</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="1">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="19">
         <v>432300</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -7229,7 +7245,8 @@
         <v>445</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
       <c r="B8" s="19">
         <v>430900</v>
       </c>
@@ -7241,30 +7258,31 @@
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G8" s="1">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H8" s="1">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="I8" s="1">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J8" s="1">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K8" s="1">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" si="0"/>
-        <v>410</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="1">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="19">
         <v>432900</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -7275,30 +7293,31 @@
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G9" s="1">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="H9" s="1">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I9" s="1">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J9" s="1">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K9" s="1">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="0"/>
-        <v>411</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="1">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" s="19">
         <v>431800</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -7309,29 +7328,30 @@
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G10" s="1">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="H10" s="1">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="I10" s="1">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="J10" s="1">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="K10" s="1">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="0"/>
-        <v>331</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="20"/>
       <c r="B11" s="19">
         <v>434100</v>
       </c>
@@ -7343,29 +7363,30 @@
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G11" s="1">
+        <v>76</v>
+      </c>
+      <c r="H11" s="1">
         <v>22</v>
       </c>
-      <c r="H11" s="1">
-        <v>23</v>
-      </c>
       <c r="I11" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J11" s="1">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K11" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L11" s="1">
         <f t="shared" si="0"/>
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="20"/>
       <c r="B12" s="19">
         <v>433300</v>
       </c>
@@ -7380,7 +7401,7 @@
         <v>11</v>
       </c>
       <c r="G12" s="1">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="H12" s="1">
         <v>37</v>
@@ -7396,11 +7417,11 @@
       </c>
       <c r="L12" s="1">
         <f t="shared" si="0"/>
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="1">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="19">
         <v>431000</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -7414,7 +7435,7 @@
         <v>7</v>
       </c>
       <c r="G13" s="1">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="H13" s="1">
         <v>39</v>
@@ -7430,10 +7451,11 @@
       </c>
       <c r="L13" s="1">
         <f t="shared" si="0"/>
-        <v>165</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="20"/>
       <c r="B14" s="19">
         <v>435600</v>
       </c>
@@ -7445,29 +7467,30 @@
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G14" s="1">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="H14" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I14" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J14" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K14" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L14" s="1">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="20"/>
       <c r="B15" s="19">
         <v>433900</v>
       </c>
@@ -7482,7 +7505,7 @@
         <v>4</v>
       </c>
       <c r="G15" s="1">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="H15" s="1">
         <v>20</v>
@@ -7498,11 +7521,11 @@
       </c>
       <c r="L15" s="1">
         <f t="shared" si="0"/>
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="20">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="19">
         <v>435601</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -7516,7 +7539,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H16" s="1">
         <v>0</v>
@@ -7532,11 +7555,12 @@
       </c>
       <c r="L16" s="1">
         <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="1">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="23"/>
+      <c r="B17" s="19">
         <v>436104</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -7549,30 +7573,30 @@
         <v>134</v>
       </c>
       <c r="F17" s="1">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="G17" s="1">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="H17" s="1">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="I17" s="1">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="J17" s="1">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="K17" s="1">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="L17" s="1">
         <f t="shared" si="0"/>
-        <v>243</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="1">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="19">
         <v>436148</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -7585,29 +7609,30 @@
         <v>133</v>
       </c>
       <c r="F18" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G18" s="1">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="H18" s="1">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="I18" s="1">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="J18" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K18" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L18" s="1">
         <f t="shared" si="0"/>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="20"/>
       <c r="B19" s="19">
         <v>431300</v>
       </c>
@@ -7622,7 +7647,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="1">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="H19" s="1">
         <v>0</v>
@@ -7638,13 +7663,13 @@
       </c>
       <c r="L19" s="1">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L21">
         <f>SUM(L4:L20)</f>
-        <v>4047</v>
+        <v>4078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar data web y corregir filtro de venta despacho
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4284" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E61F79E6-3C48-4327-9ADB-2A70172EAA85}"/>
+  <xr:revisionPtr revIDLastSave="4404" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBF294DC-7CF7-43C8-BF0B-D7E99D6FAB29}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="5" activeTab="4" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView minimized="1" xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7875" firstSheet="6" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="135">
   <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
@@ -651,11 +651,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -677,6 +673,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
@@ -1055,7 +1057,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="26" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28"/>
@@ -1854,7 +1856,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="26" t="s">
         <v>43</v>
       </c>
       <c r="C3" s="28"/>
@@ -2461,7 +2463,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="26" t="s">
         <v>44</v>
       </c>
       <c r="C3" s="28"/>
@@ -2831,7 +2833,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="26" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="28"/>
@@ -4424,7 +4426,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="26" t="s">
         <v>109</v>
       </c>
       <c r="C3" s="28"/>
@@ -4557,20 +4559,20 @@
         <v>0</v>
       </c>
       <c r="H7" s="4">
+        <v>3</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4">
         <v>4</v>
       </c>
-      <c r="I7" s="4">
-        <v>3</v>
-      </c>
-      <c r="J7" s="4">
-        <v>13</v>
-      </c>
       <c r="K7" s="4">
         <v>0</v>
       </c>
       <c r="L7" s="4">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:12">
@@ -4659,20 +4661,20 @@
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" s="4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J10" s="4">
         <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:12">
@@ -4788,25 +4790,25 @@
         <v>8</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="1">
+      <c r="F14" s="27">
         <v>0</v>
       </c>
       <c r="G14" s="4">
         <v>0</v>
       </c>
-      <c r="H14" s="1">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1">
-        <v>0</v>
-      </c>
-      <c r="K14" s="1">
-        <v>0</v>
-      </c>
-      <c r="L14" s="1">
+      <c r="H14" s="27">
+        <v>0</v>
+      </c>
+      <c r="I14" s="27">
+        <v>0</v>
+      </c>
+      <c r="J14" s="27">
+        <v>0</v>
+      </c>
+      <c r="K14" s="27">
+        <v>0</v>
+      </c>
+      <c r="L14" s="27">
         <f>SUM(F14:K14)</f>
         <v>0</v>
       </c>
@@ -4834,172 +4836,172 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="25">
         <v>36</v>
       </c>
-      <c r="G2" s="27">
+      <c r="G2" s="25">
         <v>38</v>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="25">
         <v>40</v>
       </c>
-      <c r="I2" s="27">
+      <c r="I2" s="25">
         <v>42</v>
       </c>
-      <c r="J2" s="27">
+      <c r="J2" s="25">
         <v>44</v>
       </c>
-      <c r="K2" s="27">
+      <c r="K2" s="25">
         <v>46</v>
       </c>
-      <c r="L2" s="26" t="s">
+      <c r="L2" s="24" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="2:15">
-      <c r="B3" s="20">
+      <c r="B3" s="18">
         <v>422200</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="21"/>
-      <c r="F3" s="22">
+      <c r="E3" s="19"/>
+      <c r="F3" s="20">
         <v>14</v>
       </c>
-      <c r="G3" s="22">
+      <c r="G3" s="20">
         <v>51</v>
       </c>
-      <c r="H3" s="22">
+      <c r="H3" s="20">
         <v>46</v>
       </c>
-      <c r="I3" s="22">
+      <c r="I3" s="20">
         <v>51</v>
       </c>
-      <c r="J3" s="22">
+      <c r="J3" s="20">
         <v>30</v>
       </c>
-      <c r="K3" s="22">
+      <c r="K3" s="20">
         <v>20</v>
       </c>
-      <c r="L3" s="21">
+      <c r="L3" s="19">
         <f t="shared" ref="L3:L32" si="0">SUM(F3:K3)</f>
         <v>212</v>
       </c>
     </row>
     <row r="4" spans="2:15">
-      <c r="B4" s="23">
+      <c r="B4" s="21">
         <v>420301</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="21"/>
-      <c r="F4" s="23">
+      <c r="E4" s="19"/>
+      <c r="F4" s="21">
         <v>14</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="21">
         <v>32</v>
       </c>
-      <c r="H4" s="23">
+      <c r="H4" s="21">
         <v>34</v>
       </c>
-      <c r="I4" s="23">
+      <c r="I4" s="21">
         <v>26</v>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="21">
         <v>28</v>
       </c>
-      <c r="K4" s="23">
+      <c r="K4" s="21">
         <v>8</v>
       </c>
-      <c r="L4" s="21">
+      <c r="L4" s="19">
         <f t="shared" si="0"/>
         <v>142</v>
       </c>
     </row>
     <row r="5" spans="2:15">
-      <c r="B5" s="20">
+      <c r="B5" s="18">
         <v>423600</v>
       </c>
-      <c r="C5" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="C5" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22">
+      <c r="E5" s="19"/>
+      <c r="F5" s="20">
         <v>23</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="20">
         <v>37</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="20">
         <v>16</v>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="20">
         <v>17</v>
       </c>
-      <c r="J5" s="22">
+      <c r="J5" s="20">
         <v>10</v>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="20">
         <v>16</v>
       </c>
-      <c r="L5" s="21">
+      <c r="L5" s="19">
         <f t="shared" si="0"/>
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="20">
+      <c r="B6" s="18">
         <v>423500</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="21" t="s">
+      <c r="C6" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="22">
+      <c r="E6" s="19"/>
+      <c r="F6" s="20">
         <v>8</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="20">
         <v>26</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="20">
         <v>20</v>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="20">
         <v>27</v>
       </c>
-      <c r="J6" s="22">
+      <c r="J6" s="20">
         <v>20</v>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="20">
         <v>11</v>
       </c>
-      <c r="L6" s="21">
+      <c r="L6" s="19">
         <f t="shared" si="0"/>
         <v>112</v>
       </c>
@@ -5011,127 +5013,126 @@
       </c>
     </row>
     <row r="7" spans="2:15">
-      <c r="B7" s="20">
+      <c r="B7" s="18">
         <v>421000</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="23">
+      <c r="E7" s="19"/>
+      <c r="F7" s="21">
         <v>5</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="21">
         <v>15</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="21">
         <v>15</v>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="21">
         <v>15</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="21">
         <v>10</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="21">
         <v>10</v>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="19">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="23">
+      <c r="B8" s="21">
         <v>422800</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="21"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22">
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20">
         <v>6</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="20">
         <v>31</v>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="20">
         <v>1</v>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="20">
         <v>28</v>
       </c>
-      <c r="K8" s="22"/>
-      <c r="L8" s="21">
+      <c r="K8" s="20"/>
+      <c r="L8" s="19">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
     </row>
     <row r="9" spans="2:15">
-      <c r="B9" s="23">
+      <c r="B9" s="21">
         <v>422000</v>
       </c>
-      <c r="C9" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="21" t="s">
+      <c r="C9" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="22">
+      <c r="E9" s="19"/>
+      <c r="F9" s="20">
         <v>35</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="20">
         <v>9</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="20">
         <v>12</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="20">
         <v>4</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="20">
         <v>3</v>
       </c>
-      <c r="K9" s="22"/>
-      <c r="L9" s="21">
+      <c r="K9" s="20"/>
+      <c r="L9" s="19">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="M9" s="18"/>
-      <c r="N9" s="19"/>
+      <c r="N9" s="17"/>
     </row>
     <row r="10" spans="2:15">
-      <c r="B10" s="20">
+      <c r="B10" s="18">
         <v>424400</v>
       </c>
-      <c r="C10" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="21" t="s">
+      <c r="C10" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="22">
+      <c r="E10" s="19"/>
+      <c r="F10" s="20">
         <v>16</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="20">
         <v>10</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="20">
         <v>36</v>
       </c>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="21">
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="19">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
@@ -5140,31 +5141,31 @@
       </c>
     </row>
     <row r="11" spans="2:15">
-      <c r="B11" s="20">
+      <c r="B11" s="18">
         <v>420100</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="21" t="s">
+      <c r="C11" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="22">
+      <c r="E11" s="19"/>
+      <c r="F11" s="20">
         <v>15</v>
       </c>
-      <c r="G11" s="22">
-        <v>7</v>
-      </c>
-      <c r="H11" s="22">
+      <c r="G11" s="20">
+        <v>7</v>
+      </c>
+      <c r="H11" s="20">
         <v>36</v>
       </c>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22">
+      <c r="I11" s="20"/>
+      <c r="J11" s="20">
         <v>1</v>
       </c>
-      <c r="K11" s="22"/>
-      <c r="L11" s="21">
+      <c r="K11" s="20"/>
+      <c r="L11" s="19">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
@@ -5173,35 +5174,35 @@
       </c>
     </row>
     <row r="12" spans="2:15">
-      <c r="B12" s="23">
+      <c r="B12" s="21">
         <v>420800</v>
       </c>
-      <c r="C12" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="21" t="s">
+      <c r="C12" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="21"/>
-      <c r="F12" s="23">
+      <c r="E12" s="19"/>
+      <c r="F12" s="21">
         <v>6</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="21">
         <v>11</v>
       </c>
-      <c r="H12" s="23">
+      <c r="H12" s="21">
         <v>14</v>
       </c>
-      <c r="I12" s="23">
+      <c r="I12" s="21">
         <v>13</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="21">
         <v>6</v>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="20">
         <v>6</v>
       </c>
-      <c r="L12" s="21">
+      <c r="L12" s="19">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
@@ -5210,35 +5211,35 @@
       </c>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="20">
+      <c r="B13" s="18">
         <v>420400</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22">
+      <c r="E13" s="19"/>
+      <c r="F13" s="20">
         <v>25</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="20">
         <v>4</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="20">
         <v>5</v>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="20">
         <v>4</v>
       </c>
-      <c r="J13" s="22">
+      <c r="J13" s="20">
         <v>5</v>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="20">
         <v>12</v>
       </c>
-      <c r="L13" s="21">
+      <c r="L13" s="19">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
@@ -5247,33 +5248,33 @@
       </c>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="23">
+      <c r="B14" s="21">
         <v>422101</v>
       </c>
-      <c r="C14" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="21" t="s">
+      <c r="C14" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="21"/>
-      <c r="F14" s="22">
+      <c r="E14" s="19"/>
+      <c r="F14" s="20">
         <v>14</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="20">
         <v>1</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="20">
         <v>14</v>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="20">
         <v>9</v>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="20">
         <v>14</v>
       </c>
-      <c r="K14" s="22"/>
-      <c r="L14" s="21">
+      <c r="K14" s="20"/>
+      <c r="L14" s="19">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
@@ -5282,75 +5283,74 @@
       </c>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="20">
+      <c r="B15" s="18">
         <v>424900</v>
       </c>
-      <c r="C15" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="21" t="s">
+      <c r="C15" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="20">
         <v>9</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="20">
         <v>14</v>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="21">
         <v>15</v>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="20">
         <v>6</v>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="20">
         <v>4</v>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="20">
         <v>4</v>
       </c>
-      <c r="L15" s="21">
+      <c r="L15" s="19">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="M15" s="18"/>
-      <c r="N15" s="19"/>
+      <c r="N15" s="17"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="23">
+      <c r="B16" s="21">
         <v>420160</v>
       </c>
-      <c r="C16" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="21" t="s">
+      <c r="C16" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="F16" s="22">
-        <v>7</v>
-      </c>
-      <c r="G16" s="22">
+      <c r="F16" s="20">
+        <v>7</v>
+      </c>
+      <c r="G16" s="20">
         <v>12</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="20">
         <v>9</v>
       </c>
-      <c r="I16" s="22">
+      <c r="I16" s="20">
         <v>10</v>
       </c>
-      <c r="J16" s="22">
+      <c r="J16" s="20">
         <v>6</v>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="20">
         <v>5</v>
       </c>
-      <c r="L16" s="21">
+      <c r="L16" s="19">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
@@ -5359,323 +5359,323 @@
       </c>
     </row>
     <row r="17" spans="2:13">
-      <c r="B17" s="23">
+      <c r="B17" s="21">
         <v>424600</v>
       </c>
-      <c r="C17" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="21" t="s">
+      <c r="C17" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="21"/>
-      <c r="F17" s="22">
+      <c r="E17" s="19"/>
+      <c r="F17" s="20">
         <v>3</v>
       </c>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22">
+      <c r="G17" s="20"/>
+      <c r="H17" s="20">
         <v>18</v>
       </c>
-      <c r="I17" s="22">
+      <c r="I17" s="20">
         <v>13</v>
       </c>
-      <c r="J17" s="22">
+      <c r="J17" s="20">
         <v>14</v>
       </c>
-      <c r="K17" s="22"/>
-      <c r="L17" s="21">
+      <c r="K17" s="20"/>
+      <c r="L17" s="19">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
     </row>
     <row r="18" spans="2:13">
-      <c r="B18" s="23">
+      <c r="B18" s="21">
         <v>422700</v>
       </c>
-      <c r="C18" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="21" t="s">
+      <c r="C18" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="21"/>
-      <c r="F18" s="22">
+      <c r="E18" s="19"/>
+      <c r="F18" s="20">
         <v>10</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18" s="20">
         <v>14</v>
       </c>
-      <c r="H18" s="22">
+      <c r="H18" s="20">
         <v>6</v>
       </c>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22">
+      <c r="I18" s="20"/>
+      <c r="J18" s="20">
         <v>6</v>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="20">
         <v>10</v>
       </c>
-      <c r="L18" s="21">
+      <c r="L18" s="19">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
     <row r="19" spans="2:13">
-      <c r="B19" s="23">
+      <c r="B19" s="21">
         <v>422701</v>
       </c>
-      <c r="C19" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="21" t="s">
+      <c r="C19" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="21"/>
-      <c r="F19" s="22">
+      <c r="E19" s="19"/>
+      <c r="F19" s="20">
         <v>4</v>
       </c>
-      <c r="G19" s="22">
+      <c r="G19" s="20">
         <v>3</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="20">
         <v>3</v>
       </c>
-      <c r="I19" s="22">
-        <v>7</v>
-      </c>
-      <c r="J19" s="22">
+      <c r="I19" s="20">
+        <v>7</v>
+      </c>
+      <c r="J19" s="20">
         <v>13</v>
       </c>
-      <c r="K19" s="22">
+      <c r="K19" s="20">
         <v>15</v>
       </c>
-      <c r="L19" s="21">
+      <c r="L19" s="19">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
     <row r="20" spans="2:13">
-      <c r="B20" s="23">
+      <c r="B20" s="21">
         <v>421100</v>
       </c>
-      <c r="C20" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="21" t="s">
+      <c r="C20" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="21"/>
-      <c r="F20" s="22">
+      <c r="E20" s="19"/>
+      <c r="F20" s="20">
         <v>2</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="20">
         <v>3</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="20">
         <v>5</v>
       </c>
-      <c r="I20" s="22">
-        <v>7</v>
-      </c>
-      <c r="J20" s="22">
+      <c r="I20" s="20">
+        <v>7</v>
+      </c>
+      <c r="J20" s="20">
         <v>20</v>
       </c>
-      <c r="K20" s="22">
-        <v>7</v>
-      </c>
-      <c r="L20" s="21">
+      <c r="K20" s="20">
+        <v>7</v>
+      </c>
+      <c r="L20" s="19">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
     <row r="21" spans="2:13">
-      <c r="B21" s="20">
+      <c r="B21" s="18">
         <v>423000</v>
       </c>
-      <c r="C21" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="21" t="s">
+      <c r="C21" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="22">
+      <c r="E21" s="19"/>
+      <c r="F21" s="20">
         <v>9</v>
       </c>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22">
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20">
         <v>3</v>
       </c>
-      <c r="J21" s="22">
+      <c r="J21" s="20">
         <v>20</v>
       </c>
-      <c r="K21" s="22">
+      <c r="K21" s="20">
         <v>8</v>
       </c>
-      <c r="L21" s="21">
+      <c r="L21" s="19">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
     </row>
     <row r="22" spans="2:13">
-      <c r="B22" s="23">
+      <c r="B22" s="21">
         <v>424900</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="21" t="s">
+      <c r="E22" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="F22" s="22">
+      <c r="F22" s="20">
         <v>4</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="20">
         <v>12</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="19">
         <v>13</v>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="20">
         <v>6</v>
       </c>
-      <c r="J22" s="22">
+      <c r="J22" s="20">
         <v>3</v>
       </c>
-      <c r="K22" s="22">
-        <v>0</v>
-      </c>
-      <c r="L22" s="21">
+      <c r="K22" s="20">
+        <v>0</v>
+      </c>
+      <c r="L22" s="19">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
     <row r="23" spans="2:13">
-      <c r="B23" s="23">
+      <c r="B23" s="21">
         <v>422900</v>
       </c>
-      <c r="C23" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="21" t="s">
+      <c r="C23" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="21"/>
-      <c r="F23" s="22">
+      <c r="E23" s="19"/>
+      <c r="F23" s="20">
         <v>35</v>
       </c>
-      <c r="G23" s="22">
+      <c r="G23" s="20">
         <v>1</v>
       </c>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22">
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20">
         <v>2</v>
       </c>
-      <c r="K23" s="22"/>
-      <c r="L23" s="21">
+      <c r="K23" s="20"/>
+      <c r="L23" s="19">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
     <row r="24" spans="2:13">
-      <c r="B24" s="20">
+      <c r="B24" s="18">
         <v>422500</v>
       </c>
-      <c r="C24" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="21" t="s">
+      <c r="C24" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E24" s="21"/>
-      <c r="F24" s="22">
+      <c r="E24" s="19"/>
+      <c r="F24" s="20">
         <v>8</v>
       </c>
-      <c r="G24" s="22">
+      <c r="G24" s="20">
         <v>2</v>
       </c>
-      <c r="H24" s="22">
+      <c r="H24" s="20">
         <v>4</v>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="20">
         <v>9</v>
       </c>
-      <c r="J24" s="22">
+      <c r="J24" s="20">
         <v>11</v>
       </c>
-      <c r="K24" s="22"/>
-      <c r="L24" s="21">
+      <c r="K24" s="20"/>
+      <c r="L24" s="19">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
     <row r="25" spans="2:13">
-      <c r="B25" s="20">
+      <c r="B25" s="18">
         <v>424701</v>
       </c>
-      <c r="C25" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="21" t="s">
+      <c r="C25" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="21"/>
-      <c r="F25" s="22">
-        <v>2</v>
-      </c>
-      <c r="G25" s="22">
+      <c r="E25" s="19"/>
+      <c r="F25" s="20">
+        <v>0</v>
+      </c>
+      <c r="G25" s="20">
+        <v>0</v>
+      </c>
+      <c r="H25" s="20">
+        <v>7</v>
+      </c>
+      <c r="I25" s="20">
+        <v>0</v>
+      </c>
+      <c r="J25" s="20">
+        <v>10</v>
+      </c>
+      <c r="K25" s="20">
         <v>1</v>
       </c>
-      <c r="H25" s="22">
-        <v>13</v>
-      </c>
-      <c r="I25" s="22">
+      <c r="L25" s="19">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13">
+      <c r="B26" s="21">
+        <v>421801</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20">
         <v>1</v>
       </c>
-      <c r="J25" s="22">
-        <v>16</v>
-      </c>
-      <c r="K25" s="22">
-        <v>1</v>
-      </c>
-      <c r="L25" s="21">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13">
-      <c r="B26" s="23">
-        <v>421801</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="21" t="s">
+      <c r="H26" s="20">
+        <v>4</v>
+      </c>
+      <c r="I26" s="20">
+        <v>4</v>
+      </c>
+      <c r="J26" s="20">
         <v>12</v>
       </c>
-      <c r="E26" s="21"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22">
-        <v>1</v>
-      </c>
-      <c r="H26" s="22">
-        <v>4</v>
-      </c>
-      <c r="I26" s="22">
-        <v>4</v>
-      </c>
-      <c r="J26" s="22">
-        <v>12</v>
-      </c>
-      <c r="K26" s="22">
+      <c r="K26" s="20">
         <v>11</v>
       </c>
-      <c r="L26" s="21">
+      <c r="L26" s="19">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
@@ -5684,902 +5684,1026 @@
       </c>
     </row>
     <row r="27" spans="2:13">
-      <c r="B27" s="20">
+      <c r="B27" s="18">
         <v>421400</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="21" t="s">
+      <c r="C27" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="21"/>
-      <c r="F27" s="22">
-        <v>7</v>
-      </c>
-      <c r="G27" s="22">
-        <v>0</v>
-      </c>
-      <c r="H27" s="22">
-        <v>0</v>
-      </c>
-      <c r="I27" s="22">
-        <v>0</v>
-      </c>
-      <c r="J27" s="22">
-        <v>0</v>
-      </c>
-      <c r="K27" s="22">
-        <v>24</v>
-      </c>
-      <c r="L27" s="21">
-        <f t="shared" si="0"/>
-        <v>31</v>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20">
+        <v>4</v>
+      </c>
+      <c r="G27" s="20">
+        <v>0</v>
+      </c>
+      <c r="H27" s="20">
+        <v>0</v>
+      </c>
+      <c r="I27" s="20">
+        <v>0</v>
+      </c>
+      <c r="J27" s="20">
+        <v>0</v>
+      </c>
+      <c r="K27" s="20">
+        <v>18</v>
+      </c>
+      <c r="L27" s="19">
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="2:13">
-      <c r="B28" s="23">
+      <c r="B28" s="21">
         <v>420101</v>
       </c>
-      <c r="C28" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="21" t="s">
+      <c r="C28" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E28" s="21"/>
-      <c r="F28" s="22">
-        <v>7</v>
-      </c>
-      <c r="G28" s="22">
-        <v>7</v>
-      </c>
-      <c r="H28" s="22">
-        <v>7</v>
-      </c>
-      <c r="I28" s="22">
-        <v>7</v>
-      </c>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22">
+      <c r="E28" s="19"/>
+      <c r="F28" s="20">
+        <v>7</v>
+      </c>
+      <c r="G28" s="20">
+        <v>7</v>
+      </c>
+      <c r="H28" s="20">
+        <v>7</v>
+      </c>
+      <c r="I28" s="20">
+        <v>7</v>
+      </c>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20">
         <v>2</v>
       </c>
-      <c r="L28" s="21">
+      <c r="L28" s="19">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
     <row r="29" spans="2:13">
-      <c r="B29" s="23">
+      <c r="B29" s="21">
         <v>421901</v>
       </c>
-      <c r="C29" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="21" t="s">
+      <c r="C29" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E29" s="21"/>
-      <c r="F29" s="22">
+      <c r="E29" s="19"/>
+      <c r="F29" s="20">
         <v>4</v>
       </c>
-      <c r="G29" s="22">
+      <c r="G29" s="20">
         <v>8</v>
       </c>
-      <c r="H29" s="22">
+      <c r="H29" s="20">
         <v>6</v>
       </c>
-      <c r="I29" s="22">
+      <c r="I29" s="20">
         <v>5</v>
       </c>
-      <c r="J29" s="22">
+      <c r="J29" s="20">
         <v>4</v>
       </c>
-      <c r="K29" s="22">
+      <c r="K29" s="20">
         <v>1</v>
       </c>
-      <c r="L29" s="21">
+      <c r="L29" s="19">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="2:13">
-      <c r="B30" s="23">
+      <c r="B30" s="21">
         <v>424000</v>
       </c>
-      <c r="C30" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="21" t="s">
+      <c r="C30" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E30" s="21"/>
-      <c r="F30" s="22">
-        <v>18</v>
-      </c>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22">
+      <c r="E30" s="19"/>
+      <c r="F30" s="20">
+        <v>10</v>
+      </c>
+      <c r="G30" s="20">
+        <v>0</v>
+      </c>
+      <c r="H30" s="20">
+        <v>0</v>
+      </c>
+      <c r="I30" s="20">
+        <v>0</v>
+      </c>
+      <c r="J30" s="20">
+        <v>0</v>
+      </c>
+      <c r="K30" s="20">
+        <v>0</v>
+      </c>
+      <c r="L30" s="19">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13">
+      <c r="B31" s="21">
+        <v>421902</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="K30" s="22"/>
-      <c r="L30" s="21">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="2:13">
-      <c r="B31" s="23">
-        <v>421902</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="E31" s="21"/>
-      <c r="F31" s="22">
+      <c r="E31" s="19"/>
+      <c r="F31" s="20">
         <v>2</v>
       </c>
-      <c r="G31" s="22">
+      <c r="G31" s="20">
         <v>6</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="20">
         <v>6</v>
       </c>
-      <c r="I31" s="22">
+      <c r="I31" s="20">
         <v>5</v>
       </c>
-      <c r="J31" s="22">
+      <c r="J31" s="20">
         <v>4</v>
       </c>
-      <c r="K31" s="22">
+      <c r="K31" s="20">
         <v>2</v>
       </c>
-      <c r="L31" s="21">
+      <c r="L31" s="19">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
     <row r="32" spans="2:13">
-      <c r="B32" s="23">
+      <c r="B32" s="21">
         <v>422190</v>
       </c>
-      <c r="C32" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="21" t="s">
+      <c r="C32" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="F32" s="22">
+      <c r="F32" s="20">
         <v>2</v>
       </c>
-      <c r="G32" s="22">
+      <c r="G32" s="20">
         <v>5</v>
       </c>
-      <c r="H32" s="23">
+      <c r="H32" s="21">
         <v>5</v>
       </c>
-      <c r="I32" s="22">
+      <c r="I32" s="20">
         <v>5</v>
       </c>
-      <c r="J32" s="22">
+      <c r="J32" s="20">
         <v>3</v>
       </c>
-      <c r="K32" s="22">
+      <c r="K32" s="20">
         <v>3</v>
       </c>
-      <c r="L32" s="21">
+      <c r="L32" s="19">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
     <row r="33" spans="2:12">
-      <c r="B33" s="23">
+      <c r="B33" s="21">
         <v>420802</v>
       </c>
-      <c r="C33" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="21" t="s">
+      <c r="C33" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="21"/>
-      <c r="F33" s="23">
+      <c r="E33" s="19"/>
+      <c r="F33" s="21">
         <v>1</v>
       </c>
-      <c r="G33" s="22">
+      <c r="G33" s="20">
         <v>5</v>
       </c>
-      <c r="H33" s="22">
+      <c r="H33" s="20">
         <v>5</v>
       </c>
-      <c r="I33" s="22">
+      <c r="I33" s="20">
         <v>5</v>
       </c>
-      <c r="J33" s="22">
+      <c r="J33" s="20">
         <v>3</v>
       </c>
-      <c r="K33" s="22">
+      <c r="K33" s="20">
         <v>3</v>
       </c>
-      <c r="L33" s="21">
+      <c r="L33" s="19">
         <f>SUM(G33:K33)</f>
         <v>21</v>
       </c>
     </row>
     <row r="34" spans="2:12">
-      <c r="B34" s="23">
+      <c r="B34" s="21">
         <v>420600</v>
       </c>
-      <c r="C34" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="21" t="s">
+      <c r="C34" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E34" s="21"/>
-      <c r="F34" s="22">
-        <v>17</v>
-      </c>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22">
-        <v>2</v>
-      </c>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="21">
+      <c r="E34" s="19"/>
+      <c r="F34" s="20">
+        <v>8</v>
+      </c>
+      <c r="G34" s="20">
+        <v>0</v>
+      </c>
+      <c r="H34" s="20">
+        <v>0</v>
+      </c>
+      <c r="I34" s="20">
+        <v>0</v>
+      </c>
+      <c r="J34" s="20">
+        <v>0</v>
+      </c>
+      <c r="K34" s="20">
+        <v>0</v>
+      </c>
+      <c r="L34" s="19">
         <f t="shared" ref="L34:L56" si="1">SUM(F34:K34)</f>
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="2:12">
-      <c r="B35" s="23">
+      <c r="B35" s="21">
         <v>424801</v>
       </c>
-      <c r="C35" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="21" t="s">
+      <c r="C35" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E35" s="21"/>
-      <c r="F35" s="22">
+      <c r="E35" s="19"/>
+      <c r="F35" s="20">
         <v>4</v>
       </c>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22">
+      <c r="G35" s="20">
+        <v>0</v>
+      </c>
+      <c r="H35" s="20">
         <v>10</v>
       </c>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22">
+      <c r="I35" s="20">
+        <v>0</v>
+      </c>
+      <c r="J35" s="20">
         <v>5</v>
       </c>
-      <c r="K35" s="22"/>
-      <c r="L35" s="21">
+      <c r="K35" s="20">
+        <v>0</v>
+      </c>
+      <c r="L35" s="19">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
     <row r="36" spans="2:12">
-      <c r="B36" s="23">
+      <c r="B36" s="21">
         <v>420900</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C36" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E36" s="21"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22">
+      <c r="E36" s="19"/>
+      <c r="F36" s="20">
+        <v>0</v>
+      </c>
+      <c r="G36" s="20">
         <v>5</v>
       </c>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22">
+      <c r="H36" s="20">
+        <v>0</v>
+      </c>
+      <c r="I36" s="20">
+        <v>0</v>
+      </c>
+      <c r="J36" s="20">
         <v>4</v>
       </c>
-      <c r="K36" s="22">
+      <c r="K36" s="20">
         <v>10</v>
       </c>
-      <c r="L36" s="21">
+      <c r="L36" s="19">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:12">
-      <c r="B37" s="23">
+      <c r="B37" s="21">
         <v>423900</v>
       </c>
-      <c r="C37" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="21" t="s">
+      <c r="C37" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E37" s="21"/>
-      <c r="F37" s="22">
+      <c r="E37" s="19"/>
+      <c r="F37" s="20">
         <v>2</v>
       </c>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22">
+      <c r="G37" s="20">
+        <v>0</v>
+      </c>
+      <c r="H37" s="20">
         <v>9</v>
       </c>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22">
-        <v>8</v>
-      </c>
-      <c r="K37" s="22"/>
-      <c r="L37" s="21">
+      <c r="I37" s="20">
+        <v>0</v>
+      </c>
+      <c r="J37" s="20">
+        <v>0</v>
+      </c>
+      <c r="K37" s="20">
+        <v>0</v>
+      </c>
+      <c r="L37" s="19">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" spans="2:12">
-      <c r="B38" s="23">
+      <c r="B38" s="21">
         <v>422100</v>
       </c>
-      <c r="C38" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38" s="21" t="s">
+      <c r="C38" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="21"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22">
+      <c r="E38" s="19"/>
+      <c r="F38" s="20">
+        <v>0</v>
+      </c>
+      <c r="G38" s="20">
+        <v>0</v>
+      </c>
+      <c r="H38" s="20">
+        <v>0</v>
+      </c>
+      <c r="I38" s="20">
+        <v>0</v>
+      </c>
+      <c r="J38" s="20">
         <v>5</v>
       </c>
-      <c r="K38" s="22">
+      <c r="K38" s="20">
         <v>13</v>
       </c>
-      <c r="L38" s="21">
+      <c r="L38" s="19">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
     </row>
     <row r="39" spans="2:12">
-      <c r="B39" s="23">
+      <c r="B39" s="21">
         <v>423200</v>
       </c>
-      <c r="C39" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="21" t="s">
+      <c r="C39" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E39" s="21"/>
-      <c r="F39" s="22">
+      <c r="E39" s="19"/>
+      <c r="F39" s="20">
+        <v>5</v>
+      </c>
+      <c r="G39" s="20">
+        <v>0</v>
+      </c>
+      <c r="H39" s="20">
+        <v>0</v>
+      </c>
+      <c r="I39" s="20">
+        <v>0</v>
+      </c>
+      <c r="J39" s="20">
+        <v>0</v>
+      </c>
+      <c r="K39" s="20">
         <v>8</v>
       </c>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22">
+      <c r="L39" s="19">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="2:12">
+      <c r="B40" s="21">
+        <v>422300</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20">
+        <v>8</v>
+      </c>
+      <c r="G40" s="20">
+        <v>0</v>
+      </c>
+      <c r="H40" s="20">
+        <v>0</v>
+      </c>
+      <c r="I40" s="20">
+        <v>0</v>
+      </c>
+      <c r="J40" s="20">
+        <v>0</v>
+      </c>
+      <c r="K40" s="20">
+        <v>0</v>
+      </c>
+      <c r="L40" s="19">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12">
+      <c r="B41" s="21">
+        <v>424700</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E41" s="19"/>
+      <c r="F41" s="20">
+        <v>9</v>
+      </c>
+      <c r="G41" s="20">
+        <v>0</v>
+      </c>
+      <c r="H41" s="20">
+        <v>0</v>
+      </c>
+      <c r="I41" s="20">
+        <v>0</v>
+      </c>
+      <c r="J41" s="20">
+        <v>0</v>
+      </c>
+      <c r="K41" s="20">
         <v>1</v>
       </c>
-      <c r="K39" s="22">
-        <v>8</v>
-      </c>
-      <c r="L39" s="21">
+      <c r="L41" s="19">
         <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="2:12">
-      <c r="B40" s="23">
-        <v>422300</v>
-      </c>
-      <c r="C40" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E40" s="21"/>
-      <c r="F40" s="22">
-        <v>16</v>
-      </c>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="21">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="2:12">
-      <c r="B41" s="23">
-        <v>424700</v>
-      </c>
-      <c r="C41" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E41" s="21"/>
-      <c r="F41" s="22">
-        <v>11</v>
-      </c>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22">
-        <v>5</v>
-      </c>
-      <c r="L41" s="21">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="2:12">
-      <c r="B42" s="23">
+      <c r="B42" s="21">
         <v>421301</v>
       </c>
-      <c r="C42" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="21" t="s">
+      <c r="C42" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E42" s="21"/>
-      <c r="F42" s="22">
+      <c r="E42" s="19"/>
+      <c r="F42" s="20">
         <v>3</v>
       </c>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22">
+      <c r="G42" s="20"/>
+      <c r="H42" s="20">
         <v>6</v>
       </c>
-      <c r="I42" s="22">
+      <c r="I42" s="20">
         <v>2</v>
       </c>
-      <c r="J42" s="22">
+      <c r="J42" s="20">
         <v>4</v>
       </c>
-      <c r="K42" s="22"/>
-      <c r="L42" s="21">
+      <c r="K42" s="20"/>
+      <c r="L42" s="19">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
     <row r="43" spans="2:12">
-      <c r="B43" s="23">
+      <c r="B43" s="21">
         <v>423501</v>
       </c>
-      <c r="C43" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="21" t="s">
+      <c r="C43" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E43" s="21"/>
-      <c r="F43" s="22">
+      <c r="E43" s="19"/>
+      <c r="F43" s="20">
         <v>2</v>
       </c>
-      <c r="G43" s="22">
+      <c r="G43" s="20">
         <v>3</v>
       </c>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22">
+      <c r="H43" s="20"/>
+      <c r="I43" s="20">
         <v>3</v>
       </c>
-      <c r="J43" s="22">
-        <v>0</v>
-      </c>
-      <c r="K43" s="22">
+      <c r="J43" s="20">
+        <v>0</v>
+      </c>
+      <c r="K43" s="20">
         <v>6</v>
       </c>
-      <c r="L43" s="21">
+      <c r="L43" s="19">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
     <row r="44" spans="2:12">
-      <c r="B44" s="23">
+      <c r="B44" s="21">
         <v>424200</v>
       </c>
-      <c r="C44" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" s="21" t="s">
+      <c r="C44" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E44" s="21"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23">
+      <c r="E44" s="19"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21">
         <v>1</v>
       </c>
-      <c r="H44" s="23"/>
-      <c r="I44" s="23">
+      <c r="H44" s="21"/>
+      <c r="I44" s="21">
         <v>9</v>
       </c>
-      <c r="J44" s="23">
+      <c r="J44" s="21">
         <v>1</v>
       </c>
-      <c r="K44" s="23">
+      <c r="K44" s="21">
         <v>3</v>
       </c>
-      <c r="L44" s="24">
+      <c r="L44" s="22">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
     <row r="45" spans="2:12">
-      <c r="B45" s="23">
+      <c r="B45" s="21">
         <v>424300</v>
       </c>
-      <c r="C45" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45" s="21" t="s">
+      <c r="C45" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E45" s="21"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22">
+      <c r="E45" s="19"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20">
         <v>4</v>
       </c>
-      <c r="H45" s="22">
+      <c r="H45" s="20">
         <v>2</v>
       </c>
-      <c r="I45" s="22">
+      <c r="I45" s="20">
         <v>2</v>
       </c>
-      <c r="J45" s="22"/>
-      <c r="K45" s="22">
+      <c r="J45" s="20"/>
+      <c r="K45" s="20">
         <v>5</v>
       </c>
-      <c r="L45" s="21">
+      <c r="L45" s="19">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
     <row r="46" spans="2:12">
-      <c r="B46" s="23">
+      <c r="B46" s="21">
         <v>421402</v>
       </c>
-      <c r="C46" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46" s="21" t="s">
+      <c r="C46" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E46" s="21"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22">
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20">
         <v>3</v>
       </c>
-      <c r="H46" s="22">
+      <c r="H46" s="20">
         <v>1</v>
       </c>
-      <c r="I46" s="22">
+      <c r="I46" s="20">
         <v>4</v>
       </c>
-      <c r="J46" s="22">
+      <c r="J46" s="20">
         <v>3</v>
       </c>
-      <c r="K46" s="22">
+      <c r="K46" s="20">
         <v>2</v>
       </c>
-      <c r="L46" s="21">
+      <c r="L46" s="19">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
     <row r="47" spans="2:12">
-      <c r="B47" s="23">
+      <c r="B47" s="21">
         <v>425600</v>
       </c>
-      <c r="C47" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" s="21" t="s">
+      <c r="C47" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E47" s="21"/>
-      <c r="F47" s="23">
-        <v>2</v>
-      </c>
-      <c r="G47" s="23"/>
-      <c r="H47" s="23"/>
-      <c r="I47" s="23"/>
-      <c r="J47" s="23">
-        <v>2</v>
-      </c>
-      <c r="K47" s="23">
-        <v>7</v>
-      </c>
-      <c r="L47" s="21">
+      <c r="E47" s="19"/>
+      <c r="F47" s="21">
+        <v>0</v>
+      </c>
+      <c r="G47" s="21">
+        <v>0</v>
+      </c>
+      <c r="H47" s="21">
+        <v>0</v>
+      </c>
+      <c r="I47" s="21">
+        <v>0</v>
+      </c>
+      <c r="J47" s="21">
+        <v>0</v>
+      </c>
+      <c r="K47" s="21">
+        <v>0</v>
+      </c>
+      <c r="L47" s="19">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="2:12">
-      <c r="B48" s="23">
+      <c r="B48" s="21">
         <v>420501</v>
       </c>
-      <c r="C48" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" s="21" t="s">
+      <c r="C48" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="21"/>
-      <c r="F48" s="22">
+      <c r="E48" s="19"/>
+      <c r="F48" s="20">
         <v>4</v>
       </c>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22">
+      <c r="G48" s="20">
+        <v>0</v>
+      </c>
+      <c r="H48" s="20">
+        <v>0</v>
+      </c>
+      <c r="I48" s="20">
+        <v>0</v>
+      </c>
+      <c r="J48" s="20">
         <v>5</v>
       </c>
-      <c r="K48" s="22">
+      <c r="K48" s="20">
         <v>1</v>
       </c>
-      <c r="L48" s="21">
+      <c r="L48" s="19">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="49" spans="2:16">
-      <c r="B49" s="23">
+      <c r="B49" s="21">
         <v>423408</v>
       </c>
-      <c r="C49" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49" s="21" t="s">
+      <c r="C49" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E49" s="21"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22">
+      <c r="E49" s="19"/>
+      <c r="F49" s="20">
+        <v>0</v>
+      </c>
+      <c r="G49" s="20">
+        <v>0</v>
+      </c>
+      <c r="H49" s="20">
+        <v>0</v>
+      </c>
+      <c r="I49" s="20">
+        <v>0</v>
+      </c>
+      <c r="J49" s="20">
+        <v>0</v>
+      </c>
+      <c r="K49" s="20">
+        <v>0</v>
+      </c>
+      <c r="L49" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:16">
+      <c r="B50" s="21">
+        <v>421300</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E50" s="19"/>
+      <c r="F50" s="20">
+        <v>2</v>
+      </c>
+      <c r="G50" s="20">
+        <v>0</v>
+      </c>
+      <c r="H50" s="20">
+        <v>0</v>
+      </c>
+      <c r="I50" s="20">
         <v>4</v>
       </c>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22">
-        <v>2</v>
-      </c>
-      <c r="J49" s="22">
+      <c r="J50" s="20">
+        <v>0</v>
+      </c>
+      <c r="K50" s="20">
         <v>4</v>
       </c>
-      <c r="K49" s="22"/>
-      <c r="L49" s="21">
+      <c r="L50" s="19">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="2:16">
-      <c r="B50" s="23">
-        <v>421300</v>
-      </c>
-      <c r="C50" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D50" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E50" s="21"/>
-      <c r="F50" s="22">
-        <v>2</v>
-      </c>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22">
+    <row r="51" spans="2:16">
+      <c r="B51" s="21">
+        <v>422601</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="19"/>
+      <c r="F51" s="20">
+        <v>5</v>
+      </c>
+      <c r="G51" s="20">
+        <v>0</v>
+      </c>
+      <c r="H51" s="20">
+        <v>0</v>
+      </c>
+      <c r="I51" s="20">
+        <v>0</v>
+      </c>
+      <c r="J51" s="20">
         <v>4</v>
       </c>
-      <c r="J50" s="22"/>
-      <c r="K50" s="22">
-        <v>4</v>
-      </c>
-      <c r="L50" s="21">
+      <c r="K51" s="20">
+        <v>1</v>
+      </c>
+      <c r="L51" s="19">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="2:16">
-      <c r="B51" s="23">
-        <v>422601</v>
-      </c>
-      <c r="C51" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D51" s="21" t="s">
+    <row r="52" spans="2:16">
+      <c r="B52" s="21">
+        <v>424500</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E51" s="21"/>
-      <c r="F51" s="22">
-        <v>5</v>
-      </c>
-      <c r="G51" s="22"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22">
-        <v>4</v>
-      </c>
-      <c r="K51" s="22">
-        <v>1</v>
-      </c>
-      <c r="L51" s="21">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="52" spans="2:16">
-      <c r="B52" s="23">
-        <v>424500</v>
-      </c>
-      <c r="C52" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D52" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52" s="21"/>
-      <c r="F52" s="22">
+      <c r="E52" s="19"/>
+      <c r="F52" s="20">
         <v>3</v>
       </c>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22">
+      <c r="G52" s="20">
+        <v>0</v>
+      </c>
+      <c r="H52" s="20">
+        <v>0</v>
+      </c>
+      <c r="I52" s="20">
         <v>3</v>
       </c>
-      <c r="J52" s="22">
+      <c r="J52" s="20">
         <v>3</v>
       </c>
-      <c r="K52" s="22"/>
-      <c r="L52" s="21">
+      <c r="K52" s="20">
+        <v>0</v>
+      </c>
+      <c r="L52" s="19">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
     <row r="53" spans="2:16">
-      <c r="B53" s="23">
+      <c r="B53" s="21">
         <v>424960</v>
       </c>
-      <c r="C53" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D53" s="21" t="s">
+      <c r="C53" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E53" s="21"/>
-      <c r="F53" s="22">
+      <c r="E53" s="19"/>
+      <c r="F53" s="20">
         <v>1</v>
       </c>
-      <c r="G53" s="22">
+      <c r="G53" s="20">
         <v>2</v>
       </c>
-      <c r="H53" s="23">
+      <c r="H53" s="21">
         <v>2</v>
       </c>
-      <c r="I53" s="22">
+      <c r="I53" s="20">
         <v>2</v>
       </c>
-      <c r="J53" s="22">
+      <c r="J53" s="20">
         <v>1</v>
       </c>
-      <c r="K53" s="22">
+      <c r="K53" s="20">
         <v>1</v>
       </c>
-      <c r="L53" s="24">
+      <c r="L53" s="22">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
     <row r="54" spans="2:16">
-      <c r="B54" s="23">
+      <c r="B54" s="21">
         <v>423348</v>
       </c>
-      <c r="C54" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="21" t="s">
+      <c r="C54" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E54" s="21"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="22">
+      <c r="E54" s="19"/>
+      <c r="F54" s="20">
+        <v>0</v>
+      </c>
+      <c r="G54" s="20">
         <v>2</v>
       </c>
-      <c r="H54" s="23">
+      <c r="H54" s="21">
         <v>2</v>
       </c>
-      <c r="I54" s="22">
+      <c r="I54" s="20">
         <v>1</v>
       </c>
-      <c r="J54" s="22">
+      <c r="J54" s="20">
         <v>3</v>
       </c>
-      <c r="K54" s="22"/>
-      <c r="L54" s="21">
+      <c r="K54" s="20">
+        <v>0</v>
+      </c>
+      <c r="L54" s="19">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
     <row r="55" spans="2:16">
-      <c r="B55" s="23">
+      <c r="B55" s="21">
         <v>421401</v>
       </c>
-      <c r="C55" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="21" t="s">
+      <c r="C55" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E55" s="21"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22">
+      <c r="E55" s="19"/>
+      <c r="F55" s="20">
+        <v>0</v>
+      </c>
+      <c r="G55" s="20">
         <v>2</v>
       </c>
-      <c r="H55" s="22">
+      <c r="H55" s="20">
         <v>4</v>
       </c>
-      <c r="I55" s="22"/>
-      <c r="J55" s="22"/>
-      <c r="K55" s="22">
+      <c r="I55" s="20">
+        <v>0</v>
+      </c>
+      <c r="J55" s="20">
+        <v>0</v>
+      </c>
+      <c r="K55" s="20">
         <v>1</v>
       </c>
-      <c r="L55" s="21">
+      <c r="L55" s="19">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
     </row>
     <row r="56" spans="2:16">
-      <c r="B56" s="23">
+      <c r="B56" s="21">
         <v>421900</v>
       </c>
-      <c r="C56" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" s="21" t="s">
+      <c r="C56" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E56" s="21"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="22">
+      <c r="E56" s="19"/>
+      <c r="F56" s="20">
+        <v>0</v>
+      </c>
+      <c r="G56" s="20">
+        <v>0</v>
+      </c>
+      <c r="H56" s="20">
         <v>2</v>
       </c>
-      <c r="I56" s="22"/>
-      <c r="J56" s="22">
+      <c r="I56" s="20">
+        <v>0</v>
+      </c>
+      <c r="J56" s="20">
         <v>4</v>
       </c>
-      <c r="K56" s="22"/>
-      <c r="L56" s="21">
+      <c r="K56" s="20">
+        <v>0</v>
+      </c>
+      <c r="L56" s="19">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
     <row r="57" spans="2:16">
-      <c r="B57" s="23">
+      <c r="B57" s="21">
         <v>421001</v>
       </c>
-      <c r="C57" s="21" t="s">
+      <c r="C57" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E57" s="21"/>
-      <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
+      <c r="E57" s="19"/>
+      <c r="F57" s="21">
+        <v>0</v>
+      </c>
+      <c r="G57" s="21">
+        <v>0</v>
+      </c>
       <c r="H57" s="21">
         <v>2</v>
       </c>
@@ -6601,29 +6725,29 @@
       </c>
     </row>
     <row r="58" spans="2:16">
-      <c r="B58" s="23">
+      <c r="B58" s="21">
         <v>420500</v>
       </c>
-      <c r="C58" s="21" t="s">
+      <c r="C58" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="D58" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E58" s="21"/>
-      <c r="F58" s="23"/>
-      <c r="G58" s="23">
+      <c r="E58" s="19"/>
+      <c r="F58" s="21"/>
+      <c r="G58" s="21">
         <v>1</v>
       </c>
-      <c r="H58" s="23">
+      <c r="H58" s="21">
         <v>2</v>
       </c>
-      <c r="I58" s="22"/>
-      <c r="J58" s="23">
+      <c r="I58" s="20"/>
+      <c r="J58" s="21">
         <v>2</v>
       </c>
-      <c r="K58" s="22"/>
-      <c r="L58" s="21">
+      <c r="K58" s="20"/>
+      <c r="L58" s="19">
         <f t="shared" ref="L58:L74" si="2">SUM(F58:K58)</f>
         <v>5</v>
       </c>
@@ -6632,421 +6756,421 @@
       </c>
     </row>
     <row r="59" spans="2:16">
-      <c r="B59" s="23">
+      <c r="B59" s="21">
         <v>420402</v>
       </c>
-      <c r="C59" s="21" t="s">
+      <c r="C59" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="D59" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E59" s="21"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22">
+      <c r="E59" s="19"/>
+      <c r="F59" s="20"/>
+      <c r="G59" s="20"/>
+      <c r="H59" s="20"/>
+      <c r="I59" s="20"/>
+      <c r="J59" s="20">
         <v>5</v>
       </c>
-      <c r="K59" s="22"/>
-      <c r="L59" s="21">
+      <c r="K59" s="20"/>
+      <c r="L59" s="19">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
     <row r="60" spans="2:16">
-      <c r="B60" s="23">
+      <c r="B60" s="21">
         <v>423448</v>
       </c>
-      <c r="C60" s="21" t="s">
+      <c r="C60" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D60" s="21" t="s">
+      <c r="D60" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E60" s="21"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="23"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22">
+      <c r="E60" s="19"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="21"/>
+      <c r="I60" s="20"/>
+      <c r="J60" s="20">
         <v>4</v>
       </c>
-      <c r="K60" s="22"/>
-      <c r="L60" s="21">
+      <c r="K60" s="20"/>
+      <c r="L60" s="19">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
     <row r="61" spans="2:16">
-      <c r="B61" s="23">
+      <c r="B61" s="21">
         <v>422600</v>
       </c>
-      <c r="C61" s="21" t="s">
+      <c r="C61" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="D61" s="21" t="s">
+      <c r="D61" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E61" s="21"/>
-      <c r="F61" s="23"/>
-      <c r="G61" s="23"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="23"/>
-      <c r="K61" s="23">
+      <c r="E61" s="19"/>
+      <c r="F61" s="21"/>
+      <c r="G61" s="21"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+      <c r="J61" s="21"/>
+      <c r="K61" s="21">
         <v>3</v>
       </c>
-      <c r="L61" s="21">
+      <c r="L61" s="19">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
     <row r="62" spans="2:16">
-      <c r="B62" s="23">
+      <c r="B62" s="21">
         <v>423309</v>
       </c>
-      <c r="C62" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62" s="21" t="s">
+      <c r="C62" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E62" s="21"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22">
+      <c r="E62" s="19"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="20">
         <v>1</v>
       </c>
-      <c r="H62" s="22">
+      <c r="H62" s="20">
         <v>1</v>
       </c>
-      <c r="I62" s="22">
+      <c r="I62" s="20">
         <v>1</v>
       </c>
-      <c r="J62" s="22"/>
-      <c r="K62" s="22"/>
-      <c r="L62" s="21">
+      <c r="J62" s="20"/>
+      <c r="K62" s="20"/>
+      <c r="L62" s="19">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
     <row r="63" spans="2:16">
-      <c r="B63" s="23">
+      <c r="B63" s="21">
         <v>420200</v>
       </c>
-      <c r="C63" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D63" s="21" t="s">
+      <c r="C63" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E63" s="21"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="22">
+      <c r="E63" s="19"/>
+      <c r="F63" s="20"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="20">
         <v>1</v>
       </c>
-      <c r="I63" s="22">
+      <c r="I63" s="20">
         <v>1</v>
       </c>
-      <c r="J63" s="22"/>
-      <c r="K63" s="22"/>
-      <c r="L63" s="21">
+      <c r="J63" s="20"/>
+      <c r="K63" s="20"/>
+      <c r="L63" s="19">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
     <row r="64" spans="2:16">
-      <c r="B64" s="23">
+      <c r="B64" s="21">
         <v>423308</v>
       </c>
-      <c r="C64" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" s="21" t="s">
+      <c r="C64" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E64" s="21"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22">
+      <c r="E64" s="19"/>
+      <c r="F64" s="20"/>
+      <c r="G64" s="20">
         <v>2</v>
       </c>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="22"/>
-      <c r="K64" s="22"/>
-      <c r="L64" s="21">
+      <c r="H64" s="20"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
+      <c r="K64" s="20"/>
+      <c r="L64" s="19">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
     <row r="65" spans="2:13">
-      <c r="B65" s="23">
+      <c r="B65" s="21">
         <v>422400</v>
       </c>
-      <c r="C65" s="21" t="s">
+      <c r="C65" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E65" s="21"/>
-      <c r="F65" s="23"/>
-      <c r="G65" s="23"/>
-      <c r="H65" s="23"/>
-      <c r="I65" s="23"/>
-      <c r="J65" s="23">
+      <c r="E65" s="19"/>
+      <c r="F65" s="21"/>
+      <c r="G65" s="21"/>
+      <c r="H65" s="21"/>
+      <c r="I65" s="21"/>
+      <c r="J65" s="21">
         <v>2</v>
       </c>
-      <c r="K65" s="23"/>
-      <c r="L65" s="21">
+      <c r="K65" s="21"/>
+      <c r="L65" s="19">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
     <row r="66" spans="2:13">
-      <c r="B66" s="23">
+      <c r="B66" s="21">
         <v>421800</v>
       </c>
-      <c r="C66" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" s="21" t="s">
+      <c r="C66" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E66" s="21"/>
-      <c r="F66" s="22"/>
-      <c r="G66" s="22"/>
-      <c r="H66" s="22"/>
-      <c r="I66" s="22"/>
-      <c r="J66" s="22"/>
-      <c r="K66" s="22"/>
-      <c r="L66" s="21">
+      <c r="E66" s="19"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="2:13">
-      <c r="B67" s="23">
+      <c r="B67" s="21">
         <v>423316</v>
       </c>
-      <c r="C67" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" s="21" t="s">
+      <c r="C67" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E67" s="21"/>
-      <c r="F67" s="22"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="22"/>
-      <c r="I67" s="22"/>
-      <c r="J67" s="22"/>
-      <c r="K67" s="22"/>
-      <c r="L67" s="21">
+      <c r="E67" s="19"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="20"/>
+      <c r="I67" s="20"/>
+      <c r="J67" s="20"/>
+      <c r="K67" s="20"/>
+      <c r="L67" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="68" spans="2:13">
-      <c r="B68" s="23">
+      <c r="B68" s="21">
         <v>423304</v>
       </c>
-      <c r="C68" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68" s="21" t="s">
+      <c r="C68" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E68" s="21"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="23"/>
-      <c r="I68" s="22"/>
-      <c r="J68" s="22"/>
-      <c r="K68" s="22"/>
-      <c r="L68" s="21">
+      <c r="E68" s="19"/>
+      <c r="F68" s="20"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="21"/>
+      <c r="I68" s="20"/>
+      <c r="J68" s="20"/>
+      <c r="K68" s="20"/>
+      <c r="L68" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="69" spans="2:13">
-      <c r="B69" s="23">
+      <c r="B69" s="21">
         <v>423416</v>
       </c>
-      <c r="C69" s="21" t="s">
+      <c r="C69" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D69" s="21" t="s">
+      <c r="D69" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E69" s="21"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
-      <c r="K69" s="22"/>
-      <c r="L69" s="21">
+      <c r="E69" s="19"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+      <c r="L69" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="70" spans="2:13">
-      <c r="B70" s="23">
+      <c r="B70" s="21">
         <v>420300</v>
       </c>
-      <c r="C70" s="21" t="s">
+      <c r="C70" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D70" s="21" t="s">
+      <c r="D70" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E70" s="21"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23"/>
-      <c r="I70" s="23"/>
-      <c r="J70" s="23"/>
-      <c r="K70" s="23"/>
-      <c r="L70" s="24">
+      <c r="E70" s="19"/>
+      <c r="F70" s="21"/>
+      <c r="G70" s="21"/>
+      <c r="H70" s="21"/>
+      <c r="I70" s="21"/>
+      <c r="J70" s="21"/>
+      <c r="K70" s="21"/>
+      <c r="L70" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="2:13">
-      <c r="B71" s="23">
+      <c r="B71" s="21">
         <v>422401</v>
       </c>
-      <c r="C71" s="21" t="s">
+      <c r="C71" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D71" s="21" t="s">
+      <c r="D71" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="E71" s="21"/>
-      <c r="F71" s="21"/>
-      <c r="G71" s="21"/>
-      <c r="H71" s="21"/>
-      <c r="I71" s="21"/>
-      <c r="J71" s="21"/>
-      <c r="K71" s="21"/>
-      <c r="L71" s="21">
+      <c r="E71" s="19"/>
+      <c r="F71" s="19"/>
+      <c r="G71" s="19"/>
+      <c r="H71" s="19"/>
+      <c r="I71" s="19"/>
+      <c r="J71" s="19"/>
+      <c r="K71" s="19"/>
+      <c r="L71" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="72" spans="2:13">
-      <c r="B72" s="23">
+      <c r="B72" s="21">
         <v>423800</v>
       </c>
-      <c r="C72" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="21" t="s">
+      <c r="C72" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E72" s="21" t="s">
+      <c r="E72" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="F72" s="23"/>
-      <c r="G72" s="23"/>
-      <c r="H72" s="23"/>
-      <c r="I72" s="23"/>
-      <c r="J72" s="23"/>
-      <c r="K72" s="23"/>
-      <c r="L72" s="21">
+      <c r="F72" s="21"/>
+      <c r="G72" s="21"/>
+      <c r="H72" s="21"/>
+      <c r="I72" s="21"/>
+      <c r="J72" s="21"/>
+      <c r="K72" s="21"/>
+      <c r="L72" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="73" spans="2:13">
-      <c r="B73" s="23">
+      <c r="B73" s="21">
         <v>423409</v>
       </c>
-      <c r="C73" s="21" t="s">
+      <c r="C73" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="D73" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E73" s="21"/>
-      <c r="F73" s="22"/>
-      <c r="G73" s="22"/>
-      <c r="H73" s="22"/>
-      <c r="I73" s="22"/>
-      <c r="J73" s="22"/>
-      <c r="K73" s="22"/>
-      <c r="L73" s="21">
+      <c r="E73" s="19"/>
+      <c r="F73" s="20"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="20"/>
+      <c r="I73" s="20"/>
+      <c r="J73" s="20"/>
+      <c r="K73" s="20"/>
+      <c r="L73" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="2:13">
-      <c r="B74" s="23">
+      <c r="B74" s="21">
         <v>423404</v>
       </c>
-      <c r="C74" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D74" s="21" t="s">
+      <c r="C74" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E74" s="21"/>
-      <c r="F74" s="22"/>
-      <c r="G74" s="22"/>
-      <c r="H74" s="22"/>
-      <c r="I74" s="22"/>
-      <c r="J74" s="22"/>
-      <c r="K74" s="22"/>
-      <c r="L74" s="21">
+      <c r="E74" s="19"/>
+      <c r="F74" s="20"/>
+      <c r="G74" s="20"/>
+      <c r="H74" s="20"/>
+      <c r="I74" s="20"/>
+      <c r="J74" s="20"/>
+      <c r="K74" s="20"/>
+      <c r="L74" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="75" spans="2:13">
-      <c r="B75" s="23">
+      <c r="B75" s="21">
         <v>420801</v>
       </c>
-      <c r="C75" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="21" t="s">
+      <c r="C75" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E75" s="21"/>
-      <c r="F75" s="21"/>
-      <c r="G75" s="23"/>
-      <c r="H75" s="23"/>
-      <c r="I75" s="23"/>
-      <c r="J75" s="23"/>
-      <c r="K75" s="22"/>
-      <c r="L75" s="21">
+      <c r="E75" s="19"/>
+      <c r="F75" s="19"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="21"/>
+      <c r="K75" s="20"/>
+      <c r="L75" s="19">
         <f>SUM(G75:K75)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" spans="2:13">
-      <c r="B76" s="23">
+      <c r="B76" s="21">
         <v>420160</v>
       </c>
-      <c r="C76" s="21" t="s">
+      <c r="C76" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D76" s="21" t="s">
+      <c r="D76" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E76" s="21" t="s">
+      <c r="E76" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="F76" s="22"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="22"/>
-      <c r="I76" s="22"/>
-      <c r="J76" s="22"/>
-      <c r="K76" s="22"/>
-      <c r="L76" s="21">
+      <c r="F76" s="20"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="20"/>
+      <c r="I76" s="20"/>
+      <c r="J76" s="20"/>
+      <c r="K76" s="20"/>
+      <c r="L76" s="19">
         <f>SUM(F76:K76)</f>
         <v>0</v>
       </c>
@@ -7060,9 +7184,9 @@
       </c>
     </row>
     <row r="79" spans="2:13">
-      <c r="L79" s="21">
+      <c r="L79" s="19">
         <f>SUM(L3:L78)</f>
-        <v>2086</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="83" spans="7:15">
@@ -7097,7 +7221,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="A3:L21"/>
+  <dimension ref="A3:M22"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="15"/>
@@ -7168,7 +7292,7 @@
         <v>56</v>
       </c>
       <c r="L4" s="1">
-        <f t="shared" ref="L4:L19" si="0">SUM(F4:K4)</f>
+        <f t="shared" ref="L4:M20" si="0">SUM(F4:K4)</f>
         <v>472</v>
       </c>
     </row>
@@ -7567,29 +7691,29 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G16" s="1">
+        <v>19</v>
+      </c>
+      <c r="H16" s="1">
+        <v>24</v>
+      </c>
+      <c r="I16" s="1">
         <v>17</v>
       </c>
-      <c r="H16" s="1">
-        <v>0</v>
-      </c>
-      <c r="I16" s="1">
-        <v>16</v>
-      </c>
       <c r="J16" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K16" s="1">
         <v>21</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" si="0"/>
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="16"/>
       <c r="B17" s="12">
         <v>436104</v>
@@ -7626,7 +7750,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:13">
       <c r="B18" s="12">
         <v>436148</v>
       </c>
@@ -7661,46 +7785,81 @@
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="13"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13">
       <c r="B19" s="12">
-        <v>431300</v>
+        <v>431100</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G19" s="1">
+        <v>63</v>
+      </c>
+      <c r="H19" s="1">
+        <v>64</v>
+      </c>
+      <c r="I19" s="1">
+        <v>63</v>
+      </c>
+      <c r="J19" s="1">
+        <v>42</v>
+      </c>
+      <c r="K19" s="1">
+        <v>37</v>
+      </c>
+      <c r="L19" s="1">
+        <f t="shared" si="0"/>
+        <v>299</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="13"/>
+      <c r="B20" s="12">
+        <v>431300</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
         <v>77</v>
       </c>
-      <c r="H19" s="1">
-        <v>0</v>
-      </c>
-      <c r="I19" s="1">
-        <v>0</v>
-      </c>
-      <c r="J19" s="1">
-        <v>0</v>
-      </c>
-      <c r="K19" s="1">
-        <v>0</v>
-      </c>
-      <c r="L19" s="1">
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
-      <c r="L21">
-        <f>SUM(L4:L20)</f>
-        <v>4078</v>
+    <row r="22" spans="1:13">
+      <c r="L22">
+        <f>SUM(L4:L21)</f>
+        <v>4408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar web con nueva data de pedidos y stock
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4404" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBF294DC-7CF7-43C8-BF0B-D7E99D6FAB29}"/>
+  <xr:revisionPtr revIDLastSave="4410" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12C046A9-F18B-4B18-81BA-86898131E012}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7875" firstSheet="6" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView minimized="1" xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7875" firstSheet="5" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -674,11 +674,11 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
@@ -1057,7 +1057,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.75">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="27" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28"/>
@@ -1856,7 +1856,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>43</v>
       </c>
       <c r="C3" s="28"/>
@@ -2463,7 +2463,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>44</v>
       </c>
       <c r="C3" s="28"/>
@@ -2833,7 +2833,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="28"/>
@@ -4426,7 +4426,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>109</v>
       </c>
       <c r="C3" s="28"/>
@@ -4790,25 +4790,25 @@
         <v>8</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="27">
+      <c r="F14" s="26">
         <v>0</v>
       </c>
       <c r="G14" s="4">
         <v>0</v>
       </c>
-      <c r="H14" s="27">
-        <v>0</v>
-      </c>
-      <c r="I14" s="27">
-        <v>0</v>
-      </c>
-      <c r="J14" s="27">
-        <v>0</v>
-      </c>
-      <c r="K14" s="27">
-        <v>0</v>
-      </c>
-      <c r="L14" s="27">
+      <c r="H14" s="26">
+        <v>0</v>
+      </c>
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
+      <c r="J14" s="26">
+        <v>0</v>
+      </c>
+      <c r="K14" s="26">
+        <v>0</v>
+      </c>
+      <c r="L14" s="26">
         <f>SUM(F14:K14)</f>
         <v>0</v>
       </c>
@@ -7691,26 +7691,26 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G16" s="1">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="I16" s="1">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J16" s="1">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="K16" s="1">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" si="0"/>
-        <v>102</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7859,7 +7859,7 @@
     <row r="22" spans="1:13">
       <c r="L22">
         <f>SUM(L4:L21)</f>
-        <v>4408</v>
+        <v>4342</v>
       </c>
     </row>
   </sheetData>
@@ -7873,6 +7873,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -8016,23 +8031,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8040,5 +8040,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
 </file>
</xml_diff>

<commit_message>
Actualizar stock en la web
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4688" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C678CCD-E7C4-44E8-8441-9EB48CA9A2F6}"/>
+  <xr:revisionPtr revIDLastSave="4716" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29E7183C-D8A5-4256-A00D-8961481BCC63}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7875" firstSheet="6" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="140">
   <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
@@ -255,6 +255,12 @@
   </si>
   <si>
     <t>4016</t>
+  </si>
+  <si>
+    <t>PITILLO    (BLUE)</t>
+  </si>
+  <si>
+    <t>BIOMEDIOFOCALIZADO</t>
   </si>
   <si>
     <t>4012-01</t>
@@ -471,7 +477,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -546,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -625,12 +631,64 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -690,13 +748,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1035,6 +1110,9 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -1067,27 +1145,41 @@
 </we:webextension>
 </file>
 
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{15D77760-8E18-40C7-8A74-60553030A222}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;50ce5e7d-37f8-469c-9f6f-1a80d8974e86&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FB535F-634B-4933-81FF-529A98082563}">
   <dimension ref="B2:L31"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:12" ht="18.75">
-      <c r="B2" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-    </row>
-    <row r="3" spans="2:12">
+    <row r="2" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="B2" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1122,7 +1214,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:12">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>6</v>
       </c>
@@ -1152,7 +1244,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:12">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
@@ -1180,7 +1272,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:12">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
@@ -1208,7 +1300,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:12">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>13</v>
       </c>
@@ -1234,7 +1326,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>14</v>
       </c>
@@ -1262,7 +1354,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>16</v>
       </c>
@@ -1286,7 +1378,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
@@ -1316,7 +1408,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>19</v>
       </c>
@@ -1340,7 +1432,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>21</v>
       </c>
@@ -1366,7 +1458,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>23</v>
       </c>
@@ -1394,7 +1486,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>24</v>
       </c>
@@ -1428,7 +1520,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:12">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
@@ -1454,7 +1546,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="2:12">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>26</v>
       </c>
@@ -1478,7 +1570,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:12">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>27</v>
       </c>
@@ -1510,7 +1602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:12">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="6" t="s">
         <v>28</v>
       </c>
@@ -1534,7 +1626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:12">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
@@ -1562,7 +1654,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:12">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="6" t="s">
         <v>31</v>
       </c>
@@ -1594,7 +1686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:12">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="6" t="s">
         <v>32</v>
       </c>
@@ -1618,7 +1710,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:12">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="6" t="s">
         <v>33</v>
       </c>
@@ -1642,7 +1734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:12">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="6" t="s">
         <v>34</v>
       </c>
@@ -1666,7 +1758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="2:12">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="6" t="s">
         <v>35</v>
       </c>
@@ -1690,7 +1782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:12">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
         <v>36</v>
       </c>
@@ -1714,7 +1806,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:12">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="6" t="s">
         <v>37</v>
       </c>
@@ -1738,7 +1830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:12">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="6" t="s">
         <v>38</v>
       </c>
@@ -1764,7 +1856,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="2:12">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="6" t="s">
         <v>39</v>
       </c>
@@ -1790,7 +1882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:12">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="6" t="s">
         <v>40</v>
       </c>
@@ -1812,7 +1904,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="2:12">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="6" t="s">
         <v>41</v>
       </c>
@@ -1834,7 +1926,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:12">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
         <v>42</v>
       </c>
@@ -1869,24 +1961,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011174A9-0248-46ED-981A-FD90D8DB99B2}">
   <dimension ref="B3:L20"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-    </row>
-    <row r="4" spans="2:12">
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
@@ -1921,7 +2013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:12">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="9">
         <v>389201</v>
       </c>
@@ -1955,7 +2047,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="2:12">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="9">
         <v>380200</v>
       </c>
@@ -1989,7 +2081,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="2:12">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="9">
         <v>383400</v>
       </c>
@@ -2023,7 +2115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="9">
         <v>382100</v>
       </c>
@@ -2057,7 +2149,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="9">
         <v>388000</v>
       </c>
@@ -2091,7 +2183,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="9">
         <v>389300</v>
       </c>
@@ -2125,7 +2217,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="9">
         <v>385371</v>
       </c>
@@ -2159,7 +2251,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="9">
         <v>386501</v>
       </c>
@@ -2193,7 +2285,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="9">
         <v>385304</v>
       </c>
@@ -2227,7 +2319,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="9">
         <v>388300</v>
       </c>
@@ -2261,7 +2353,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="2:12">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="9">
         <v>387900</v>
       </c>
@@ -2295,7 +2387,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="2:12">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="9">
         <v>385800</v>
       </c>
@@ -2329,7 +2421,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="2:12">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="9">
         <v>381801</v>
       </c>
@@ -2363,7 +2455,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="2:12">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="9">
         <v>389401</v>
       </c>
@@ -2397,7 +2489,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="2:12">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="9">
         <v>382101</v>
       </c>
@@ -2431,7 +2523,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:12">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="9">
         <v>389700</v>
       </c>
@@ -2476,24 +2568,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE2264EF-F28E-4311-81D5-A7BF6F5FC77F}">
   <dimension ref="B3:L15"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-    </row>
-    <row r="4" spans="2:12">
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
@@ -2528,7 +2620,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:12">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>45</v>
       </c>
@@ -2562,7 +2654,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="2:12">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>47</v>
       </c>
@@ -2592,7 +2684,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="2:12">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>48</v>
       </c>
@@ -2622,7 +2714,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>49</v>
       </c>
@@ -2652,7 +2744,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>50</v>
       </c>
@@ -2680,7 +2772,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>51</v>
       </c>
@@ -2706,7 +2798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>52</v>
       </c>
@@ -2734,7 +2826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>53</v>
       </c>
@@ -2760,7 +2852,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>54</v>
       </c>
@@ -2784,7 +2876,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>55</v>
       </c>
@@ -2808,7 +2900,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:12">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>56</v>
       </c>
@@ -2843,69 +2935,71 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFAA1C20-0AB4-435A-AEDE-B6C824B1C346}">
   <dimension ref="B3:L49"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="2" max="3" width="11.453125" style="31"/>
+    <col min="4" max="4" width="16" style="31" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="27" t="s">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-    </row>
-    <row r="4" spans="2:12">
-      <c r="B4" s="5" t="s">
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="34"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="27">
         <v>36</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="27">
         <v>38</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="27">
         <v>40</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="27">
         <v>42</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="27">
         <v>44</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="27">
         <v>46</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="27" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:12">
-      <c r="B5" s="6" t="s">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B5" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="C5" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E5" s="7"/>
@@ -2932,14 +3026,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="2:12">
-      <c r="B6" s="6" t="s">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B6" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="C6" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="7"/>
@@ -2966,14 +3060,14 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="2:12">
-      <c r="B7" s="6" t="s">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B7" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="C7" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="28" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="7"/>
@@ -3000,14 +3094,14 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
-      <c r="B8" s="6" t="s">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B8" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="7"/>
@@ -3034,14 +3128,14 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
-      <c r="B9" s="6" t="s">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B9" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="7"/>
@@ -3068,14 +3162,14 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
-      <c r="B10" s="6" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E10" s="7"/>
@@ -3102,14 +3196,14 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
-      <c r="B11" s="6" t="s">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="28" t="s">
         <v>65</v>
       </c>
       <c r="E11" s="7"/>
@@ -3136,14 +3230,14 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
-      <c r="B12" s="6" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E12" s="7"/>
@@ -3170,17 +3264,19 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
-      <c r="B13" s="6" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="7"/>
+      <c r="C13" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>69</v>
+      </c>
       <c r="F13" s="7">
         <v>18</v>
       </c>
@@ -3204,14 +3300,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
-      <c r="B14" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="7" t="s">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B14" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="7"/>
@@ -3238,14 +3334,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:12">
-      <c r="B15" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="7" t="s">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B15" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E15" s="7"/>
@@ -3272,14 +3368,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="2:12">
-      <c r="B16" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="7" t="s">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B16" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E16" s="7"/>
@@ -3306,14 +3402,14 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="2:12">
-      <c r="B17" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="7" t="s">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B17" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="7"/>
@@ -3340,14 +3436,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="2:12">
-      <c r="B18" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="7" t="s">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B18" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E18" s="7"/>
@@ -3374,14 +3470,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:12">
-      <c r="B19" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="7" t="s">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B19" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="7"/>
@@ -3408,14 +3504,14 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="2:12">
-      <c r="B20" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="7" t="s">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B20" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="7"/>
@@ -3442,14 +3538,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:12">
-      <c r="B21" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C21" s="7" t="s">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B21" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="7"/>
@@ -3476,14 +3572,14 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="2:12">
-      <c r="B22" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="7" t="s">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B22" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E22" s="7"/>
@@ -3510,14 +3606,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="2:12">
-      <c r="B23" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C23" s="7" t="s">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B23" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="28" t="s">
         <v>22</v>
       </c>
       <c r="E23" s="7"/>
@@ -3544,14 +3640,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:12">
-      <c r="B24" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C24" s="7" t="s">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B24" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="7"/>
@@ -3578,14 +3674,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:12">
-      <c r="B25" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="7" t="s">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B25" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E25" s="7"/>
@@ -3612,15 +3708,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:12">
-      <c r="B26" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>81</v>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B26" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7">
@@ -3646,14 +3742,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:12">
-      <c r="B27" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="7" t="s">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B27" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E27" s="7"/>
@@ -3680,14 +3776,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="2:12">
-      <c r="B28" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="7" t="s">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B28" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="E28" s="7"/>
@@ -3714,15 +3810,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:12">
-      <c r="B29" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>85</v>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B29" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7">
@@ -3748,14 +3844,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:12">
-      <c r="B30" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C30" s="7" t="s">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B30" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E30" s="7"/>
@@ -3782,14 +3878,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:12">
-      <c r="B31" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="7" t="s">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B31" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E31" s="7"/>
@@ -3816,14 +3912,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12">
-      <c r="B32" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="7" t="s">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B32" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E32" s="7"/>
@@ -3850,14 +3946,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:12">
-      <c r="B33" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" s="7" t="s">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B33" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E33" s="7"/>
@@ -3884,14 +3980,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:12">
-      <c r="B34" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="7" t="s">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B34" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E34" s="7"/>
@@ -3918,14 +4014,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:12">
-      <c r="B35" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="7" t="s">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B35" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E35" s="7"/>
@@ -3952,15 +4048,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:12">
-      <c r="B36" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>93</v>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B36" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="28" t="s">
+        <v>95</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7">
@@ -3986,14 +4082,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:12">
-      <c r="B37" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="7" t="s">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B37" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E37" s="7"/>
@@ -4020,14 +4116,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:12">
-      <c r="B38" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38" s="7" t="s">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B38" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E38" s="7"/>
@@ -4054,14 +4150,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:12">
-      <c r="B39" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="7" t="s">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B39" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="28" t="s">
         <v>8</v>
       </c>
       <c r="E39" s="7"/>
@@ -4088,14 +4184,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:12">
-      <c r="B40" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" s="7" t="s">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B40" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E40" s="7"/>
@@ -4122,14 +4218,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:12">
-      <c r="B41" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="7" t="s">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B41" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E41" s="7"/>
@@ -4156,14 +4252,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:12">
-      <c r="B42" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="7" t="s">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B42" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="28" t="s">
         <v>46</v>
       </c>
       <c r="E42" s="7"/>
@@ -4190,14 +4286,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:12">
-      <c r="B43" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C43" s="7" t="s">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B43" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="C43" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="28" t="s">
         <v>10</v>
       </c>
       <c r="E43" s="7"/>
@@ -4224,14 +4320,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:12">
-      <c r="B44" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" s="7" t="s">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B44" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E44" s="7"/>
@@ -4258,14 +4354,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:12">
-      <c r="B45" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45" s="7" t="s">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B45" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="28" t="s">
         <v>29</v>
       </c>
       <c r="E45" s="7"/>
@@ -4292,14 +4388,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:12">
-      <c r="B46" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46" s="7" t="s">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B46" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="C46" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" s="28" t="s">
         <v>22</v>
       </c>
       <c r="E46" s="7"/>
@@ -4326,15 +4422,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:12">
-      <c r="B47" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>105</v>
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B47" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="28" t="s">
+        <v>107</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7">
@@ -4360,15 +4456,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:12">
-      <c r="B48" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>107</v>
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B48" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="28" t="s">
+        <v>109</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7">
@@ -4394,14 +4490,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:12">
-      <c r="B49" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49" s="7" t="s">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B49" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="C49" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="28" t="s">
         <v>22</v>
       </c>
       <c r="E49" s="7"/>
@@ -4439,24 +4535,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E9EB22C-7ED7-4D45-8EA1-BD18A384D586}">
   <dimension ref="B3:L17"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-    </row>
-    <row r="4" spans="2:12">
+    <row r="3" spans="2:12" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" s="10" t="s">
         <v>1</v>
       </c>
@@ -4491,12 +4587,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:12">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>12</v>
@@ -4525,9 +4621,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="2:12">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>7</v>
@@ -4557,9 +4653,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="2:12">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>7</v>
@@ -4591,9 +4687,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>15</v>
@@ -4625,9 +4721,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>15</v>
@@ -4659,9 +4755,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>7</v>
@@ -4693,9 +4789,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>7</v>
@@ -4727,9 +4823,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>7</v>
@@ -4761,9 +4857,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>7</v>
@@ -4795,7 +4891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="1">
         <v>416500</v>
       </c>
@@ -4829,9 +4925,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="10:10">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J17" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -4845,13 +4941,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
   <dimension ref="A2:P127"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="16" max="16" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B2" s="26" t="s">
         <v>1</v>
       </c>
@@ -4886,7 +4982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B3" s="20">
         <v>422200</v>
       </c>
@@ -4920,7 +5016,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B4" s="20">
         <v>420301</v>
       </c>
@@ -4954,7 +5050,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B5" s="20">
         <v>423600</v>
       </c>
@@ -4988,7 +5084,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B6" s="20">
         <v>423500</v>
       </c>
@@ -5022,10 +5118,10 @@
         <v>112</v>
       </c>
       <c r="M6" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B7" s="20">
         <v>421000</v>
       </c>
@@ -5059,7 +5155,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B8" s="20">
         <v>422800</v>
       </c>
@@ -5089,10 +5185,10 @@
         <v>66</v>
       </c>
       <c r="N8" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B9" s="20">
         <v>422000</v>
       </c>
@@ -5125,7 +5221,7 @@
       </c>
       <c r="N9" s="17"/>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="16"/>
       <c r="B10" s="20">
         <v>424400</v>
@@ -5160,10 +5256,10 @@
         <v>47</v>
       </c>
       <c r="O10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="16"/>
       <c r="B11" s="20">
         <v>420100</v>
@@ -5198,10 +5294,10 @@
         <v>41</v>
       </c>
       <c r="O11" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="16"/>
       <c r="B12" s="20">
         <v>420800</v>
@@ -5236,10 +5332,10 @@
         <v>54</v>
       </c>
       <c r="N12" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="16"/>
       <c r="B13" s="20">
         <v>420400</v>
@@ -5274,10 +5370,10 @@
         <v>17</v>
       </c>
       <c r="O13" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B14" s="20">
         <v>422101</v>
       </c>
@@ -5309,10 +5405,10 @@
         <v>52</v>
       </c>
       <c r="O14" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
       <c r="B15" s="20">
         <v>424900</v>
@@ -5324,7 +5420,7 @@
         <v>29</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F15" s="19">
         <v>6</v>
@@ -5350,7 +5446,7 @@
       </c>
       <c r="N15" s="17"/>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B16" s="20">
         <v>420160</v>
       </c>
@@ -5361,7 +5457,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F16" s="19">
         <v>7</v>
@@ -5386,10 +5482,10 @@
         <v>49</v>
       </c>
       <c r="O16" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="16"/>
       <c r="B17" s="20">
         <v>424600</v>
@@ -5424,7 +5520,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="16"/>
       <c r="B18" s="20">
         <v>422700</v>
@@ -5459,7 +5555,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B19" s="20">
         <v>422701</v>
       </c>
@@ -5493,7 +5589,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B20" s="20">
         <v>421100</v>
       </c>
@@ -5527,7 +5623,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="16"/>
       <c r="B21" s="20">
         <v>423000</v>
@@ -5562,18 +5658,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B22" s="20">
         <v>424900</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>29</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F22" s="19">
         <v>4</v>
@@ -5598,7 +5694,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B23" s="20">
         <v>422900</v>
       </c>
@@ -5626,7 +5722,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B24" s="20">
         <v>422500</v>
       </c>
@@ -5660,9 +5756,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="16"/>
-      <c r="B25" s="28">
+      <c r="B25" s="20">
         <v>424701</v>
       </c>
       <c r="C25" s="18" t="s">
@@ -5695,7 +5791,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B26" s="20">
         <v>421801</v>
       </c>
@@ -5727,12 +5823,12 @@
         <v>32</v>
       </c>
       <c r="M26" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="16"/>
-      <c r="B27" s="28">
+      <c r="B27" s="20">
         <v>421400</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -5742,7 +5838,7 @@
         <v>20</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F27" s="19">
         <v>4</v>
@@ -5767,7 +5863,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B28" s="20">
         <v>420101</v>
       </c>
@@ -5799,7 +5895,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B29" s="20">
         <v>421901</v>
       </c>
@@ -5833,7 +5929,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B30" s="20">
         <v>424000</v>
       </c>
@@ -5867,7 +5963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B31" s="20">
         <v>421902</v>
       </c>
@@ -5901,7 +5997,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B32" s="20">
         <v>422190</v>
       </c>
@@ -5912,7 +6008,7 @@
         <v>10</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F32" s="19">
         <v>2</v>
@@ -5937,7 +6033,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B33" s="20">
         <v>420802</v>
       </c>
@@ -5971,7 +6067,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A34" s="16"/>
       <c r="B34" s="20">
         <v>420600</v>
       </c>
@@ -5983,29 +6080,29 @@
       </c>
       <c r="E34" s="18"/>
       <c r="F34" s="19">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G34" s="19">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H34" s="19">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I34" s="19">
         <v>0</v>
       </c>
       <c r="J34" s="19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K34" s="19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L34" s="18">
         <f t="shared" ref="L34:L56" si="1">SUM(F34:K34)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B35" s="20">
         <v>424801</v>
       </c>
@@ -6039,7 +6136,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="16"/>
       <c r="B36" s="20">
         <v>420900</v>
@@ -6074,7 +6171,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B37" s="20">
         <v>423900</v>
       </c>
@@ -6108,7 +6205,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B38" s="20">
         <v>422100</v>
       </c>
@@ -6142,7 +6239,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B39" s="20">
         <v>423200</v>
       </c>
@@ -6176,7 +6273,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B40" s="20">
         <v>422300</v>
       </c>
@@ -6210,7 +6307,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B41" s="20">
         <v>424700</v>
       </c>
@@ -6244,7 +6341,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B42" s="20">
         <v>421301</v>
       </c>
@@ -6274,7 +6371,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B43" s="20">
         <v>423501</v>
       </c>
@@ -6306,7 +6403,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B44" s="20">
         <v>424200</v>
       </c>
@@ -6336,7 +6433,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B45" s="20">
         <v>424300</v>
       </c>
@@ -6366,7 +6463,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="16"/>
       <c r="B46" s="20">
         <v>421402</v>
@@ -6401,7 +6498,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B47" s="20">
         <v>425600</v>
       </c>
@@ -6435,7 +6532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B48" s="20">
         <v>420501</v>
       </c>
@@ -6469,7 +6566,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B49" s="20">
         <v>423408</v>
       </c>
@@ -6503,7 +6600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B50" s="20">
         <v>421300</v>
       </c>
@@ -6537,7 +6634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B51" s="20">
         <v>422601</v>
       </c>
@@ -6571,7 +6668,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B52" s="20">
         <v>424500</v>
       </c>
@@ -6605,7 +6702,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B53" s="20">
         <v>424960</v>
       </c>
@@ -6639,7 +6736,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B54" s="20">
         <v>423348</v>
       </c>
@@ -6673,7 +6770,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" s="16"/>
       <c r="B55" s="20">
         <v>421401</v>
@@ -6708,7 +6805,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B56" s="20">
         <v>421900</v>
       </c>
@@ -6742,7 +6839,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B57" s="20">
         <v>421001</v>
       </c>
@@ -6776,15 +6873,15 @@
         <v>6</v>
       </c>
       <c r="M57" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B58" s="20">
         <v>420500</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D58" s="18" t="s">
         <v>20</v>
@@ -6807,10 +6904,10 @@
         <v>5</v>
       </c>
       <c r="P58" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B59" s="20">
         <v>420402</v>
       </c>
@@ -6844,12 +6941,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B60" s="20">
         <v>423448</v>
       </c>
       <c r="C60" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D60" s="18" t="s">
         <v>12</v>
@@ -6868,12 +6965,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B61" s="20">
         <v>422600</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D61" s="18" t="s">
         <v>8</v>
@@ -6892,7 +6989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:16">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B62" s="20">
         <v>423309</v>
       </c>
@@ -6920,7 +7017,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:16">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B63" s="20">
         <v>420200</v>
       </c>
@@ -6946,7 +7043,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:16">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B64" s="20">
         <v>423308</v>
       </c>
@@ -6970,7 +7067,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="2:13">
+    <row r="65" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B65" s="20">
         <v>422400</v>
       </c>
@@ -6994,7 +7091,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="2:13">
+    <row r="66" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B66" s="20">
         <v>421800</v>
       </c>
@@ -7016,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:13">
+    <row r="67" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B67" s="20">
         <v>423316</v>
       </c>
@@ -7038,7 +7135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:13">
+    <row r="68" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B68" s="20">
         <v>423304</v>
       </c>
@@ -7060,12 +7157,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="2:13">
+    <row r="69" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B69" s="20">
         <v>423416</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D69" s="18" t="s">
         <v>12</v>
@@ -7082,7 +7179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:13">
+    <row r="70" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B70" s="20">
         <v>420300</v>
       </c>
@@ -7104,7 +7201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="2:13">
+    <row r="71" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B71" s="20">
         <v>422401</v>
       </c>
@@ -7126,7 +7223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:13">
+    <row r="72" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B72" s="20">
         <v>423800</v>
       </c>
@@ -7137,7 +7234,7 @@
         <v>29</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F72" s="20"/>
       <c r="G72" s="20"/>
@@ -7150,12 +7247,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:13">
+    <row r="73" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B73" s="20">
         <v>423409</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D73" s="18" t="s">
         <v>12</v>
@@ -7172,7 +7269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="2:13">
+    <row r="74" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B74" s="20">
         <v>423404</v>
       </c>
@@ -7194,7 +7291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="2:13">
+    <row r="75" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B75" s="20">
         <v>420801</v>
       </c>
@@ -7216,18 +7313,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:13">
+    <row r="76" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B76" s="20">
         <v>420160</v>
       </c>
       <c r="C76" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D76" s="18" t="s">
         <v>8</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F76" s="19"/>
       <c r="G76" s="19"/>
@@ -7240,38 +7337,38 @@
         <v>0</v>
       </c>
       <c r="M76" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="77" spans="2:13">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E77" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="79" spans="2:13">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.35">
       <c r="L79" s="18">
         <f>SUM(L3:L78)</f>
-        <v>1868</v>
-      </c>
-    </row>
-    <row r="83" spans="7:15">
+        <v>1897</v>
+      </c>
+    </row>
+    <row r="83" spans="7:15" x14ac:dyDescent="0.35">
       <c r="O83" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="86" spans="7:15">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="86" spans="7:15" x14ac:dyDescent="0.35">
       <c r="G86" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="87" spans="7:15">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="87" spans="7:15" x14ac:dyDescent="0.35">
       <c r="H87" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="127" spans="11:11">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="127" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K127" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -7281,19 +7378,20 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
   <dimension ref="A3:M73"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" style="15"/>
+    <col min="2" max="2" width="11.453125" style="15"/>
     <col min="5" max="5" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B3" s="14" t="s">
         <v>1</v>
       </c>
@@ -7328,7 +7426,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="16"/>
       <c r="B4" s="12">
         <v>430100</v>
@@ -7363,7 +7461,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="12">
         <v>432100</v>
@@ -7398,7 +7496,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="16"/>
       <c r="B6" s="12">
         <v>431400</v>
@@ -7433,7 +7531,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="16"/>
       <c r="B7" s="12">
         <v>432300</v>
@@ -7442,7 +7540,7 @@
         <v>7</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1">
@@ -7468,7 +7566,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="16"/>
       <c r="B8" s="12">
         <v>430900</v>
@@ -7503,7 +7601,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="16"/>
       <c r="B9" s="12">
         <v>432900</v>
@@ -7538,7 +7636,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="16"/>
       <c r="B10" s="12">
         <v>431800</v>
@@ -7547,7 +7645,7 @@
         <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1">
@@ -7573,7 +7671,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="16"/>
       <c r="B11" s="12">
         <v>434100</v>
@@ -7608,7 +7706,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="16"/>
       <c r="B12" s="12">
         <v>433300</v>
@@ -7617,7 +7715,7 @@
         <v>7</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1">
@@ -7643,7 +7741,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="16"/>
       <c r="B13" s="12">
         <v>431000</v>
@@ -7678,7 +7776,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="16"/>
       <c r="B14" s="12">
         <v>435600</v>
@@ -7713,7 +7811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="16"/>
       <c r="B15" s="12">
         <v>433900</v>
@@ -7748,7 +7846,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="16"/>
       <c r="B16" s="12">
         <v>433901</v>
@@ -7760,7 +7858,7 @@
         <v>12</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F16" s="1">
         <v>12</v>
@@ -7785,7 +7883,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="16"/>
       <c r="B17" s="12">
         <v>435601</v>
@@ -7820,7 +7918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="16"/>
       <c r="B18" s="12">
         <v>436104</v>
@@ -7832,7 +7930,7 @@
         <v>12</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -7841,23 +7939,23 @@
         <v>0</v>
       </c>
       <c r="H18" s="1">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I18" s="1">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J18" s="1">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L18" s="1">
         <f t="shared" si="0"/>
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="16"/>
       <c r="B19" s="12">
         <v>436148</v>
@@ -7869,7 +7967,7 @@
         <v>12</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -7895,7 +7993,7 @@
       </c>
       <c r="M19" s="1"/>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="16"/>
       <c r="B20" s="12">
         <v>436167</v>
@@ -7907,7 +8005,7 @@
         <v>12</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F20" s="1">
         <v>8</v>
@@ -7932,7 +8030,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="16"/>
       <c r="B21" s="12">
         <v>431100</v>
@@ -7967,13 +8065,13 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="16"/>
       <c r="B22" s="12">
         <v>434000</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>29</v>
@@ -7983,28 +8081,28 @@
         <v>0</v>
       </c>
       <c r="G22" s="1">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="H22" s="1">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="I22" s="1">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J22" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K22" s="1">
         <v>3</v>
       </c>
       <c r="L22" s="1">
         <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B23" s="12">
         <v>431300</v>
@@ -8039,161 +8137,161 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B24"/>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B25"/>
       <c r="K25" t="s">
         <v>5</v>
       </c>
       <c r="L25" s="25">
         <f>SUM(L4:L24)</f>
-        <v>3010</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13">
+        <v>2911</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B26"/>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B27"/>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B28"/>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B29"/>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B30"/>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B31"/>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B32"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B34"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B35"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B36"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B37"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B38"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B39"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B40"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B41"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B42"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B43"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B44"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B45"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B46"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B47"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B48"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B54"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B55"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B56"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B57"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B58"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B59"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B60"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B61"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B62"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B63"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B64"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B65"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B66"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B67"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B68"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B69"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B70"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B71"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B72"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B73"/>
     </row>
   </sheetData>
@@ -8207,18 +8305,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8366,13 +8464,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar stock desde inventario OneDrive
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5744" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{221A2367-9071-4A25-BAED-758C850E60ED}"/>
+  <xr:revisionPtr revIDLastSave="5746" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2118AE89-3CE6-4A46-92AE-CB2E2DC6AB13}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -6476,6 +6476,7 @@
       </c>
     </row>
     <row r="29" spans="1:15">
+      <c r="A29" s="9"/>
       <c r="B29" s="13">
         <v>422700</v>
       </c>
@@ -6962,6 +6963,7 @@
       </c>
     </row>
     <row r="43" spans="1:12">
+      <c r="A43" s="9"/>
       <c r="B43" s="13">
         <v>421402</v>
       </c>

</xml_diff>

<commit_message>
Auto-actualizar web con TRAZABILIDAD2.CSV
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6133" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E50B3D8-3D92-4E75-92C0-66E6EB640488}"/>
+  <xr:revisionPtr revIDLastSave="6136" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2183FD87-D6AE-423F-B199-494A5A32D221}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -1413,21 +1413,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1444,6 +1429,21 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -1852,7 +1852,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.600000000000001">
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="88" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="93"/>
@@ -2668,19 +2668,19 @@
   <sheetData>
     <row r="2" spans="2:15" ht="15"/>
     <row r="3" spans="2:15" ht="15">
-      <c r="B3" s="82" t="s">
+      <c r="B3" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="83"/>
-      <c r="L3" s="84"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="91"/>
       <c r="N3" s="64">
         <v>46029</v>
       </c>
@@ -3254,7 +3254,7 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15"/>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="92" t="s">
         <v>44</v>
       </c>
       <c r="C3" s="94"/>
@@ -3632,7 +3632,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.600000000000001">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="92" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="94"/>
@@ -5239,7 +5239,7 @@
   <sheetData>
     <row r="2" spans="2:14" ht="15"/>
     <row r="3" spans="2:14" ht="18.75">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="92" t="s">
         <v>112</v>
       </c>
       <c r="C3" s="94"/>
@@ -8609,7 +8609,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:Q88"/>
+  <dimension ref="B3:Q89"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="7.7109375" style="8" customWidth="1"/>
@@ -8651,13 +8651,13 @@
       <c r="L3" s="3">
         <v>44</v>
       </c>
-      <c r="M3" s="88">
+      <c r="M3" s="83">
         <v>46</v>
       </c>
-      <c r="N3" s="87" t="s">
+      <c r="N3" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="90" t="s">
+      <c r="O3" s="85" t="s">
         <v>160</v>
       </c>
       <c r="P3" s="55" t="s">
@@ -8669,7 +8669,7 @@
     </row>
     <row r="4" spans="2:17" ht="15">
       <c r="B4" s="26"/>
-      <c r="C4" s="86">
+      <c r="C4" s="81">
         <v>430100</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -8697,14 +8697,14 @@
       <c r="L4" s="1">
         <v>51</v>
       </c>
-      <c r="M4" s="89">
+      <c r="M4" s="84">
         <v>31</v>
       </c>
       <c r="N4" s="59">
         <f>SUM(H4:M4)</f>
         <v>272</v>
       </c>
-      <c r="O4" s="91" t="s">
+      <c r="O4" s="86" t="s">
         <v>164</v>
       </c>
       <c r="P4" s="56">
@@ -8716,7 +8716,7 @@
     </row>
     <row r="5" spans="2:17" ht="15">
       <c r="B5" s="25"/>
-      <c r="C5" s="86">
+      <c r="C5" s="81">
         <v>431400</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -8744,14 +8744,14 @@
       <c r="L5" s="1">
         <v>34</v>
       </c>
-      <c r="M5" s="89">
+      <c r="M5" s="84">
         <v>36</v>
       </c>
       <c r="N5" s="59">
         <f>SUM(H5:M5)</f>
         <v>257</v>
       </c>
-      <c r="O5" s="92">
+      <c r="O5" s="87">
         <v>46208</v>
       </c>
       <c r="P5" s="56">
@@ -8763,7 +8763,7 @@
     </row>
     <row r="6" spans="2:17" ht="15">
       <c r="B6" s="27"/>
-      <c r="C6" s="86">
+      <c r="C6" s="81">
         <v>432900</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -8791,14 +8791,14 @@
       <c r="L6" s="1">
         <v>36</v>
       </c>
-      <c r="M6" s="89">
+      <c r="M6" s="84">
         <v>43</v>
       </c>
       <c r="N6" s="59">
         <f>SUM(H6:M6)</f>
         <v>251</v>
       </c>
-      <c r="O6" s="91" t="s">
+      <c r="O6" s="86" t="s">
         <v>168</v>
       </c>
       <c r="P6" s="56">
@@ -8810,7 +8810,7 @@
     </row>
     <row r="7" spans="2:17" ht="15">
       <c r="B7" s="25"/>
-      <c r="C7" s="86">
+      <c r="C7" s="81">
         <v>430900</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -8840,14 +8840,14 @@
       <c r="L7" s="1">
         <v>32</v>
       </c>
-      <c r="M7" s="89">
+      <c r="M7" s="84">
         <v>36</v>
       </c>
       <c r="N7" s="59">
         <f>SUM(H7:M7)</f>
         <v>178</v>
       </c>
-      <c r="O7" s="91" t="s">
+      <c r="O7" s="86" t="s">
         <v>171</v>
       </c>
       <c r="P7" s="13" t="s">
@@ -8859,7 +8859,7 @@
     </row>
     <row r="8" spans="2:17" ht="15">
       <c r="B8" s="28"/>
-      <c r="C8" s="86">
+      <c r="C8" s="81">
         <v>431800</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -8887,14 +8887,14 @@
       <c r="L8" s="1">
         <v>30</v>
       </c>
-      <c r="M8" s="89">
+      <c r="M8" s="84">
         <v>22</v>
       </c>
       <c r="N8" s="59">
         <f>SUM(H8:M8)</f>
         <v>171</v>
       </c>
-      <c r="O8" s="91" t="s">
+      <c r="O8" s="86" t="s">
         <v>175</v>
       </c>
       <c r="P8" s="13" t="s">
@@ -8906,7 +8906,7 @@
     </row>
     <row r="9" spans="2:17" ht="15">
       <c r="B9" s="27"/>
-      <c r="C9" s="86">
+      <c r="C9" s="81">
         <v>432100</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -8936,14 +8936,14 @@
       <c r="L9" s="1">
         <v>33</v>
       </c>
-      <c r="M9" s="89">
+      <c r="M9" s="84">
         <v>33</v>
       </c>
       <c r="N9" s="59">
         <f>SUM(H9:M9)</f>
         <v>194</v>
       </c>
-      <c r="O9" s="91" t="s">
+      <c r="O9" s="86" t="s">
         <v>179</v>
       </c>
       <c r="P9" s="13" t="s">
@@ -8955,7 +8955,7 @@
     </row>
     <row r="10" spans="2:17" ht="15">
       <c r="B10" s="25"/>
-      <c r="C10" s="86">
+      <c r="C10" s="81">
         <v>432300</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -8983,20 +8983,20 @@
       <c r="L10" s="1">
         <v>28</v>
       </c>
-      <c r="M10" s="89">
+      <c r="M10" s="84">
         <v>25</v>
       </c>
       <c r="N10" s="59">
         <f>SUM(H10:M10)</f>
         <v>149</v>
       </c>
-      <c r="O10" s="91"/>
+      <c r="O10" s="86"/>
       <c r="P10" s="13"/>
       <c r="Q10" s="54"/>
     </row>
     <row r="11" spans="2:17" ht="15">
       <c r="B11" s="25"/>
-      <c r="C11" s="86">
+      <c r="C11" s="81">
         <v>433900</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -9024,7 +9024,7 @@
       <c r="L11" s="1">
         <v>15</v>
       </c>
-      <c r="M11" s="89">
+      <c r="M11" s="84">
         <v>20</v>
       </c>
       <c r="N11" s="11">
@@ -9060,14 +9060,14 @@
       <c r="L12" s="1">
         <v>12</v>
       </c>
-      <c r="M12" s="89">
+      <c r="M12" s="84">
         <v>15</v>
       </c>
       <c r="N12" s="59">
         <f>SUM(H12:M12)</f>
         <v>93</v>
       </c>
-      <c r="O12" s="91"/>
+      <c r="O12" s="86"/>
       <c r="P12" s="13"/>
       <c r="Q12" s="54"/>
     </row>
@@ -9101,14 +9101,14 @@
       <c r="L13" s="1">
         <v>7</v>
       </c>
-      <c r="M13" s="89">
+      <c r="M13" s="84">
         <v>14</v>
       </c>
       <c r="N13" s="59">
         <f>SUM(H13:M13)</f>
         <v>93</v>
       </c>
-      <c r="O13" s="91"/>
+      <c r="O13" s="86"/>
       <c r="P13" s="13"/>
       <c r="Q13" s="54"/>
     </row>
@@ -9140,14 +9140,14 @@
       <c r="L14" s="1">
         <v>13</v>
       </c>
-      <c r="M14" s="89">
+      <c r="M14" s="84">
         <v>5</v>
       </c>
       <c r="N14" s="59">
         <f>SUM(H14:M14)</f>
         <v>92</v>
       </c>
-      <c r="O14" s="91"/>
+      <c r="O14" s="86"/>
       <c r="P14" s="13"/>
       <c r="Q14" s="54"/>
     </row>
@@ -9181,14 +9181,14 @@
       <c r="L15" s="1">
         <v>10</v>
       </c>
-      <c r="M15" s="89">
+      <c r="M15" s="84">
         <v>9</v>
       </c>
       <c r="N15" s="59">
         <f>SUM(H15:M15)</f>
         <v>79</v>
       </c>
-      <c r="O15" s="91"/>
+      <c r="O15" s="86"/>
       <c r="P15" s="13"/>
       <c r="Q15" s="54"/>
     </row>
@@ -9220,7 +9220,7 @@
       <c r="L16" s="1">
         <v>13</v>
       </c>
-      <c r="M16" s="89">
+      <c r="M16" s="84">
         <v>24</v>
       </c>
       <c r="N16" s="11">
@@ -9258,14 +9258,14 @@
       <c r="L17" s="1">
         <v>14</v>
       </c>
-      <c r="M17" s="89">
+      <c r="M17" s="84">
         <v>13</v>
       </c>
       <c r="N17" s="59">
         <f>SUM(H17:M17)</f>
         <v>73</v>
       </c>
-      <c r="O17" s="91"/>
+      <c r="O17" s="86"/>
       <c r="P17" s="13"/>
       <c r="Q17" s="54"/>
     </row>
@@ -9297,14 +9297,14 @@
       <c r="L18" s="1">
         <v>12</v>
       </c>
-      <c r="M18" s="89">
+      <c r="M18" s="84">
         <v>18</v>
       </c>
       <c r="N18" s="59">
         <f>SUM(H18:M18)</f>
         <v>70</v>
       </c>
-      <c r="O18" s="91"/>
+      <c r="O18" s="86"/>
       <c r="P18" s="13"/>
       <c r="Q18" s="54"/>
     </row>
@@ -9338,7 +9338,7 @@
       <c r="L19" s="1">
         <v>13</v>
       </c>
-      <c r="M19" s="89">
+      <c r="M19" s="84">
         <v>12</v>
       </c>
       <c r="N19" s="11">
@@ -9374,7 +9374,7 @@
       <c r="L20" s="1">
         <v>17</v>
       </c>
-      <c r="M20" s="89">
+      <c r="M20" s="84">
         <v>0</v>
       </c>
       <c r="N20" s="11">
@@ -9384,7 +9384,7 @@
     </row>
     <row r="21" spans="2:17" s="8" customFormat="1" ht="15">
       <c r="B21" s="26"/>
-      <c r="C21" s="86">
+      <c r="C21" s="81">
         <v>431300</v>
       </c>
       <c r="D21" s="61" t="s">
@@ -9453,7 +9453,7 @@
       <c r="L22" s="1">
         <v>6</v>
       </c>
-      <c r="M22" s="89">
+      <c r="M22" s="84">
         <v>3</v>
       </c>
       <c r="N22" s="11">
@@ -9489,7 +9489,7 @@
       <c r="L23" s="1">
         <v>3</v>
       </c>
-      <c r="M23" s="89">
+      <c r="M23" s="84">
         <v>0</v>
       </c>
       <c r="N23" s="11">
@@ -9525,7 +9525,7 @@
       <c r="L24" s="1">
         <v>1</v>
       </c>
-      <c r="M24" s="89">
+      <c r="M24" s="84">
         <v>12</v>
       </c>
       <c r="N24" s="11">
@@ -9563,7 +9563,7 @@
       <c r="L25" s="1">
         <v>4</v>
       </c>
-      <c r="M25" s="89">
+      <c r="M25" s="84">
         <v>3</v>
       </c>
       <c r="N25" s="11">
@@ -9599,7 +9599,7 @@
       <c r="L26" s="1">
         <v>3</v>
       </c>
-      <c r="M26" s="89">
+      <c r="M26" s="84">
         <v>1</v>
       </c>
       <c r="N26" s="11">
@@ -9635,7 +9635,7 @@
       <c r="L27" s="1">
         <v>2</v>
       </c>
-      <c r="M27" s="89">
+      <c r="M27" s="84">
         <v>5</v>
       </c>
       <c r="N27" s="11">
@@ -9673,7 +9673,7 @@
       <c r="L28" s="1">
         <v>1</v>
       </c>
-      <c r="M28" s="89">
+      <c r="M28" s="84">
         <v>2</v>
       </c>
       <c r="N28" s="11">
@@ -9711,7 +9711,7 @@
       <c r="L29" s="1">
         <v>0</v>
       </c>
-      <c r="M29" s="89">
+      <c r="M29" s="84">
         <v>2</v>
       </c>
       <c r="N29" s="11">
@@ -9749,7 +9749,7 @@
       <c r="L30" s="1">
         <v>1</v>
       </c>
-      <c r="M30" s="89">
+      <c r="M30" s="84">
         <v>0</v>
       </c>
       <c r="N30" s="11">
@@ -9787,7 +9787,7 @@
       <c r="L31" s="1">
         <v>0</v>
       </c>
-      <c r="M31" s="89">
+      <c r="M31" s="84">
         <v>0</v>
       </c>
       <c r="N31" s="11">
@@ -9823,7 +9823,7 @@
       <c r="L32" s="1">
         <v>0</v>
       </c>
-      <c r="M32" s="89">
+      <c r="M32" s="84">
         <v>0</v>
       </c>
       <c r="N32" s="11">
@@ -9861,7 +9861,7 @@
       <c r="L33" s="1">
         <v>0</v>
       </c>
-      <c r="M33" s="89">
+      <c r="M33" s="84">
         <v>0</v>
       </c>
       <c r="N33" s="11">
@@ -9897,7 +9897,7 @@
       <c r="L34" s="1">
         <v>0</v>
       </c>
-      <c r="M34" s="89">
+      <c r="M34" s="84">
         <v>0</v>
       </c>
       <c r="N34" s="11">
@@ -9935,7 +9935,7 @@
       <c r="L35" s="1">
         <v>0</v>
       </c>
-      <c r="M35" s="89">
+      <c r="M35" s="84">
         <v>0</v>
       </c>
       <c r="N35" s="11">
@@ -9971,7 +9971,7 @@
       <c r="L36" s="1">
         <v>0</v>
       </c>
-      <c r="M36" s="89">
+      <c r="M36" s="84">
         <v>0</v>
       </c>
       <c r="N36" s="11">
@@ -10007,7 +10007,7 @@
       <c r="L37" s="1">
         <v>0</v>
       </c>
-      <c r="M37" s="89">
+      <c r="M37" s="84">
         <v>0</v>
       </c>
       <c r="N37" s="11">
@@ -10045,7 +10045,7 @@
       <c r="L38" s="1">
         <v>0</v>
       </c>
-      <c r="M38" s="89">
+      <c r="M38" s="84">
         <v>0</v>
       </c>
       <c r="N38" s="11">
@@ -10054,9 +10054,11 @@
       </c>
     </row>
     <row r="39" spans="2:14" ht="15">
+      <c r="B39"/>
       <c r="C39" s="30"/>
     </row>
     <row r="40" spans="2:14" ht="15">
+      <c r="B40"/>
       <c r="C40" s="30"/>
       <c r="M40" t="s">
         <v>5</v>
@@ -10067,148 +10069,199 @@
       </c>
     </row>
     <row r="41" spans="2:14" ht="15">
+      <c r="B41"/>
       <c r="C41" s="30"/>
     </row>
     <row r="42" spans="2:14" ht="15">
+      <c r="B42"/>
       <c r="C42" s="30"/>
     </row>
     <row r="43" spans="2:14" ht="15">
+      <c r="B43"/>
       <c r="C43" s="30"/>
     </row>
     <row r="44" spans="2:14" ht="15">
+      <c r="B44"/>
       <c r="C44" s="30"/>
     </row>
     <row r="45" spans="2:14" ht="15">
+      <c r="B45"/>
       <c r="C45" s="30"/>
     </row>
     <row r="46" spans="2:14" ht="15">
+      <c r="B46"/>
       <c r="C46" s="30"/>
     </row>
     <row r="47" spans="2:14" ht="15">
+      <c r="B47"/>
       <c r="C47" s="30"/>
     </row>
     <row r="48" spans="2:14" ht="15">
+      <c r="B48"/>
       <c r="C48" s="30"/>
     </row>
-    <row r="49" spans="3:3" ht="15">
+    <row r="49" spans="2:3" ht="15">
+      <c r="B49"/>
       <c r="C49" s="30"/>
     </row>
-    <row r="50" spans="3:3" ht="15">
+    <row r="50" spans="2:3" ht="15">
+      <c r="B50"/>
       <c r="C50" s="30"/>
     </row>
-    <row r="51" spans="3:3" ht="15">
+    <row r="51" spans="2:3" ht="15">
+      <c r="B51"/>
       <c r="C51" s="30"/>
     </row>
-    <row r="52" spans="3:3" ht="15">
+    <row r="52" spans="2:3" ht="15">
+      <c r="B52"/>
       <c r="C52" s="30"/>
     </row>
-    <row r="53" spans="3:3" ht="15">
+    <row r="53" spans="2:3" ht="15">
+      <c r="B53"/>
       <c r="C53" s="30"/>
     </row>
-    <row r="54" spans="3:3" ht="15">
+    <row r="54" spans="2:3" ht="15">
+      <c r="B54"/>
       <c r="C54" s="30"/>
     </row>
-    <row r="55" spans="3:3" ht="15">
+    <row r="55" spans="2:3" ht="15">
+      <c r="B55"/>
       <c r="C55" s="30"/>
     </row>
-    <row r="56" spans="3:3" ht="15">
+    <row r="56" spans="2:3" ht="15">
+      <c r="B56"/>
       <c r="C56" s="30"/>
     </row>
-    <row r="57" spans="3:3" ht="15">
+    <row r="57" spans="2:3" ht="15">
+      <c r="B57"/>
       <c r="C57" s="30"/>
     </row>
-    <row r="58" spans="3:3" ht="15">
+    <row r="58" spans="2:3" ht="15">
+      <c r="B58" s="30"/>
       <c r="C58" s="30"/>
     </row>
-    <row r="59" spans="3:3" ht="15">
+    <row r="59" spans="2:3" ht="15">
+      <c r="B59" s="30"/>
       <c r="C59" s="30"/>
     </row>
-    <row r="60" spans="3:3" ht="15">
+    <row r="60" spans="2:3" ht="15">
+      <c r="B60" s="30"/>
       <c r="C60" s="30"/>
     </row>
-    <row r="61" spans="3:3" ht="15">
+    <row r="61" spans="2:3" ht="15">
+      <c r="B61" s="30"/>
       <c r="C61" s="30"/>
     </row>
-    <row r="62" spans="3:3" ht="15">
+    <row r="62" spans="2:3" ht="15">
+      <c r="B62" s="30"/>
       <c r="C62" s="30"/>
     </row>
-    <row r="63" spans="3:3" ht="15">
+    <row r="63" spans="2:3" ht="15">
+      <c r="B63" s="30"/>
       <c r="C63" s="30"/>
     </row>
-    <row r="64" spans="3:3" ht="15">
+    <row r="64" spans="2:3" ht="15">
+      <c r="B64" s="30"/>
       <c r="C64" s="30"/>
     </row>
-    <row r="65" spans="3:3" ht="15">
+    <row r="65" spans="2:3" ht="15">
+      <c r="B65" s="30"/>
       <c r="C65" s="30"/>
     </row>
-    <row r="66" spans="3:3" ht="15">
+    <row r="66" spans="2:3" ht="15">
+      <c r="B66" s="30"/>
       <c r="C66" s="30"/>
     </row>
-    <row r="67" spans="3:3" ht="15">
+    <row r="67" spans="2:3" ht="15">
+      <c r="B67" s="30"/>
       <c r="C67" s="30"/>
     </row>
-    <row r="68" spans="3:3" ht="15">
+    <row r="68" spans="2:3" ht="15">
+      <c r="B68" s="30"/>
       <c r="C68" s="30"/>
     </row>
-    <row r="69" spans="3:3" ht="15">
+    <row r="69" spans="2:3" ht="15">
+      <c r="B69" s="30"/>
       <c r="C69" s="30"/>
     </row>
-    <row r="70" spans="3:3" ht="15">
+    <row r="70" spans="2:3" ht="15">
+      <c r="B70" s="30"/>
       <c r="C70" s="30"/>
     </row>
-    <row r="71" spans="3:3" ht="15">
+    <row r="71" spans="2:3" ht="15">
+      <c r="B71" s="30"/>
       <c r="C71" s="30"/>
     </row>
-    <row r="72" spans="3:3" ht="15">
+    <row r="72" spans="2:3" ht="15">
+      <c r="B72" s="30"/>
       <c r="C72" s="30"/>
     </row>
-    <row r="73" spans="3:3" ht="15">
+    <row r="73" spans="2:3" ht="15">
+      <c r="B73" s="30"/>
       <c r="C73" s="30"/>
     </row>
-    <row r="74" spans="3:3" ht="15">
+    <row r="74" spans="2:3" ht="15">
+      <c r="B74" s="30"/>
       <c r="C74" s="30"/>
     </row>
-    <row r="75" spans="3:3" ht="15">
+    <row r="75" spans="2:3" ht="15">
+      <c r="B75" s="30"/>
       <c r="C75" s="30"/>
     </row>
-    <row r="76" spans="3:3" ht="15">
+    <row r="76" spans="2:3" ht="15">
+      <c r="B76" s="30"/>
       <c r="C76" s="30"/>
     </row>
-    <row r="77" spans="3:3" ht="15">
+    <row r="77" spans="2:3" ht="15">
+      <c r="B77" s="30"/>
       <c r="C77" s="30"/>
     </row>
-    <row r="78" spans="3:3" ht="15">
+    <row r="78" spans="2:3" ht="15">
+      <c r="B78" s="30"/>
       <c r="C78" s="30"/>
     </row>
-    <row r="79" spans="3:3" ht="15">
+    <row r="79" spans="2:3" ht="15">
+      <c r="B79" s="30"/>
       <c r="C79" s="30"/>
     </row>
-    <row r="80" spans="3:3" ht="15">
+    <row r="80" spans="2:3" ht="15">
+      <c r="B80" s="30"/>
       <c r="C80" s="30"/>
     </row>
-    <row r="81" spans="3:3" ht="15">
+    <row r="81" spans="2:3" ht="15">
+      <c r="B81" s="30"/>
       <c r="C81" s="30"/>
     </row>
-    <row r="82" spans="3:3" ht="15">
+    <row r="82" spans="2:3" ht="15">
+      <c r="B82" s="30"/>
       <c r="C82" s="30"/>
     </row>
-    <row r="83" spans="3:3" ht="15">
+    <row r="83" spans="2:3" ht="15">
+      <c r="B83" s="30"/>
       <c r="C83" s="30"/>
     </row>
-    <row r="84" spans="3:3" ht="15">
+    <row r="84" spans="2:3" ht="15">
+      <c r="B84" s="30"/>
       <c r="C84" s="30"/>
     </row>
-    <row r="85" spans="3:3" ht="15">
+    <row r="85" spans="2:3" ht="15">
+      <c r="B85" s="30"/>
       <c r="C85" s="30"/>
     </row>
-    <row r="86" spans="3:3" ht="15">
+    <row r="86" spans="2:3" ht="15">
+      <c r="B86" s="30"/>
       <c r="C86" s="30"/>
     </row>
-    <row r="87" spans="3:3" ht="15">
+    <row r="87" spans="2:3" ht="15">
+      <c r="B87" s="30"/>
       <c r="C87" s="30"/>
     </row>
-    <row r="88" spans="3:3" ht="15">
+    <row r="88" spans="2:3" ht="15">
+      <c r="B88" s="30"/>
       <c r="C88" s="30"/>
+    </row>
+    <row r="89" spans="2:3">
+      <c r="B89" s="30"/>
     </row>
   </sheetData>
   <autoFilter ref="C3:N25" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
@@ -10311,21 +10364,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -10469,8 +10507,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10478,5 +10531,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
 </file>
</xml_diff>

<commit_message>
Actualizar pedidos e inventario 10-07-2026
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6136" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2183FD87-D6AE-423F-B199-494A5A32D221}"/>
+  <xr:revisionPtr revIDLastSave="6176" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C5F5BB8-13F2-4461-873E-DA2B1780F711}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
@@ -20,7 +20,8 @@
     <sheet name="COLE 41" sheetId="9" r:id="rId5"/>
     <sheet name="COLE 42" sheetId="4" r:id="rId6"/>
     <sheet name="COLE 43" sheetId="10" r:id="rId7"/>
-    <sheet name="Resumen" sheetId="11" r:id="rId8"/>
+    <sheet name="COLE 44" sheetId="12" r:id="rId8"/>
+    <sheet name="Resumen" sheetId="11" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cole 37'!$B$3:$L$3</definedName>
@@ -30,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'COLE 42'!$B$2:$L$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'COLE 43'!$C$3:$N$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cole39!$B$4:$L$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'COLE 43'!$B$2:$Q$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'COLE 43'!$A$3:$N$11</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="204">
   <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
@@ -542,6 +543,9 @@
   </si>
   <si>
     <t>ingreso bod</t>
+  </si>
+  <si>
+    <t>TRASPASAR</t>
   </si>
   <si>
     <t>MISSY PLUS</t>
@@ -1207,7 +1211,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1266,9 +1270,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1409,7 +1410,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1428,6 +1428,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1852,87 +1879,87 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.600000000000001">
-      <c r="B2" s="88" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="93"/>
-      <c r="L2" s="93"/>
+      <c r="B2" s="95" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="100"/>
+      <c r="D2" s="100"/>
+      <c r="E2" s="100"/>
+      <c r="F2" s="100"/>
+      <c r="G2" s="100"/>
+      <c r="H2" s="100"/>
+      <c r="I2" s="100"/>
+      <c r="J2" s="100"/>
+      <c r="K2" s="100"/>
+      <c r="L2" s="100"/>
     </row>
     <row r="3" spans="2:12" ht="15">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="D3" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="46" t="s">
+      <c r="E3" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="46">
+      <c r="F3" s="43">
         <v>36</v>
       </c>
-      <c r="G3" s="46">
+      <c r="G3" s="43">
         <v>38</v>
       </c>
-      <c r="H3" s="46">
+      <c r="H3" s="43">
         <v>40</v>
       </c>
-      <c r="I3" s="46">
+      <c r="I3" s="43">
         <v>42</v>
       </c>
-      <c r="J3" s="46">
+      <c r="J3" s="43">
         <v>44</v>
       </c>
-      <c r="K3" s="46">
+      <c r="K3" s="43">
         <v>46</v>
       </c>
-      <c r="L3" s="46" t="s">
+      <c r="L3" s="43" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="15">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="42" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="42" t="s">
+      <c r="C4" s="39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42">
+      <c r="E4" s="39"/>
+      <c r="F4" s="39">
         <v>18</v>
       </c>
-      <c r="G4" s="42">
+      <c r="G4" s="39">
         <v>28</v>
       </c>
-      <c r="H4" s="42">
+      <c r="H4" s="39">
         <v>9</v>
       </c>
-      <c r="I4" s="42">
+      <c r="I4" s="39">
         <v>6</v>
       </c>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="43">
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="40">
         <f t="shared" ref="L4:L31" si="0">SUM(F4:K4)</f>
         <v>61</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="15">
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="41" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1954,13 +1981,13 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="32">
+      <c r="L5" s="29">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="15">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="41" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1982,13 +2009,13 @@
       <c r="K6" s="5">
         <v>3</v>
       </c>
-      <c r="L6" s="32">
+      <c r="L6" s="29">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
     <row r="7" spans="2:12" ht="15">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="41" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -2008,13 +2035,13 @@
       <c r="K7" s="5">
         <v>8</v>
       </c>
-      <c r="L7" s="32">
+      <c r="L7" s="29">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="15">
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="41" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -2036,13 +2063,13 @@
         <v>1</v>
       </c>
       <c r="K8" s="5"/>
-      <c r="L8" s="32">
+      <c r="L8" s="29">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15">
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="41" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -2060,13 +2087,13 @@
         <v>15</v>
       </c>
       <c r="K9" s="5"/>
-      <c r="L9" s="32">
+      <c r="L9" s="29">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15">
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="41" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -2090,13 +2117,13 @@
       <c r="K10" s="5">
         <v>1</v>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="29">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="15">
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="41" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -2114,13 +2141,13 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="L11" s="32">
+      <c r="L11" s="29">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="15">
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="41" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -2140,13 +2167,13 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="L12" s="32">
+      <c r="L12" s="29">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="2:12" ht="15">
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="41" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -2168,13 +2195,13 @@
         <v>1</v>
       </c>
       <c r="K13" s="5"/>
-      <c r="L13" s="32">
+      <c r="L13" s="29">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="2:12" ht="15">
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="41" t="s">
         <v>24</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -2202,13 +2229,13 @@
       <c r="K14" s="5">
         <v>3</v>
       </c>
-      <c r="L14" s="32">
+      <c r="L14" s="29">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="2:12" ht="15">
-      <c r="B15" s="44" t="s">
+      <c r="B15" s="41" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -2228,13 +2255,13 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
-      <c r="L15" s="32">
+      <c r="L15" s="29">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="15">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="41" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -2252,13 +2279,13 @@
       <c r="K16" s="5">
         <v>11</v>
       </c>
-      <c r="L16" s="32">
+      <c r="L16" s="29">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
     <row r="17" spans="2:12" ht="15">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="41" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -2284,13 +2311,13 @@
       <c r="K17" s="5">
         <v>1</v>
       </c>
-      <c r="L17" s="32">
+      <c r="L17" s="29">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="2:12" ht="15">
-      <c r="B18" s="44" t="s">
+      <c r="B18" s="41" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -2308,13 +2335,13 @@
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
-      <c r="L18" s="32">
+      <c r="L18" s="29">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="15">
-      <c r="B19" s="44" t="s">
+      <c r="B19" s="41" t="s">
         <v>30</v>
       </c>
       <c r="C19" s="5" t="s">
@@ -2336,13 +2363,13 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
-      <c r="L19" s="32">
+      <c r="L19" s="29">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="2:12" ht="15">
-      <c r="B20" s="44" t="s">
+      <c r="B20" s="41" t="s">
         <v>31</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -2368,13 +2395,13 @@
       <c r="K20" s="5">
         <v>1</v>
       </c>
-      <c r="L20" s="32">
+      <c r="L20" s="29">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="15">
-      <c r="B21" s="44" t="s">
+      <c r="B21" s="41" t="s">
         <v>32</v>
       </c>
       <c r="C21" s="5" t="s">
@@ -2392,13 +2419,13 @@
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
-      <c r="L21" s="32">
+      <c r="L21" s="29">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="2:12" ht="15">
-      <c r="B22" s="44" t="s">
+      <c r="B22" s="41" t="s">
         <v>33</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -2416,13 +2443,13 @@
       <c r="K22" s="5">
         <v>6</v>
       </c>
-      <c r="L22" s="32">
+      <c r="L22" s="29">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
     <row r="23" spans="2:12" ht="15">
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="41" t="s">
         <v>34</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -2440,13 +2467,13 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
-      <c r="L23" s="32">
+      <c r="L23" s="29">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="24" spans="2:12" ht="15">
-      <c r="B24" s="44" t="s">
+      <c r="B24" s="41" t="s">
         <v>35</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -2464,13 +2491,13 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
-      <c r="L24" s="32">
+      <c r="L24" s="29">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="25" spans="2:12" ht="15">
-      <c r="B25" s="44" t="s">
+      <c r="B25" s="41" t="s">
         <v>36</v>
       </c>
       <c r="C25" s="5" t="s">
@@ -2488,13 +2515,13 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
-      <c r="L25" s="32">
+      <c r="L25" s="29">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="2:12" ht="15">
-      <c r="B26" s="44" t="s">
+      <c r="B26" s="41" t="s">
         <v>37</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -2512,13 +2539,13 @@
       <c r="K26" s="5">
         <v>3</v>
       </c>
-      <c r="L26" s="32">
+      <c r="L26" s="29">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
     <row r="27" spans="2:12" ht="15">
-      <c r="B27" s="44" t="s">
+      <c r="B27" s="41" t="s">
         <v>38</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -2538,13 +2565,13 @@
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
-      <c r="L27" s="32">
+      <c r="L27" s="29">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="2:12" ht="15">
-      <c r="B28" s="44" t="s">
+      <c r="B28" s="41" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="5" t="s">
@@ -2564,13 +2591,13 @@
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
-      <c r="L28" s="32">
+      <c r="L28" s="29">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="2:12" ht="15">
-      <c r="B29" s="44" t="s">
+      <c r="B29" s="41" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="5" t="s">
@@ -2586,13 +2613,13 @@
       </c>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
-      <c r="L29" s="32">
+      <c r="L29" s="29">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="2:12" ht="15">
-      <c r="B30" s="44" t="s">
+      <c r="B30" s="41" t="s">
         <v>41</v>
       </c>
       <c r="C30" s="5" t="s">
@@ -2608,31 +2635,31 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
-      <c r="L30" s="32">
+      <c r="L30" s="29">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="2:12" ht="15">
-      <c r="B31" s="45" t="s">
+      <c r="B31" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="33" t="s">
+      <c r="C31" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33">
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30">
         <v>1</v>
       </c>
-      <c r="K31" s="33"/>
-      <c r="L31" s="34">
+      <c r="K31" s="30"/>
+      <c r="L31" s="31">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -2668,97 +2695,97 @@
   <sheetData>
     <row r="2" spans="2:15" ht="15"/>
     <row r="3" spans="2:15" ht="15">
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="96" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="91"/>
-      <c r="N3" s="64">
+      <c r="C3" s="97"/>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="97"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="98"/>
+      <c r="N3" s="61">
         <v>46029</v>
       </c>
-      <c r="O3" s="65">
+      <c r="O3" s="62">
         <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="4" spans="2:15" ht="15">
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="37">
+      <c r="F4" s="34">
         <v>36</v>
       </c>
-      <c r="G4" s="37">
+      <c r="G4" s="34">
         <v>38</v>
       </c>
-      <c r="H4" s="37">
+      <c r="H4" s="34">
         <v>40</v>
       </c>
-      <c r="I4" s="37">
+      <c r="I4" s="34">
         <v>42</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="34">
         <v>44</v>
       </c>
-      <c r="K4" s="37">
+      <c r="K4" s="34">
         <v>46</v>
       </c>
-      <c r="L4" s="37" t="s">
+      <c r="L4" s="34" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="2:15" ht="15">
-      <c r="B5" s="66">
+      <c r="B5" s="63">
         <v>389201</v>
       </c>
-      <c r="C5" s="39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="39" t="s">
+      <c r="C5" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35">
+      <c r="E5" s="32"/>
+      <c r="F5" s="32">
         <v>4</v>
       </c>
-      <c r="G5" s="35">
+      <c r="G5" s="32">
         <v>29</v>
       </c>
-      <c r="H5" s="35">
+      <c r="H5" s="32">
         <v>27</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="32">
         <v>30</v>
       </c>
-      <c r="J5" s="35">
+      <c r="J5" s="32">
         <v>23</v>
       </c>
-      <c r="K5" s="35">
+      <c r="K5" s="32">
         <v>16</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L5" s="33">
         <f t="shared" ref="L5:L19" si="0">SUM(F5:K5)</f>
         <v>129</v>
       </c>
     </row>
     <row r="6" spans="2:15" ht="15">
-      <c r="B6" s="63">
+      <c r="B6" s="60">
         <v>380200</v>
       </c>
       <c r="C6" s="20" t="s">
@@ -2786,13 +2813,13 @@
       <c r="K6" s="5">
         <v>2</v>
       </c>
-      <c r="L6" s="32">
+      <c r="L6" s="29">
         <f t="shared" si="0"/>
         <v>137</v>
       </c>
     </row>
     <row r="7" spans="2:15" ht="15">
-      <c r="B7" s="68">
+      <c r="B7" s="65">
         <v>382100</v>
       </c>
       <c r="C7" s="20" t="s">
@@ -2818,13 +2845,13 @@
       <c r="K7" s="5">
         <v>0</v>
       </c>
-      <c r="L7" s="32">
+      <c r="L7" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:15" ht="15">
-      <c r="B8" s="63">
+      <c r="B8" s="60">
         <v>388000</v>
       </c>
       <c r="C8" s="20" t="s">
@@ -2852,13 +2879,13 @@
       <c r="K8" s="5">
         <v>0</v>
       </c>
-      <c r="L8" s="32">
+      <c r="L8" s="29">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:15" ht="15">
-      <c r="B9" s="63">
+      <c r="B9" s="60">
         <v>389300</v>
       </c>
       <c r="C9" s="20" t="s">
@@ -2886,13 +2913,13 @@
       <c r="K9" s="5">
         <v>18</v>
       </c>
-      <c r="L9" s="32">
+      <c r="L9" s="29">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
     </row>
     <row r="10" spans="2:15" ht="15">
-      <c r="B10" s="63">
+      <c r="B10" s="60">
         <v>385371</v>
       </c>
       <c r="C10" s="20" t="s">
@@ -2920,13 +2947,13 @@
       <c r="K10" s="5">
         <v>2</v>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="29">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
     </row>
     <row r="11" spans="2:15" ht="15">
-      <c r="B11" s="63">
+      <c r="B11" s="60">
         <v>386501</v>
       </c>
       <c r="C11" s="20" t="s">
@@ -2954,13 +2981,13 @@
       <c r="K11" s="5">
         <v>0</v>
       </c>
-      <c r="L11" s="32">
+      <c r="L11" s="29">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="2:15" ht="15">
-      <c r="B12" s="63">
+      <c r="B12" s="60">
         <v>385304</v>
       </c>
       <c r="C12" s="20" t="s">
@@ -2988,13 +3015,13 @@
       <c r="K12" s="5">
         <v>0</v>
       </c>
-      <c r="L12" s="32">
+      <c r="L12" s="29">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="2:15" ht="15">
-      <c r="B13" s="63">
+      <c r="B13" s="60">
         <v>388300</v>
       </c>
       <c r="C13" s="20" t="s">
@@ -3022,13 +3049,13 @@
       <c r="K13" s="5">
         <v>0</v>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="29">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
     <row r="14" spans="2:15" ht="15">
-      <c r="B14" s="63">
+      <c r="B14" s="60">
         <v>387900</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -3056,13 +3083,13 @@
       <c r="K14" s="5">
         <v>0</v>
       </c>
-      <c r="L14" s="32">
+      <c r="L14" s="29">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="2:15" ht="15">
-      <c r="B15" s="63">
+      <c r="B15" s="60">
         <v>385800</v>
       </c>
       <c r="C15" s="20" t="s">
@@ -3090,13 +3117,13 @@
       <c r="K15" s="5">
         <v>0</v>
       </c>
-      <c r="L15" s="32">
+      <c r="L15" s="29">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="2:15" ht="15">
-      <c r="B16" s="63">
+      <c r="B16" s="60">
         <v>381801</v>
       </c>
       <c r="C16" s="20" t="s">
@@ -3124,13 +3151,13 @@
       <c r="K16" s="5">
         <v>0</v>
       </c>
-      <c r="L16" s="32">
+      <c r="L16" s="29">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="2:12" ht="15">
-      <c r="B17" s="63">
+      <c r="B17" s="60">
         <v>389401</v>
       </c>
       <c r="C17" s="20" t="s">
@@ -3158,13 +3185,13 @@
       <c r="K17" s="5">
         <v>0</v>
       </c>
-      <c r="L17" s="32">
+      <c r="L17" s="29">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
     </row>
     <row r="18" spans="2:12" ht="15">
-      <c r="B18" s="63">
+      <c r="B18" s="60">
         <v>382101</v>
       </c>
       <c r="C18" s="20" t="s">
@@ -3192,41 +3219,41 @@
       <c r="K18" s="5">
         <v>0</v>
       </c>
-      <c r="L18" s="32">
+      <c r="L18" s="29">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="15">
-      <c r="B19" s="67">
+      <c r="B19" s="64">
         <v>389700</v>
       </c>
-      <c r="C19" s="40" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="40" t="s">
+      <c r="C19" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33">
+      <c r="E19" s="30"/>
+      <c r="F19" s="30">
         <v>6</v>
       </c>
-      <c r="G19" s="33">
-        <v>0</v>
-      </c>
-      <c r="H19" s="33">
-        <v>0</v>
-      </c>
-      <c r="I19" s="33">
-        <v>0</v>
-      </c>
-      <c r="J19" s="33">
-        <v>0</v>
-      </c>
-      <c r="K19" s="33">
-        <v>0</v>
-      </c>
-      <c r="L19" s="34">
+      <c r="G19" s="30">
+        <v>0</v>
+      </c>
+      <c r="H19" s="30">
+        <v>0</v>
+      </c>
+      <c r="I19" s="30">
+        <v>0</v>
+      </c>
+      <c r="J19" s="30">
+        <v>0</v>
+      </c>
+      <c r="K19" s="30">
+        <v>0</v>
+      </c>
+      <c r="L19" s="31">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -3254,85 +3281,85 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15"/>
     <row r="3" spans="2:12" ht="18.75">
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="95"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="102"/>
     </row>
     <row r="4" spans="2:12" ht="15">
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="50">
+      <c r="F4" s="47">
         <v>36</v>
       </c>
-      <c r="G4" s="50">
+      <c r="G4" s="47">
         <v>38</v>
       </c>
-      <c r="H4" s="50">
+      <c r="H4" s="47">
         <v>40</v>
       </c>
-      <c r="I4" s="50">
+      <c r="I4" s="47">
         <v>42</v>
       </c>
-      <c r="J4" s="50">
+      <c r="J4" s="47">
         <v>44</v>
       </c>
-      <c r="K4" s="50">
+      <c r="K4" s="47">
         <v>46</v>
       </c>
-      <c r="L4" s="51" t="s">
+      <c r="L4" s="48" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="15">
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35">
+      <c r="E5" s="32"/>
+      <c r="F5" s="32">
         <v>15</v>
       </c>
-      <c r="G5" s="35">
+      <c r="G5" s="32">
         <v>15</v>
       </c>
-      <c r="H5" s="35">
+      <c r="H5" s="32">
         <v>19</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="32">
         <v>20</v>
       </c>
-      <c r="J5" s="35">
+      <c r="J5" s="32">
         <v>15</v>
       </c>
-      <c r="K5" s="35">
+      <c r="K5" s="32">
         <v>11</v>
       </c>
-      <c r="L5" s="35">
+      <c r="L5" s="32">
         <f t="shared" ref="L5:L15" si="0">SUM(F5:K5)</f>
         <v>95</v>
       </c>
@@ -3632,19 +3659,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.600000000000001">
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="99" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="95"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="102"/>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="21" t="s">
@@ -5239,55 +5266,55 @@
   <sheetData>
     <row r="2" spans="2:14" ht="15"/>
     <row r="3" spans="2:14" ht="18.75">
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="95"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="102"/>
     </row>
     <row r="4" spans="2:14" ht="15">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="52">
+      <c r="F4" s="49">
         <v>36</v>
       </c>
-      <c r="G4" s="52">
+      <c r="G4" s="49">
         <v>38</v>
       </c>
-      <c r="H4" s="52">
+      <c r="H4" s="49">
         <v>40</v>
       </c>
-      <c r="I4" s="52">
+      <c r="I4" s="49">
         <v>42</v>
       </c>
-      <c r="J4" s="52">
+      <c r="J4" s="49">
         <v>44</v>
       </c>
-      <c r="K4" s="52">
+      <c r="K4" s="49">
         <v>46</v>
       </c>
-      <c r="L4" s="52" t="s">
+      <c r="L4" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="64">
+      <c r="M4" s="61">
         <v>46029</v>
       </c>
       <c r="N4" t="s">
@@ -5295,10 +5322,10 @@
       </c>
     </row>
     <row r="5" spans="2:14" ht="15">
-      <c r="B5" s="69" t="s">
+      <c r="B5" s="66" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="75" t="s">
+      <c r="C5" s="72" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -5329,46 +5356,46 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="15">
-      <c r="B6" s="70" t="s">
+      <c r="B6" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="C6" s="76" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="71" t="s">
+      <c r="C6" s="73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="E6" s="71" t="s">
+      <c r="E6" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="71">
+      <c r="F6" s="68">
         <v>5</v>
       </c>
-      <c r="G6" s="71">
+      <c r="G6" s="68">
         <v>11</v>
       </c>
-      <c r="H6" s="71">
+      <c r="H6" s="68">
         <v>12</v>
       </c>
-      <c r="I6" s="71">
+      <c r="I6" s="68">
         <v>6</v>
       </c>
-      <c r="J6" s="71">
+      <c r="J6" s="68">
         <v>6</v>
       </c>
-      <c r="K6" s="71">
+      <c r="K6" s="68">
         <v>2</v>
       </c>
-      <c r="L6" s="71">
+      <c r="L6" s="68">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="2:14" ht="15">
-      <c r="B7" s="69" t="s">
+      <c r="B7" s="66" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="77" t="s">
+      <c r="C7" s="74" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="12" t="s">
@@ -5399,10 +5426,10 @@
       </c>
     </row>
     <row r="8" spans="2:14" ht="15">
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="66" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="77" t="s">
+      <c r="C8" s="74" t="s">
         <v>119</v>
       </c>
       <c r="D8" s="12" t="s">
@@ -5433,10 +5460,10 @@
       </c>
     </row>
     <row r="9" spans="2:14" ht="15">
-      <c r="B9" s="69" t="s">
+      <c r="B9" s="66" t="s">
         <v>120</v>
       </c>
-      <c r="C9" s="77" t="s">
+      <c r="C9" s="74" t="s">
         <v>119</v>
       </c>
       <c r="D9" s="12" t="s">
@@ -5472,7 +5499,7 @@
       <c r="B10" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="C10" s="78" t="s">
+      <c r="C10" s="75" t="s">
         <v>119</v>
       </c>
       <c r="D10" s="11" t="s">
@@ -5503,7 +5530,7 @@
       </c>
     </row>
     <row r="11" spans="2:14" ht="15">
-      <c r="B11" s="69" t="s">
+      <c r="B11" s="66" t="s">
         <v>123</v>
       </c>
       <c r="C11" s="12" t="s">
@@ -5537,7 +5564,7 @@
       </c>
     </row>
     <row r="12" spans="2:14" ht="15">
-      <c r="B12" s="69" t="s">
+      <c r="B12" s="66" t="s">
         <v>124</v>
       </c>
       <c r="C12" s="12" t="s">
@@ -5571,7 +5598,7 @@
       </c>
     </row>
     <row r="13" spans="2:14" ht="15">
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="66" t="s">
         <v>125</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -5607,43 +5634,43 @@
       </c>
     </row>
     <row r="14" spans="2:14" ht="15">
-      <c r="B14" s="72" t="s">
+      <c r="B14" s="69" t="s">
         <v>127</v>
       </c>
-      <c r="C14" s="73" t="s">
+      <c r="C14" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="D14" s="73" t="s">
+      <c r="D14" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="73" t="s">
+      <c r="E14" s="70" t="s">
         <v>128</v>
       </c>
-      <c r="F14" s="73">
-        <v>0</v>
-      </c>
-      <c r="G14" s="73">
+      <c r="F14" s="70">
+        <v>0</v>
+      </c>
+      <c r="G14" s="70">
         <v>1</v>
       </c>
-      <c r="H14" s="73">
-        <v>0</v>
-      </c>
-      <c r="I14" s="73">
-        <v>0</v>
-      </c>
-      <c r="J14" s="73">
-        <v>0</v>
-      </c>
-      <c r="K14" s="73">
-        <v>0</v>
-      </c>
-      <c r="L14" s="74">
+      <c r="H14" s="70">
+        <v>0</v>
+      </c>
+      <c r="I14" s="70">
+        <v>0</v>
+      </c>
+      <c r="J14" s="70">
+        <v>0</v>
+      </c>
+      <c r="K14" s="70">
+        <v>0</v>
+      </c>
+      <c r="L14" s="71">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="2:14" ht="15">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="50" t="s">
         <v>129</v>
       </c>
       <c r="C15" s="12" t="s">
@@ -5677,10 +5704,10 @@
       </c>
     </row>
     <row r="16" spans="2:14" ht="15">
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="70" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -5711,7 +5738,7 @@
       </c>
     </row>
     <row r="17" spans="2:12" ht="15">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="50" t="s">
         <v>131</v>
       </c>
       <c r="C17" s="12" t="s">
@@ -5745,7 +5772,7 @@
       </c>
     </row>
     <row r="18" spans="2:12" ht="15">
-      <c r="B18" s="54">
+      <c r="B18" s="51">
         <v>416500</v>
       </c>
       <c r="C18" s="12" t="s">
@@ -8609,18 +8636,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
-  <dimension ref="B3:Q89"/>
+  <dimension ref="A3:BU89"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="7.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="31"/>
+    <col min="2" max="2" width="7.7109375" style="28" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="28"/>
     <col min="6" max="6" width="17" customWidth="1"/>
     <col min="7" max="7" width="16.140625" customWidth="1"/>
-    <col min="15" max="16" width="11.42578125" style="30"/>
-    <col min="17" max="17" width="15.42578125" style="30" customWidth="1"/>
+    <col min="15" max="16" width="11.42578125" style="27"/>
+    <col min="17" max="17" width="15.42578125" style="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:17" ht="15">
+    <row r="3" spans="1:17" ht="15">
       <c r="C3" s="7" t="s">
         <v>1</v>
       </c>
@@ -8651,25 +8678,30 @@
       <c r="L3" s="3">
         <v>44</v>
       </c>
-      <c r="M3" s="83">
+      <c r="M3" s="79">
         <v>46</v>
       </c>
-      <c r="N3" s="82" t="s">
+      <c r="N3" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="85" t="s">
+      <c r="O3" s="81" t="s">
         <v>160</v>
       </c>
-      <c r="P3" s="55" t="s">
+      <c r="P3" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="Q3" s="58" t="s">
+      <c r="Q3" s="55" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="15">
-      <c r="B4" s="26"/>
-      <c r="C4" s="81">
+    <row r="4" spans="1:17" ht="15">
+      <c r="A4" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="94">
+        <v>44</v>
+      </c>
+      <c r="C4" s="77">
         <v>430100</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -8680,43 +8712,48 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="H4" s="1">
+        <v>11</v>
+      </c>
+      <c r="I4" s="1">
+        <v>57</v>
+      </c>
+      <c r="J4" s="1">
+        <v>48</v>
+      </c>
+      <c r="K4" s="1">
+        <v>50</v>
+      </c>
+      <c r="L4" s="1">
+        <v>45</v>
+      </c>
+      <c r="M4" s="80">
+        <v>29</v>
+      </c>
+      <c r="N4" s="56">
+        <f>SUM(H4:M4)</f>
+        <v>240</v>
+      </c>
+      <c r="O4" s="82" t="s">
+        <v>165</v>
+      </c>
+      <c r="P4" s="53">
+        <v>46178</v>
+      </c>
+      <c r="Q4" s="54">
+        <v>46361</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="15">
+      <c r="A5" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="H4" s="1">
-        <v>13</v>
-      </c>
-      <c r="I4" s="1">
-        <v>61</v>
-      </c>
-      <c r="J4" s="1">
-        <v>58</v>
-      </c>
-      <c r="K4" s="1">
-        <v>58</v>
-      </c>
-      <c r="L4" s="1">
-        <v>51</v>
-      </c>
-      <c r="M4" s="84">
-        <v>31</v>
-      </c>
-      <c r="N4" s="59">
-        <f>SUM(H4:M4)</f>
-        <v>272</v>
-      </c>
-      <c r="O4" s="86" t="s">
-        <v>164</v>
-      </c>
-      <c r="P4" s="56">
-        <v>46178</v>
-      </c>
-      <c r="Q4" s="57">
-        <v>46361</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17" ht="15">
-      <c r="B5" s="25"/>
-      <c r="C5" s="81">
+      <c r="B5" s="94">
+        <v>44</v>
+      </c>
+      <c r="C5" s="77">
         <v>431400</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -8727,7 +8764,7 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H5" s="1">
         <v>26</v>
@@ -8744,26 +8781,31 @@
       <c r="L5" s="1">
         <v>34</v>
       </c>
-      <c r="M5" s="84">
+      <c r="M5" s="80">
         <v>36</v>
       </c>
-      <c r="N5" s="59">
+      <c r="N5" s="56">
         <f>SUM(H5:M5)</f>
         <v>257</v>
       </c>
-      <c r="O5" s="87">
+      <c r="O5" s="83">
         <v>46208</v>
       </c>
-      <c r="P5" s="56">
+      <c r="P5" s="53">
         <v>46361</v>
       </c>
-      <c r="Q5" s="54" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" ht="15">
-      <c r="B6" s="27"/>
-      <c r="C6" s="81">
+      <c r="Q5" s="51" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="15">
+      <c r="A6" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="94">
+        <v>44</v>
+      </c>
+      <c r="C6" s="77">
         <v>432900</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -8774,43 +8816,48 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H6" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I6" s="1">
+        <v>40</v>
+      </c>
+      <c r="J6" s="1">
+        <v>47</v>
+      </c>
+      <c r="K6" s="1">
+        <v>50</v>
+      </c>
+      <c r="L6" s="1">
+        <v>30</v>
+      </c>
+      <c r="M6" s="80">
+        <v>41</v>
+      </c>
+      <c r="N6" s="56">
+        <f>SUM(H6:M6)</f>
+        <v>219</v>
+      </c>
+      <c r="O6" s="82" t="s">
+        <v>169</v>
+      </c>
+      <c r="P6" s="53">
+        <v>46178</v>
+      </c>
+      <c r="Q6" s="51" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="15">
+      <c r="A7" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" s="94">
         <v>44</v>
       </c>
-      <c r="J6" s="1">
-        <v>57</v>
-      </c>
-      <c r="K6" s="1">
-        <v>58</v>
-      </c>
-      <c r="L6" s="1">
-        <v>36</v>
-      </c>
-      <c r="M6" s="84">
-        <v>43</v>
-      </c>
-      <c r="N6" s="59">
-        <f>SUM(H6:M6)</f>
-        <v>251</v>
-      </c>
-      <c r="O6" s="86" t="s">
-        <v>168</v>
-      </c>
-      <c r="P6" s="56">
-        <v>46178</v>
-      </c>
-      <c r="Q6" s="54" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" ht="15">
-      <c r="B7" s="25"/>
-      <c r="C7" s="81">
+      <c r="C7" s="77">
         <v>430900</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -8820,10 +8867,10 @@
         <v>12</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
@@ -8840,73 +8887,83 @@
       <c r="L7" s="1">
         <v>32</v>
       </c>
-      <c r="M7" s="84">
+      <c r="M7" s="80">
         <v>36</v>
       </c>
-      <c r="N7" s="59">
+      <c r="N7" s="56">
         <f>SUM(H7:M7)</f>
         <v>178</v>
       </c>
-      <c r="O7" s="86" t="s">
-        <v>171</v>
+      <c r="O7" s="82" t="s">
+        <v>172</v>
       </c>
       <c r="P7" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q7" s="54" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="8" spans="2:17" ht="15">
-      <c r="B8" s="28"/>
-      <c r="C8" s="81">
+      <c r="Q7" s="51" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="15">
+      <c r="A8" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="94">
+        <v>44</v>
+      </c>
+      <c r="C8" s="77">
         <v>431800</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="H8" s="1">
+        <v>11</v>
+      </c>
+      <c r="I8" s="1">
+        <v>37</v>
+      </c>
+      <c r="J8" s="1">
+        <v>26</v>
+      </c>
+      <c r="K8" s="1">
+        <v>21</v>
+      </c>
+      <c r="L8" s="1">
+        <v>24</v>
+      </c>
+      <c r="M8" s="80">
+        <v>20</v>
+      </c>
+      <c r="N8" s="56">
+        <f>SUM(H8:M8)</f>
+        <v>139</v>
+      </c>
+      <c r="O8" s="82" t="s">
+        <v>176</v>
+      </c>
+      <c r="P8" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q8" s="51" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="15">
+      <c r="A9" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="H8" s="1">
-        <v>13</v>
-      </c>
-      <c r="I8" s="1">
-        <v>41</v>
-      </c>
-      <c r="J8" s="1">
-        <v>36</v>
-      </c>
-      <c r="K8" s="1">
-        <v>29</v>
-      </c>
-      <c r="L8" s="1">
-        <v>30</v>
-      </c>
-      <c r="M8" s="84">
-        <v>22</v>
-      </c>
-      <c r="N8" s="59">
-        <f>SUM(H8:M8)</f>
-        <v>171</v>
-      </c>
-      <c r="O8" s="86" t="s">
-        <v>175</v>
-      </c>
-      <c r="P8" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q8" s="54" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" ht="15">
-      <c r="B9" s="27"/>
-      <c r="C9" s="81">
+      <c r="B9" s="94">
+        <v>44</v>
+      </c>
+      <c r="C9" s="77">
         <v>432100</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -8916,10 +8973,10 @@
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H9" s="1">
         <v>8</v>
@@ -8936,37 +8993,42 @@
       <c r="L9" s="1">
         <v>33</v>
       </c>
-      <c r="M9" s="84">
+      <c r="M9" s="80">
         <v>33</v>
       </c>
-      <c r="N9" s="59">
+      <c r="N9" s="56">
         <f>SUM(H9:M9)</f>
         <v>194</v>
       </c>
-      <c r="O9" s="86" t="s">
-        <v>179</v>
+      <c r="O9" s="82" t="s">
+        <v>180</v>
       </c>
       <c r="P9" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="Q9" s="54" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="10" spans="2:17" ht="15">
-      <c r="B10" s="25"/>
-      <c r="C10" s="81">
+      <c r="Q9" s="51" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="15">
+      <c r="A10" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="94">
+        <v>44</v>
+      </c>
+      <c r="C10" s="77">
         <v>432300</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H10" s="1">
         <v>10</v>
@@ -8983,20 +9045,25 @@
       <c r="L10" s="1">
         <v>28</v>
       </c>
-      <c r="M10" s="84">
+      <c r="M10" s="80">
         <v>25</v>
       </c>
-      <c r="N10" s="59">
+      <c r="N10" s="56">
         <f>SUM(H10:M10)</f>
         <v>149</v>
       </c>
-      <c r="O10" s="86"/>
+      <c r="O10" s="82"/>
       <c r="P10" s="13"/>
-      <c r="Q10" s="54"/>
-    </row>
-    <row r="11" spans="2:17" ht="15">
-      <c r="B11" s="25"/>
-      <c r="C11" s="81">
+      <c r="Q10" s="51"/>
+    </row>
+    <row r="11" spans="1:17" ht="15">
+      <c r="A11" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="94">
+        <v>44</v>
+      </c>
+      <c r="C11" s="77">
         <v>433900</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -9007,7 +9074,7 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H11" s="1">
         <v>8</v>
@@ -9024,7 +9091,7 @@
       <c r="L11" s="1">
         <v>15</v>
       </c>
-      <c r="M11" s="84">
+      <c r="M11" s="80">
         <v>20</v>
       </c>
       <c r="N11" s="11">
@@ -9032,9 +9099,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="15">
-      <c r="B12" s="79"/>
-      <c r="C12" s="29">
+    <row r="12" spans="1:17" ht="15">
+      <c r="B12" s="91"/>
+      <c r="C12" s="26">
         <v>431100</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -9060,20 +9127,20 @@
       <c r="L12" s="1">
         <v>12</v>
       </c>
-      <c r="M12" s="84">
+      <c r="M12" s="80">
         <v>15</v>
       </c>
-      <c r="N12" s="59">
+      <c r="N12" s="56">
         <f>SUM(H12:M12)</f>
         <v>93</v>
       </c>
-      <c r="O12" s="86"/>
+      <c r="O12" s="82"/>
       <c r="P12" s="13"/>
-      <c r="Q12" s="54"/>
-    </row>
-    <row r="13" spans="2:17" ht="15">
-      <c r="B13" s="25"/>
-      <c r="C13" s="29">
+      <c r="Q12" s="51"/>
+    </row>
+    <row r="13" spans="1:17" ht="15">
+      <c r="B13" s="88"/>
+      <c r="C13" s="26">
         <v>436204</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -9083,7 +9150,7 @@
         <v>8</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1">
@@ -9101,27 +9168,27 @@
       <c r="L13" s="1">
         <v>7</v>
       </c>
-      <c r="M13" s="84">
+      <c r="M13" s="80">
         <v>14</v>
       </c>
-      <c r="N13" s="59">
+      <c r="N13" s="56">
         <f>SUM(H13:M13)</f>
         <v>93</v>
       </c>
-      <c r="O13" s="86"/>
+      <c r="O13" s="82"/>
       <c r="P13" s="13"/>
-      <c r="Q13" s="54"/>
-    </row>
-    <row r="14" spans="2:17" ht="15">
-      <c r="B14" s="25"/>
-      <c r="C14" s="29">
+      <c r="Q13" s="51"/>
+    </row>
+    <row r="14" spans="1:17" ht="15">
+      <c r="B14" s="88"/>
+      <c r="C14" s="26">
         <v>432501</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -9140,20 +9207,20 @@
       <c r="L14" s="1">
         <v>13</v>
       </c>
-      <c r="M14" s="84">
+      <c r="M14" s="80">
         <v>5</v>
       </c>
-      <c r="N14" s="59">
+      <c r="N14" s="56">
         <f>SUM(H14:M14)</f>
         <v>92</v>
       </c>
-      <c r="O14" s="86"/>
+      <c r="O14" s="82"/>
       <c r="P14" s="13"/>
-      <c r="Q14" s="54"/>
-    </row>
-    <row r="15" spans="2:17" ht="15">
-      <c r="B15" s="25"/>
-      <c r="C15" s="29">
+      <c r="Q14" s="51"/>
+    </row>
+    <row r="15" spans="1:17" ht="15">
+      <c r="B15" s="88"/>
+      <c r="C15" s="26">
         <v>436248</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -9163,7 +9230,7 @@
         <v>8</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1">
@@ -9181,27 +9248,27 @@
       <c r="L15" s="1">
         <v>10</v>
       </c>
-      <c r="M15" s="84">
+      <c r="M15" s="80">
         <v>9</v>
       </c>
-      <c r="N15" s="59">
+      <c r="N15" s="56">
         <f>SUM(H15:M15)</f>
         <v>79</v>
       </c>
-      <c r="O15" s="86"/>
+      <c r="O15" s="82"/>
       <c r="P15" s="13"/>
-      <c r="Q15" s="54"/>
-    </row>
-    <row r="16" spans="2:17" ht="15">
-      <c r="B16" s="25"/>
-      <c r="C16" s="29">
+      <c r="Q15" s="51"/>
+    </row>
+    <row r="16" spans="1:17" ht="15">
+      <c r="B16" s="88"/>
+      <c r="C16" s="26">
         <v>432500</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -9220,7 +9287,7 @@
       <c r="L16" s="1">
         <v>13</v>
       </c>
-      <c r="M16" s="84">
+      <c r="M16" s="80">
         <v>24</v>
       </c>
       <c r="N16" s="11">
@@ -9228,9 +9295,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="2:17" ht="15">
-      <c r="B17" s="25"/>
-      <c r="C17" s="29">
+    <row r="17" spans="2:73" ht="15">
+      <c r="B17" s="88"/>
+      <c r="C17" s="26">
         <v>433700</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -9240,7 +9307,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1">
@@ -9258,27 +9325,27 @@
       <c r="L17" s="1">
         <v>14</v>
       </c>
-      <c r="M17" s="84">
+      <c r="M17" s="80">
         <v>13</v>
       </c>
-      <c r="N17" s="59">
+      <c r="N17" s="56">
         <f>SUM(H17:M17)</f>
         <v>73</v>
       </c>
-      <c r="O17" s="86"/>
+      <c r="O17" s="82"/>
       <c r="P17" s="13"/>
-      <c r="Q17" s="54"/>
-    </row>
-    <row r="18" spans="2:17" ht="15">
-      <c r="B18" s="27"/>
-      <c r="C18" s="80">
+      <c r="Q17" s="51"/>
+    </row>
+    <row r="18" spans="2:73" ht="15">
+      <c r="B18" s="89"/>
+      <c r="C18" s="76">
         <v>433300</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -9297,20 +9364,20 @@
       <c r="L18" s="1">
         <v>12</v>
       </c>
-      <c r="M18" s="84">
+      <c r="M18" s="80">
         <v>18</v>
       </c>
-      <c r="N18" s="59">
+      <c r="N18" s="56">
         <f>SUM(H18:M18)</f>
         <v>70</v>
       </c>
-      <c r="O18" s="86"/>
+      <c r="O18" s="82"/>
       <c r="P18" s="13"/>
-      <c r="Q18" s="54"/>
-    </row>
-    <row r="19" spans="2:17" ht="15">
-      <c r="B19" s="25"/>
-      <c r="C19" s="29">
+      <c r="Q18" s="51"/>
+    </row>
+    <row r="19" spans="2:73" ht="15">
+      <c r="B19" s="88"/>
+      <c r="C19" s="26">
         <v>436604</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -9338,7 +9405,7 @@
       <c r="L19" s="1">
         <v>13</v>
       </c>
-      <c r="M19" s="84">
+      <c r="M19" s="80">
         <v>12</v>
       </c>
       <c r="N19" s="11">
@@ -9346,9 +9413,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="2:17" ht="15">
-      <c r="B20" s="25"/>
-      <c r="C20" s="29">
+    <row r="20" spans="2:73" ht="15">
+      <c r="B20" s="88"/>
+      <c r="C20" s="26">
         <v>431000</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -9374,7 +9441,7 @@
       <c r="L20" s="1">
         <v>17</v>
       </c>
-      <c r="M20" s="84">
+      <c r="M20" s="80">
         <v>0</v>
       </c>
       <c r="N20" s="11">
@@ -9382,50 +9449,106 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="2:17" s="8" customFormat="1" ht="15">
-      <c r="B21" s="26"/>
-      <c r="C21" s="81">
+    <row r="21" spans="2:73" s="8" customFormat="1" ht="15">
+      <c r="B21" s="87"/>
+      <c r="C21" s="77">
         <v>431300</v>
       </c>
-      <c r="D21" s="61" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="61" t="s">
+      <c r="D21" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="F21" s="61"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61">
-        <v>0</v>
-      </c>
-      <c r="I21" s="61">
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="58">
+        <v>0</v>
+      </c>
+      <c r="I21" s="58">
         <v>2</v>
       </c>
-      <c r="J21" s="61">
+      <c r="J21" s="58">
         <v>21</v>
       </c>
-      <c r="K21" s="61">
+      <c r="K21" s="58">
         <v>5</v>
       </c>
-      <c r="L21" s="61">
-        <v>7</v>
-      </c>
-      <c r="M21" s="60">
+      <c r="L21" s="58">
+        <v>7</v>
+      </c>
+      <c r="M21" s="57">
         <v>10</v>
       </c>
-      <c r="N21" s="59">
+      <c r="N21" s="56">
         <f>SUM(H21:M21)</f>
         <v>45</v>
       </c>
-      <c r="O21" s="30"/>
-      <c r="P21" s="30"/>
-      <c r="Q21" s="62" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="22" spans="2:17" ht="15">
-      <c r="B22" s="25"/>
-      <c r="C22" s="29">
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="59" t="s">
+        <v>190</v>
+      </c>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
+      <c r="W21"/>
+      <c r="X21"/>
+      <c r="Y21"/>
+      <c r="Z21"/>
+      <c r="AA21"/>
+      <c r="AB21"/>
+      <c r="AC21"/>
+      <c r="AD21"/>
+      <c r="AE21"/>
+      <c r="AF21"/>
+      <c r="AG21"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
+      <c r="AJ21"/>
+      <c r="AK21"/>
+      <c r="AL21"/>
+      <c r="AM21"/>
+      <c r="AN21"/>
+      <c r="AO21"/>
+      <c r="AP21"/>
+      <c r="AQ21"/>
+      <c r="AR21"/>
+      <c r="AS21"/>
+      <c r="AT21"/>
+      <c r="AU21"/>
+      <c r="AV21"/>
+      <c r="AW21"/>
+      <c r="AX21"/>
+      <c r="AY21"/>
+      <c r="AZ21"/>
+      <c r="BA21"/>
+      <c r="BB21"/>
+      <c r="BC21"/>
+      <c r="BD21"/>
+      <c r="BE21"/>
+      <c r="BF21"/>
+      <c r="BG21"/>
+      <c r="BH21"/>
+      <c r="BI21"/>
+      <c r="BJ21"/>
+      <c r="BK21"/>
+      <c r="BL21"/>
+      <c r="BM21"/>
+      <c r="BN21"/>
+      <c r="BO21"/>
+      <c r="BP21"/>
+      <c r="BQ21"/>
+      <c r="BR21"/>
+      <c r="BS21"/>
+      <c r="BT21"/>
+      <c r="BU21"/>
+    </row>
+    <row r="22" spans="2:73" ht="15">
+      <c r="B22" s="88"/>
+      <c r="C22" s="26">
         <v>433901</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -9435,7 +9558,7 @@
         <v>12</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1">
@@ -9453,7 +9576,7 @@
       <c r="L22" s="1">
         <v>6</v>
       </c>
-      <c r="M22" s="84">
+      <c r="M22" s="80">
         <v>3</v>
       </c>
       <c r="N22" s="11">
@@ -9461,9 +9584,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:17" ht="15">
-      <c r="B23" s="25"/>
-      <c r="C23" s="29">
+    <row r="23" spans="2:73" ht="15">
+      <c r="B23" s="88"/>
+      <c r="C23" s="26">
         <v>434000</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -9489,7 +9612,7 @@
       <c r="L23" s="1">
         <v>3</v>
       </c>
-      <c r="M23" s="84">
+      <c r="M23" s="80">
         <v>0</v>
       </c>
       <c r="N23" s="11">
@@ -9497,9 +9620,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:17" ht="15">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29">
+    <row r="24" spans="2:73" ht="15">
+      <c r="B24" s="90"/>
+      <c r="C24" s="26">
         <v>434100</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -9525,7 +9648,7 @@
       <c r="L24" s="1">
         <v>1</v>
       </c>
-      <c r="M24" s="84">
+      <c r="M24" s="80">
         <v>12</v>
       </c>
       <c r="N24" s="11">
@@ -9533,9 +9656,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="2:17" ht="15">
-      <c r="B25" s="28"/>
-      <c r="C25" s="29">
+    <row r="25" spans="2:73" ht="15">
+      <c r="B25" s="90"/>
+      <c r="C25" s="26">
         <v>434801</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -9563,7 +9686,7 @@
       <c r="L25" s="1">
         <v>4</v>
       </c>
-      <c r="M25" s="84">
+      <c r="M25" s="80">
         <v>3</v>
       </c>
       <c r="N25" s="11">
@@ -9571,8 +9694,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="2:17" ht="15">
-      <c r="B26" s="9"/>
+    <row r="26" spans="2:73" ht="15">
+      <c r="B26" s="92"/>
       <c r="C26" s="7">
         <v>431900</v>
       </c>
@@ -9599,7 +9722,7 @@
       <c r="L26" s="1">
         <v>3</v>
       </c>
-      <c r="M26" s="84">
+      <c r="M26" s="80">
         <v>1</v>
       </c>
       <c r="N26" s="11">
@@ -9607,9 +9730,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="2:17" ht="15">
-      <c r="B27" s="26"/>
-      <c r="C27" s="29">
+    <row r="27" spans="2:73" ht="15">
+      <c r="B27" s="87"/>
+      <c r="C27" s="26">
         <v>432200</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -9635,7 +9758,7 @@
       <c r="L27" s="1">
         <v>2</v>
       </c>
-      <c r="M27" s="84">
+      <c r="M27" s="80">
         <v>5</v>
       </c>
       <c r="N27" s="11">
@@ -9643,9 +9766,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="2:17" ht="15">
-      <c r="B28" s="25"/>
-      <c r="C28" s="29">
+    <row r="28" spans="2:73" ht="15">
+      <c r="B28" s="88"/>
+      <c r="C28" s="26">
         <v>434861</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -9655,7 +9778,7 @@
         <v>8</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1">
@@ -9673,7 +9796,7 @@
       <c r="L28" s="1">
         <v>1</v>
       </c>
-      <c r="M28" s="84">
+      <c r="M28" s="80">
         <v>2</v>
       </c>
       <c r="N28" s="11">
@@ -9681,8 +9804,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:17" ht="15">
-      <c r="B29" s="9"/>
+    <row r="29" spans="2:73" ht="15">
+      <c r="B29" s="92"/>
       <c r="C29" s="7">
         <v>436167</v>
       </c>
@@ -9693,7 +9816,7 @@
         <v>12</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1">
@@ -9711,7 +9834,7 @@
       <c r="L29" s="1">
         <v>0</v>
       </c>
-      <c r="M29" s="84">
+      <c r="M29" s="80">
         <v>2</v>
       </c>
       <c r="N29" s="11">
@@ -9719,9 +9842,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="2:17" ht="15">
-      <c r="B30" s="26"/>
-      <c r="C30" s="29">
+    <row r="30" spans="2:73" ht="15">
+      <c r="B30" s="87"/>
+      <c r="C30" s="26">
         <v>434860</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -9749,7 +9872,7 @@
       <c r="L30" s="1">
         <v>1</v>
       </c>
-      <c r="M30" s="84">
+      <c r="M30" s="80">
         <v>0</v>
       </c>
       <c r="N30" s="11">
@@ -9757,9 +9880,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:17" ht="15">
-      <c r="B31" s="25"/>
-      <c r="C31" s="29">
+    <row r="31" spans="2:73" ht="15">
+      <c r="B31" s="88"/>
+      <c r="C31" s="26">
         <v>436104</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -9769,7 +9892,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1">
@@ -9787,7 +9910,7 @@
       <c r="L31" s="1">
         <v>0</v>
       </c>
-      <c r="M31" s="84">
+      <c r="M31" s="80">
         <v>0</v>
       </c>
       <c r="N31" s="11">
@@ -9795,9 +9918,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="2:17" ht="15">
-      <c r="B32" s="25"/>
-      <c r="C32" s="29">
+    <row r="32" spans="2:73" ht="15">
+      <c r="B32" s="88"/>
+      <c r="C32" s="26">
         <v>432202</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -9823,7 +9946,7 @@
       <c r="L32" s="1">
         <v>0</v>
       </c>
-      <c r="M32" s="84">
+      <c r="M32" s="80">
         <v>0</v>
       </c>
       <c r="N32" s="11">
@@ -9832,8 +9955,8 @@
       </c>
     </row>
     <row r="33" spans="2:14" ht="15">
-      <c r="B33" s="25"/>
-      <c r="C33" s="29">
+      <c r="B33" s="88"/>
+      <c r="C33" s="26">
         <v>434800</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -9861,7 +9984,7 @@
       <c r="L33" s="1">
         <v>0</v>
       </c>
-      <c r="M33" s="84">
+      <c r="M33" s="80">
         <v>0</v>
       </c>
       <c r="N33" s="11">
@@ -9870,8 +9993,8 @@
       </c>
     </row>
     <row r="34" spans="2:14" ht="15">
-      <c r="B34" s="59"/>
-      <c r="C34" s="29">
+      <c r="B34" s="93"/>
+      <c r="C34" s="26">
         <v>432201</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -9897,7 +10020,7 @@
       <c r="L34" s="1">
         <v>0</v>
       </c>
-      <c r="M34" s="84">
+      <c r="M34" s="80">
         <v>0</v>
       </c>
       <c r="N34" s="11">
@@ -9906,8 +10029,8 @@
       </c>
     </row>
     <row r="35" spans="2:14" ht="15">
-      <c r="B35" s="59"/>
-      <c r="C35" s="29">
+      <c r="B35" s="93"/>
+      <c r="C35" s="26">
         <v>436148</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -9935,7 +10058,7 @@
       <c r="L35" s="1">
         <v>0</v>
       </c>
-      <c r="M35" s="84">
+      <c r="M35" s="80">
         <v>0</v>
       </c>
       <c r="N35" s="11">
@@ -9944,8 +10067,8 @@
       </c>
     </row>
     <row r="36" spans="2:14" ht="15">
-      <c r="B36" s="26"/>
-      <c r="C36" s="29">
+      <c r="B36" s="87"/>
+      <c r="C36" s="26">
         <v>435601</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -9971,7 +10094,7 @@
       <c r="L36" s="1">
         <v>0</v>
       </c>
-      <c r="M36" s="84">
+      <c r="M36" s="80">
         <v>0</v>
       </c>
       <c r="N36" s="11">
@@ -9980,8 +10103,8 @@
       </c>
     </row>
     <row r="37" spans="2:14" ht="15">
-      <c r="B37" s="59"/>
-      <c r="C37" s="29">
+      <c r="B37" s="93"/>
+      <c r="C37" s="26">
         <v>435600</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -10007,7 +10130,7 @@
       <c r="L37" s="1">
         <v>0</v>
       </c>
-      <c r="M37" s="84">
+      <c r="M37" s="80">
         <v>0</v>
       </c>
       <c r="N37" s="11">
@@ -10016,10 +10139,10 @@
       </c>
     </row>
     <row r="38" spans="2:14" ht="15">
-      <c r="B38" s="59" t="s">
+      <c r="B38" s="93" t="s">
         <v>136</v>
       </c>
-      <c r="C38" s="29">
+      <c r="C38" s="26">
         <v>432300</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -10045,7 +10168,7 @@
       <c r="L38" s="1">
         <v>0</v>
       </c>
-      <c r="M38" s="84">
+      <c r="M38" s="80">
         <v>0</v>
       </c>
       <c r="N38" s="11">
@@ -10054,214 +10177,214 @@
       </c>
     </row>
     <row r="39" spans="2:14" ht="15">
-      <c r="B39"/>
-      <c r="C39" s="30"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
     </row>
     <row r="40" spans="2:14" ht="15">
-      <c r="B40"/>
-      <c r="C40" s="30"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
       <c r="M40" t="s">
         <v>5</v>
       </c>
       <c r="N40" s="17">
         <f>SUM(N4:N39)</f>
-        <v>2443</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="41" spans="2:14" ht="15">
-      <c r="B41"/>
-      <c r="C41" s="30"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
     </row>
     <row r="42" spans="2:14" ht="15">
-      <c r="B42"/>
-      <c r="C42" s="30"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
     </row>
     <row r="43" spans="2:14" ht="15">
-      <c r="B43"/>
-      <c r="C43" s="30"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
     </row>
     <row r="44" spans="2:14" ht="15">
-      <c r="B44"/>
-      <c r="C44" s="30"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
     </row>
     <row r="45" spans="2:14" ht="15">
-      <c r="B45"/>
-      <c r="C45" s="30"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
     </row>
     <row r="46" spans="2:14" ht="15">
-      <c r="B46"/>
-      <c r="C46" s="30"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
     </row>
     <row r="47" spans="2:14" ht="15">
-      <c r="B47"/>
-      <c r="C47" s="30"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
     </row>
     <row r="48" spans="2:14" ht="15">
-      <c r="B48"/>
-      <c r="C48" s="30"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
     </row>
     <row r="49" spans="2:3" ht="15">
-      <c r="B49"/>
-      <c r="C49" s="30"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
     </row>
     <row r="50" spans="2:3" ht="15">
-      <c r="B50"/>
-      <c r="C50" s="30"/>
+      <c r="B50" s="27"/>
+      <c r="C50" s="27"/>
     </row>
     <row r="51" spans="2:3" ht="15">
-      <c r="B51"/>
-      <c r="C51" s="30"/>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
     </row>
     <row r="52" spans="2:3" ht="15">
-      <c r="B52"/>
-      <c r="C52" s="30"/>
+      <c r="B52" s="27"/>
+      <c r="C52" s="27"/>
     </row>
     <row r="53" spans="2:3" ht="15">
-      <c r="B53"/>
-      <c r="C53" s="30"/>
+      <c r="B53" s="27"/>
+      <c r="C53" s="27"/>
     </row>
     <row r="54" spans="2:3" ht="15">
-      <c r="B54"/>
-      <c r="C54" s="30"/>
+      <c r="B54" s="27"/>
+      <c r="C54" s="27"/>
     </row>
     <row r="55" spans="2:3" ht="15">
-      <c r="B55"/>
-      <c r="C55" s="30"/>
+      <c r="B55" s="27"/>
+      <c r="C55" s="27"/>
     </row>
     <row r="56" spans="2:3" ht="15">
-      <c r="B56"/>
-      <c r="C56" s="30"/>
+      <c r="B56" s="27"/>
+      <c r="C56" s="27"/>
     </row>
     <row r="57" spans="2:3" ht="15">
-      <c r="B57"/>
-      <c r="C57" s="30"/>
+      <c r="B57" s="27"/>
+      <c r="C57" s="27"/>
     </row>
     <row r="58" spans="2:3" ht="15">
-      <c r="B58" s="30"/>
-      <c r="C58" s="30"/>
+      <c r="B58" s="27"/>
+      <c r="C58" s="27"/>
     </row>
     <row r="59" spans="2:3" ht="15">
-      <c r="B59" s="30"/>
-      <c r="C59" s="30"/>
+      <c r="B59" s="27"/>
+      <c r="C59" s="27"/>
     </row>
     <row r="60" spans="2:3" ht="15">
-      <c r="B60" s="30"/>
-      <c r="C60" s="30"/>
+      <c r="B60" s="27"/>
+      <c r="C60" s="27"/>
     </row>
     <row r="61" spans="2:3" ht="15">
-      <c r="B61" s="30"/>
-      <c r="C61" s="30"/>
+      <c r="B61" s="27"/>
+      <c r="C61" s="27"/>
     </row>
     <row r="62" spans="2:3" ht="15">
-      <c r="B62" s="30"/>
-      <c r="C62" s="30"/>
+      <c r="B62" s="27"/>
+      <c r="C62" s="27"/>
     </row>
     <row r="63" spans="2:3" ht="15">
-      <c r="B63" s="30"/>
-      <c r="C63" s="30"/>
+      <c r="B63" s="27"/>
+      <c r="C63" s="27"/>
     </row>
     <row r="64" spans="2:3" ht="15">
-      <c r="B64" s="30"/>
-      <c r="C64" s="30"/>
+      <c r="B64" s="27"/>
+      <c r="C64" s="27"/>
     </row>
     <row r="65" spans="2:3" ht="15">
-      <c r="B65" s="30"/>
-      <c r="C65" s="30"/>
+      <c r="B65" s="27"/>
+      <c r="C65" s="27"/>
     </row>
     <row r="66" spans="2:3" ht="15">
-      <c r="B66" s="30"/>
-      <c r="C66" s="30"/>
+      <c r="B66" s="27"/>
+      <c r="C66" s="27"/>
     </row>
     <row r="67" spans="2:3" ht="15">
-      <c r="B67" s="30"/>
-      <c r="C67" s="30"/>
+      <c r="B67" s="27"/>
+      <c r="C67" s="27"/>
     </row>
     <row r="68" spans="2:3" ht="15">
-      <c r="B68" s="30"/>
-      <c r="C68" s="30"/>
+      <c r="B68" s="27"/>
+      <c r="C68" s="27"/>
     </row>
     <row r="69" spans="2:3" ht="15">
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
     </row>
     <row r="70" spans="2:3" ht="15">
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
     </row>
     <row r="71" spans="2:3" ht="15">
-      <c r="B71" s="30"/>
-      <c r="C71" s="30"/>
+      <c r="B71" s="27"/>
+      <c r="C71" s="27"/>
     </row>
     <row r="72" spans="2:3" ht="15">
-      <c r="B72" s="30"/>
-      <c r="C72" s="30"/>
+      <c r="B72" s="27"/>
+      <c r="C72" s="27"/>
     </row>
     <row r="73" spans="2:3" ht="15">
-      <c r="B73" s="30"/>
-      <c r="C73" s="30"/>
+      <c r="B73" s="27"/>
+      <c r="C73" s="27"/>
     </row>
     <row r="74" spans="2:3" ht="15">
-      <c r="B74" s="30"/>
-      <c r="C74" s="30"/>
+      <c r="B74" s="27"/>
+      <c r="C74" s="27"/>
     </row>
     <row r="75" spans="2:3" ht="15">
-      <c r="B75" s="30"/>
-      <c r="C75" s="30"/>
+      <c r="B75" s="27"/>
+      <c r="C75" s="27"/>
     </row>
     <row r="76" spans="2:3" ht="15">
-      <c r="B76" s="30"/>
-      <c r="C76" s="30"/>
+      <c r="B76" s="27"/>
+      <c r="C76" s="27"/>
     </row>
     <row r="77" spans="2:3" ht="15">
-      <c r="B77" s="30"/>
-      <c r="C77" s="30"/>
+      <c r="B77" s="27"/>
+      <c r="C77" s="27"/>
     </row>
     <row r="78" spans="2:3" ht="15">
-      <c r="B78" s="30"/>
-      <c r="C78" s="30"/>
+      <c r="B78" s="27"/>
+      <c r="C78" s="27"/>
     </row>
     <row r="79" spans="2:3" ht="15">
-      <c r="B79" s="30"/>
-      <c r="C79" s="30"/>
+      <c r="B79" s="27"/>
+      <c r="C79" s="27"/>
     </row>
     <row r="80" spans="2:3" ht="15">
-      <c r="B80" s="30"/>
-      <c r="C80" s="30"/>
+      <c r="B80" s="27"/>
+      <c r="C80" s="27"/>
     </row>
     <row r="81" spans="2:3" ht="15">
-      <c r="B81" s="30"/>
-      <c r="C81" s="30"/>
+      <c r="B81" s="27"/>
+      <c r="C81" s="27"/>
     </row>
     <row r="82" spans="2:3" ht="15">
-      <c r="B82" s="30"/>
-      <c r="C82" s="30"/>
+      <c r="B82" s="27"/>
+      <c r="C82" s="27"/>
     </row>
     <row r="83" spans="2:3" ht="15">
-      <c r="B83" s="30"/>
-      <c r="C83" s="30"/>
+      <c r="B83" s="27"/>
+      <c r="C83" s="27"/>
     </row>
     <row r="84" spans="2:3" ht="15">
-      <c r="B84" s="30"/>
-      <c r="C84" s="30"/>
+      <c r="B84" s="27"/>
+      <c r="C84" s="27"/>
     </row>
     <row r="85" spans="2:3" ht="15">
-      <c r="B85" s="30"/>
-      <c r="C85" s="30"/>
+      <c r="B85" s="27"/>
+      <c r="C85" s="27"/>
     </row>
     <row r="86" spans="2:3" ht="15">
-      <c r="B86" s="30"/>
-      <c r="C86" s="30"/>
+      <c r="B86" s="27"/>
+      <c r="C86" s="27"/>
     </row>
     <row r="87" spans="2:3" ht="15">
-      <c r="B87" s="30"/>
-      <c r="C87" s="30"/>
+      <c r="B87" s="27"/>
+      <c r="C87" s="27"/>
     </row>
     <row r="88" spans="2:3" ht="15">
-      <c r="B88" s="30"/>
-      <c r="C88" s="30"/>
+      <c r="B88" s="27"/>
+      <c r="C88" s="27"/>
     </row>
     <row r="89" spans="2:3">
-      <c r="B89" s="30"/>
+      <c r="B89" s="27"/>
     </row>
   </sheetData>
   <autoFilter ref="C3:N25" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
@@ -10275,32 +10398,757 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD0FCA9-A906-4FEF-9843-D37FAC686B1F}">
+  <dimension ref="B4:N52"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="4" spans="2:14">
+      <c r="C4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H4" s="3">
+        <v>36</v>
+      </c>
+      <c r="I4" s="3">
+        <v>38</v>
+      </c>
+      <c r="J4" s="3">
+        <v>40</v>
+      </c>
+      <c r="K4" s="3">
+        <v>42</v>
+      </c>
+      <c r="L4" s="3">
+        <v>44</v>
+      </c>
+      <c r="M4" s="79">
+        <v>46</v>
+      </c>
+      <c r="N4" s="78" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14">
+      <c r="B5" s="84"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="80"/>
+      <c r="N5" s="56">
+        <f>SUM(H5:M5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14">
+      <c r="B6" s="56"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="80"/>
+      <c r="N6" s="56">
+        <f>SUM(H6:M6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14">
+      <c r="B7" s="85"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="80"/>
+      <c r="N7" s="56">
+        <f>SUM(H7:M7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14">
+      <c r="B8" s="56"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="80"/>
+      <c r="N8" s="56">
+        <f>SUM(H8:M8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14">
+      <c r="B9" s="86"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="80"/>
+      <c r="N9" s="56">
+        <f>SUM(H9:M9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14">
+      <c r="B10" s="85"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="80"/>
+      <c r="N10" s="56">
+        <f>SUM(H10:M10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14">
+      <c r="B11" s="56"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="80"/>
+      <c r="N11" s="56">
+        <f>SUM(H11:M11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14">
+      <c r="B12" s="56"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="80"/>
+      <c r="N12" s="11">
+        <f>SUM(H12:M12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14">
+      <c r="B13" s="84"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="80"/>
+      <c r="N13" s="56">
+        <f>SUM(H13:M13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14">
+      <c r="B14" s="56"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="80"/>
+      <c r="N14" s="56">
+        <f>SUM(H14:M14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14">
+      <c r="B15" s="56"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="80"/>
+      <c r="N15" s="56">
+        <f>SUM(H15:M15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14">
+      <c r="B16" s="56"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="80"/>
+      <c r="N16" s="56">
+        <f>SUM(H16:M16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14">
+      <c r="B17" s="56"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="80"/>
+      <c r="N17" s="11">
+        <f>SUM(H17:M17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14">
+      <c r="B18" s="56"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="80"/>
+      <c r="N18" s="56">
+        <f>SUM(H18:M18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14">
+      <c r="B19" s="85"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="80"/>
+      <c r="N19" s="56">
+        <f>SUM(H19:M19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14">
+      <c r="B20" s="56"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="80"/>
+      <c r="N20" s="11">
+        <f t="shared" ref="N20:N21" si="0">SUM(H20:M20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14">
+      <c r="B21" s="56"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="80"/>
+      <c r="N21" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14">
+      <c r="B22" s="84"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="58"/>
+      <c r="K22" s="58"/>
+      <c r="L22" s="58"/>
+      <c r="M22" s="57"/>
+      <c r="N22" s="56">
+        <f>SUM(H22:M22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14">
+      <c r="B23" s="56"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="80"/>
+      <c r="N23" s="11">
+        <f>SUM(H23:M23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14">
+      <c r="B24" s="56"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="80"/>
+      <c r="N24" s="11">
+        <f>SUM(H24:M24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14">
+      <c r="B25" s="86"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="80"/>
+      <c r="N25" s="11">
+        <f>SUM(H25:M25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14">
+      <c r="B26" s="86"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="80"/>
+      <c r="N26" s="11">
+        <f>SUM(H26:M26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14">
+      <c r="B27" s="8"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="80"/>
+      <c r="N27" s="11">
+        <f>SUM(H27:M27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14">
+      <c r="B28" s="84"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="80"/>
+      <c r="N28" s="11">
+        <f>SUM(H28:M28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14">
+      <c r="B29" s="56"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="80"/>
+      <c r="N29" s="11">
+        <f>SUM(H29:M29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14">
+      <c r="B30" s="8"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="80"/>
+      <c r="N30" s="11">
+        <f>SUM(H30:M30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14">
+      <c r="B31" s="84"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="80"/>
+      <c r="N31" s="11">
+        <f>SUM(H31:M31)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14">
+      <c r="B32" s="56"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="80"/>
+      <c r="N32" s="11">
+        <f>SUM(H32:M32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14">
+      <c r="B33" s="56"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="80"/>
+      <c r="N33" s="11">
+        <f>SUM(H33:M33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14">
+      <c r="B34" s="56"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="80"/>
+      <c r="N34" s="11">
+        <f>SUM(H34:M34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:14">
+      <c r="B35" s="56"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="80"/>
+      <c r="N35" s="11">
+        <f>SUM(H35:M35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14">
+      <c r="B36" s="56"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="80"/>
+      <c r="N36" s="11">
+        <f>SUM(H36:M36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:14">
+      <c r="B37" s="84"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="80"/>
+      <c r="N37" s="11">
+        <f>SUM(H37:M37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14">
+      <c r="B38" s="56"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="80"/>
+      <c r="N38" s="11">
+        <f>SUM(H38:M38)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:14">
+      <c r="B39" s="56"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="80"/>
+      <c r="N39" s="11">
+        <f>SUM(H39:M39)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14">
+      <c r="B40" s="8"/>
+      <c r="C40" s="28"/>
+    </row>
+    <row r="41" spans="2:14">
+      <c r="C41" s="27"/>
+      <c r="M41" t="s">
+        <v>5</v>
+      </c>
+      <c r="N41" s="17">
+        <f>SUM(N5:N40)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14">
+      <c r="C42" s="27"/>
+    </row>
+    <row r="43" spans="2:14">
+      <c r="C43" s="27"/>
+    </row>
+    <row r="44" spans="2:14">
+      <c r="C44" s="27"/>
+    </row>
+    <row r="45" spans="2:14">
+      <c r="C45" s="27"/>
+    </row>
+    <row r="46" spans="2:14">
+      <c r="C46" s="27"/>
+    </row>
+    <row r="47" spans="2:14">
+      <c r="C47" s="27"/>
+    </row>
+    <row r="48" spans="2:14">
+      <c r="C48" s="27"/>
+    </row>
+    <row r="49" spans="3:3">
+      <c r="C49" s="27"/>
+    </row>
+    <row r="50" spans="3:3">
+      <c r="C50" s="27"/>
+    </row>
+    <row r="51" spans="3:3">
+      <c r="C51" s="27"/>
+    </row>
+    <row r="52" spans="3:3">
+      <c r="C52" s="27"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CDB450F-F8E7-45C9-9C2C-71F0E42E1F9B}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="B3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="B5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C5">
         <f>'COLE 43'!N40</f>
-        <v>2443</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="B6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C6">
         <f>'COLE 42'!L83</f>
@@ -10309,7 +11157,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="B7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C7">
         <f>'COLE 41'!L24</f>
@@ -10318,7 +11166,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="B8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C8">
         <f>'COLE 40'!L52</f>
@@ -10327,7 +11175,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="B9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C9">
         <f>cole39!L19</f>
@@ -10336,7 +11184,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="B10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C10">
         <f>'cole 38'!L22</f>
@@ -10345,7 +11193,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="B11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C11">
         <f>'cole 37'!L34</f>
@@ -10355,7 +11203,7 @@
     <row r="16" spans="1:3">
       <c r="C16">
         <f>SUM(C5:C15)</f>
-        <v>6303</v>
+        <v>6207</v>
       </c>
     </row>
   </sheetData>
@@ -10364,6 +11212,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -10507,29 +11370,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
 </file>
</xml_diff>

<commit_message>
Revertir grafico - restaurar web sin chart
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7389" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBE356FF-4435-43DF-A6BA-AB12F1304117}"/>
+  <xr:revisionPtr revIDLastSave="7666" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE97BF9F-6776-40A3-9BE2-68698F20B12E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView minimized="1" xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" firstSheet="6" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="197">
   <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
@@ -577,9 +577,6 @@
   </si>
   <si>
     <t>WIDE LEG</t>
-  </si>
-  <si>
-    <t>4370-04</t>
   </si>
   <si>
     <t>PATRICIA DARK</t>
@@ -655,6 +652,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -1274,7 +1274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1484,6 +1484,44 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1509,51 +1547,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -1961,19 +1954,19 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
     <row r="2" spans="2:12" ht="18.600000000000001">
-      <c r="B2" s="87" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="115"/>
-      <c r="L2" s="115"/>
+      <c r="B2" s="105" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
+      <c r="L2" s="110"/>
     </row>
     <row r="3" spans="2:12">
       <c r="B3" s="40" t="s">
@@ -2762,86 +2755,93 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CDB450F-F8E7-45C9-9C2C-71F0E42E1F9B}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <cols>
+    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="B3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="B3" t="s">
+    <row r="5" spans="1:5">
+      <c r="B5" t="s">
         <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="B5" t="s">
-        <v>191</v>
       </c>
       <c r="C5">
         <f>'COLE 43'!N43</f>
-        <v>1336</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="B6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C6">
         <f>'COLE 42 otoño'!L84</f>
-        <v>1682</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>1646</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="B7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C7">
         <f>'COLE 41 Alto v'!L21</f>
         <v>186</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="B8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C8">
         <f>'COLE 40 prima'!L50</f>
         <v>730</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="B9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C9">
         <f>cole39!L19</f>
         <v>289</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="B10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C10">
         <f>'cole 38'!L22</f>
         <v>588</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5">
       <c r="B11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C11">
         <f>'cole 37'!L34</f>
         <v>375</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
-      <c r="C16">
-        <f>SUM(C5:C15)</f>
-        <v>5186</v>
+    <row r="12" spans="1:5">
+      <c r="C12">
+        <f>SUM(C5:C11)</f>
+        <v>4587</v>
+      </c>
+      <c r="E12" s="100">
+        <f>C12*20000</f>
+        <v>91740000</v>
       </c>
     </row>
   </sheetData>
@@ -2864,19 +2864,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:15">
-      <c r="B3" s="88" t="s">
+      <c r="B3" s="106" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
-      <c r="K3" s="89"/>
-      <c r="L3" s="90"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="107"/>
+      <c r="L3" s="108"/>
       <c r="N3" s="52">
         <v>46029</v>
       </c>
@@ -3447,19 +3447,19 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
     <row r="3" spans="2:12" ht="18.600000000000001">
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="109" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="117"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="112"/>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="42" t="s">
@@ -3831,19 +3831,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:12" ht="18.600000000000001">
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="109" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="117"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="112"/>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="18" t="s">
@@ -5437,19 +5437,19 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:14" ht="18.600000000000001">
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="109" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="117"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="112"/>
     </row>
     <row r="4" spans="2:14">
       <c r="B4" s="46" t="s">
@@ -5992,7 +5992,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112103A-CDAB-4900-9F11-1B2050D63174}">
-  <dimension ref="A2:L132"/>
+  <dimension ref="A2:N132"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="5" max="5" width="19.140625" customWidth="1"/>
@@ -6001,19 +6001,20 @@
     <col min="8" max="8" width="8" customWidth="1"/>
     <col min="9" max="10" width="9" customWidth="1"/>
     <col min="11" max="11" width="7.5703125" customWidth="1"/>
+    <col min="14" max="14" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="18.600000000000001">
-      <c r="E2" s="84" t="s">
+      <c r="E2" s="102" t="s">
         <v>132</v>
       </c>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
-      <c r="L2" s="86"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="104"/>
     </row>
     <row r="3" spans="1:12">
       <c r="B3" s="15" t="s">
@@ -6068,23 +6069,23 @@
         <v>0</v>
       </c>
       <c r="G4" s="10">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H4" s="10">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I4" s="10">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J4" s="10">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K4" s="10">
         <v>11</v>
       </c>
       <c r="L4" s="9">
         <f t="shared" ref="L4:L35" si="0">SUM(F4:K4)</f>
-        <v>70</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -6139,7 +6140,7 @@
         <v>135</v>
       </c>
       <c r="F6" s="10">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" s="10">
         <v>28</v>
@@ -6158,7 +6159,7 @@
       </c>
       <c r="L6" s="9">
         <f t="shared" si="0"/>
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -6179,13 +6180,13 @@
         <v>9</v>
       </c>
       <c r="G7" s="10">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H7" s="10">
         <v>16</v>
       </c>
       <c r="I7" s="10">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J7" s="10">
         <v>17</v>
@@ -6195,7 +6196,7 @@
       </c>
       <c r="L7" s="9">
         <f t="shared" si="0"/>
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -6440,7 +6441,7 @@
         <v>10</v>
       </c>
       <c r="H14" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I14" s="10">
         <v>15</v>
@@ -6453,7 +6454,7 @@
       </c>
       <c r="L14" s="9">
         <f t="shared" si="0"/>
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -6480,7 +6481,7 @@
         <v>17</v>
       </c>
       <c r="I15" s="10">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J15" s="10">
         <v>14</v>
@@ -6490,7 +6491,7 @@
       </c>
       <c r="L15" s="9">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -6513,20 +6514,20 @@
         <v>0</v>
       </c>
       <c r="H16" s="10">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I16" s="10">
         <v>7</v>
       </c>
       <c r="J16" s="10">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K16" s="10">
         <v>0</v>
       </c>
       <c r="L16" s="9">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -7257,7 +7258,7 @@
         <v>12</v>
       </c>
       <c r="L36" s="9">
-        <f t="shared" ref="L36:L67" si="1">SUM(F36:K36)</f>
+        <f t="shared" ref="L36:L57" si="1">SUM(F36:K36)</f>
         <v>17</v>
       </c>
     </row>
@@ -8207,7 +8208,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I63" s="10">
         <v>1</v>
@@ -8220,7 +8221,7 @@
       </c>
       <c r="L63" s="9">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -8702,7 +8703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:12">
+    <row r="81" spans="2:14">
       <c r="B81" s="11">
         <v>420160</v>
       </c>
@@ -8726,23 +8727,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:12">
+    <row r="82" spans="2:14">
       <c r="E82" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="84" spans="2:12">
+    <row r="84" spans="2:14">
       <c r="L84" s="9">
         <f>SUM(L4:L83)</f>
-        <v>1682</v>
-      </c>
-    </row>
-    <row r="91" spans="2:12">
+        <v>1646</v>
+      </c>
+      <c r="N84" s="100"/>
+    </row>
+    <row r="91" spans="2:14">
       <c r="G91" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="92" spans="2:12">
+    <row r="92" spans="2:14">
       <c r="H92" t="s">
         <v>157</v>
       </c>
@@ -8779,7 +8781,7 @@
     <col min="3" max="3" width="9.42578125" style="25" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" customWidth="1"/>
     <col min="5" max="5" width="14.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
     <col min="7" max="7" width="14.140625" customWidth="1"/>
     <col min="8" max="13" width="7.85546875" customWidth="1"/>
     <col min="14" max="14" width="8.85546875" customWidth="1"/>
@@ -8791,22 +8793,22 @@
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
       <c r="B2"/>
-      <c r="C2" s="84" t="s">
+      <c r="C2" s="102" t="s">
         <v>158</v>
       </c>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="86"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="104"/>
       <c r="K2" s="24"/>
       <c r="L2" s="24"/>
       <c r="M2" s="24"/>
       <c r="N2" s="24"/>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" ht="14.45">
       <c r="B3"/>
       <c r="C3" s="6" t="s">
         <v>1</v>
@@ -8845,8 +8847,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
-      <c r="B4" s="96"/>
+    <row r="4" spans="1:14" ht="14.45">
+      <c r="B4" s="84"/>
       <c r="C4" s="74">
         <v>435500</v>
       </c>
@@ -8861,30 +8863,30 @@
         <v>160</v>
       </c>
       <c r="H4" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I4" s="1">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="J4" s="1">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="K4" s="1">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L4" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M4" s="69">
-        <v>10</v>
-      </c>
-      <c r="N4" s="105">
-        <f t="shared" ref="N4:N42" si="0">SUM(H4:M4)</f>
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="B5" s="96"/>
+        <v>7</v>
+      </c>
+      <c r="N4" s="9">
+        <f>SUM(H4:M4)</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="14.45">
+      <c r="B5" s="84"/>
       <c r="C5" s="74">
         <v>438000</v>
       </c>
@@ -8899,30 +8901,30 @@
         <v>162</v>
       </c>
       <c r="H5" s="1">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I5" s="1">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="J5" s="1">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="K5" s="1">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="L5" s="1">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="M5" s="69">
-        <v>14</v>
-      </c>
-      <c r="N5" s="105">
-        <f t="shared" si="0"/>
-        <v>122</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="B6" s="96"/>
+        <v>5</v>
+      </c>
+      <c r="N5" s="9">
+        <f>SUM(H5:M5)</f>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="14.45">
+      <c r="B6" s="84"/>
       <c r="C6" s="74">
         <v>438002</v>
       </c>
@@ -8939,348 +8941,348 @@
         <v>162</v>
       </c>
       <c r="H6" s="1">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I6" s="1">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="J6" s="1">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="K6" s="1">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="L6" s="1">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="M6" s="69">
-        <v>7</v>
-      </c>
-      <c r="N6" s="105">
-        <f t="shared" si="0"/>
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>5</v>
+      </c>
+      <c r="N6" s="9">
+        <f>SUM(H6:M6)</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="14.45">
       <c r="A7" s="75" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="92">
+      <c r="B7" s="83">
         <v>44</v>
       </c>
-      <c r="C7" s="95">
+      <c r="C7" s="74">
         <v>433900</v>
       </c>
-      <c r="D7" s="93" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="93" t="s">
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="93"/>
-      <c r="G7" s="93" t="s">
+      <c r="F7" s="1"/>
+      <c r="G7" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="H7" s="93">
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>10</v>
+      </c>
+      <c r="J7" s="1">
+        <v>15</v>
+      </c>
+      <c r="K7" s="1">
+        <v>18</v>
+      </c>
+      <c r="L7" s="1">
+        <v>15</v>
+      </c>
+      <c r="M7" s="69">
+        <v>20</v>
+      </c>
+      <c r="N7" s="9">
+        <f>SUM(H7:M7)</f>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="14.45">
+      <c r="A8" s="85"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="74">
+        <v>436604</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0</v>
+      </c>
+      <c r="M8" s="69">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9">
+        <f>SUM(H8:M8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="14.45">
+      <c r="A9" s="85"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="74">
+        <v>436104</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1</v>
+      </c>
+      <c r="J9" s="1">
+        <v>3</v>
+      </c>
+      <c r="K9" s="1">
+        <v>5</v>
+      </c>
+      <c r="L9" s="1">
+        <v>1</v>
+      </c>
+      <c r="M9" s="69">
+        <v>4</v>
+      </c>
+      <c r="N9" s="9">
+        <f>SUM(H9:M9)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="14.45">
+      <c r="A10" s="85"/>
+      <c r="B10" s="84"/>
+      <c r="C10" s="74">
+        <v>437801</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>0</v>
+      </c>
+      <c r="M10" s="69">
+        <v>0</v>
+      </c>
+      <c r="N10" s="9">
+        <f>SUM(H10:M10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="14.45">
+      <c r="A11" s="85"/>
+      <c r="B11" s="84"/>
+      <c r="C11" s="74">
+        <v>433300</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1</v>
+      </c>
+      <c r="L11" s="1">
+        <v>10</v>
+      </c>
+      <c r="M11" s="69">
+        <v>16</v>
+      </c>
+      <c r="N11" s="9">
+        <f>SUM(H11:M11)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="14.45">
+      <c r="A12" s="85"/>
+      <c r="B12" s="84"/>
+      <c r="C12" s="74">
+        <v>436648</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1">
+        <v>9</v>
+      </c>
+      <c r="I12" s="1">
+        <v>12</v>
+      </c>
+      <c r="J12" s="1">
         <v>8</v>
       </c>
-      <c r="I7" s="93">
-        <v>20</v>
-      </c>
-      <c r="J7" s="93">
-        <v>20</v>
-      </c>
-      <c r="K7" s="93">
+      <c r="K12" s="1">
+        <v>8</v>
+      </c>
+      <c r="L12" s="1">
+        <v>6</v>
+      </c>
+      <c r="M12" s="69">
+        <v>9</v>
+      </c>
+      <c r="N12" s="9">
+        <f>SUM(H12:M12)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="14.45">
+      <c r="A13" s="85"/>
+      <c r="B13" s="84"/>
+      <c r="C13" s="74">
+        <v>435601</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>9</v>
+      </c>
+      <c r="J13" s="1">
         <v>18</v>
       </c>
-      <c r="L7" s="93">
+      <c r="K13" s="1">
+        <v>5</v>
+      </c>
+      <c r="L13" s="1">
         <v>15</v>
       </c>
-      <c r="M7" s="94">
-        <v>20</v>
-      </c>
-      <c r="N7" s="105">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="97"/>
-      <c r="B8" s="96"/>
-      <c r="C8" s="95">
-        <v>436604</v>
-      </c>
-      <c r="D8" s="93" t="s">
+      <c r="M13" s="69">
+        <v>4</v>
+      </c>
+      <c r="N13" s="9">
+        <f>SUM(H13:M13)</f>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="14.45">
+      <c r="A14" s="85"/>
+      <c r="B14" s="84"/>
+      <c r="C14" s="88">
+        <v>432301</v>
+      </c>
+      <c r="D14" s="89" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="93" t="s">
+      <c r="E14" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="93" t="s">
-        <v>166</v>
-      </c>
-      <c r="G8" s="93" t="s">
-        <v>167</v>
-      </c>
-      <c r="H8" s="93">
-        <v>11</v>
-      </c>
-      <c r="I8" s="93">
-        <v>16</v>
-      </c>
-      <c r="J8" s="93">
-        <v>11</v>
-      </c>
-      <c r="K8" s="93">
-        <v>12</v>
-      </c>
-      <c r="L8" s="93">
-        <v>6</v>
-      </c>
-      <c r="M8" s="94">
-        <v>10</v>
-      </c>
-      <c r="N8" s="105">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="97"/>
-      <c r="B9" s="96"/>
-      <c r="C9" s="95">
-        <v>436104</v>
-      </c>
-      <c r="D9" s="93" t="s">
-        <v>119</v>
-      </c>
-      <c r="E9" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="93" t="s">
-        <v>153</v>
-      </c>
-      <c r="G9" s="93" t="s">
-        <v>167</v>
-      </c>
-      <c r="H9" s="93">
-        <v>10</v>
-      </c>
-      <c r="I9" s="93">
-        <v>11</v>
-      </c>
-      <c r="J9" s="93">
-        <v>11</v>
-      </c>
-      <c r="K9" s="93">
-        <v>10</v>
-      </c>
-      <c r="L9" s="93">
-        <v>12</v>
-      </c>
-      <c r="M9" s="94">
-        <v>8</v>
-      </c>
-      <c r="N9" s="105">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="97"/>
-      <c r="B10" s="96"/>
-      <c r="C10" s="95">
-        <v>437801</v>
-      </c>
-      <c r="D10" s="93" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" s="93" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
-      <c r="H10" s="93">
-        <v>9</v>
-      </c>
-      <c r="I10" s="93">
-        <v>11</v>
-      </c>
-      <c r="J10" s="93">
-        <v>13</v>
-      </c>
-      <c r="K10" s="93">
-        <v>11</v>
-      </c>
-      <c r="L10" s="93">
-        <v>8</v>
-      </c>
-      <c r="M10" s="94">
-        <v>7</v>
-      </c>
-      <c r="N10" s="105">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="97"/>
-      <c r="B11" s="96"/>
-      <c r="C11" s="95">
-        <v>433300</v>
-      </c>
-      <c r="D11" s="93" t="s">
-        <v>119</v>
-      </c>
-      <c r="E11" s="93" t="s">
-        <v>168</v>
-      </c>
-      <c r="F11" s="93"/>
-      <c r="G11" s="93" t="s">
-        <v>169</v>
-      </c>
-      <c r="H11" s="93">
-        <v>0</v>
-      </c>
-      <c r="I11" s="93">
-        <v>11</v>
-      </c>
-      <c r="J11" s="93">
-        <v>10</v>
-      </c>
-      <c r="K11" s="93">
-        <v>7</v>
-      </c>
-      <c r="L11" s="93">
-        <v>10</v>
-      </c>
-      <c r="M11" s="94">
-        <v>17</v>
-      </c>
-      <c r="N11" s="105">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="97"/>
-      <c r="B12" s="96"/>
-      <c r="C12" s="95">
-        <v>436648</v>
-      </c>
-      <c r="D12" s="93" t="s">
-        <v>119</v>
-      </c>
-      <c r="E12" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="93" t="s">
-        <v>151</v>
-      </c>
-      <c r="G12" s="93"/>
-      <c r="H12" s="93">
-        <v>9</v>
-      </c>
-      <c r="I12" s="93">
-        <v>12</v>
-      </c>
-      <c r="J12" s="93">
-        <v>8</v>
-      </c>
-      <c r="K12" s="93">
-        <v>8</v>
-      </c>
-      <c r="L12" s="93">
-        <v>6</v>
-      </c>
-      <c r="M12" s="94">
-        <v>9</v>
-      </c>
-      <c r="N12" s="105">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="A13" s="97"/>
-      <c r="B13" s="96"/>
-      <c r="C13" s="95">
-        <v>435601</v>
-      </c>
-      <c r="D13" s="93" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="93" t="s">
-        <v>170</v>
-      </c>
-      <c r="G13" s="93"/>
-      <c r="H13" s="93">
-        <v>0</v>
-      </c>
-      <c r="I13" s="93">
-        <v>9</v>
-      </c>
-      <c r="J13" s="93">
-        <v>18</v>
-      </c>
-      <c r="K13" s="93">
-        <v>5</v>
-      </c>
-      <c r="L13" s="93">
-        <v>15</v>
-      </c>
-      <c r="M13" s="94">
-        <v>4</v>
-      </c>
-      <c r="N13" s="105">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="97"/>
-      <c r="B14" s="96"/>
-      <c r="C14" s="100">
-        <v>432301</v>
-      </c>
-      <c r="D14" s="101" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" s="101" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="101"/>
-      <c r="G14" s="101" t="s">
+      <c r="F14" s="89"/>
+      <c r="G14" s="89" t="s">
         <v>171</v>
       </c>
-      <c r="H14" s="101">
-        <v>7</v>
-      </c>
-      <c r="I14" s="101">
-        <v>9</v>
-      </c>
-      <c r="J14" s="101">
-        <v>10</v>
-      </c>
-      <c r="K14" s="101">
-        <v>9</v>
-      </c>
-      <c r="L14" s="101">
-        <v>9</v>
-      </c>
-      <c r="M14" s="102">
-        <v>7</v>
-      </c>
-      <c r="N14" s="106">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="B15" s="98"/>
+      <c r="H14" s="89">
+        <v>0</v>
+      </c>
+      <c r="I14" s="89">
+        <v>0</v>
+      </c>
+      <c r="J14" s="89">
+        <v>0</v>
+      </c>
+      <c r="K14" s="89">
+        <v>0</v>
+      </c>
+      <c r="L14" s="89">
+        <v>0</v>
+      </c>
+      <c r="M14" s="90">
+        <v>0</v>
+      </c>
+      <c r="N14" s="87">
+        <f>SUM(H14:M14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="14.45">
+      <c r="B15" s="86"/>
       <c r="C15" s="11">
         <v>431100</v>
       </c>
@@ -9298,27 +9300,27 @@
         <v>2</v>
       </c>
       <c r="I15" s="9">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J15" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K15" s="9">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L15" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M15" s="9">
         <v>12</v>
       </c>
-      <c r="N15" s="105">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="B16" s="98"/>
+      <c r="N15" s="9">
+        <f>SUM(H15:M15)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="14.45">
+      <c r="B16" s="86"/>
       <c r="C16" s="11">
         <v>433700</v>
       </c>
@@ -9350,13 +9352,13 @@
       <c r="M16" s="9">
         <v>8</v>
       </c>
-      <c r="N16" s="105">
-        <f t="shared" si="0"/>
+      <c r="N16" s="9">
+        <f>SUM(H16:M16)</f>
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
-      <c r="B17" s="109"/>
+    <row r="17" spans="1:14" ht="14.45">
+      <c r="B17" s="94"/>
       <c r="C17" s="11">
         <v>436500</v>
       </c>
@@ -9371,68 +9373,68 @@
         <v>171</v>
       </c>
       <c r="H17" s="9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I17" s="9">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K17" s="9">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L17" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M17" s="9">
-        <v>1</v>
-      </c>
-      <c r="N17" s="105">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
-      <c r="B18" s="92"/>
-      <c r="C18" s="112">
+        <v>0</v>
+      </c>
+      <c r="N17" s="9">
+        <f>SUM(H17:M17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="14.45">
+      <c r="B18" s="83"/>
+      <c r="C18" s="96">
         <v>434000</v>
       </c>
-      <c r="D18" s="113" t="s">
+      <c r="D18" s="97" t="s">
         <v>119</v>
       </c>
-      <c r="E18" s="113" t="s">
+      <c r="E18" s="97" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="113"/>
-      <c r="G18" s="113" t="s">
+      <c r="F18" s="97"/>
+      <c r="G18" s="97" t="s">
         <v>169</v>
       </c>
-      <c r="H18" s="113">
-        <v>0</v>
-      </c>
-      <c r="I18" s="113">
-        <v>9</v>
-      </c>
-      <c r="J18" s="113">
-        <v>12</v>
-      </c>
-      <c r="K18" s="113">
-        <v>7</v>
-      </c>
-      <c r="L18" s="113">
-        <v>3</v>
-      </c>
-      <c r="M18" s="113">
-        <v>0</v>
-      </c>
-      <c r="N18" s="114">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
-      <c r="B19" s="98"/>
+      <c r="H18" s="97">
+        <v>0</v>
+      </c>
+      <c r="I18" s="97">
+        <v>0</v>
+      </c>
+      <c r="J18" s="97">
+        <v>0</v>
+      </c>
+      <c r="K18" s="97">
+        <v>0</v>
+      </c>
+      <c r="L18" s="97">
+        <v>0</v>
+      </c>
+      <c r="M18" s="97">
+        <v>0</v>
+      </c>
+      <c r="N18" s="97">
+        <f>SUM(H18:M18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="14.45">
+      <c r="B19" s="86"/>
       <c r="C19" s="11">
         <v>432500</v>
       </c>
@@ -9464,54 +9466,54 @@
       <c r="M19" s="9">
         <v>21</v>
       </c>
-      <c r="N19" s="105">
-        <f t="shared" si="0"/>
+      <c r="N19" s="9">
+        <f>SUM(H19:M19)</f>
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
-      <c r="A20" s="97"/>
-      <c r="B20" s="98"/>
-      <c r="C20" s="111">
+    <row r="20" spans="1:14" ht="14.45">
+      <c r="A20" s="85"/>
+      <c r="B20" s="86"/>
+      <c r="C20" s="11">
         <v>436248</v>
       </c>
-      <c r="D20" s="105" t="s">
+      <c r="D20" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="E20" s="105" t="s">
+      <c r="E20" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="105" t="s">
+      <c r="F20" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="G20" s="105" t="s">
+      <c r="G20" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="H20" s="105">
-        <v>0</v>
-      </c>
-      <c r="I20" s="105">
+      <c r="H20" s="9">
+        <v>0</v>
+      </c>
+      <c r="I20" s="9">
         <v>2</v>
       </c>
-      <c r="J20" s="105">
+      <c r="J20" s="9">
         <v>3</v>
       </c>
-      <c r="K20" s="105">
+      <c r="K20" s="9">
         <v>11</v>
       </c>
-      <c r="L20" s="105">
+      <c r="L20" s="9">
         <v>1</v>
       </c>
-      <c r="M20" s="105">
+      <c r="M20" s="9">
         <v>12</v>
       </c>
-      <c r="N20" s="105">
-        <f t="shared" si="0"/>
+      <c r="N20" s="9">
+        <f>SUM(H20:M20)</f>
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
-      <c r="B21" s="98"/>
+    <row r="21" spans="1:14" ht="14.45">
+      <c r="B21" s="86"/>
       <c r="C21" s="11">
         <v>436148</v>
       </c>
@@ -9541,52 +9543,52 @@
       <c r="M21" s="9">
         <v>5</v>
       </c>
-      <c r="N21" s="105">
+      <c r="N21" s="9">
         <f>SUM(H21:M21)</f>
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
-      <c r="B22" s="92"/>
-      <c r="C22" s="110" t="s">
-        <v>174</v>
-      </c>
-      <c r="D22" s="103" t="s">
+    <row r="22" spans="1:14" ht="14.45">
+      <c r="B22" s="83"/>
+      <c r="C22" s="95">
+        <v>437004</v>
+      </c>
+      <c r="D22" s="91" t="s">
         <v>119</v>
       </c>
-      <c r="E22" s="103" t="s">
+      <c r="E22" s="91" t="s">
         <v>173</v>
       </c>
-      <c r="F22" s="103"/>
-      <c r="G22" s="103" t="s">
+      <c r="F22" s="91"/>
+      <c r="G22" s="91" t="s">
         <v>167</v>
       </c>
-      <c r="H22" s="103">
+      <c r="H22" s="91">
         <v>2</v>
       </c>
-      <c r="I22" s="103">
+      <c r="I22" s="91">
         <v>5</v>
       </c>
-      <c r="J22" s="103">
-        <v>7</v>
-      </c>
-      <c r="K22" s="103">
+      <c r="J22" s="91">
+        <v>7</v>
+      </c>
+      <c r="K22" s="91">
         <v>6</v>
       </c>
-      <c r="L22" s="103">
+      <c r="L22" s="91">
         <v>4</v>
       </c>
-      <c r="M22" s="103">
+      <c r="M22" s="91">
         <v>2</v>
       </c>
-      <c r="N22" s="107">
-        <f t="shared" si="0"/>
+      <c r="N22" s="91">
+        <f>SUM(H22:M22)</f>
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
-      <c r="B23" s="92"/>
-      <c r="C23" s="104">
+    <row r="23" spans="1:14" ht="14.45">
+      <c r="B23" s="83"/>
+      <c r="C23" s="92">
         <v>436148</v>
       </c>
       <c r="D23" s="9" t="s">
@@ -9617,14 +9619,14 @@
       <c r="M23" s="9">
         <v>5</v>
       </c>
-      <c r="N23" s="105">
-        <f t="shared" si="0"/>
+      <c r="N23" s="9">
+        <f>SUM(H23:M23)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
-      <c r="B24" s="92"/>
-      <c r="C24" s="104">
+    <row r="24" spans="1:14" ht="14.45">
+      <c r="B24" s="83"/>
+      <c r="C24" s="92">
         <v>431000</v>
       </c>
       <c r="D24" s="9" t="s">
@@ -9635,7 +9637,7 @@
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H24" s="9">
         <v>0</v>
@@ -9644,7 +9646,7 @@
         <v>1</v>
       </c>
       <c r="J24" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K24" s="9">
         <v>0</v>
@@ -9655,14 +9657,14 @@
       <c r="M24" s="9">
         <v>15</v>
       </c>
-      <c r="N24" s="105">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14">
-      <c r="B25" s="92"/>
-      <c r="C25" s="104">
+      <c r="N24" s="9">
+        <f>SUM(H24:M24)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="14.45">
+      <c r="B25" s="83"/>
+      <c r="C25" s="92">
         <v>435300</v>
       </c>
       <c r="D25" s="9" t="s">
@@ -9693,14 +9695,14 @@
       <c r="M25" s="9">
         <v>3</v>
       </c>
-      <c r="N25" s="105">
-        <f t="shared" si="0"/>
+      <c r="N25" s="9">
+        <f>SUM(H25:M25)</f>
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
-      <c r="B26" s="92"/>
-      <c r="C26" s="104">
+    <row r="26" spans="1:14" ht="14.45">
+      <c r="B26" s="83"/>
+      <c r="C26" s="92">
         <v>436606</v>
       </c>
       <c r="D26" s="9" t="s">
@@ -9710,37 +9712,37 @@
         <v>22</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>167</v>
       </c>
       <c r="H26" s="9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I26" s="9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J26" s="9">
         <v>0</v>
       </c>
       <c r="K26" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L26" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" s="9">
-        <v>4</v>
-      </c>
-      <c r="N26" s="105">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14">
-      <c r="B27" s="92"/>
-      <c r="C27" s="104">
+        <v>0</v>
+      </c>
+      <c r="N26" s="9">
+        <f>SUM(H26:M26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="14.45">
+      <c r="B27" s="83"/>
+      <c r="C27" s="92">
         <v>434100</v>
       </c>
       <c r="D27" s="9" t="s">
@@ -9771,14 +9773,14 @@
       <c r="M27" s="9">
         <v>12</v>
       </c>
-      <c r="N27" s="105">
-        <f t="shared" si="0"/>
+      <c r="N27" s="9">
+        <f>SUM(H27:M27)</f>
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
-      <c r="B28" s="92"/>
-      <c r="C28" s="104">
+    <row r="28" spans="1:14" ht="14.45">
+      <c r="B28" s="83"/>
+      <c r="C28" s="92">
         <v>432100</v>
       </c>
       <c r="D28" s="9" t="s">
@@ -9809,21 +9811,21 @@
       <c r="M28" s="9">
         <v>3</v>
       </c>
-      <c r="N28" s="105">
-        <f t="shared" si="0"/>
+      <c r="N28" s="9">
+        <f>SUM(H28:M28)</f>
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
-      <c r="B29" s="92"/>
-      <c r="C29" s="104">
+    <row r="29" spans="1:14" ht="14.45">
+      <c r="B29" s="83"/>
+      <c r="C29" s="92">
         <v>431800</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>119</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9" t="s">
@@ -9833,28 +9835,28 @@
         <v>0</v>
       </c>
       <c r="I29" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J29" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K29" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L29" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M29" s="9">
-        <v>2</v>
-      </c>
-      <c r="N29" s="105">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14">
-      <c r="B30" s="92"/>
-      <c r="C30" s="104">
+        <v>0</v>
+      </c>
+      <c r="N29" s="9">
+        <f>SUM(H29:M29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="14.45">
+      <c r="B30" s="83"/>
+      <c r="C30" s="92">
         <v>433901</v>
       </c>
       <c r="D30" s="9" t="s">
@@ -9885,14 +9887,14 @@
       <c r="M30" s="9">
         <v>1</v>
       </c>
-      <c r="N30" s="105">
-        <f t="shared" si="0"/>
+      <c r="N30" s="9">
+        <f>SUM(H30:M30)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
-      <c r="B31" s="92"/>
-      <c r="C31" s="104">
+    <row r="31" spans="1:14" ht="14.45">
+      <c r="B31" s="83"/>
+      <c r="C31" s="92">
         <v>436167</v>
       </c>
       <c r="D31" s="9" t="s">
@@ -9902,7 +9904,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G31" s="9"/>
       <c r="H31" s="9">
@@ -9923,165 +9925,165 @@
       <c r="M31" s="9">
         <v>3</v>
       </c>
-      <c r="N31" s="105">
-        <f t="shared" si="0"/>
+      <c r="N31" s="9">
+        <f>SUM(H31:M31)</f>
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
-      <c r="B32" s="96"/>
-      <c r="C32" s="108">
+    <row r="32" spans="1:14" ht="14.45">
+      <c r="B32" s="84"/>
+      <c r="C32" s="93">
         <v>432200</v>
       </c>
-      <c r="D32" s="99" t="s">
+      <c r="D32" s="87" t="s">
         <v>119</v>
       </c>
-      <c r="E32" s="99" t="s">
+      <c r="E32" s="87" t="s">
         <v>12</v>
       </c>
-      <c r="F32" s="99"/>
-      <c r="G32" s="99" t="s">
+      <c r="F32" s="87"/>
+      <c r="G32" s="87" t="s">
         <v>160</v>
       </c>
-      <c r="H32" s="99">
+      <c r="H32" s="87">
         <v>3</v>
       </c>
-      <c r="I32" s="99">
-        <v>3</v>
-      </c>
-      <c r="J32" s="99">
-        <v>0</v>
-      </c>
-      <c r="K32" s="99">
-        <v>0</v>
-      </c>
-      <c r="L32" s="99">
-        <v>0</v>
-      </c>
-      <c r="M32" s="99">
+      <c r="I32" s="87">
         <v>2</v>
       </c>
-      <c r="N32" s="105">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="2:14">
-      <c r="B33" s="96"/>
-      <c r="C33" s="108">
+      <c r="J32" s="87">
+        <v>0</v>
+      </c>
+      <c r="K32" s="87">
+        <v>0</v>
+      </c>
+      <c r="L32" s="87">
+        <v>0</v>
+      </c>
+      <c r="M32" s="87">
+        <v>2</v>
+      </c>
+      <c r="N32" s="9">
+        <f>SUM(H32:M32)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14" ht="14.45">
+      <c r="B33" s="84"/>
+      <c r="C33" s="93">
         <v>431300</v>
       </c>
-      <c r="D33" s="99" t="s">
+      <c r="D33" s="87" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="99" t="s">
+      <c r="E33" s="87" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="99" t="s">
+      <c r="F33" s="87" t="s">
+        <v>178</v>
+      </c>
+      <c r="G33" s="87" t="s">
+        <v>165</v>
+      </c>
+      <c r="H33" s="87">
+        <v>0</v>
+      </c>
+      <c r="I33" s="87">
+        <v>0</v>
+      </c>
+      <c r="J33" s="87">
+        <v>4</v>
+      </c>
+      <c r="K33" s="87">
+        <v>0</v>
+      </c>
+      <c r="L33" s="87">
+        <v>0</v>
+      </c>
+      <c r="M33" s="87">
+        <v>2</v>
+      </c>
+      <c r="N33" s="9">
+        <f>SUM(H33:M33)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14" ht="14.45">
+      <c r="B34" s="84"/>
+      <c r="C34" s="93">
+        <v>435600</v>
+      </c>
+      <c r="D34" s="87" t="s">
+        <v>119</v>
+      </c>
+      <c r="E34" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" s="87"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="87">
+        <v>0</v>
+      </c>
+      <c r="I34" s="87">
+        <v>0</v>
+      </c>
+      <c r="J34" s="87">
+        <v>0</v>
+      </c>
+      <c r="K34" s="87">
+        <v>0</v>
+      </c>
+      <c r="L34" s="87">
+        <v>0</v>
+      </c>
+      <c r="M34" s="87">
+        <v>0</v>
+      </c>
+      <c r="N34" s="9">
+        <f>SUM(H34:M34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:14" ht="14.45">
+      <c r="B35" s="84"/>
+      <c r="C35" s="93">
+        <v>432261</v>
+      </c>
+      <c r="D35" s="87" t="s">
+        <v>119</v>
+      </c>
+      <c r="E35" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="87" t="s">
         <v>179</v>
       </c>
-      <c r="G33" s="99" t="s">
-        <v>165</v>
-      </c>
-      <c r="H33" s="99">
-        <v>0</v>
-      </c>
-      <c r="I33" s="99">
-        <v>0</v>
-      </c>
-      <c r="J33" s="99">
-        <v>5</v>
-      </c>
-      <c r="K33" s="99">
-        <v>0</v>
-      </c>
-      <c r="L33" s="99">
-        <v>0</v>
-      </c>
-      <c r="M33" s="99">
-        <v>2</v>
-      </c>
-      <c r="N33" s="105">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="2:14">
-      <c r="B34" s="96"/>
-      <c r="C34" s="108">
-        <v>435600</v>
-      </c>
-      <c r="D34" s="99" t="s">
-        <v>119</v>
-      </c>
-      <c r="E34" s="99" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="99"/>
-      <c r="G34" s="99"/>
-      <c r="H34" s="99">
-        <v>1</v>
-      </c>
-      <c r="I34" s="99">
-        <v>0</v>
-      </c>
-      <c r="J34" s="99">
-        <v>0</v>
-      </c>
-      <c r="K34" s="99">
-        <v>0</v>
-      </c>
-      <c r="L34" s="99">
-        <v>6</v>
-      </c>
-      <c r="M34" s="99">
-        <v>0</v>
-      </c>
-      <c r="N34" s="105">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="2:14">
-      <c r="B35" s="96"/>
-      <c r="C35" s="108">
-        <v>432261</v>
-      </c>
-      <c r="D35" s="99" t="s">
-        <v>119</v>
-      </c>
-      <c r="E35" s="99" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="99" t="s">
-        <v>180</v>
-      </c>
-      <c r="G35" s="99"/>
-      <c r="H35" s="99">
-        <v>3</v>
-      </c>
-      <c r="I35" s="99">
-        <v>0</v>
-      </c>
-      <c r="J35" s="99">
-        <v>3</v>
-      </c>
-      <c r="K35" s="99">
-        <v>0</v>
-      </c>
-      <c r="L35" s="99">
-        <v>0</v>
-      </c>
-      <c r="M35" s="99">
-        <v>0</v>
-      </c>
-      <c r="N35" s="105">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="2:14">
-      <c r="B36" s="92"/>
+      <c r="G35" s="87"/>
+      <c r="H35" s="87">
+        <v>0</v>
+      </c>
+      <c r="I35" s="87">
+        <v>0</v>
+      </c>
+      <c r="J35" s="87">
+        <v>0</v>
+      </c>
+      <c r="K35" s="87">
+        <v>0</v>
+      </c>
+      <c r="L35" s="87">
+        <v>0</v>
+      </c>
+      <c r="M35" s="87">
+        <v>0</v>
+      </c>
+      <c r="N35" s="9">
+        <f>SUM(H35:M35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14" ht="14.45">
+      <c r="B36" s="83"/>
       <c r="C36" s="11">
         <v>434801</v>
       </c>
@@ -10115,13 +10117,13 @@
       <c r="M36" s="9">
         <v>0</v>
       </c>
-      <c r="N36" s="106">
-        <f t="shared" si="0"/>
+      <c r="N36" s="87">
+        <f>SUM(H36:M36)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="2:14">
-      <c r="B37" s="92"/>
+    <row r="37" spans="2:14" ht="14.45">
+      <c r="B37" s="83"/>
       <c r="C37" s="11">
         <v>436116</v>
       </c>
@@ -10132,7 +10134,7 @@
         <v>12</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G37" s="9"/>
       <c r="H37" s="9">
@@ -10151,15 +10153,15 @@
         <v>2</v>
       </c>
       <c r="M37" s="9">
-        <v>2</v>
-      </c>
-      <c r="N37" s="106">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" spans="2:14">
-      <c r="B38" s="92"/>
+        <v>1</v>
+      </c>
+      <c r="N37" s="87">
+        <f>SUM(H37:M37)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14" ht="14.45">
+      <c r="B38" s="83"/>
       <c r="C38" s="11">
         <v>434861</v>
       </c>
@@ -10191,13 +10193,13 @@
       <c r="M38" s="9">
         <v>2</v>
       </c>
-      <c r="N38" s="106">
-        <f t="shared" si="0"/>
+      <c r="N38" s="87">
+        <f>SUM(H38:M38)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="2:14">
-      <c r="B39" s="92"/>
+    <row r="39" spans="2:14" ht="14.45">
+      <c r="B39" s="83"/>
       <c r="C39" s="11">
         <v>431900</v>
       </c>
@@ -10212,10 +10214,10 @@
         <v>165</v>
       </c>
       <c r="H39" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
@@ -10224,18 +10226,18 @@
         <v>0</v>
       </c>
       <c r="L39" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M39" s="9">
         <v>0</v>
       </c>
-      <c r="N39" s="106">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="2:14">
-      <c r="B40" s="92"/>
+      <c r="N39" s="87">
+        <f>SUM(H39:M39)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" ht="14.45">
+      <c r="B40" s="83"/>
       <c r="C40" s="11">
         <v>436168</v>
       </c>
@@ -10246,7 +10248,7 @@
         <v>12</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G40" s="9"/>
       <c r="H40" s="9">
@@ -10267,13 +10269,13 @@
       <c r="M40" s="9">
         <v>0</v>
       </c>
-      <c r="N40" s="106">
-        <f t="shared" si="0"/>
+      <c r="N40" s="87">
+        <f>SUM(H40:M40)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="2:14">
-      <c r="B41" s="92"/>
+    <row r="41" spans="2:14" ht="14.45">
+      <c r="B41" s="83"/>
       <c r="C41" s="11">
         <v>434800</v>
       </c>
@@ -10305,13 +10307,13 @@
       <c r="M41" s="9">
         <v>0</v>
       </c>
-      <c r="N41" s="106">
-        <f t="shared" si="0"/>
+      <c r="N41" s="87">
+        <f>SUM(H41:M41)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="2:14">
-      <c r="B42" s="92"/>
+    <row r="42" spans="2:14" ht="14.45">
+      <c r="B42" s="83"/>
       <c r="C42" s="11">
         <v>432202</v>
       </c>
@@ -10343,174 +10345,174 @@
       <c r="M42" s="9">
         <v>0</v>
       </c>
-      <c r="N42" s="106">
-        <f t="shared" si="0"/>
+      <c r="N42" s="87">
+        <f>SUM(H42:M42)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="2:14">
+    <row r="43" spans="2:14" ht="14.45">
       <c r="C43" s="24"/>
       <c r="M43" t="s">
         <v>5</v>
       </c>
       <c r="N43" s="14">
         <f>SUM(N4:N42)</f>
-        <v>1336</v>
-      </c>
-    </row>
-    <row r="44" spans="2:14">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14" ht="14.45">
       <c r="C44" s="24"/>
     </row>
-    <row r="45" spans="2:14">
+    <row r="45" spans="2:14" ht="14.45">
       <c r="C45" s="24"/>
     </row>
-    <row r="46" spans="2:14">
+    <row r="46" spans="2:14" ht="14.45">
       <c r="C46" s="24"/>
     </row>
-    <row r="47" spans="2:14">
+    <row r="47" spans="2:14" ht="14.45">
       <c r="C47" s="24"/>
     </row>
-    <row r="48" spans="2:14">
+    <row r="48" spans="2:14" ht="14.45">
       <c r="C48" s="24"/>
     </row>
-    <row r="49" spans="3:3">
+    <row r="49" spans="3:3" ht="14.45">
       <c r="C49" s="24"/>
     </row>
-    <row r="50" spans="3:3">
+    <row r="50" spans="3:3" ht="14.45">
       <c r="C50" s="24"/>
     </row>
-    <row r="51" spans="3:3">
+    <row r="51" spans="3:3" ht="14.45">
       <c r="C51" s="24"/>
     </row>
-    <row r="52" spans="3:3">
+    <row r="52" spans="3:3" ht="14.45">
       <c r="C52" s="24"/>
     </row>
-    <row r="53" spans="3:3">
+    <row r="53" spans="3:3" ht="14.45">
       <c r="C53" s="24"/>
     </row>
-    <row r="54" spans="3:3">
+    <row r="54" spans="3:3" ht="14.45">
       <c r="C54" s="24"/>
     </row>
-    <row r="55" spans="3:3">
+    <row r="55" spans="3:3" ht="14.45">
       <c r="C55" s="24"/>
     </row>
-    <row r="56" spans="3:3">
+    <row r="56" spans="3:3" ht="14.45">
       <c r="C56" s="24"/>
     </row>
-    <row r="57" spans="3:3">
+    <row r="57" spans="3:3" ht="14.45">
       <c r="C57" s="24"/>
     </row>
-    <row r="58" spans="3:3">
+    <row r="58" spans="3:3" ht="14.45">
       <c r="C58" s="24"/>
     </row>
-    <row r="59" spans="3:3">
+    <row r="59" spans="3:3" ht="14.45">
       <c r="C59" s="24"/>
     </row>
-    <row r="60" spans="3:3">
+    <row r="60" spans="3:3" ht="14.45">
       <c r="C60" s="24"/>
     </row>
-    <row r="61" spans="3:3">
+    <row r="61" spans="3:3" ht="14.45">
       <c r="C61" s="24"/>
     </row>
-    <row r="62" spans="3:3">
+    <row r="62" spans="3:3" ht="14.45">
       <c r="C62" s="24"/>
     </row>
-    <row r="63" spans="3:3">
+    <row r="63" spans="3:3" ht="14.45">
       <c r="C63" s="24"/>
     </row>
-    <row r="64" spans="3:3">
+    <row r="64" spans="3:3" ht="14.45">
       <c r="C64" s="24"/>
     </row>
-    <row r="65" spans="3:3">
+    <row r="65" spans="3:3" ht="14.45">
       <c r="C65" s="24"/>
     </row>
-    <row r="66" spans="3:3">
+    <row r="66" spans="3:3" ht="14.45">
       <c r="C66" s="24"/>
     </row>
-    <row r="67" spans="3:3">
+    <row r="67" spans="3:3" ht="14.45">
       <c r="C67" s="24"/>
     </row>
-    <row r="68" spans="3:3">
+    <row r="68" spans="3:3" ht="14.45">
       <c r="C68" s="24"/>
     </row>
-    <row r="69" spans="3:3">
+    <row r="69" spans="3:3" ht="14.45">
       <c r="C69" s="24"/>
     </row>
-    <row r="70" spans="3:3">
+    <row r="70" spans="3:3" ht="14.45">
       <c r="C70" s="24"/>
     </row>
-    <row r="71" spans="3:3">
+    <row r="71" spans="3:3" ht="14.45">
       <c r="C71" s="24"/>
     </row>
-    <row r="72" spans="3:3">
+    <row r="72" spans="3:3" ht="14.45">
       <c r="C72" s="24"/>
     </row>
-    <row r="73" spans="3:3">
+    <row r="73" spans="3:3" ht="14.45">
       <c r="C73" s="24"/>
     </row>
-    <row r="74" spans="3:3">
+    <row r="74" spans="3:3" ht="14.45">
       <c r="C74" s="24"/>
     </row>
-    <row r="75" spans="3:3">
+    <row r="75" spans="3:3" ht="14.45">
       <c r="C75" s="24"/>
     </row>
-    <row r="76" spans="3:3">
+    <row r="76" spans="3:3" ht="14.45">
       <c r="C76" s="24"/>
     </row>
-    <row r="77" spans="3:3">
+    <row r="77" spans="3:3" ht="14.45">
       <c r="C77" s="24"/>
     </row>
-    <row r="78" spans="3:3">
+    <row r="78" spans="3:3" ht="14.45">
       <c r="C78" s="24"/>
     </row>
-    <row r="79" spans="3:3">
+    <row r="79" spans="3:3" ht="14.45">
       <c r="C79" s="24"/>
     </row>
-    <row r="80" spans="3:3">
+    <row r="80" spans="3:3" ht="14.45">
       <c r="C80" s="24"/>
     </row>
-    <row r="81" spans="3:3">
+    <row r="81" spans="3:3" ht="14.45">
       <c r="C81" s="24"/>
     </row>
-    <row r="82" spans="3:3">
+    <row r="82" spans="3:3" ht="14.45">
       <c r="C82" s="24"/>
     </row>
-    <row r="83" spans="3:3">
+    <row r="83" spans="3:3" ht="14.45">
       <c r="C83" s="24"/>
     </row>
-    <row r="84" spans="3:3">
+    <row r="84" spans="3:3" ht="14.45">
       <c r="C84" s="24"/>
     </row>
-    <row r="85" spans="3:3">
+    <row r="85" spans="3:3" ht="14.45">
       <c r="C85" s="24"/>
     </row>
-    <row r="86" spans="3:3">
+    <row r="86" spans="3:3" ht="14.45">
       <c r="C86" s="24"/>
     </row>
-    <row r="87" spans="3:3">
+    <row r="87" spans="3:3" ht="14.45">
       <c r="C87" s="24"/>
     </row>
-    <row r="88" spans="3:3">
+    <row r="88" spans="3:3" ht="14.45">
       <c r="C88" s="24"/>
     </row>
-    <row r="89" spans="3:3">
+    <row r="89" spans="3:3" ht="14.45">
       <c r="C89" s="24"/>
     </row>
-    <row r="90" spans="3:3">
+    <row r="90" spans="3:3" ht="14.45">
       <c r="C90" s="24"/>
     </row>
-    <row r="91" spans="3:3">
+    <row r="91" spans="3:3" ht="14.45">
       <c r="C91" s="24"/>
     </row>
-    <row r="92" spans="3:3"/>
-    <row r="93" spans="3:3"/>
-    <row r="94" spans="3:3"/>
-    <row r="95" spans="3:3"/>
-    <row r="96" spans="3:3"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
+    <row r="92" spans="3:3" ht="14.45"/>
+    <row r="93" spans="3:3" ht="14.45"/>
+    <row r="94" spans="3:3" ht="14.45"/>
+    <row r="95" spans="3:3" ht="14.45"/>
+    <row r="96" spans="3:3" ht="14.45"/>
+    <row r="97" ht="14.45"/>
+    <row r="98" ht="14.45"/>
+    <row r="99" ht="14.45"/>
+    <row r="100" ht="14.45"/>
   </sheetData>
   <autoFilter ref="C3:N17" xr:uid="{B5734B30-2D58-4B23-A8DD-CE4A8B965AA0}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:N17">
@@ -10527,13 +10529,12 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD0FCA9-A906-4FEF-9843-D37FAC686B1F}">
-  <dimension ref="B1:N72"/>
+  <dimension ref="B1:N74"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="7"/>
     <col min="3" max="3" width="11.5703125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="7.140625" customWidth="1"/>
@@ -10552,16 +10553,16 @@
     </row>
     <row r="3" spans="2:14" ht="18.600000000000001">
       <c r="B3"/>
-      <c r="D3" s="84" t="s">
-        <v>183</v>
-      </c>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="86"/>
+      <c r="D3" s="102" t="s">
+        <v>182</v>
+      </c>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="104"/>
     </row>
     <row r="4" spans="2:14">
       <c r="B4"/>
@@ -10603,7 +10604,7 @@
       </c>
     </row>
     <row r="5" spans="2:14">
-      <c r="B5" s="83"/>
+      <c r="B5" s="101"/>
       <c r="C5" s="23">
         <v>444800</v>
       </c>
@@ -10614,116 +10615,116 @@
         <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>165</v>
       </c>
       <c r="H5" s="78">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="I5" s="78">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="J5" s="78">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="K5" s="78">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="L5" s="78">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="M5" s="80">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="N5" s="73">
-        <f>SUM(H5:M5)</f>
-        <v>709</v>
+        <f t="shared" ref="N5:N10" si="0">SUM(H5:M5)</f>
+        <v>585</v>
       </c>
     </row>
     <row r="6" spans="2:14">
-      <c r="B6" s="83"/>
+      <c r="B6" s="101"/>
       <c r="C6" s="23">
-        <v>443000</v>
+        <v>445500</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="H6" s="78">
-        <v>28</v>
-      </c>
-      <c r="I6" s="78">
+        <v>169</v>
+      </c>
+      <c r="H6" s="4">
+        <v>29</v>
+      </c>
+      <c r="I6" s="4">
+        <v>52</v>
+      </c>
+      <c r="J6" s="4">
+        <v>62</v>
+      </c>
+      <c r="K6" s="4">
+        <v>58</v>
+      </c>
+      <c r="L6" s="4">
         <v>40</v>
       </c>
-      <c r="J6" s="78">
-        <v>60</v>
-      </c>
-      <c r="K6" s="78">
-        <v>65</v>
-      </c>
-      <c r="L6" s="78">
-        <v>64</v>
-      </c>
-      <c r="M6" s="80">
-        <v>47</v>
+      <c r="M6" s="79">
+        <v>34</v>
       </c>
       <c r="N6" s="73">
         <f>SUM(H6:M6)</f>
-        <v>304</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="2:14">
-      <c r="B7" s="83"/>
+      <c r="B7" s="101"/>
       <c r="C7" s="23">
-        <v>445500</v>
+        <v>443000</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>184</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="H7" s="4">
-        <v>31</v>
-      </c>
-      <c r="I7" s="4">
-        <v>56</v>
-      </c>
-      <c r="J7" s="4">
-        <v>65</v>
-      </c>
-      <c r="K7" s="4">
-        <v>62</v>
-      </c>
-      <c r="L7" s="4">
-        <v>42</v>
-      </c>
-      <c r="M7" s="79">
+        <v>165</v>
+      </c>
+      <c r="H7" s="78">
+        <v>3</v>
+      </c>
+      <c r="I7" s="78">
+        <v>4</v>
+      </c>
+      <c r="J7" s="78">
+        <v>21</v>
+      </c>
+      <c r="K7" s="78">
+        <v>29</v>
+      </c>
+      <c r="L7" s="78">
+        <v>46</v>
+      </c>
+      <c r="M7" s="80">
         <v>35</v>
       </c>
       <c r="N7" s="73">
-        <f>SUM(H7:M7)</f>
-        <v>291</v>
+        <f t="shared" si="0"/>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="2:14">
-      <c r="B8" s="83"/>
+      <c r="B8" s="98"/>
       <c r="C8" s="23">
         <v>441800</v>
       </c>
@@ -10734,36 +10735,36 @@
         <v>29</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>169</v>
       </c>
       <c r="H8" s="78">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I8" s="78">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="J8" s="78">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="K8" s="78">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="L8" s="78">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="M8" s="80">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="N8" s="73">
-        <f>SUM(H8:M8)</f>
-        <v>268</v>
+        <f t="shared" si="0"/>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="2:14">
-      <c r="B9" s="83"/>
+      <c r="B9" s="101"/>
       <c r="C9" s="23">
         <v>448400</v>
       </c>
@@ -10774,34 +10775,34 @@
         <v>12</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="78">
         <v>5</v>
       </c>
       <c r="I9" s="78">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J9" s="78">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="K9" s="78">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L9" s="78">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="M9" s="80">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N9" s="73">
-        <f>SUM(H9:M9)</f>
-        <v>193</v>
+        <f t="shared" si="0"/>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="2:14">
-      <c r="B10" s="73"/>
+      <c r="B10" s="99"/>
       <c r="C10" s="23">
         <v>447900</v>
       </c>
@@ -10812,7 +10813,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>169</v>
@@ -10821,23 +10822,23 @@
         <v>0</v>
       </c>
       <c r="I10" s="78">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J10" s="78">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="K10" s="78">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="L10" s="78">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="M10" s="80">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="N10" s="73">
-        <f>SUM(H10:M10)</f>
-        <v>178</v>
+        <f t="shared" si="0"/>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="2:14">
@@ -10853,33 +10854,33 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H11" s="78">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I11" s="78">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="J11" s="78">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="K11" s="78">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="L11" s="78">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="M11" s="80">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="N11" s="73">
-        <f t="shared" ref="N11:N12" si="0">SUM(H11:M11)</f>
-        <v>167</v>
+        <f t="shared" ref="N11:N12" si="1">SUM(H11:M11)</f>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="2:14">
-      <c r="B12" s="82"/>
+      <c r="B12" s="99"/>
       <c r="C12" s="23">
         <v>447600</v>
       </c>
@@ -10894,30 +10895,30 @@
         <v>165</v>
       </c>
       <c r="H12" s="78">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I12" s="78">
+        <v>9</v>
+      </c>
+      <c r="J12" s="78">
+        <v>16</v>
+      </c>
+      <c r="K12" s="78">
+        <v>18</v>
+      </c>
+      <c r="L12" s="78">
+        <v>13</v>
+      </c>
+      <c r="M12" s="80">
         <v>28</v>
       </c>
-      <c r="J12" s="78">
-        <v>32</v>
-      </c>
-      <c r="K12" s="78">
-        <v>40</v>
-      </c>
-      <c r="L12" s="78">
-        <v>22</v>
-      </c>
-      <c r="M12" s="80">
-        <v>35</v>
-      </c>
       <c r="N12" s="73">
-        <f t="shared" si="0"/>
-        <v>162</v>
+        <f t="shared" si="1"/>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="2:14">
-      <c r="B13" s="83"/>
+      <c r="B13" s="98"/>
       <c r="C13" s="23">
         <v>443101</v>
       </c>
@@ -10935,147 +10936,145 @@
         <v>0</v>
       </c>
       <c r="I13" s="78">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="J13" s="78">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K13" s="78">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="L13" s="78">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="M13" s="80">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="N13" s="73">
-        <f t="shared" ref="N13" si="1">SUM(H13:M13)</f>
-        <v>160</v>
+        <f t="shared" ref="N13" si="2">SUM(H13:M13)</f>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="2:14">
       <c r="B14" s="82"/>
       <c r="C14" s="23">
-        <v>445400</v>
+        <v>447400</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>184</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="H14" s="78">
+        <v>5</v>
+      </c>
+      <c r="I14" s="78">
+        <v>15</v>
+      </c>
+      <c r="J14" s="78">
+        <v>22</v>
+      </c>
+      <c r="K14" s="78">
+        <v>21</v>
+      </c>
+      <c r="L14" s="78">
+        <v>15</v>
+      </c>
+      <c r="M14" s="80">
         <v>8</v>
       </c>
-      <c r="I14" s="78">
-        <v>23</v>
-      </c>
-      <c r="J14" s="78">
-        <v>34</v>
-      </c>
-      <c r="K14" s="78">
-        <v>29</v>
-      </c>
-      <c r="L14" s="78">
-        <v>27</v>
-      </c>
-      <c r="M14" s="80">
-        <v>16</v>
-      </c>
       <c r="N14" s="73">
-        <f t="shared" ref="N14:N27" si="2">SUM(H14:M14)</f>
-        <v>137</v>
+        <f t="shared" ref="N14:N28" si="3">SUM(H14:M14)</f>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="2:14">
-      <c r="B15" s="82"/>
+      <c r="B15" s="99"/>
       <c r="C15" s="23">
-        <v>447400</v>
+        <v>443100</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="1"/>
+        <v>173</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>183</v>
+      </c>
       <c r="G15" s="1" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
       <c r="H15" s="78">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I15" s="78">
+        <v>12</v>
+      </c>
+      <c r="J15" s="78">
+        <v>17</v>
+      </c>
+      <c r="K15" s="78">
+        <v>16</v>
+      </c>
+      <c r="L15" s="78">
         <v>18</v>
       </c>
-      <c r="J15" s="78">
-        <v>25</v>
-      </c>
-      <c r="K15" s="78">
-        <v>24</v>
-      </c>
-      <c r="L15" s="78">
-        <v>17</v>
-      </c>
       <c r="M15" s="80">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="N15" s="73">
-        <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14">
+        <f t="shared" si="3"/>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" ht="15">
       <c r="B16" s="82"/>
       <c r="C16" s="23">
-        <v>443100</v>
+        <v>443400</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>119</v>
+        <v>15</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>184</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="H16" s="78">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I16" s="78">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J16" s="78">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="K16" s="78">
         <v>25</v>
       </c>
       <c r="L16" s="78">
+        <v>13</v>
+      </c>
+      <c r="M16" s="80">
         <v>4</v>
       </c>
-      <c r="M16" s="80">
-        <v>20</v>
-      </c>
       <c r="N16" s="73">
-        <f t="shared" si="2"/>
-        <v>99</v>
+        <f>SUM(H16:M16)</f>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="2:14">
-      <c r="B17" s="82"/>
+      <c r="B17" s="99"/>
       <c r="C17" s="23">
-        <v>447200</v>
+        <v>445400</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>119</v>
@@ -11083,85 +11082,87 @@
       <c r="E17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1" t="s">
+        <v>183</v>
+      </c>
       <c r="G17" s="1" t="s">
-        <v>187</v>
+        <v>165</v>
       </c>
       <c r="H17" s="78">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I17" s="78">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J17" s="78">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="K17" s="78">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L17" s="78">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="M17" s="80">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N17" s="73">
-        <f t="shared" si="2"/>
-        <v>37</v>
+        <f>SUM(H17:M17)</f>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="2:14">
       <c r="B18" s="82"/>
       <c r="C18" s="23">
-        <v>445300</v>
+        <v>447200</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H18" s="78">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I18" s="78">
         <v>0</v>
       </c>
-      <c r="J18" s="78">
-        <v>2</v>
+      <c r="J18" s="78" t="s">
+        <v>155</v>
       </c>
       <c r="K18" s="78">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L18" s="78">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M18" s="80">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="N18" s="73">
-        <f>SUM(H18:M18)</f>
-        <v>22</v>
+        <f t="shared" si="3"/>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:14">
       <c r="B19" s="82"/>
       <c r="C19" s="23">
-        <v>447201</v>
+        <v>445300</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H19" s="78">
         <v>0</v>
@@ -11170,39 +11171,39 @@
         <v>0</v>
       </c>
       <c r="J19" s="78">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" s="78">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L19" s="78">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M19" s="80">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N19" s="73">
-        <f t="shared" ref="N19:N21" si="3">SUM(H19:M19)</f>
-        <v>18</v>
+        <f t="shared" si="3"/>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="2:14">
       <c r="B20" s="82"/>
       <c r="C20" s="23">
-        <v>447300</v>
+        <v>447201</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>119</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>188</v>
+        <v>12</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="H20" s="78">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I20" s="78">
         <v>0</v>
@@ -11211,39 +11212,59 @@
         <v>0</v>
       </c>
       <c r="K20" s="78">
+        <v>1</v>
+      </c>
+      <c r="L20" s="78">
+        <v>5</v>
+      </c>
+      <c r="M20" s="80">
+        <v>12</v>
+      </c>
+      <c r="N20" s="73">
+        <f t="shared" ref="N20:N22" si="4">SUM(H20:M20)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14">
+      <c r="B21" s="82"/>
+      <c r="C21" s="23">
+        <v>447300</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H21" s="78">
+        <v>7</v>
+      </c>
+      <c r="I21" s="78">
+        <v>0</v>
+      </c>
+      <c r="J21" s="78">
+        <v>0</v>
+      </c>
+      <c r="K21" s="78">
         <v>2</v>
       </c>
-      <c r="L20" s="78">
+      <c r="L21" s="78">
         <v>4</v>
       </c>
-      <c r="M20" s="80">
-        <v>0</v>
-      </c>
-      <c r="N20" s="73">
-        <f t="shared" si="3"/>
+      <c r="M21" s="80">
+        <v>0</v>
+      </c>
+      <c r="N21" s="73">
+        <f t="shared" si="4"/>
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="2:14">
-      <c r="B21" s="49"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="78"/>
-      <c r="I21" s="78"/>
-      <c r="J21" s="78"/>
-      <c r="K21" s="78"/>
-      <c r="L21" s="78"/>
-      <c r="M21" s="80"/>
-      <c r="N21" s="73">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="2:14" hidden="1">
-      <c r="B22" s="72"/>
+    <row r="22" spans="2:14">
+      <c r="B22" s="49"/>
       <c r="C22" s="23"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -11256,12 +11277,12 @@
       <c r="L22" s="78"/>
       <c r="M22" s="80"/>
       <c r="N22" s="73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:14" hidden="1">
-      <c r="B23" s="49"/>
+      <c r="B23" s="72"/>
       <c r="C23" s="23"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -11274,7 +11295,7 @@
       <c r="L23" s="78"/>
       <c r="M23" s="80"/>
       <c r="N23" s="73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -11292,7 +11313,7 @@
       <c r="L24" s="78"/>
       <c r="M24" s="80"/>
       <c r="N24" s="73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -11309,8 +11330,8 @@
       <c r="K25" s="78"/>
       <c r="L25" s="78"/>
       <c r="M25" s="80"/>
-      <c r="N25" s="11">
-        <f t="shared" si="2"/>
+      <c r="N25" s="73">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -11327,13 +11348,13 @@
       <c r="K26" s="78"/>
       <c r="L26" s="78"/>
       <c r="M26" s="80"/>
-      <c r="N26" s="73">
-        <f t="shared" si="2"/>
+      <c r="N26" s="11">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:14" hidden="1">
-      <c r="B27" s="71"/>
+      <c r="B27" s="49"/>
       <c r="C27" s="23"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -11346,12 +11367,12 @@
       <c r="L27" s="78"/>
       <c r="M27" s="80"/>
       <c r="N27" s="73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:14" hidden="1">
-      <c r="B28" s="49"/>
+      <c r="B28" s="71"/>
       <c r="C28" s="23"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -11363,8 +11384,8 @@
       <c r="K28" s="78"/>
       <c r="L28" s="78"/>
       <c r="M28" s="80"/>
-      <c r="N28" s="11">
-        <f t="shared" ref="N28:N29" si="4">SUM(H28:M28)</f>
+      <c r="N28" s="73">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -11382,43 +11403,43 @@
       <c r="L29" s="78"/>
       <c r="M29" s="80"/>
       <c r="N29" s="11">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="N29:N30" si="5">SUM(H29:M29)</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="2:14" hidden="1">
-      <c r="B30" s="70"/>
+      <c r="B30" s="49"/>
       <c r="C30" s="23"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="81"/>
-      <c r="N30" s="73">
-        <f t="shared" ref="N30:N38" si="5">SUM(H30:M30)</f>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="78"/>
+      <c r="I30" s="78"/>
+      <c r="J30" s="78"/>
+      <c r="K30" s="78"/>
+      <c r="L30" s="78"/>
+      <c r="M30" s="80"/>
+      <c r="N30" s="11">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:14" hidden="1">
-      <c r="B31" s="49"/>
+      <c r="B31" s="70"/>
       <c r="C31" s="23"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="78"/>
-      <c r="I31" s="78"/>
-      <c r="J31" s="78"/>
-      <c r="K31" s="78"/>
-      <c r="L31" s="78"/>
-      <c r="M31" s="80"/>
-      <c r="N31" s="11">
-        <f t="shared" si="5"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="50"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="81"/>
+      <c r="N31" s="73">
+        <f t="shared" ref="N31:N39" si="6">SUM(H31:M31)</f>
         <v>0</v>
       </c>
     </row>
@@ -11436,12 +11457,12 @@
       <c r="L32" s="78"/>
       <c r="M32" s="80"/>
       <c r="N32" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="2:14" hidden="1">
-      <c r="B33" s="72"/>
+      <c r="B33" s="49"/>
       <c r="C33" s="23"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -11454,7 +11475,7 @@
       <c r="L33" s="78"/>
       <c r="M33" s="80"/>
       <c r="N33" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -11472,12 +11493,13 @@
       <c r="L34" s="78"/>
       <c r="M34" s="80"/>
       <c r="N34" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="2:14" hidden="1">
-      <c r="C35" s="6"/>
+      <c r="B35" s="72"/>
+      <c r="C35" s="23"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -11489,13 +11511,12 @@
       <c r="L35" s="78"/>
       <c r="M35" s="80"/>
       <c r="N35" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="2:14" hidden="1">
-      <c r="B36" s="70"/>
-      <c r="C36" s="23"/>
+      <c r="C36" s="6"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -11507,12 +11528,12 @@
       <c r="L36" s="78"/>
       <c r="M36" s="80"/>
       <c r="N36" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="2:14" hidden="1">
-      <c r="B37" s="49"/>
+      <c r="B37" s="70"/>
       <c r="C37" s="23"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -11525,7 +11546,7 @@
       <c r="L37" s="78"/>
       <c r="M37" s="80"/>
       <c r="N37" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -11543,28 +11564,42 @@
       <c r="L38" s="78"/>
       <c r="M38" s="80"/>
       <c r="N38" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="2:14" hidden="1">
-      <c r="B39"/>
-      <c r="C39" s="25"/>
-    </row>
-    <row r="40" spans="2:14">
+      <c r="B39" s="49"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
+      <c r="J39" s="78"/>
+      <c r="K39" s="78"/>
+      <c r="L39" s="78"/>
+      <c r="M39" s="80"/>
+      <c r="N39" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" hidden="1">
       <c r="B40"/>
       <c r="C40" s="25"/>
-      <c r="M40" t="s">
-        <v>5</v>
-      </c>
-      <c r="N40" s="14">
-        <f>SUM(N5:N39)</f>
-        <v>2858</v>
-      </c>
     </row>
     <row r="41" spans="2:14">
       <c r="B41"/>
       <c r="C41" s="25"/>
+      <c r="M41" t="s">
+        <v>5</v>
+      </c>
+      <c r="N41" s="14">
+        <f>SUM(N5:N40)</f>
+        <v>2086</v>
+      </c>
     </row>
     <row r="42" spans="2:14">
       <c r="B42"/>
@@ -11608,6 +11643,7 @@
     </row>
     <row r="52" spans="2:3">
       <c r="B52"/>
+      <c r="C52" s="25"/>
     </row>
     <row r="53" spans="2:3">
       <c r="B53"/>
@@ -11666,7 +11702,11 @@
     <row r="71" spans="2:2">
       <c r="B71"/>
     </row>
-    <row r="72" spans="2:2" ht="15"/>
+    <row r="72" spans="2:2">
+      <c r="B72"/>
+    </row>
+    <row r="73" spans="2:2" ht="15"/>
+    <row r="74" spans="2:2" ht="15"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:K3"/>
@@ -11691,6 +11731,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -11834,23 +11883,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
 </file>
</xml_diff>

<commit_message>
Mejoras visuales dashboard y Estado de Resultado detallado
- Dashboard: colores por sección (Pedidos/Produccion/Venta/Finanzas), badges íconos, sin línea separadora
- Ocultar header título y buscador, solo muestra badge fecha
- PVC: T44 por defecto, total Σ Diferencia dinámico, botón imprimir, hover legible
- Estado de Resultado: tabs Resumen/Por mes, tabla mensual con sub-cuentas colapsables
- Parser ER actualizado para capturar cuentas detalladas del CSV

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/INVENTARIO 01-04 COMPLETO.xlsx
+++ b/seed/INVENTARIO 01-04 COMPLETO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mohicanojeans-my.sharepoint.com/personal/controleinventarios_mohicanojeans_onmicrosoft_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7666" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE97BF9F-6776-40A3-9BE2-68698F20B12E}"/>
+  <xr:revisionPtr revIDLastSave="7766" documentId="8_{7153A978-015E-4100-A25B-FE4B86BBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45677B50-5048-47A2-AB33-F5B2D15D4E28}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" firstSheet="6" activeTab="6" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
+    <workbookView minimized="1" xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" firstSheet="6" activeTab="5" xr2:uid="{DFBB1149-B842-467A-B253-B2263D43B28E}"/>
   </bookViews>
   <sheets>
     <sheet name="cole 37" sheetId="2" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="199">
   <si>
     <t>INVENTARIO COLECCIÓN 37</t>
   </si>
@@ -459,6 +459,9 @@
     <t>bLUE</t>
   </si>
   <si>
+    <t>18-08-26</t>
+  </si>
+  <si>
     <t>MARENGO</t>
   </si>
   <si>
@@ -481,6 +484,9 @@
   </si>
   <si>
     <t>GRIS</t>
+  </si>
+  <si>
+    <t>18-08-2026</t>
   </si>
   <si>
     <t>OXIDADO</t>
@@ -1274,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1547,6 +1553,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -1957,16 +1964,16 @@
       <c r="B2" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="110"/>
-      <c r="L2" s="110"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
     </row>
     <row r="3" spans="2:12">
       <c r="B3" s="40" t="s">
@@ -2763,17 +2770,17 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="B3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C5">
         <f>'COLE 43'!N43</f>
@@ -2782,16 +2789,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="B6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C6">
         <f>'COLE 42 otoño'!L84</f>
-        <v>1646</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="B7" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C7">
         <f>'COLE 41 Alto v'!L21</f>
@@ -2800,7 +2807,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="B8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C8">
         <f>'COLE 40 prima'!L50</f>
@@ -2809,7 +2816,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="B9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C9">
         <f>cole39!L19</f>
@@ -2818,7 +2825,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="B10" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C10">
         <f>'cole 38'!L22</f>
@@ -2827,7 +2834,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="B11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C11">
         <f>'cole 37'!L34</f>
@@ -2837,11 +2844,11 @@
     <row r="12" spans="1:5">
       <c r="C12">
         <f>SUM(C5:C11)</f>
-        <v>4587</v>
+        <v>4158</v>
       </c>
       <c r="E12" s="100">
         <f>C12*20000</f>
-        <v>91740000</v>
+        <v>83160000</v>
       </c>
     </row>
   </sheetData>
@@ -3450,16 +3457,16 @@
       <c r="B3" s="109" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="113"/>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="42" t="s">
@@ -3834,16 +3841,16 @@
       <c r="B3" s="109" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="113"/>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" s="18" t="s">
@@ -5440,16 +5447,16 @@
       <c r="B3" s="109" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="113"/>
     </row>
     <row r="4" spans="2:14">
       <c r="B4" s="46" t="s">
@@ -6089,7 +6096,9 @@
       </c>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="8"/>
+      <c r="A5" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B5" s="11">
         <v>424900</v>
       </c>
@@ -6100,33 +6109,35 @@
         <v>29</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F5" s="10">
+        <v>8</v>
+      </c>
+      <c r="G5" s="10">
+        <v>12</v>
+      </c>
+      <c r="H5" s="11">
+        <v>12</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10">
+        <v>10</v>
+      </c>
+      <c r="K5" s="10">
+        <v>4</v>
+      </c>
+      <c r="L5" s="9">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="10">
-        <v>15</v>
-      </c>
-      <c r="G5" s="10">
-        <v>29</v>
-      </c>
-      <c r="H5" s="11">
-        <v>34</v>
-      </c>
-      <c r="I5" s="10">
-        <v>23</v>
-      </c>
-      <c r="J5" s="10">
-        <v>19</v>
-      </c>
-      <c r="K5" s="10">
-        <v>5</v>
-      </c>
-      <c r="L5" s="9">
-        <f t="shared" si="0"/>
-        <v>125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="8"/>
       <c r="B6" s="11">
         <v>423600</v>
       </c>
@@ -6137,34 +6148,36 @@
         <v>29</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F6" s="10">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G6" s="10">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H6" s="10">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="I6" s="10">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J6" s="10">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K6" s="10">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L6" s="9">
         <f t="shared" si="0"/>
-        <v>103</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:12">
-      <c r="A7" s="8"/>
-      <c r="B7" s="11">
+      <c r="A7" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="92">
         <v>423500</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -6174,33 +6187,35 @@
         <v>8</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F7" s="10">
         <v>9</v>
       </c>
       <c r="G7" s="10">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H7" s="10">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I7" s="10">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J7" s="10">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K7" s="10">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L7" s="9">
         <f t="shared" si="0"/>
-        <v>86</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="8"/>
+      <c r="A8" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B8" s="11">
         <v>420301</v>
       </c>
@@ -6211,10 +6226,10 @@
         <v>10</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F8" s="11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G8" s="11">
         <v>11</v>
@@ -6226,18 +6241,20 @@
         <v>21</v>
       </c>
       <c r="J8" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K8" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L8" s="9">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="8"/>
+      <c r="A9" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B9" s="11">
         <v>421000</v>
       </c>
@@ -6248,29 +6265,29 @@
         <v>20</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F9" s="11">
+        <v>0</v>
+      </c>
+      <c r="G9" s="11">
+        <v>10</v>
+      </c>
+      <c r="H9" s="11">
         <v>5</v>
       </c>
-      <c r="G9" s="11">
-        <v>15</v>
-      </c>
-      <c r="H9" s="11">
-        <v>15</v>
-      </c>
       <c r="I9" s="11">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J9" s="11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K9" s="11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L9" s="9">
         <f t="shared" si="0"/>
-        <v>70</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -6322,7 +6339,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F11" s="11">
         <v>6</v>
@@ -6348,8 +6365,10 @@
       </c>
     </row>
     <row r="12" spans="1:12">
-      <c r="A12" s="8"/>
-      <c r="B12" s="11">
+      <c r="A12" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="92">
         <v>422000</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -6359,32 +6378,35 @@
         <v>8</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F12" s="10">
         <v>32</v>
       </c>
       <c r="G12" s="10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H12" s="10">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I12" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J12" s="10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K12" s="10">
         <v>0</v>
       </c>
       <c r="L12" s="9">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" s="110" t="s">
+        <v>134</v>
+      </c>
       <c r="B13" s="11">
         <v>421400</v>
       </c>
@@ -6398,30 +6420,32 @@
         <v>61</v>
       </c>
       <c r="F13" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G13" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="10">
+        <v>0</v>
+      </c>
+      <c r="I13" s="10">
+        <v>0</v>
+      </c>
+      <c r="J13" s="10">
         <v>5</v>
       </c>
-      <c r="I13" s="10">
-        <v>5</v>
-      </c>
-      <c r="J13" s="10">
-        <v>10</v>
-      </c>
       <c r="K13" s="10">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L13" s="9">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:12">
-      <c r="A14" s="8"/>
+      <c r="A14" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B14" s="11">
         <v>424400</v>
       </c>
@@ -6432,19 +6456,19 @@
         <v>8</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F14" s="10">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G14" s="10">
         <v>10</v>
       </c>
       <c r="H14" s="10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I14" s="10">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J14" s="10">
         <v>0</v>
@@ -6454,11 +6478,13 @@
       </c>
       <c r="L14" s="9">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:12">
-      <c r="A15" s="8"/>
+      <c r="A15" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B15" s="11">
         <v>424600</v>
       </c>
@@ -6469,32 +6495,35 @@
         <v>10</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F15" s="10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G15" s="10">
         <v>0</v>
       </c>
       <c r="H15" s="10">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I15" s="10">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="J15" s="10">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K15" s="10">
         <v>0</v>
       </c>
       <c r="L15" s="9">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:12">
+      <c r="A16" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B16" s="11">
         <v>422101</v>
       </c>
@@ -6505,32 +6534,35 @@
         <v>8</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F16" s="10">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G16" s="10">
         <v>0</v>
       </c>
       <c r="H16" s="10">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I16" s="10">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J16" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K16" s="10">
         <v>0</v>
       </c>
       <c r="L16" s="9">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:12">
+      <c r="A17" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B17" s="11">
         <v>422701</v>
       </c>
@@ -6541,32 +6573,35 @@
         <v>22</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F17" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G17" s="10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H17" s="10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I17" s="10">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J17" s="10">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K17" s="10">
+        <v>10</v>
+      </c>
+      <c r="L17" s="9">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="L17" s="9">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
     </row>
     <row r="18" spans="1:12">
+      <c r="A18" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B18" s="11">
         <v>420160</v>
       </c>
@@ -6577,29 +6612,29 @@
         <v>8</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F18" s="10">
         <v>0</v>
       </c>
       <c r="G18" s="10">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H18" s="10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I18" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J18" s="10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K18" s="10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L18" s="9">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -6650,7 +6685,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F20" s="10">
         <v>35</v>
@@ -6676,7 +6711,9 @@
       </c>
     </row>
     <row r="21" spans="1:12">
-      <c r="A21" s="8"/>
+      <c r="A21" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="B21" s="11">
         <v>420100</v>
       </c>
@@ -6696,7 +6733,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="10">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="I21" s="10">
         <v>0</v>
@@ -6709,7 +6746,7 @@
       </c>
       <c r="L21" s="9">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -6724,7 +6761,7 @@
         <v>29</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F22" s="10">
         <v>7</v>
@@ -6761,7 +6798,7 @@
         <v>29</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F23" s="10">
         <v>7</v>
@@ -6798,7 +6835,7 @@
         <v>12</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F24" s="10">
         <v>1</v>
@@ -6834,7 +6871,7 @@
         <v>22</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F25" s="10">
         <v>1</v>
@@ -6860,6 +6897,9 @@
       </c>
     </row>
     <row r="26" spans="1:12">
+      <c r="A26" s="8" t="s">
+        <v>143</v>
+      </c>
       <c r="B26" s="11">
         <v>421801</v>
       </c>
@@ -6870,7 +6910,7 @@
         <v>12</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F26" s="10">
         <v>0</v>
@@ -6879,10 +6919,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I26" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J26" s="10">
         <v>11</v>
@@ -6892,7 +6932,7 @@
       </c>
       <c r="L26" s="9">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -6907,7 +6947,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F27" s="10">
         <v>2</v>
@@ -6981,7 +7021,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F29" s="10">
         <v>2</v>
@@ -7015,10 +7055,10 @@
         <v>7</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F30" s="10">
         <v>5</v>
@@ -7055,7 +7095,7 @@
         <v>12</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F31" s="10">
         <v>22</v>
@@ -7091,7 +7131,7 @@
         <v>10</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F32" s="10">
         <v>2</v>
@@ -7127,7 +7167,7 @@
         <v>8</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F33" s="10">
         <v>5</v>
@@ -7164,7 +7204,7 @@
         <v>12</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F34" s="11">
         <v>1</v>
@@ -7200,7 +7240,7 @@
         <v>20</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F35" s="10">
         <v>0</v>
@@ -7237,7 +7277,7 @@
         <v>12</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F36" s="10">
         <v>0</v>
@@ -7274,7 +7314,7 @@
         <v>22</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F37" s="10">
         <v>0</v>
@@ -7310,7 +7350,7 @@
         <v>10</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F38" s="10">
         <v>0</v>
@@ -7384,7 +7424,7 @@
         <v>20</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F40" s="10">
         <v>3</v>
@@ -7421,7 +7461,7 @@
         <v>22</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F41" s="10">
         <v>0</v>
@@ -7452,13 +7492,13 @@
         <v>422600</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F42" s="11">
         <v>3</v>
@@ -7494,7 +7534,7 @@
         <v>8</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F43" s="10">
         <v>0</v>
@@ -7913,7 +7953,7 @@
         <v>10</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F55" s="10">
         <v>0</v>
@@ -8054,7 +8094,7 @@
         <v>10</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F59" s="10">
         <v>0</v>
@@ -8091,7 +8131,7 @@
         <v>10</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F60" s="10">
         <v>2</v>
@@ -8162,7 +8202,7 @@
         <v>12</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F62" s="10">
         <v>0</v>
@@ -8199,7 +8239,7 @@
         <v>12</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F63" s="10">
         <v>0</v>
@@ -8363,7 +8403,7 @@
         <v>20</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F68" s="10">
         <v>0</v>
@@ -8646,7 +8686,7 @@
         <v>29</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F78" s="11"/>
       <c r="G78" s="11"/>
@@ -8714,7 +8754,7 @@
         <v>8</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F81" s="10"/>
       <c r="G81" s="10"/>
@@ -8729,29 +8769,29 @@
     </row>
     <row r="82" spans="2:14">
       <c r="E82" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="84" spans="2:14">
       <c r="L84" s="9">
         <f>SUM(L4:L83)</f>
-        <v>1646</v>
+        <v>1217</v>
       </c>
       <c r="N84" s="100"/>
     </row>
     <row r="91" spans="2:14">
       <c r="G91" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="92" spans="2:14">
       <c r="H92" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="132" spans="11:11">
       <c r="K132" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -8794,7 +8834,7 @@
     <row r="2" spans="1:14" ht="15" customHeight="1">
       <c r="B2"/>
       <c r="C2" s="102" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D2" s="103"/>
       <c r="E2" s="103"/>
@@ -8823,7 +8863,7 @@
         <v>4</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H3" s="3">
         <v>36</v>
@@ -8860,7 +8900,7 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H4" s="1">
         <v>8</v>
@@ -8894,11 +8934,11 @@
         <v>119</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H5" s="1">
         <v>10</v>
@@ -8932,13 +8972,13 @@
         <v>119</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H6" s="1">
         <v>9</v>
@@ -8965,7 +9005,7 @@
     </row>
     <row r="7" spans="1:14" ht="14.45">
       <c r="A7" s="75" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" s="83">
         <v>44</v>
@@ -8981,7 +9021,7 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
@@ -9019,10 +9059,10 @@
         <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
@@ -9060,10 +9100,10 @@
         <v>12</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
@@ -9135,11 +9175,11 @@
         <v>119</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
@@ -9177,7 +9217,7 @@
         <v>22</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1">
@@ -9216,7 +9256,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1">
@@ -9256,7 +9296,7 @@
       </c>
       <c r="F14" s="89"/>
       <c r="G14" s="89" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H14" s="89">
         <v>0</v>
@@ -9294,7 +9334,7 @@
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H15" s="9">
         <v>2</v>
@@ -9332,7 +9372,7 @@
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H16" s="9">
         <v>0</v>
@@ -9370,7 +9410,7 @@
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H17" s="9">
         <v>0</v>
@@ -9408,7 +9448,7 @@
       </c>
       <c r="F18" s="97"/>
       <c r="G18" s="97" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H18" s="97">
         <v>0</v>
@@ -9442,11 +9482,11 @@
         <v>119</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H19" s="9">
         <v>0</v>
@@ -9484,10 +9524,10 @@
         <v>8</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H20" s="9">
         <v>0</v>
@@ -9557,11 +9597,11 @@
         <v>119</v>
       </c>
       <c r="E22" s="91" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F22" s="91"/>
       <c r="G22" s="91" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H22" s="91">
         <v>2</v>
@@ -9598,7 +9638,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G23" s="9"/>
       <c r="H23" s="9">
@@ -9637,7 +9677,7 @@
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H24" s="9">
         <v>0</v>
@@ -9675,7 +9715,7 @@
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H25" s="9">
         <v>1</v>
@@ -9712,10 +9752,10 @@
         <v>22</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H26" s="9">
         <v>0</v>
@@ -9753,7 +9793,7 @@
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H27" s="9">
         <v>0</v>
@@ -9791,7 +9831,7 @@
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H28" s="9">
         <v>0</v>
@@ -9825,11 +9865,11 @@
         <v>119</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H29" s="9">
         <v>0</v>
@@ -9867,7 +9907,7 @@
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H30" s="9">
         <v>0</v>
@@ -9904,7 +9944,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G31" s="9"/>
       <c r="H31" s="9">
@@ -9943,7 +9983,7 @@
       </c>
       <c r="F32" s="87"/>
       <c r="G32" s="87" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H32" s="87">
         <v>3</v>
@@ -9980,10 +10020,10 @@
         <v>12</v>
       </c>
       <c r="F33" s="87" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G33" s="87" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H33" s="87">
         <v>0</v>
@@ -10056,7 +10096,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="87" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G35" s="87"/>
       <c r="H35" s="87">
@@ -10094,10 +10134,10 @@
         <v>8</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H36" s="9">
         <v>1</v>
@@ -10134,7 +10174,7 @@
         <v>12</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G37" s="9"/>
       <c r="H37" s="9">
@@ -10172,7 +10212,7 @@
         <v>8</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G38" s="9"/>
       <c r="H38" s="9">
@@ -10211,7 +10251,7 @@
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H39" s="9">
         <v>0</v>
@@ -10248,7 +10288,7 @@
         <v>12</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G40" s="9"/>
       <c r="H40" s="9">
@@ -10287,7 +10327,7 @@
       </c>
       <c r="F41" s="9"/>
       <c r="G41" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H41" s="9">
         <v>0</v>
@@ -10325,7 +10365,7 @@
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H42" s="9">
         <v>0</v>
@@ -10554,7 +10594,7 @@
     <row r="3" spans="2:14" ht="18.600000000000001">
       <c r="B3"/>
       <c r="D3" s="102" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E3" s="103"/>
       <c r="F3" s="103"/>
@@ -10579,7 +10619,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H4" s="3">
         <v>36</v>
@@ -10615,10 +10655,10 @@
         <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H5" s="78">
         <v>30</v>
@@ -10655,10 +10695,10 @@
         <v>29</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H6" s="4">
         <v>29</v>
@@ -10695,10 +10735,10 @@
         <v>12</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H7" s="78">
         <v>3</v>
@@ -10735,10 +10775,10 @@
         <v>29</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H8" s="78">
         <v>4</v>
@@ -10775,7 +10815,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="78">
@@ -10813,10 +10853,10 @@
         <v>12</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H10" s="78">
         <v>0</v>
@@ -10854,7 +10894,7 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H11" s="78">
         <v>7</v>
@@ -10892,29 +10932,29 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H12" s="78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I12" s="78">
         <v>9</v>
       </c>
       <c r="J12" s="78">
+        <v>14</v>
+      </c>
+      <c r="K12" s="78">
         <v>16</v>
       </c>
-      <c r="K12" s="78">
-        <v>18</v>
-      </c>
       <c r="L12" s="78">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M12" s="80">
         <v>28</v>
       </c>
       <c r="N12" s="73">
         <f t="shared" si="1"/>
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="2:14">
@@ -10926,11 +10966,11 @@
         <v>119</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H13" s="78">
         <v>0</v>
@@ -10968,16 +11008,16 @@
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H14" s="78">
         <v>5</v>
       </c>
       <c r="I14" s="78">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J14" s="78">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="K14" s="78">
         <v>21</v>
@@ -10990,7 +11030,7 @@
       </c>
       <c r="N14" s="73">
         <f t="shared" ref="N14:N28" si="3">SUM(H14:M14)</f>
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="2:14">
@@ -11002,13 +11042,13 @@
         <v>119</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H15" s="78">
         <v>2</v>
@@ -11017,20 +11057,20 @@
         <v>12</v>
       </c>
       <c r="J15" s="78">
+        <v>16</v>
+      </c>
+      <c r="K15" s="78">
+        <v>15</v>
+      </c>
+      <c r="L15" s="78">
         <v>17</v>
-      </c>
-      <c r="K15" s="78">
-        <v>16</v>
-      </c>
-      <c r="L15" s="78">
-        <v>18</v>
       </c>
       <c r="M15" s="80">
         <v>18</v>
       </c>
       <c r="N15" s="73">
         <f t="shared" si="3"/>
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="2:14" ht="15">
@@ -11046,7 +11086,7 @@
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H16" s="78">
         <v>11</v>
@@ -11083,32 +11123,32 @@
         <v>12</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H17" s="78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="78">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J17" s="78">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K17" s="78">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L17" s="78">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M17" s="80">
         <v>8</v>
       </c>
       <c r="N17" s="73">
         <f>SUM(H17:M17)</f>
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="2:14">
@@ -11124,7 +11164,7 @@
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H18" s="78">
         <v>13</v>
@@ -11133,7 +11173,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="78" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K18" s="78">
         <v>6</v>
@@ -11162,7 +11202,7 @@
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H19" s="78">
         <v>0</v>
@@ -11200,7 +11240,7 @@
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H20" s="78">
         <v>0</v>
@@ -11234,11 +11274,11 @@
         <v>119</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H21" s="78">
         <v>7</v>
@@ -11598,7 +11638,7 @@
       </c>
       <c r="N41" s="14">
         <f>SUM(N5:N40)</f>
-        <v>2086</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="42" spans="2:14">
@@ -11731,15 +11771,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074A930493430584FA0AAA82464888454" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a8d20479ec654229e6693fc7a42d8396">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87cd4242d2fb989be9a9d15ec31d7a56" ns3:_="">
     <xsd:import namespace="eee826e9-b1fc-4e67-86a4-7fdd0eb0488d"/>
@@ -11883,14 +11914,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F435606-CC94-4D7E-AC45-9A1C80658731}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5440EA7-5A09-4509-9BD3-E23F1F6F33D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3DF54EF-1C4E-4303-AAC9-B10BE11AC9B0}"/>
 </file>
</xml_diff>